<commit_message>
One-time adding zipped statements subdirectory
Easy transfer to Treasury workstation

Also updated master spreadsheet readme to have documentation on cleaning procedure outside of your typical removal of procedural passages with little economic meaning, UTF-8 encoding, and so on.
</commit_message>
<xml_diff>
--- a/fomcCommunication_master.xlsx
+++ b/fomcCommunication_master.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranlephu/Documents/github/fomc-communication/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6795C98-FEFA-464F-9D6F-B2F7DF797809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0BCF0BF-5CC4-A641-85C0-1CCE6608D5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="1" r:id="rId1"/>
     <sheet name="master" sheetId="3" r:id="rId2"/>
     <sheet name="statements" sheetId="2" r:id="rId3"/>
-    <sheet name="speeches" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1053" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="278">
   <si>
     <t>Explanation:</t>
   </si>
@@ -176,102 +175,12 @@
     <t>statement, press conference, chair speech, vice-chair speech</t>
   </si>
   <si>
-    <t>speech_date</t>
-  </si>
-  <si>
-    <t>speech_time</t>
-  </si>
-  <si>
     <t>fomc_meeting/[communication]_date</t>
   </si>
   <si>
     <t>FOMC meeting or general communication at time t, recorded as dd-mm-yy</t>
   </si>
   <si>
-    <t>speaker</t>
-  </si>
-  <si>
-    <t>The United States is currently confronting a set of forces pulling us in divergent directions. The rapid acceleration of computer and telecommunication technologies, can reasonably be expected to appreciably raise our productivity and standards of living in the twenty-first century certainly, and quite possibly in some of the remaining years of this century. In the short run, however, the fallout from rapidly changing technology has created a marked degree of uncertainty and insecurity among a significant segment of our work force. It should not be surprising to find that when the stock of plant and equipment with which most Americans have to interact in their day-by-day job routines is turning over rapidly, human skills are subject to obsolescence at a rate perhaps unprecedented in American history. Almost six years ago I stressed to this Association the dramatic trends toward an ever increasing conceptualization of our Gross Domestic Product, the substitution, in effect, of ideas for physical matter in the creation of economic value. This afternoon I should like to update and extend the implications of these extraordinary forces which are driving the American economy. The roots of increasing conceptualization of output lie deep in human history, but the pace of such substitution probably picked up in the early stages of the industrial revolution, when science and machines created new leverage for human energy. Nonetheless, even as recently as the middle of this century, the symbols of American economic strength were our output of such products as steel, motor vehicles, and heavy machineryâ€”items for which sizable proportions of production costs reflected the value of raw materials and the sheer manual labor required to manipulate them. Since then, trends towards conceptualization have focused today's views of economic leadership increasingly on downsized, smaller, less palpable evidence of output, requiring more technologically sophisticated labor input. Our radios used to be activated by large vacuum tubes; today we have elegantly designed pocket-sized transistors to perform the same functionâ€”but with the higher quality of sound and greater reliability that consumers now expect. Thin fiber optic cable has replaced huge tonnages of copper wire. Advances in architecture and engineering, as well as the development of lighter but stronger materials, now give us the same working space but in buildings with significantly less concrete, glass, and steel tonnage than was required in an earlier era. The process of conceptualization in output, seems to have accelerated in recent decades with the advent of the semiconductor, the microprocessor, the computer, and the satellite. These technologies have become especially significant since my visit in 1989. Under the circumstances, it has puzzled many of us that the growth of output as customarily measured has not evidenced a corresponding pickup. Of course, output may not be measured correctly. Indeed, the financial markets are suggesting that we increasingly expense items which should be capitalized and hence underestimate the growth of our GDP and productivity. But it also is possible that some of the frenetic pace of change is wheel spinningâ€”changing production inputs without increasing output â€”rather than real advances in productivity. A number of commentators, particularly Professor David of Stanford University, have suggested that much of the wheel spinning, if that is what it is, reflects the extended time it typically has taken to translate a major new technology into increased productivity and higher standards of living. It may be that the big increases in productivity growing out of the introduction of computers and communications equipment still lie ahead. Past innovations, such as the advent of electricity or the invention of the gasoline-powered motor required considerable infrastructure before their full potential could be realized. Electricity, when it substituted for steam power late last century, was applied to production processes suited to steam. Gravity was used to move goods vertically in the steam environment and that could not initially change with the advent of electric power. It was only when horizontal factories, newly designed for optimal use of electric power, began to dominate our industrial system many years after electricity's initial introduction, that productivity clearly accelerated. Similarly, it was only when modern highways and gasoline service stations became extensive that the lower cost of motor vehicle transportation became evident. It is possible that the computer-telecommunications revolution is too new to as yet fundamentally improve standards of living overall. Moreover, to be fully effective, innovations also require a considerable amount of human investment on the part of workers who have to deal with these devices on a day-to-day basis. On this score, I sense that we still may not have progressed very far, relative to potential. Compared to the facility with which the average citizen handles another complex deviceâ€”the automobileâ€”most workers and consumers still appear to possess only rudimentary skills when it comes to making computers do what is wanted of them. Mass acceptance and full exploitation of computer technologiesâ€”the analogue of what was accomplished in making cars that were affordable, standardized, and easily operatedâ€”probably still lie ahead. In the meantime, we have a situation in which there are some serious mismatches between the skills of workers and technologies that have changed considerably and still are advancing rapidly, and these mismatches are affecting pay differentials between the skilled and the unskilled. As conceptualization of output has moved apace, the relative economic value of intellectual skill has clearly increased. During the past fifteen years, for example, the earnings of college graduates have increased relative to those who are high school graduates, and, in turn, high school graduates have continued to open up their advantage over those who are high school dropouts. In fact, a significant minority of our labor force has experienced real wage decreases, and this development surely is one factor in the unease that is all too prevalent, as well as in the apparent stretching of the distribution of incomes in recent years. Exaggerating this income dispersing trend is the growing evidence of what is being called a "winner take all society" in which the best in any activity tends to take an increasingly larger share of a market. The best actors, the best basketball players, the best business innovators, earn far more than average. The reason is that the major advances in telecommunications technologies have allowed any skill a far wider market than a generation ago. New visual communications allows talent to offer their services throughout the world. Who wants second best when the best is available at nearly the same price? Who buys the records of the fourth or fifth best tenors in the world singing an aria from Don Giovanni? The few top performers take most of the market. A century ago, such performers could not readily compete outside their localized area. Fortunately, the rapidly changing technologies have engendered an increased degree of competitive intensity which may very well cap, and perhaps reverse, the trend toward winner-take- all and other forces increasing income dispersion. Once proud hi-tech firms are being upended by new technologies developed by upstarts. But even the latter are lately looking over their shoulders at other upstarts with still newer technologies. The outsized rewards to high skills induce others to emulate them, and hence staying at the top has become ever more precarious. More generally entrenched economic advantage is being increasingly challenged by a global competition which shows no signs of abating. In addition, we must be alert in coming years to the need to improve the skills and earning power of those who appear to be falling behind. In the long run, better child-rearing and better schools are essential. But in the shorter run, on-the-job training is a critical necessityâ€”to overcome the educational deficiencies of all too many of our young people, and to renew the skills of workers who have fallen behind the rapidly rising curve of technological change. It has become quite apparent that many firms have concluded that it makes more sense to invest in such training than to bid up wage scales in a zero-sum competition for the existing limited pool of well-qualified workers. As a bottom line, though, workers in many kinds of pursuits probably had better look forward to a lot of hard work acquiring and maintaining the skills needed to cope with a rapidly evolving economy. The notion that early education could be crafted to support the needs of one's lifework, is rapidly changing. Education is increasingly becoming a lifetime activity. Over time, as workers acquire new skills and as computer applications continue to become evermore user friendly, the present income mismatches should diminish. To be sure, the most visible force of recent change, the continuous downsizing of microprocessors, and hence computer and telecommunications equipment, may increasingly encounter physical limits. But almost as surely, new technologies, not now visible, will emerge. We can anticipate change to be pervasive and, if competitive forces are allowed free rein, and our fiscal problems resolved, we can expect ever higher living standards for all Americans. Will Americans adjust to a frenetic pace of change and allow it to happen? While we have in the past, and almost surely will in the future, it is important that we recognize that adjustment is not automatic. We have episodes in recent human history where, for example, pressures of change were not easily absorbed and people chose what appeared to be a greater degree of security rather than competitive challenge. Competitive forces, especially those driven by technological change, create uncertainty and dislodgment, but they also bring with them an enhanced quality of living and the increased economic abundance so necessary to confront the problems that exist in societies throughout the world.</t>
-  </si>
-  <si>
-    <t>Many of you may not know that Henry Cisneros is an alumnus of the Federal Reserve System Immediately before joining the President's cabinet, the Secretary served as the Deputy Chairman of the Board of Directors of the Dallas Federal Reserve Bank He was always generous with his time and expertise, and I am delighted to be able, in some small way, to reciprocate I probably do not have to convince this audience that housing plays a central role in the economy and, more important, in the life of every person in our country Although significant housing problems and challenges remain, the progress this nation has made during the past 50 years in expanding and improving our housing has been enormous Since World War II we have doubled the number of houses and apartments nationwide By almost all measures, housing quality has improved and overcrowding has diminished And the proportion of families and individuals who are home owners has risen from about half to nearly two-thirds But the housing progress has not come evenly over the years The housing sector of the economy has been both an accelerator and a brake for economic growth. Because housing construction is highly cyclical and particularly sensitive to credit conditions, its importance in the economy--and the attention we at the Federal Reserve devote to it--are greater than its typical 4 percent share of gross domestic product would suggest Financial innovations and regulatory changes of the past two decades have somewhat eased the burden placed on housing when monetary policy must be tightened to contain inflation "Disintermediation" is a word not often heard in the 1990s The proliferation of new mortgage instruments and the maturation of the secondary mortgage market have reduced the vulnerability of housing demand to interest rate variations and to regional differences in interest rates resulting from geographic mismatches in the demand for, and supply of, home mortgage credit But the housing finance system has not been trouble-free in recent years One stress point has been in lending for real estate acquisition, development, and construction Readily available credit during the mid- 1980s, combined with excessive optimism by developers, contributed to overbuilding, especially of income properties The overbuilding resulted in sharp cutbacks in real estate lending across the board toward the end of the decade During this period some undoubtedly worthy projects-- even single-family developments --were denied credit The credit crunch served as a reminder of the burden placed on housing by boom-and-bust cycles Large swings in the pace of activity cause both inefficiencies in production and disruptions in consumers' planning One positive result from that difficult episode, born of necessity, was that developers broadened their base of financing by seeking out new credit sources and exploring new ways of funding their projects and operations This broadened base should help provide some added stability to real estate development in the future Despite the whole array of improvements in our system of mortgage finance, housing continues to play a disproportionate role in the ups and downs of our economy For instance, as the nation came out of the recession at the beginning of this decade, housing accounted directly for nearly one-fifth of the total growth in output during the subsequent two years, a share not much different from the average of previous recoveries Given the long-term nature of a housing commitment and the heavy use of credit, housing remains a sector more dependent than most on financial markets and consumer confidence, two determinants that can change quickly To be sure, the past three years have been good ones for housing Starts exceeded 1-1/4 million each year Single-family construction--most of which is destined for owner-occupancy--was particularly strong and accounted for an unusually large share of all starts, as the multifamily sector continued to work off the excess supply built up during the 1980s Indeed, all of the key indicators of the new home market-- starts, permits, and sales--have been running above their averages for the 1980s The existing home market also has been quite healthy overall, although the story varies some by region It is no coincidence that this good time for housing has come when inflation has been moderate and income growth has been reasonably steady These are precisely the conditions that promote housing affordabality, consumer confidence, and healthy lending institutions Expectations of subdued inflation have held the speculative component of housing demand in check and have contained the inflationary premiums required by mortgage lenders One result is that the proportion of its monthly income that the typical household must devote to mortgage payments on a new house is now the lowest in more than twenty years And the steady expansion of the economy has given consumers the confidence they need to be willing to make the long-term commitment typically involved in home purchase Along with the housing production gains of the past three years has come an increase in the rate of homeownership The proportion of all households that own their home, at 65 1 percent late last year, is the highest since the early 1980s More than economics comes into play in interpreting the prevalence and changes in homeownership Surveys have repeatedly found that most Americans aspire to homeownership as a value in itself Homeownership undoubtedly means different things to different people. For many, it probably means more space For others, it means more amenities For perhaps most, the "pride of ownership" often brings with it a sense of financial security, residential stability, and community status While this aspiration underlies the market, economics and demography drive changes in the ownership rate As you know, the ownership rate dipped during the 1980s, after four decades of gradual increase The first reason for the reversal was that consumers were less able to buy Income growth lagged, and interest rates remained high throughout the first half of the decade even after coming down from the peaks in 1980 and 1981 Housing was far less affordable, requiring a bigger commitment of household income Confidence was down as well Furthermore, households had less financial reason to buy Smaller gains m house prices and absolute declines in some major markets greatly diminished the investment return from owner-occupied housing In addition to the improvement m the economic conditions for home purchase in the past few years, demography-- specifically the aging of the population--also has given a boost to the single-family market As the baby boomers mature, they anticipate fewer future changes in their jobs, marital status, and family size This expected stability makes the selection of owner - occupied housing, with its substantial transactions costs, more appropriate It is worth noting, however, that despite some recent gains, the ownership rate among younger adults remains below that of their parents, when they were young adults Houses remain the single most important store of wealth for much of the population Consumers view their home equity as a cushion against possible hard times And many consumers also tap their home equity directly for various purposes, including home improvements, auto purchases, college tuition, and debt consolidation Home equity lines of credit, rare just ten years ago, are now held by roughly 5 million homeowners Even as we work to expand opportunities for homeownership, we need to keep renters in mind, recognizing that they, too, are full partners in our communities Our population is diverse Owning is not the right choice for everyone Someone anticipating a move in the near term or a big change in income--in either direction--probably is well advised to avoid the transactions costs of buying and selling And owning does involve financial risks Housing does not appreciate in all places at all times, the risks of capital loss are real While owning affords stability m some respects, renting offers flexibility, freedom of movement to new job or personal opportunities, and less of a responsibility for monitoring and maintaining the physical plant Indeed, the Partnership's action plan extends beyond promoting homeownership Many of the specifics are intended to expand housing opportunities for both owners and renters, One recurring theme among the 100 specific actions to which you have committed is to take advantage of technological advances Electronic technology clearly has improved the operation of the mortgage market, enabling the faster flow of more information at much lower cost than in a paper-based industry Technology has changed the underwriting, originating, and servicing of mortgages and has enabled more efficient pricing of a wider variety of mortgage products tailored for increasingly specialized segments of the market Of particular note, technology has aided the measurement and pricing of risk on low-downpayment loans to first-time homebuyers and in this tangible way has broadened the potential market for homeownership The full and timely flow of information is critical to all participants in this market, and the Partnership's emphasis on this strategy is well-placed Buying a house and taking out a mortgage is complicated and often intimidating to consumers, especially those of limited means At the Federal Reserve, through our regional Reserve Banks, working with community groups, we have long attempted to provide information on the process of home buying and mortgage borrowing Since 1990, the Federal Reserve has sponsored or co-sponsored more than 600 conferences, seminars, and informational meetings on affordable housing, fair lending, and related community- development In our own attempt to improve understanding through technology, last year the Board produced and broadcast teleseminars on the basics of homeownership to first-time homebuyers across the country Today, the information contained in those live broadcasts is available in videotape format to potential homebuyers, financial institutions, and civic and nonprofit groups And the Atlanta Fed recently developed a software product, called "Partners," that helps bankers determine borrower loan eligibility and pursue creative techniques for qualifying low- and moderate-income borrowers More than 30,000 copies of the software have been distributed nationwide, and the program recently became available on the Internet These efforts, together with the wide range of initiatives of almost all other participants in the mortgage and housing industries, appear to be bearing fruit In 1994, the latest full year for which statistics from the Home Mortgage Disclosure Act data are available, originations of conventional home purchase loans to lower income households expanded at more than twice the rate of lending to higher income households Anecdotal information suggests that these gains have continued The most far-reaching and lasting way in which the Fed can promote expansion of housing opportunities is by doing what we can to provide a stable platform for economic growth As I have mentioned, neither inflation nor boom and bust cycles are friends of housing Steady, sustainable growth in economic output, and thus incomes, provides consumers with the economic means and confidence required for the long-term decisions inherent in housing choices Under any conceivable scenario, the housing sector will continue to be critical to the overall performance of the economy Population projections have been revised upward in recent years By most estimates, Generation X, augmented by a continuing flow of immigrants, should keep the demographic component of housing demand growing about as rapidly during the next several years as it has since 1980 This impetus is important, because over the long run the number of housing units built depends more on demographics than on financial markets, even though interest rates certainly can and do affect the short-run timing of housing construction Among the important issues facing our nation, deficit reduction has particularly significant implications for housing In the past year, long-term interest rates have moved down as the outlook for deficit reduction have improved and have fluctuated with the ebbs and flows of the budget negotiations The stakes for housing--and for long- term growth of our economy--are high Our economic prospects in coming years will hinge on our ability to increase national saving and to ensure that such saving is invested wisely Making a serious commitment to balancing the budget within the foreseeable future is an essential first step--but only a first step Making good on our commitment by resisting the temptation to depart from that path will be a significant challenge. Budgets of governments at all levels --federal, state and local--seem certain to be under pressure for years to come Thus, approaches such as the National Homeownership Strategy, with its emphasis on voluntary cooperation among the private, public, and community sectors, are particularly timely As professionals in the housing and mortgage industries, you know how best to cut costs of production and financing, how best to open markets by reducing regulatory and discriminatory barriers, and how best to expand opportunities through education, information, and technology I applaud and encourage your efforts</t>
-  </si>
-  <si>
-    <t>I appreciate the opportunity to appear before this Committee to present the Federal Reserve's semiannual report on monetary policy The United States economy performed reasonably well in 1995 One-and-three-quarter million new jobs were added to payrolls over the year, and the unemployment rate was at the lowest sustained level in five years Despite the relatively high level of resource utilization, inflation remained well contained, with the consumer price index rising less than 3 percent--the fifth year running at 3 percent or below A reduction in inflation expectations, together with anticipation of significant progress toward eliminating federal budget deficits, was reflected in financial markets, where long-term interest rates dropped sharply and stock prices rose dramatically over the year This outcome was influenced in part by monetary policy actions taken by the Federal Reserve in recent years Responding to evidence that inflationary pressures were building, we progressively raised short-term interest rates over 1994 and early 1995 Rates had been purposely held at quite low, stimulative levels in 1993 We moved in 1994 to levels more consistent with sustainable growth Our intent was to be preemptive--to head off an incipient increase in inflationary pressures and to forestall the emergence of imbalances that so often in the past have undermined economic expansions As we entered the spring of 1995, it became increasingly evident that our policy was likely to succeed Although various price indexes were rising a bit more rapidly, there were indications that pressures would not continue to intensify, and might even reverse to a degree Moderating overall demand growth left businesses with excess inventories In response, firms initiated production cutbacks to prevent serious inventory imbalances, and the growth of economic activity slowed substantially With inflation pressures apparently receding, the previous degree of restraint in monetary policy was no longer deemed necessary, and the Federal Open Market Committee consequently implemented a small reduction in reserve market pressures last July During the summer and early fall, aggregate demand growth strengthened As a result, business stocks of raw materials and finished goods appeared somewhat better aligned with sales In sum, the economy, as hoped, appeared to have moved onto a trajectory that could be maintained-- one less steep than in 1994, when the rate of growth was clearly unsustainable, but one that nevertheless would imply continued significant growth in employment and incomes Importantly, the performance of the economy seemed to be consistent with maintaining low inflation Despite the step-up in growth and the relatively high levels of resource utilization, measured inflation abated a little, and many of the signs that had been pointing toward greater price pressures gradually disappeared Expectations of both near- and longer-term inflation fell substantially over the second half of the year, as gauged by survey results as well as by the downward movements in longer-term interest rates The fall in bond rates was also encouraged by improving prospects for significant progress in reducing the federal budget deficit The declines in actual and expected inflation meant that maintaining the existing nominal federal funds rate would raise real short-term interest rates, implying a slight effective firming in the stance of monetary policy Such a shift would have been particularly inappropriate because economic growth near the end of the year seemed to be slowing, and some FOMC members were concerned about the risks of prolonged sluggishness Consequently, the Committee decided in December that a further reduction in the funds rate was warranted Information becoming available in late December and January raised additional questions about the prospective pace of expansion The situation was difficult to judge, partly because economic statistics were more sparse than usual, owing mainly to the government shutdowns In addition, harsh weather in January disrupted both data flows and patterns of economic activity But several indicators-- including initial claims for unemployment insurance, purchasing managers' surveys, and consumer confidence measures --appeared to signal some softening in the economy Consonant with this pattern, some Reserve Bank Presidents reported that they seemed to be detecting anecdotal indications of weakness in the expansion within their districts with somewhat greater frequency than previously Moreover, growth in several of our major trading partners seemed to be lagging, which could tend to moderate demand for exports A number of factors have prompted the recent tendency toward renewed weakness Some are clearly quite transitory-- related, for example, to bad weather or the Federal government shutdown Others may be somewhat more significant, but still temporary The constraint on government spending while permanent budget authorizations are being negotiated is one Another may be a temporary reduction in output in some industries as businesses have further adjusted inventories to disappointing sales As I noted last July, the change in the pace of inventory investment when the economy shifts gears can be substantial Inventory investment surged in 1994 and into the early months of 1995, but proceeded to fall markedly throughout the rest of the year This has placed significant downward pressure on output, which should lift as inventory adjustments subside But for the moment, the pressures remain, in the motor vehicle industry and elsewhere Ultimately, of course, it is the path of final demand after the temporary influences work themselves out that determines the trajectory of the economy There are some factors, such as high consumer debt levels, that may be working to restrain spending But as I shall be detailing shortly, a number of fundamentals point to an economy basically on track for sustained growth, so any weakness is likely to be temporary Nonetheless, the Committee decided in late January that the evidence suggested sufficient risk of subpar performance going forward to warrant another slight easing of the stance of monetary policy Given the subdued trends in costs and wages, the odds that such a move would boost inflation pressures seemed low In assessing the likely course of the economy and the appropriate stance of policy, one question is the significance, if any, of the age of the business expansion Some analysts, viewing recent weakness, have observed that the expansion is approaching the start of its sixth year and is now one of the longer peacetime spans of growth in the past half century Economic expansions, however, do not necessarily die of old age Although the factors governing each individual business cycle are not always clear, expansions usually end because serious imbalances eventually develop When aggregate demand exceeds the economy's potential, for example, inflationary pressures pick up The inevitable increase in market interest rates, as inflation expectations rise and price pressures intensify, depresses final demand Lagging demand in turn sets off an inventory correction that frequently triggers a downturn in the economy As I noted, we acted in 1994 to forestall such a process Monetary policy began to tighten in advance of the buildup of inflationary pressures and, at least to date, these pressures appear to have been held in check Capital expenditures by households and firms can also contribute significantly to the development of cycle-ending imbalances The level of stocks of such real assets have effects on output very similar to those of business inventories In typical cycles, capital expenditures tend to grow rapidly in the early stages of recovery Pent-up demands coming out of a recession by consumers and businesses are satisfied by rapid growth of spending on capital assets There is a limit, however, on, say, how many cars people choose to own, or how many square feet of floor space retailers need to service customers Spending on such assets generally tends to grow more slowly after the pent-up demand is met As with business inventories, the downshifting of spending on consumer durable goods or business plant and equipment may not occur smoothly The dynamics of expanding output and rising profit expectations often create a degree of exuberance which, as in much of human nature, tends on occasion to excess--in this case, in the form of a temporary over-accumulation of assets The ensuing correction in demand for such assets triggers production adjustments that can significantly mute growth for a time or even cause a downturn if the imbalances are large enough The current extent of any asset overhang is difficult to determine The growth of demand for durables and some categories of capital goods evidently has slowed, but the available evidence does not suggest a degree of saturation in capital assets that would tip the economy into a downturn Moreover, financial conditions are likely to be generally supportive of spending The low level of long-term interest rates should have an especially favorable effect Low rates increase the affordability of housing for consumers and foster investment in productive plant and equipment by businesses The decline in interest rates also has contributed to a pronounced rise in stock prices The spread of mutual fund investments has meant that the gain in wealth as financial asset prices have risen has been shared by an ever-wider segment of households These developments should tend to counter, in part, the depressing effects on spending of rising debt burdens In addition, with the condition of most financial institutions strong, lenders are likely to remain willing to extend credit to firms and households on favorable terms We have seen some move by lenders toward tighter standards, but these actions are a modest correction after a marked swing toward ease and should not constrain the availability of funds to creditworthy borrowers Against this backdrop, Federal Reserve policymakers expect the most likely outcome for 1996 as a whole is further moderate growth On the new chain-weighted basis, the central tendency of the forecasts of Board members and Reserve Bank Presidents is for real gross domestic product to expand 2 to 2-1/4 percent on a fourth- quarter to fourth-quarter basis, similar to the Administration's outlook With output expanding roughly in line with standard estimates of the increase in the productive capacity of the economy, the unemployment rate is expected to remain around recent levels, as is also forecast by the Administration The Federal Open Market Committee expects a continuation of reasonably good inflation performance in 1996 The success during 1995 in keeping the increase in the consumer price index below 3 percent in the fifth year of an expansion illustrates that an extended period of growth with low inflation is possible And most on the Committee anticipate consumer price inflation at or somewhat below 3 percent in 1996 Although well-known biases in the CPI, as well as the more favorable price performance of business equipment, which is not included in that index, indicate that the true rate of inflation for the whole economy would be significantly lower than 3 percent, the Committee recognized that its expectations for inflation do not imply that price stability has as yet been reached Nonetheless, keeping inflation from rising significantly during economic expansions will permit a gradual ratcheting down of inflation over the course of successive business cycles that will eventually result in the achievement of price stability To emphasize its continued commitment to price stability, the Committee chose to reaffirm the relatively low ranges for money growth in 1996 that it had selected on a provisional basis last July These ranges are identical to those employed in 1995--1 to 5 percent for M2 and 2 to 6 percent for M3 The Committee also reaffirmed the 3 to 7 percent range for debt Patterns of money growth and velocity have been erratic in recent years, but should the monetary aggregates at some point re-establish their previous trend relationships with nominal income, average growth near the center of these ranges should be consistent with the eventual achievement of price stability Determining whether further changes to the stance of monetary policy will be necessary in the months ahead to foster progress toward our goals will be a continuing challenge In formulating monetary policy, while we have in mind a forecast of the most likely outcome, we must also evaluate the consequences of other possible developments Thus, it is sometimes the case that we take out monetary policy "insurance" when we perceive an imbalance in the net costs or benefits of coming out on one side or the other of the most probable scenario For example, in our most recent actions, we saw a decline in the federal funds rate as not increasing inflationary risks unacceptably. while addressing the downside risks to the most likely forecast In assessing the costs and benefits of adjustments to the stance of policy, members of the Committee recognize that policy affects the economy and inflation with a lag and thus needs to be formulated with a focus on the future Over the past year, we have kept firmly in mind our goals of containing inflation in the near term and moving over time toward price stability, and they will continue to guide us in the period ahead Structural forces may be assisting us in this regard Increases in producers' costs and in output prices proved to be a little lower last year than many had anticipated While it is too soon to draw any definitive conclusions, this experience provides some tentative evidence that basic, ongoing changes In the structure of the economy may be helping to hold down price pressures These changes stem from the introduction of new technologies Into a wide variety of production processes throughout the economy Successive generations of these new technologies are being quickly embodied in the nation's capital stock and older technologies are, at a somewhat slower pace, being phased out As a consequence, the nation's capital stock Is turning over at an increasingly rapid pace, not primarily because of physical deterioration but reflecting technological and economic obsolescence The more rapid advance of Information and communications technology and the associated acceleration in the turnover of the capital stock are being mirrored in a brisk restructuring of firms In line with their adoption of new organizational structures and technologies, many enterprises are finding that their needs for various forms of labor are evolving just as quickly In some cases, the job skills that were adequate only five years ago are no longer as relevant Partly for that reason, most corporate restructurings have involved a significant number of permanent dismissals The phenomenon of restructuring can be especially unfortunate for those workers directly caught up in the process Many dedicated, long-term workers In all types of American businesses--including long- established, stable, and profitable firms--have been let go An important consequence of the layoffs and dismissals associated with restructuring activity Is a significant and widely reported Increase in the sense of job insecurity Concern about employment has been manifested in unusually low levels of indicators of labor unrest Work stoppages, for example, were at a fifty-year low last year And contract negotiators for labor unions have sought to obtain greater job security for their members through very long- term labor contracts, including some with virtually unprecedented lengths of five or six years Of particular relevance to the inflation outlook, the sense of job insecurity is having a pronounced effect in damping labor costs For example, the increase in the employment cost index for compensation in the private sector, which includes both wage and salary payments and benefit costs, slowed further in 1995, to 2-3/4 percent, despite labor market conditions that, by historical stan- dards, were fairly tight With productivity also expanding, the increase in unit labor costs was even lower In manufacturing, such costs have actually been falling in recent years While the link between labor costs, which account for two-thirds of consolidated business sector costs, and prices is not rigid, these very limited increases in labor expenses nonetheless constitute a significant restraint on inflation In addition to its effect on labor costs, the more rapid pace of technological change is reducing business costs through other channels Initially most important, the downsizing of products resulting from semiconductor technologies, together with the Increasing proportion of national output accounted for by high-tech products, has reduced costs of transporting the average unit of GDP Quite simply, small products can be moved more quickly and at lower cost More recently, dramatic advances in telecommunications technologies have lowered the costs of production for a variety of products by slashing further the information component of those costs Increasingly, the physical distance between communications endpomts is becoming less relevant in determining the difficulty and cost of transporting information Once fiber-optic and satellite technologies are in place, the added resource cost of another 200 or 2,000 miles is often quite trivial As a consequence, the movement of inputs and outputs across geographic distance is progressively becoming a smaller component of overall business expenses, particularly as intellectual-- and therefore immaterial--products become proportionately more important in the economy This enables an average business firm to broaden markets and sales far beyond its original domicile Accordingly, fixed costs are spread more widely For the world market as a whole, the specialization of labor is enhanced to the benefit of standards of living of all market participants To be sure, advancing technology, with its profound implications for the nature of the economy, is nothing new, and the pace of improvement has never been even But it is possible that we may be in the midst of a quickening of the process It is possible that the rate at which earlier computer technologies are being applied to new production processes is still increasing This would explain the recent decline in the growth of unit costs Nonetheless, we have to be careful in projecting a further acceleration in the application of technology indefinitely into the future, as would be required for technological change to depress the rate of increase in unit business costs even more Similarly, suppressed wage cost growth as a consequence of job insecurity can be carried only so far At some point in the future, the tradeoff of subdued wage growth for job security has to come to an end While it is difficult to judge the time frame on such adjustments, the risks to cost and price inflation going forward are not entirely skewed to the downside, especially with the economy so recently operating at high levels of resource utilization In light of the quickened pace of technological change, the question arises whether the U S economy can expand more rapidly on an ongoing basis than the 2 to 2-1/4 percent range for measured GDP forecasted for 1996 by government agencies and most private forecasters without adding to inflationary pressures, which in turn would undermine growth The Federal Reserve would certainly welcome faster growth-- provided that it is sustainable The particular rate of maximum sustainable growth in an economy as complex and ever-changing as ours is difficult to pin down Fortunately, the Federal Reserve does not need to have a firm judgment on such an estimate, for persistent deviations of actual growth from that of capacity potential will soon send signals that a policy adjustment is needed Should the nation's true growth potential exceed actual growth, for example, the disparity and lessened strain would be signaled in shorter lead times on the delivery of materials, declining overtime, and ebbing inflationary pressures Conversely, actual growth in excess of the economy's true potential would soon result in tightened markets and other distortions which, as history amply demonstrates, would propel the economy into recession Consequently, we must be cautious in reaching conclusions that growth in productivity and hence of potential output has as yet risen to match the evident step-up in technological advance The hypothesis that advancing technology has enhanced productivity growth would be more persuasive if national data on productivity increases showed a distinct improvement To a degree, the lack of any marked pickup may be a shortcoming of the statistics rather than a refutation of the hypothesis Faulty data could be arising in part because business purchases are increasingly concentrated in items that are expensed but which market prices suggest should be capitalized Growing disparities between book capital and its valuation in equity markets may in part reflect widening effects of this misclassification If this problem is indeed growing, we may be underestimating the growth of our GDP and productivity This classification problem compounds other difficulties with measuring output in the increasingly important service sector The output of services --and the productivity of labor in that sector--is particularly hard to measure In part, the statisticians have simply thrown up their hands, gauging output in some service industries just in terms of labor input By construction, such a procedure will miss improvements in productivity caused by other inputs In manufacturing, where output is more tangible and therefore easier to assess, measured productivity has been rising briskly, suggesting that technological advances are indeed having some effect Nonetheless, there is still a nagging inconsistency The evidence of significant restructurings and improvements in technology and real costs within business establishments does not seem to be fully reflected in our national productivity measurements It is possible that some of the frenetic pace of business restructuring is mere wheel spinning-- changing production inputs without increasing output-- rather than real increases in productivity One cause of the wheel spinning, if that is what it is, may be that it takes some time for firms to adapt in such a way that major new technology is translated into increased output In an intriguing parallel, electric motors in the late nineteenth century were well-known as a technology, but were initially integrated into production systems that were designed for steam-driven power plants It wasn't until the gradual conversion of previously vertical factories into horizontal facilities, mainly in the 1920s, that firms were able to take full advantage of the synergies implicit in the electric dynamo, thus achieving dramatic productivity increases Analogously, existing production systems today to some degree cannot be integrated easily with new information and communication technologies Some existing equipment is not capable of control by computer, for example Thus, it may be that the full advantage of even the current generation of information and communication equipment will be exploited over a span of quite a few years and only after a considerably updated stock of physical capital has been put in place While the Federal Reserve does not need to establish targets- - and definitely not limits--for long-term growth, it is helpful in coming to shorter-run policy insights to have some judgments about the growth in potential GDP in the past and what it is likely to be in the future Judgments of potential, quite naturally, are based on experience Through the four quarters of 1994, for example, real GDP, pressed by strong demand, rose 3-1/2 percent If that were the true rate of increase in the economy's long-run potential, then we would have expected no change in rates of resource utilization Instead, industrial capacity utilization rose nearly 3 percentage points and the unemployment rate dropped a percentage point Moreover, we began to see signs of strains on facilities, deliveries of materials slowed appreciably and factory overtime rose sharply These signs of developing pressures on capacity suggest that the growth rate in economic potential in 1994 was below 3-1/2 percent In general, as we get close to presumed potential, we are required to step up our surveillance for inflationary pressures Estimates of potential growth necessarily recognize that expansion in the economy over time comes essentially from three factors--growth in population, increases in labor force participation, and gains in average labor productivity Of these factors, the first two are determined basically by demographic and social factors and seem unlikely to change dramatically over the next few years Thus, the source of any significant pickup of output growth would need to be a more rapid pace of productivity growth Here, the uncertainty of the pace of conversion of rapid technological advance into productivity gains is crucial to the determination To be fully effective in achieving potential productivity improvements, technological innovations also require a considerable amount of human investment on the part of workers who have to deal with these devices on a day-to-day basis On this score, we still may not have progressed very far Many workers still possess only rudimentary skills in manipulating advanced information technology In these circumstances, firms and employees alike need to recognize that obtaining the potential rewards of the new technologies in the years ahead will require a renewed commitment to effective education and training, especially on-the-job training This is especially the case if we are to prevent the disruptions to lives and the nation's capacity to produce that arise from mismatches between jobs and workers We need to improve the preparation for the job market our schools do, but even better schools are unlikely to be able to provide adequate skills to support a lifetime of work Indeed, the need to ensure that our labor force has the ongoing education and training necessary to compete in an increasingly sophisticated world economy is a critical task for the years ahead Our nation faces many important and difficult challenges in economic policy Nonetheless, we have made significant and fundamental gains in macroeconomic performance in recent years that enhance the prospects for maximum sustainable economic growth Inflation, as measured by the consumer price index, has been gradually reduced from a peak of more than 13 percent in 1979 to 2-1/2 percent last year Lower rates of inflation have brought a variety of benefits to the economy, including lower long-term interest rates, a sense of greater economic stability, an improved environment for household and business planning, and more robust investment in capital expenditures The years ahead should see further progress against inflation and the eventual achievement of price stability We have also made considerable progress on the fiscal front Over the past ten years and especially since 1993, our elected political leaders, through sometimes prolonged and even painful negotiations, have been successful in reaching several agreements that have significantly narrowed the budget deficit But more remains to be done As I have emphasized many times, lower budget deficits are the surest and most direct way to increase national saving Higher national saving would help to reduce real interest rates further, promoting more rapid accumulation of productive capital embodying recent technological advances Agreement is widely shared that attaining a higher national saving rate quite soon is crucial, particularly in view of the anticipated shift in the nation's demographics m the first few decades of the next century Lower inflation and reduced budget deficits will by no means solve all of the economic problems we face But the achievement of price stability and federal budget balance or surplus will provide the best possible macroeconomic climate in which the nation can address other economic challenges</t>
-  </si>
-  <si>
-    <t>I am pleased to participate once again in the Federal Reserve Bank of Atlanta's annual Financial Markets Conference Now in its fifth year, this conference has earned a reputation for bringing together groups of distinguished academics, practitioners, and policymakers to discuss important policy issues This year's program promises to enhance that reputation The principal topic of the program is the transparency and liquidity of derivatives More precisely, it is the implications of the relative opaqueness and illiquidity of many customized, over-the counter (OTC) derivatives for risk management, public disclosure, and relationships between counterparties By choosing this topic, this conference distinguishes itself from the many others on derivatives and risk management In effect, the conference focuses our attention on the challenges that lie ahead rather than on the very impressive advances that have been made in recent years In my remarks today I shall attempt to set the stage for the sessions that follow I shall begin by clarifying the characteristics of OTC derivatives that determine their transparency and liquidity and that tend to make a significant portion of these instruments opaque and illiquid Then I shall identify some of the challenges that are created by the use of opaque and illiquid financial instruments I shall conclude by offering some suggestions on how to meet them Before beginning I want to emphasize that by discussing these difficulties and challenges I do not mean to call into question the benefits of OTC derivatives or the utility of the risk management techniques that derivatives dealers have developed I would note that bank loans pose essentially the same difficulties Like OTC derivatives, bank loans are customized, privately negotiated agreements that, despite increases in availability of price information and in trading activity, still quite often lack transparency and liquidity This unquestionably makes the risks of many bank loans rather difficult to quantify and to manage Yet no one seriously questions the public benefits of bank loans, and most would agree that efforts to apply modern risk management techniques to bank loans should be supported and encouraged Indeed, it is my hope and expectation that by addressing the challenges posed by the lack of transparency and liquidity of the more customized OTC derivatives, the way will be paved for significant and parallel advances in the management of the risks of bank loans and the many other relatively opaque and illiquid instruments The intermediation and unbundling of credit risks and market risks are critical functions of a financial system These functions can be achieved only partially through standardized instruments and organized exchanges Hence, more opaque and illiquid financial instruments serve an invaluable function in our economy The use of such instruments entails higher risks which, of necessity, are reflected in higher intermediation costs As advances in risk management are achieved, however, these risks and related costs can be expected to decline At the outset I should clarify what I mean by transparency and liquidity By the transparency of a financial instrument I mean the degree of certainty with which one can determine its "fair value," which the Financial Accounting Standards Board (FASB) defines as "the amount at which the instrument could be exchanged in a current transaction between willing parties, other than in a forced or liquidation sale " Thus, fair values are a matter of conjecture rather than fact, they cannot be known, but must be estimated FASB has noted that quoted market prices, when available, are the best indicators of fair values As I shall note later, however, even quoted market prices are not always reliable indicators of the values at which transactions could be executed Moreover, quoted market prices simply are not available for many financial instruments, despite a rapid expansion of sources of price information, such as broker screens When quoted market prices are unavailable, fair values typically are estimated on the basis of quoted market prices for related instruments Such estimates require assumptions about relationships between fair values of different instruments Inaccurate or outdated assumptions inevitably heighten uncertainty about potential transactions prices By the liquidity of a financial instrument, I mean the percentage of its fair value that could be realized in a forced or liquidation sale A perfectly liquid financial instrument is one whose fair value could if necessary, be realized instantaneously Few financial instruments, however, are perfectly liquid For most instruments, time is required to search out a counterparty who is willing to transact at the fair value of the instrument In general, the less time that is available to complete the transaction, the smaller is the percentage of fair value that can be realized Also, the percentage of fair value that can be realized tends to decrease with the size of the transaction By these definitions, many OTC derivatives are neither highly transparent nor highly liquid The defining characteristic of OTC derivatives is the customization of terms through private negotiations between counterparties To be sure, broker screens provide market quotations for the more standardized or "plain vanilla" OTC derivatives, and these account for a large portion of outstanding contracts Even for plain vanilla derivatives, however, the estimation of fair values generally involves adjustments to market quotations to reflect operating, hedging, and other potential costs For more customized OTC derivatives, the estimation of fair values often involves use of a mathematical model that relates fair values of the customized instruments to available market quotations for more standardized products For example, the fair values of OTC options often are estimated using pricing models that utilize market quotations for the underlying asset and implied price volatilities from exchange-traded or plain-vanilla OTC options as inputs Especially for more complex options, the choice of a pricing model and of certain inputs to the model includes important elements of art as well as science Assumptions must be made, for example, about the shape of the sampling distributions of prices and price volatilities of the underlying assets The growing availability of independent valuation services allows users of complex instruments to assess whether or not their price estimates are consistent with other estimates But for many instruments the range of estimates can be quite wide Moreover, estimates are estimates Without timely transactions prices for very similar instruments, the accuracy of the estimates remains questionable In principle, the value of an OTC derivative can be promptly realized either by terminating the contract or by transferring it to another counterparty In practice, however, either procedure is likely to be time-consuming and may require the counterparty seeking to liquidate the contract to accept something less than the fair value In either case, the prior consent of the original counterparty usually must be obtained Counterparties typically require prior consent for termination because termination would require them to bear the costs of replacing the terminated contract with a new contract In general, the more customized the contract, the greater will be the cost of replacement, for which the counterparty will expect compensation Prior consent typically is also required for a transfer, so as to protect the other counterparty against the possibility of a transfer to a less creditworthy counterparty Although accommodating a transfer request generally would be less costly than the cost of accommodating a termination request, the counterparty may nonetheless seek compensation This discussion suggests that the opaqueness and illiquidity of many OTC derivatives stems from both the customization of contract terms and differences in creditworthiness across counterparties Users of the more customized OTC derivatives, in particular, are forced to accept a trade-off between the benefits of individually tailored contract terms and credit relationships and the costs of opaqueness and llliquidity This trade-off can perhaps be seen more clearly by comparing the benefits and costs of exchange-traded derivatives and OTC derivatives Exchange-traded derivatives are highly transparent and liquid, but these advantages are not achieved costlessly The terms of contracts traded on exchanges are very standardized In addition, credit risk is standardized by substitution of the exchange's clearing house as the central counterparty to every trade The standardization of contract terms limits the precision with which users can manage their risk exposures The standardization of credit risk requires the clearing house to impose costly margin requirements that are not yet routinely imposed in OTC transactions Users of highly customized OTC derivatives evidently perceive the benefits of tailoring contract terms and counterparty credit relationships as exceeding the costs associated with less transparency and liquidity Otherwise they would choose more standardized contracts, either of the plain vanilla OTC or exchange-traded variety Over time, the terms of this trade-off between the benefits of customization of contract terms and credit relationships and the costs of opaqueness and illiquidity are likely to improve In recent years, futures and options exchanges have successfully introduced so- called "flex" products that allow for greater tailoring of terms than traditional exchange offerings At the same time, the use of bilateral margining agreements for OTC derivatives has been spreading Existing proposals to create facilities for the centralized administration of such bilateral margining agreements may prove to be the first step toward the creation of clearing houses for OTC derivatives In general, I expect that we shall see further convergence between the characteristics of OTC and exchange-traded derivatives But I believe that it would be a mistake for policymakers to attempt to force this process Economic forces will ensure that market participants will seek to implement exchange or clearing house arrangements if they can enhance liquidity and transparency while maintaining most of the benefits of customized contracts Implications for Risk Management The development of OTC derivatives unquestionably has stimulated very significant improvements in financial risk management practices In particular, concerns about the risks associated with use of OTC derivatives prompted the Group of Thirty to sponsor development and publication in July 1993 of a set of recommended risk management practices that have been extremely effective in fostering improvements Critical elements of the G-30 risk management framework are accurate assessments of the fair values of financial instruments and portfolios and the use of risk measures that presume significant portfolio liquidity The authors of the G-30 study recognized that a series of difficulties arise in applying this framework to financial instruments that are relatively opaque and illiquid, including the more customized OTC derivatives But the study's discussion of practices and procedures necessary to address these difficulties was rather vague Our banking supervisors report that at the most sophisticated U S banks the relevant practices have been rapidly evolving but remain diverse In part, the diversity reflects differences in risk profiles and business strategies, but varying levels of refinement also are apparent Opaqueness and illiquidity affect each of the critical elements of risk management--valuation, risk measurement, and risk control The critical first step in risk management is determining the current market value of the portfolio Earlier I noted that market quotations simply are not available for many financial instruments I should emphasize that these include not only the more customized OTC derivatives but also thinly traded securities, as many investors in mortgage-backed securities discovered in early 1994 Values of these instruments must be estimated on the basis of market quotations for other, more standardized instruments This requires use of mathematical or economic models that relate the values of the customized instrument to the values of more standardized instruments Sophisticated risk managers recognize the uncertainty and the potential for error in valuation methods for opaque instruments and seek to compensate for various sources of error by creating reserves Among the reserves that institutions often create are reserves for additional hedging costs, for uncertainty about the accuracy of models, especially in valuing new or especially complex products, and, quite explicitly, for illiquidity The values of these reserves can be quite significant, especially in the aggregate In addition, some institutions establish a credit risk reserve that is intended to incorporate credit quality into fair values While these reserving practices can be described within a broad common framework, there appears to be no common understanding within the industry of the circumstances in which many of these reserves should be created or on their appropriate size Risk measurement is the assessment of potential future changes in portfolio values Opaqueness affects the measurement of both market risk and credit risk Consistent with the recommendations of the G-30, sophisticated managers typically measure market risk by value-at-risk ("VaR"), often defined as the amount of losses over one day that would be expected to occur only one day out of a hundred In practice, VaR measures typically assume that the values of all instruments in a portfolio are determined by a common set of underlying risk factors --interest rates, exchange rates, commodity prices, and stock indexes --most of which are readily hedgeable But the sensitivity of customized instruments to these factors sometimes is difficult to assess Furthermore, the values of such instruments may be influenced importantly by risk factors other than common hedgeable factors recognized in VaR measures One can hope that these residual risks are well diversified, but, absent a means of measuring them, this may be nothing more than wishful thinking Unfortunately, the measurement of these risks requires accurate measures of fair values which, by definition, are problematic in the case of opaque instruments The difficulties in valuing some financial instruments also make accurate measurement of credit risk quite difficult In the case of OTC derivatives, much progress has been made in modeling potential future claims on counterparties, which often are termed potential future credit exposures However, as is the case for any financial instrument, the credit risk of an OTC derivative depends on the creditworthiness of the counterparty If the holder seeks to transfer an OTC derivative, the amount that a transferee will be willing to pay for the contract will depend on market discount rates then applying to claims on the counterparty Likewise, the amount that the counterparty will be willing to pay in a negotiated termination will depend on the cost at which the counterparty could replace the terminated contract, which will depend on these same future discount rates The development of techniques for estimating potential future discount rates remains at the frontier of risk measurement Even in the best of circumstances--in which the counterparty has issued actively traded corporate bonds --techniques extracting estimates of the relevant discount factors remain at an early stage of development Assessments of the liquidity of financial instruments are critical to efforts to control risks VaR measurements often are translated into position limits for traders, which are a critical element of internal risk controls When VaR is measured using a one- day horizon, it is implicitly assumed that risk exposures in the portfolio can, if necessary, be offset within a day This assumption does not require that all of the financial instruments in the portfolio can be liquidated within a day Rather, it merely assumes that the hedgeable risk exposures that are the focus of VaR measures can be offset that quickly, presumably through use of highly liquid instruments such as exchange-traded derivatives Still, even the most liquid markets may experience periods of illiquidity As noted in the title of today's first session, one needs to consider the consequences if everyone can't get into the lifeboat at the same time Furthermore, as I have suggested, the unhedgeable instrument-speciflc risks of illiquid instruments cannot be ignored Losses stemming from an inability to offset or close out portfolios promptly are among the risks that sophisticated risk managers seek to assess through so- called "stress tests " However, stress testing is another area in which our bank supervisors observe considerable diversity of practice Consensus has not yet emerged on how to identify scenarios that pose the greatest risk of loss or, as important, on appropriate responses to test results As I have noted, some banks establish reserves to cover the potential costs of llliquidity Others supplement VaR-based risk limits with instrument-specific position limits In principle, stress tests could be used to evaluate the size of such reserves and limits Implications for Public Disclosure The opaqueness and llliquidity of customized OTC derivatives and other financial instruments create uncertainty about the financial position and performance--the net worth, earnings, and risk profile-- of users of such instruments Concerns about such uncertainty often are termed concerns about the transparency of financial statements, a concept that is broader than the concept of transparency I have been using thus far These concerns have prompted issuance in recent years of a series of new accounting standards and proposals by the FASB and the Securities and Exchange Commission The most recent changes have required disclosure of accounting policies for derivatives, of the purposes (trading or hedging) for which derivatives are used, and of fair values of derivatives, either carried on the balance sheet or in supplemental schedules FASB has encouraged disclosures of quantitative information on market risk, and the SEC recently has proposed to require such disclosures I have discussed the difficulties involved in determining fair values for the more customized OTC derivatives and the diversity of valuation practices actually employed An implication of this discussion is that market participants could better assess the financial position of users if more information were disclosed on valuation policies, including the size of the various reserves, if material, and how those reserves are determined Fuller disclosure would reduce not only uncertainty but also the danger that reserves could be manipulated to reduce the volatility of reported earnings My discussion of risk measurement issues suggests that disclosure of quantitative measures of market risk, such as value-at- risk is enlightening only when accompanied by a thorough discussion of how the risk measures were calculated and how they related to actual performance Moreover, no single quantitative measure can summarize all aspects of such a complex concept as market risk These conclusions are fully consistent with an analysis of appropriate public disclosures of market and credit risks (the Fisher Report) that was released in September 1994 by the Euro-currency Standing Committee of the Group of Ten central banks Implications for Counterparty Relationships The opaqueness and illiquidity of some OTC derivatives also have contributed to tensions between counterparties, tensions that in some instances have produced litigation or threats of litigation As I noted earlier, even when a market quotation is available, there may be uncertainty and confusion about what the quotation is intended to convey and how it should be interpreted In particular, there may be confusion about whether a quotation represents an estimate of the fair market value of an instrument or a firm offer to transact in the instrument at the quoted price By definition, transaction prices of illiquid instruments can be different, possibly significantly different from fair market values A fair market value is an estimate of the price at which a transaction might be executed with a willing counterparty As I have emphasized, estimation errors are to be expected, especially for more customized, illiquid contracts Moreover, a price concession may be necessary to produce a willing counterparty Consequently, the price at which a transaction can be executed cannot be inferred from estimates of fair market value Transactions prices can be determined only by contacting potential counterparties and soliciting offers to transact Moreover when soliciting quotations it is essential that it be made clear to potential counterparties that a transactions price, rather than a fair market value estimate or a nonbinding "indicative" price quotation is desired Likewise, counterparties that receive requests for quotations should determine clearly what type of quotation is desired before responding Addressing the Challenges Posed by Opaqueness and Illiquidity Before concluding, I would like to offer a few brief suggestions for addressing the challenges I have identified On the risk management front, there should be more public discussion of valuation difficulties and best practices for addressing those difficulties This would appear to be an area in which an industry initiative by derivatives dealers or by accounting or consulting firms would be quite useful Regarding public disclosure, I remain convinced of the usefulness of the central recommendation of the aforementioned Fisher Report, which called for financial intermediaries to move in the direction of disclosing to the public the quantitative measures of market risk and credit risk that the firm's management relies upon A November 1995 review by the Basle Supervisors Committee and the Technical Committee of IOSCO found that internationally active banks and securities firms had made progress in implementing the Fisher Report's recommendations, but the Report also concluded that further efforts were needed by intermediaries in many G-10 countries Finally, I believe the problems that opaqueness can create for counterparty relationships can best be addressed by heightening awareness of potential ambiguities associated with market quotations and encouraging clarity in communications between counterparties The initiative on valuation that I have suggested would clearly contribute to an understanding of the differences between fair value estimates and transactions prices Conclusion In my remarks today I have tried to identify the challenges posed by the opaqueness and illiquidity of some OTC derivatives and of many other financial instruments as well I have done so on the assumption that the long debate on derivatives has reached a stage of maturity at which we can openly discuss difficulties and challenges without running the risk of a legislative or regulatory overreaction In any event, I am confident that, in the long run, frank discussions like those that I expect to take place at this conference offer the most effective hedge against that risk</t>
-  </si>
-  <si>
-    <t>This is the fifth time I have addressed the I B M annual convention Over those years, both the problems facing community banks and the environment in which they operate have changed quite a bit Today, I would like to discuss some of the broader challenges facing America's community bankers, and how one of those challengesâ€”technologyâ€”affects the economy more generally If we had surveyed the members of this association over the last few years about their most significant concerns, the list at one time or another would certainly have included loan quality, interest rate risk, the increasing layering of regulations, and supervisory rigidity Some of these are no longer issues, others have been greatly reduced in importance, and a few have been incorporated into day-to-day operations so as to be only a dull pain But I would venture the guess that the three concerns that community bankers have continued to discuss among themselves as the fundamental challenges to their survival are interstate banking, ongoing industry consolidation, and relentless technological change Many pundits have concluded that these forces will destroy small banks by making them quaint symbols of the past I think these prognosticators are plain wrong The evidence seems clear that, despite these powerful forces, well-managed community banks will not only survive, but will continue to be among the more innovative in our nation's financial system Community banks will maintain their significant contribution to economic growth by providing specialized and flexible financial services to small businesses, households, and others But I must quickly add that ignoring the fundamental changes going on in financial delivery systemsâ€”and not adapting to themâ€”could well contribute to the demise of the individual bank so inclined Such unresponsive banksâ€”and some still exist, at least for the time beingâ€”are not, by definition, showing the creativity that has characterized community banking, and there is no reason policymakers should be concerned about their individual competitive demise The Riegle-Neal Interstate Banking and Branching Act of 1994 already allows nationwide interstate banking through bank holding companies and will allow interstate branching next year This Act will accelerate, but not fundamentally change, what has been a fact of life for several years interstate banking Indeed, about one-fourth of domestic deposits are already held by out-of-state banking organizations I do not mean to understate the importance of interstate branching when I say the more significant contribution of Riegle-Neal is permitting interstate operations everywhere on the same basisâ€”except for branching in states opting out of interstate branching, so far only Texas Prior to the 1994 federal legislation, the lack of uniformity in interstate banking laws had hindered the equitable erosion of the anticompetitive state laws designed to protect local banks from out-of-market competition But whether by prior state modification or as the result of federal legislation, those banks whose profitability, and hence survival, had before depended solely on protection from geographical competition will not survive in the new environment As you know, entry from out-of-market, let alone out-of-state, has been almost entirely by acquisition of existing local rivals rather than the creation of de novo banks or branches With the number of rivals in local markets unchanged, out-of-market acquirers generally have not been able to increase the market share of their acquired institutions Apparently, knowledge of local markets and old fashioned banking skills have been more than a match for the new entrants I might note that the long-held fear that out-of-state rivals will cut prices on services to build market share is not supported by the evidence we have regarding fees Federal Reserve sponsored surveys of bank fees indicate that, on average, the highest fees in local markets are levied by out-of-state banking organizations who, in turn, are not charging significantly lower fees than they charge in their home markets Let me be clear I am not saying that the impact of a substitute rival leaves competitive pressures in local markets totally unchanged Although some bankers have indicated that it is easier to compete against a large out-of-market firm than the same size local firm that knows the market, I believe that generally local banks have found it necessary to respond to the new, perhaps more aggressive, entrant that purchased an already existing competitor Nonetheless, it seems clear that well-managed community banks have done well in such markets by drawing on their expertise and knowledge and managing their costs, and I see no reason why this will change To be sure, branch banks and multi-bank holding companies can offer some services that local banks cannot, such as services over a wider area Even here I would note, however, that ten states already permit independent state banks to form agency relationships with other banks for deposit gathering, loan collection, and other services in order to match many of the things branch systems can offer Twenty-one states permit such agency relationships among state banks in the same holding company I expect other states to follow soon And while, to date, not many banks have opted to use these powers, there is reason to expect them to do so as part of the continuing innovative response and leadership that is the hallmark of the dual banking system Most interstate banking has been accomplished, as I noted, by acquisition rather than by establishing de novo offices Acquisitions by out-of-market organizations result in a consolidation of the total number of banks in the country, but no change in the number of local market rivals Much of the recent merger activity, however, has been in-market consolidation, resulting in both a reduction of the total number of banks and in the number of rivals in local markets Community bankers have been active participants in this form of merger activity For both large and small banks, these in-market acquisitions, like interstate mergers, are intended to create efficiencies of scale and scope by eliminating redundancies and duplications, and by leveraging the different skills from the component banks Often the stated reasons for such mergers include phrases like "better control of the market," which is, let us admit, a not very cryptic code for reducing competitive pressure, often in pricing Like the Justice Department, the Federal Reserve and the other banking agencies, however, are required by law to ensure that mergers do not significantly reduce competition in local markets Indeed, the mergers that are substantially inconsistent with Justice Department and agency guidelines never even result in formal applications In addition, approval of an in-market merger is often conditional on the divestiture of offices in local markets in which the surviving bank would otherwise become excessively dominant In part for these reasons, even with the well-publicized wave of very large consolidations, local market concentration ratios have risen only marginally It is in these local markets where the competitive battle is fought among community banks and the regional and giant banks Application of the banking and antitrust laws may have mitigated the competitive impact of in-market mergers on the other banks in the local market But more important, in my judgment, has been the economics of the marketplace that limit the competitive strengths of merged banks The best evidence we have is that economies of scaleâ€”that is, the efficiencies that are alleged to come with greater sizeâ€”are quite limited Indeed, in explaining performance, differences in management effectiveness among banks of similar size dominate any efficiencies (or inefficiencies) that are connected directly to size per se Within each groupâ€”community banks, regionals, and giantsâ€”the cost differences associated with management skills are much more dramatic than the cost differences between size groups And, for reasons we do not fully understand, efficient banks that acquire inefficient banks do not seem to be able consistently to transfer their efficiencies to the consolidated unit This result, it seems to me, cannot hold much longer As you know better than I, the ongoing powerful competitive pressures will make survival of the inefficient banks in all size categories unlikely In contrast to the record of earlier years, some of the recent consolidations have brought not only cost-savings, but apparently efficiencies as well In the new competitive environment, all acquirers are cutting costs, but it is important to underline that cost cutting does not result in efficiency gains, which require that revenues fall by less than costs (or rise by more than costs) Be that as it may, it appears that resultant cost savings and any associated increased efficiencies are less the mechanical/technical dividends of scale, and more the result of actions that could have been taken separately by the component banks Interestingly, many of these efforts, such as reducing management overhead or eliminating unprofitable lines, may have not been feasible without the substantial rearrangement implicit in a consolidation Whatever the reason, consolidation in some casesâ€”not allâ€”seems to have resulted in efficiencies More and more, I believe, the surviving banksâ€”large and smallâ€”will have to be efficient in all the dimensions of that term, and will be under constant pressure to remain so For these reasons, most forecasts of the future United States banking structure project a substantial reduction in the number of American banks But these same projections also predict that thousands of banks will survive the consolidation trend, reflecting both their individual efficiencies and competitive skills, on the one hand, and the preferences of the marketplace on the other Such analysis, done by the Federal Reserve Board's staff and others, merely reinforces my own view that the franchise value of the U S community bankâ€”based on its intimate and personalized knowledge of local markets and customers, its organizational flexibility, and, most of all, its management skillsâ€”will remain high, assuring that community banks continue to play a significant role in the U S financial system Other observers are not so sanguine, arguing that changing technology may be the real slayer of banks, especially community banks This argument has at least two strands One is that technology reduces the degree of financial intermediation needed by society because it permits economic units to directly create their own financial contracts as both asset and liability holders Banks, it is argued, will be replaced by virtual banks, and the future J P Morgan will not ask for your person to see my person, but will ask your computer to see my computer The other strand of the argument is that it takes substantial resources and skills to develop and use the new technology, and that because small banks do not have such resources they will not be able to maintain their position Let's look at the second argument first This very conventionâ€”whose theme is "Tech World"â€”belies this thesis I know that a critical reason for you attending this convention is to hear the scintillating speeches, such as mine, but the displays of equipment and software are not irrelevant Not only is the technology for sale, often by larger banks, but the services that come from that technology are also for sale The community bank of today is as different from a small bank of 20 years ago as is the giant bank from its predecessor Both have fundamentally changed the way they do business, provide the customer service, and manage risk by using computer technology For example, smaller banks are among the end-users of derivatives to hedge risk, even as the larger banks are the dealers in such instruments Both are using the fruits of the new technology There is no question that technology is among the critical causes of the financial revolution that has swept the world in the last two decades It has changed the way banks do business and has increased the number and kinds of bank competitors But to conclude that banksâ€”especially community banksâ€”will not continue to be significant participants in the financial system does not square with the facts Community banks have always focussed on local face-to-face customer contacts Yet as technology has deepened, we find that most large banks are increasing, not decreasing, their branch systems as they relearn what community banks have always known Meeting customer demands on the customers' terms remains the name of the game and the customer continues to demonstrate his desire to deal with an institution that is conveniently located Moreover, community banks have already showed their skill in using technology to meet customer preferences I fail to see why community banks will not continue to do so Small does not mean unadaptable, and it certainly does not mean inefficient In sum, as you think about interstate banking, consolidation, and changing technology, I urge you to continue to worry, because concerned management means efficient management But don't worry too much because your efficiencies suggest that you will more than hold your own against intra- and interstate competition and consolidation, virtually regardless of technological change The same relentless pressures of technological change that has revolutionized banking and the financial system has also been at work in the economy at large The pressures to improve productivity and contain costs range far beyond the financial system And they seem to have been effective Increases in producers' costs and in output prices, for example, proved to be a little lower last year than many had anticipated While it is too soon to draw any definitive conclusions, this experience provides some tentative evidence that basic, ongoing changes in the structure of the economy may be helping to hold down business costs and price pressures Successive generations of new technologies are being quickly embodied in the nation's capital stock and older technologies are, at a somewhat slower pace, being phased out As a consequence, the nation's capital stock is turning over at an increasingly rapid pace, not primarily because of physical deterioration, but reflecting technological and economic obsolescence The more rapid pace of technological change is reducing business costs through a variety of channels One important channel, the downsizing of products resulting from semiconductor technologies, together with the increasing proportion of national output accounted for by high-tech products, has reduced costs of transporting the average unit of GDP Quite simply, small products can be moved more quickly and at lower cost More recently, dramatic advances in telecommunications technologies have lowered the costs of production for a variety of products by slashing further the information component of those costs Increasingly, the physical distance between communications endpoints is becoming less relevant in determining the difficulty and cost of transporting information Once fiber-optic and satellite technologies are in place, the added resource cost of another 200 or 2,000 miles is often quite trivial As a consequence, the movement of inputs and outputs across geographic distance is progressively becoming a smaller component of overall business expenses, particularly as intellectualâ€”and therefore immaterialâ€”products become proportionately more important in the economy This enables an average business firm to broaden markets and sales far beyond its original domicile Accordingly, fixed costs are spread more widely For the world market as a whole, the specialization of labor is enhanced to the benefit of standards of living of all market participants One would think that the evident step-up in technological advance would have been matched by a pickup in the growth of productivity nationwide It certainly has been the case in banking However, to paraphrase Nobel Laureate Robert Solow, we see technological advance everywhere but in the productivity statistics To a degree, the lack of any marked improvement in the national data on productivity growth may be a shortcoming of the statistics Faulty data could be arising in part because business purchases are increasingly concentrated in items that are expensed but which market prices suggest should be capitalized Growing disparities between book capital and its valuation in equity markets may in part reflect widening effects of this misclassification If this problem is indeed growing, we may be underestimating the growth of our GDP and productivity This classification problem compounds other difficulties with measuring output in the increasingly important service sector The output of servicesâ€”and the productivity of labor in that sectorâ€”is particularly hard to measure In part, the statisticians have simply thrown up their hands, gauging output in some service industries just in terms of labor input Should medical output, for example, be measured by the number of physicians, nurses, and other medical personnel at work, or by the dramatic advances in medical outcomes In manufacturing, where output is more tangible and therefore easier to assess, measured productivity has been rising briskly, suggesting that technological advances are indeed having some effect Nonetheless, there is still a nagging inconsistency The evidence of significant improvements in technology and reductions of real costs within business establishments does not seem to be fully reflected in our national productivity measurements It is possible that some of the frenetic pace of business restructuring is mere wheel spinningâ€”changing production inputs without increasing outputâ€”rather than real increases in productivity One cause of the wheel spinning, if that is what it is, may be that it takes some time for firms to adapt in such a way that major new technology is translated into increased output In an intriguing parallel, electric motors in the late nineteenth century were well-known as a technology, but were initially integrated into production systems that were designed for steam-driven power plants It wasn't until the gradual conversion of previously vertical factories into horizontal facilities, mainly in the 1920s, that firms were able to take full advantage of the synergies implicit in the electric dynamo, thus achieving dramatic productivity increases Analogously, existing production systems today to some degree cannot be integrated easily with new information and communication technologies Some existing equipment is not capable of control by computer, for example Thus, it may be that the full advantage of even the current generation of information and communication equipment will be exploited over a span of quite a few years and only after a considerably updated stock of physical capital has been put in place Our nation faces many important and difficult challenges in economic policy Nonetheless, we have made significant and fundamental gains in macroeconomic performance in recent years that enhance the prospects for maximum sustainable economic growth And, as technological advances are absorbed more and more into the way firms do business, the years ahead should see improved productivity growth, further progress against inflation, and a macroeconomic climate in which the nation, the financial system, and the banking community can address its other economic challenges</t>
-  </si>
-  <si>
-    <t>Mr Chairman, you have invited me to appear before this Committee to discuss the Savings Association Insurance Fund I testified before this Committee last August and September, and our position on the difficult issues raised by an undercapitalized SAIF has not changed I would like to review some of the issues and principles raised in that earlier statement, as well as, of course, respond to the request for my views on the policy options raised in the Chairman's letter of invitation The deposit insurance provided by BIF and SAIF is identical For identical insurance, depository institutions are rational to seek the one available at the lowest cost Since a substantial difference in deposit premiums exists between SAIF and BIF, SAIF institutions will pursue BIF insurance unless there is some other reason to remain with their current fund It is critical to underline that even if there were no problem with two different insurance premiums, the existing deposit insurance system, with its reliance on two funds, is inherently unstable Congress can attempt to legislate barriers that try to stop institutions from shifting deposits between entities insured by the other fund, but the history of efforts to legislate against such strong financial incentives is not encouraging Under the current system, we are, in effect, attempting to use government to enforce two different prices for the same itemâ€”namely, government-mandated deposit insurance Such price differences only create efforts by market participants to arbitrage the difference Given the large financial gains to SAIF institutions if they move deposits to BIF, they will continually strive to do so The only winners created by continuation of the current deposit premium difference between SAIF and BIF deposits will be those depositories able to "game" the system, and leave SAIF first The solution to this problem is to end this game and merge SAIF and BIF The merger of the savings and loan charter into a commercial bank-like charter also should be undertaken as soon as practicable The specific details of a charter consolidation are less important than making measurable progress in developing a set of insured depository institutions subject to as identical set of rules and incentives as possible However, at a minimum, removal of tax incentives that inhibit more diversified thrift portfolios should be enacted along with legislation recapitalizing the SAIF Such legislation is part of the Balanced Budget Act Mr Chairman, you requested my views on each of five options The principles outlined earlier, in my judgment, apply in evaluating each of them The same price should apply for the same deposit insurance and insured depository institutions should not be artificially induced to specialize Implementation of these principles implies that the premium differential should be eliminated, the SAIF fund should be recapitalized and then merged with the BIF, the bad debt reserve recapture should be repealed, and the thrift charter replaced with a bank-like charter The first option would have the taxpayer pick up both the FICO obligation and the cost of recapitalizing the SAIF The Congress did decide in 1989 in favor of taxpayer funding of the failed deposit insurer of the savings and loan industry Up to now, you have chosen not to use the same option for FICO or SAIF The decision, of course, is a political one The second option of resubmittmg the legislation that was included in the Balanced Budget Act would be a major step forward, although it leaves merger of the insurance funds and the bank-thrift charter to a second step I believe that the third option of no action is simply not viable economically, for reasons noted earlier I have no view on the fourth option of using Fannie Mae or Freddie Mac to fund FICO Like the fourth option, the fifth option, to fund FICO from Oakar and Sassar premiums, does not result in elimination of either the premium differential or of the separate insurance funds offering the same insurance, though it does delay FICO insolvency We should not lose sight of first principles A deposit insurance system that focuses the attention of banks and thrifts on the relative status of their funds, and a system that rewards those who can jump ship first, is, to say the least, counterproductive What is needed is a deposit insurance system whose status is unquestioned so that the depositories can appropriately focus their attention on the extension and management of credit in our economy</t>
-  </si>
-  <si>
-    <t>I appreciate the opportunity to appear before this Committee once again As you know, I discussed current economic conditions and the outlook rather extensively in appearances before House and Senate Banking Committees just over a month ago Today, I would like to provide a brief update of comments that I made then and reiterate my views on some key issues that are important for our nation's economic prospects over the medium term. A month ago, the economy clearly had been perceived as soft over the latter part of 1995 and early weeks of 1996 There were uncertainties, however, both about the factors that might have given rise to the softness in activity and the degree to which that softness might persist Although not all of the uncertainties have been resolved, recent data have confirmed the expectation that a good bit of the economic sluggishness of late 1995 was related to inventory investment The efforts of businesses to re-establish more desirable relationships between their holdings of inventories and their actual and prospective levels of sales held down production. Toward the end of last year, the inventory adjustments reached a point at which stocks actually were being reduced in the aggregate Although January, with its unusually severe weather, apparently resulted in goods being bottled up for a time in some parts of the economy, the underlying picture, as best we can discern, seems to be one in which much, but perhaps not all, of the needed inventory correction already has been accomplished Ultimately, of course, the inventories that businesses want to hold will depend on the growth of final demand At present, there are some factors, such as high consumer debt levels, that still may be working to restrain spending But the recent data seem to indicate that those restraining influences are not so strong as to seriously jeopardize the continued expansion of the economy. Data for February showed increases in sales of motor vehicles and other types of goods that are purchased at retail, and housing starts rose further last month. In the business sector, real outlays for fixed capital still appear to be trending up. The labor market reports for February provided additional evidence that the economy is moving past the disruptions that had slowed it in previous months Payroll employment surged in February, more than reversing the losses of January, and the unemployment rate, after having ticked up in January, dropped back last month It is possible that the February data may have exaggerated the strength of the labor market to some extent, as we've not seen a similar degree of strength in other labor market indicators, such as initial claims for unemployment insurance But even so, the current economic expansion seems to have exhibited staying power The strike that has recently affected the motor vehicle industry is likely to result in additional volatility over the near term, but like the disruptions of this past winter, it should not have a great impact on underlying trends in the economy The most recent reports on inflation also have been reasonably encouraging. Price increases at the consumer level have been moderate, on average, in the early part of 1996, and the twelve-month change in the CPI has remained near recent lows. In addition, producer prices have been well-behaved early this year, the prices of finished goods changed little over the first two months of the year, and materials prices in the PPI continued to edge down While monetary policy, as always, will need to be alert to inflation risks as we move forward, the recent economic data suggest that the economy should be able to continue operating at a high level of resource utilization, sustaining growth without risking a reversal of progress that has been made toward the goal of price stability As I noted last month, structural forces may be assisting us in this regard Introduction of new technologies into a wide variety of production processes is affecting production costs and business pricing throughout the economy Successive generations of these new technologies are being quickly embodied in the nation's capital stock, and older technologies are, at a somewhat slower pace, being phased out As a consequence, the nation's capital stock is turning over at an increasingly rapid pace, not primarily because of physical deterioration but reflecting technological and economic obsolescence A major challenge that we face during this period of rapid technical change is that of altering, with minimal disruption, not only the existing organizational structures and production methods of firms but, even more important, the skills of the labor force At present, the more rapid advance of information and communications technology and the associated acceleration in the turnover of the capital stock are being mirrored in a brisk restructuring of firms In line with their adoption of new organizational structures and technologies, many enterprises are finding that their needs for various forms of labor are evolving just as quickly In some cases, job skills that were adequate only five years ago are no longer as relevant Partly for that reason, most corporate restructurings have involved a significant number of permanent dismissals It would be neither feasible nor desirable to try to restrain the technical forces that lie behind the huge structural changes that are playing themselves out in the business world and in the workplace But we can take steps that will help ease the transition between the old and the new Firms and employees alike need to recognize that obtaining the potential rewards of the new technologies in the years ahead will require a renewed commitment to effective education and training, especially on-the-job training Such a commitment is essential if we are to prevent the disruptions to lives and the nation's capacity to produce that arise from mismatches between jobs and workers We need to improve the preparation for the job market our schools do, but even better schools are unlikely to be able to provide adequate skills to support a lifetime of work Indeed, ensuring that our labor force has the ongoing education and training necessary to compete in an increasingly sophisticated world economy is a critical task for the years ahead Fortunately, economic successes of the past decade or so have put us in a better position to meet the challenges that remain We have made significant and fundamental gains in macroeconomic performance in recent years that enhance the prospects for maximum sustainable economic growth Inflation, as measured by the consumer price index, has been gradually reduced from a peak of more than 13 percent in 1979 to about 2-1/2 percent last year Lower rates of inflation have brought a variety of benefits to the economy, including lower long-term interest rates, a sense of greater economic stability, an improved environment for household and business planning, and more robust investment in capital expenditures Hopefully, the years ahead will see further progress against inflation and the eventual achievement of price stability We have also made considerable progress on the fiscal front. Over the past ten years and especially since 1993, our elected political leaders, through sometimes prolonged and even painful negotiations, have been successful in reaching several agreements that have significantly narrowed the budget deficit But more remains to be done As I have emphasized many times, lower budget deficits are the surest and most direct way to increase national saving. Higher national saving would help to reduce real interest rates further, promoting more rapid accumulation of productive capital embodying recent technological advances Agreement is widely shared that attaining a higher national saving rate quite soon is crucial, particularly in view of the anticipated shift in the nation's demographics in the first few decades of the next century As recent events in financial markets seem to have demonstrated, delay in taking meaningful action on the budget comes at a cost Although the backup of long-term interest rates this year surely has been in large part a reflection of an economy on firmer footing than many market participants had thought, long-term rates also have been affected by perceptions in the market that priorities may be shifting away from deficit reduction Lower inflation and reduced budget deficits will by no means solve all of the economic problems we face But the achievement of price stability and federal budget balance or surplus will provide the best possible macroeconomic climate in which the nation can address other economic challenges, including those that arise as side effects of the otherwise beneficial and highly desirable process of technological advance</t>
-  </si>
-  <si>
-    <t>Good morning It is a pleasure to once more address this impressive conference Through the years the Chicago Federal Reserve Bank has consistently identified the most important issues that policymakers are confronting. It has done so again The rapidity of technological change, the globalization of finance, and the institutional expansion of financial competition are changing the banking environment so dramatically that regulators, of necessity, must continually re-evaluate their strategy and procedures It is useful, I think, to begin a discussion of "what should regulators do " by reminding ourselves just why there is bank regulation, by which I mean regulation designed to assure a minimum level of prudential soundness At bottom, of course, is the historical experience of the effects on the real economy of financial market disruptions and bank failures, especially when the disruptions and failures spread beyond the initial impetus Perhaps equally important is the unintended market response to a safety net designed to address systemic concerns and protect "small" depositors Deposit insurance and the discount window, by changing the terms under which banks deal with their creditors, distort the signals and incentives that banks receive from the market, creating a substantial potential for excessive risk-taking by banks In response, bank regulators have been forced to try to minimize this moral hazard that, in the absence of the safety net, the market itself would police The problems that arise from the short-circuiting of the pressures of market discipline have led us increasingly to understand that the ideal strategy for supervision and regulation is to simulate the market responses that would occur if there were no safety net, but without giving up the basic requirement that financial market disruptions be minimized Such a realization highlights the basic tensions between stability and risk taking, between regulation and market forces, between government guarantees and business choices Our goal is, in effect, to make the safety net moot in order to give wider range to market forces But our constraint is to avoid systemic risk, by which â€” as I have noted at this conference before â€” I do not mean a zero bank failure rate Far from it For we should not forget that the basic economic function of these regulated entities is to take risk If we minimize risk taking in order to reduce failure rates to zero, we will, by definition, have eliminated the purpose of the banking system Since dramatic institutional and regulatory change is rare, the challenge is to develop evolutionary modifications that balance risk-taking and stability, market incentives and regulations Happily there are, I think, reasons to be optimistic that this can be done The source of my optimism, as I will explain, is the potential to harness one of the main forces that is also challenging our current regulatory structure technology Supervisors and regulators have already begun to do so by emphasizing risk management procedures at individual banks and, most recently, by proposing the use of internal risk models for purposes of allocating capital for trading risk Nonetheless, the most fundamental recent change â€” to which the others are simply modifications â€” is the adoption of risk-based capital The risk-based capital accord of 1988 was a genuine step forward at the time However, compromises were inevitably made to achieve consensus The regulators knew the shortcomings, but were â€” in my view, correctly â€” willing to compromise in order to establish both a meaningful capital floor and to recognize, in a rough way, differences in risks for broad categories of assets The capital rules were especially helpful to halt â€” and reverse â€” the secular decline in bank capital ratios Moreover, the Fed was â€” and continues to be â€” supportive of prompt corrective action that builds upon the accord by requiring specific regulatory responses at different risk-based capital ratios In recent years, however, the weaknesses in the risk-based capital structure have become ever more evident its sole focus on credit risk, its one-size-fits all risk weight for nonmortgage loans, its inability to adjust weights for hedges, portfolio diversification, and management controls, and the difficulties of folding in interest rate risk, to name a few Most, if not all, of these problems were known before adoption Most, if not all, are addressed judgmentally by the supervisors in their case-by-case onsite examination and review Nonetheless, despite these efforts and greater attention to internal bank risk management and control, our current procedures are linked too closely, in my view, to the risk-based capital ratio At the same time, the market place has become more complicated in ways that risk-based capital rules cannot handle, even with the increasing complexity of the rules These market complexities, however, would not have occurred without the same technology that has recently made it possible to quantify risks that only a short time ago we could just conceptualize Like internal models for measuring risk on trading positions, quantifiable measures for other risks make it possible for banks and others to choose more carefully their risk positions and better link those positions to the appropriate capital levels Consider securitization, which, of course, has been evolving for several years, but is, in an important sense, a paradigm of the evolving risk management techniques in financial markets In a typical secuntization, the sponsoring entity â€” which is often a bank â€” establishes a special purpose vehicle, or conduit, that acquires a loan pool from an originator Frequently, to exploit regulatory loopholes, the conduit itself originates the loans The conduit then issues varying tranches of securities to fund the loan pool It achieves double- or tnple-A ratings on most of these securities by providing for their credit enhancement, typically by having the sponsor purchase the most junior securities, which are structured to absorb virtually all of the credit risk inherent in the underlying loan pool The sponsoring bank retains all of the residual spread between the return on the loan pool and the costs incurred by the conduit, including the interest and noninterest costs on the loan-backed securities For present purposes, what is most critical about secuntizations is that the participants â€” the originator and the credit enhancer (who are often one and the same), as well as the purchasers of the senior securities â€” all need to have a fairly clear and quantifiable idea of their risk exposure Typically, however, bank loans are opaque to outsiders, making such knowledge hard, if not impossible, to come by Nevertheless, this problem often can be overcome by using loan portfolios with standard loan contracts having well-known characteristics â€” like credit card and auto loans â€” or by overcollateralizing, or by providing appropriate levels of credit enhancement Most often a combination of these is used While perhaps not designed originally with the purpose in mind, one method for making such loans more amenable to securitization is credit scoring Credit scoring applies formal statistical procedures to the credit decision process By subjecting loans to uniform underwriting standards, credit scoring facilitates analysis of the credit risk inherent in a securitized loan pool Such procedures are being applied to an ever wider array of bank loans, including, most notably, small business loans In the future, one can thus expect to see an increasing volume of secuntized small business loans that are not guaranteed by the SBA It is also worth emphasizing that the credit scoring exercise â€” and the market evaluation accompanying secuntizations of loan pools â€” requires that banks capture, monitor, study, and present historical loss data on a large volume of their loans The development of such data bases was a necessary prerequisite to mortgage, credit card, and auto loan securitization Such data bases will be equally critical not only to the evolving technology of internal risk management at banks and for secuntization of other loan pools, but, as I will be noting shortly, also for evaluations of risk by the supervisor/regulator A brief digression may be useful at this point A common misunderstanding of credit scoring and securitization is that both will cause banks to refrain from making the nonstandard loans that their special knowledge has made possible, including the credits that, in the past, I have referred to as character loans It is also sometimes argued that secuntization of loans will undermine the economic franchise of banking, driving down spreads on the last profitable credit function in the banks' economic franchise But such a result is not at all preordained, especially for those banks willing and able to take advantage of new technologies Of course, the new technologies of loan standardization and credit scoring can be viewed as chipping away at the monopoly rents associated with specialized knowledge of the local loan customer In effect, barriers to entry are lowered when the new technologies allow nonlocal competitors to offer standardized products through nationwide marketing campaigns using toll-free "800" telephone numbers But the by-products of standardization and credit-scoring include lower underwriting expenses and the more accurate estimation of loss probability distributions These byproducts act to offset the effects of a reduction in barriers to entry, both by raising profits on existing operations and by opening up opportunities with customers previously not served Better and quantifiable estimates of risk are tantamount to risk reduction Moreover, securitization, by expanding lower cost funding sources, increases the ability of banks to make more loans and to diversify their risks Risk reduction, lower funding costs, and lower noninterest costs in making the credit decision, all act to increase banks' risk-adjusted rate of return In addition, banks can, will, and do, continue to make the nonstandard loan based on judgment and asymmetrical information, retaining the resultant whole loan in their portfolios Indeed, the new technology should enable banks efficiently to evaluate borrowers they could not assess in a cost-efficient way before Thus, new banking opportunities will be opened The new procedures I have just described also induce banks to price all loans â€” but especially nonstandard loans â€” more accurately to reflect their true costs and risks This, too, works to increase risk-adjusted rates of return and results in a better allocation of resources True, some banks, unwilling or unable to adapt to the changing technology, will lose market share and perhaps suffer lower rates of return But the banks that embrace the cost-cutting and risk-reducing effects of the technology will, in my judgment, tend to find it a rewarding experience Beyond credit scoring and securitization, larger banks are moving into new areas of risk evaluation for internal management purposes, including the quantification of credit risk Most large banking organizations have â€” or are developing â€” procedures for allocating capital against various types of loans, based on estimates of credit risk for various categories For example, in middle market lending at these institutions, a first step is to classify loans into various rating categories â€” usually 1 to 10, with 1-rated loans being equivalent to tripleâ€”A securities and 10-rated loans about to be written off as loss Periodically, each loan is re-evaluated and re-categorized if necessary Such categorizations have been done for some time, but the more sophisticated banks are going an important step beyond this point They are using historical data to estimate the mean and variance of defaults and actual losses on each grade of loan The result can be interpreted as attempting to infer the loss probability distribution for each category or subportfolio of loans, and for the entire loan portfolio Consider how such information can be used Estimates of expected losses and the probability distribution of unexpected losses are critical for pricing credits correctly and deciding whether competitive market rates thus imply withdrawing, cutting back, or expanding various types of credit A prerequisite, however, is the judgment by management as to the proper amount of capital to allocate to each of the subportfolios or risk categories so that risk-adjusted rates of return can be calculated The most common approach is to allocate sufficient capital so that the probability of actual credit loss exceeding the allocated capital is no greater than, say, one-half percent This probability "target," in turn, could be arbitrarily chosen or selected to be consistent with, say, maintaining a double-A bond rating on the bank's own debt These capital allocations, as I noted, are for internal management, not regulatory, purposes But I am impressed with what they teach us, the regulators, and what they imply for regulatory capital The internal capital allocations used by banks range from less than 2 percent for highly rated loans to 20 percent or more for the most risky credits In addition, credit enhancements, such as most junior positions in secuntized loan pools, can have theoretical capital allocations that widen still further the range of appropriate internal capital allocations Compare this wide range of internal capital allocations with the 8 percent, one-size-fits-all Basle standard In fact the average risk-based capital ratio for U S banks approaches 12 percent for large banks, far above the 8 percent minimum Nonetheless, consider the contradiction implicit when a bank with a 12 percent risk weighted capital ratio may be viewed by the public as having a strong capital position when the bank's own capital allocation models suggest that it should have 15 percent capital, or more The supervisor, I believe, is not being misled in most such cases, and is making the appropriate judgmental adjustments Moreover, the markets clearly make such adjustments I note that the banks with very high risk-based capital ratios still do not achieve tripleâ€”A ratings on their debt, and some do not even have single-A ratings One can conceive of a bank following a portfolio policy that would engender an average internal capital allocation that would be well below our 8 percent minimum In such a case, our rules would significantly disadvantage the bank and induce it to find loopholes and to engage in regulatory arbitrage to avoid the standard But consider a bank carrying capital considerably above what the regulatory guidelines suggest, but below what the bank's own internal capital allocation procedures imply Such a bank has no reason to adjust its position for regulatory purposes if the supervisor does not see through the veil of nominally high regulatory capital As I noted, I believe that supervisors generally have been able to do so But should they fail to see through that veil, in an environment of increasingly complicated financial transactions, there could be a serious inconsistency between our desired regulatory soundness standard and actual bank risk levels Federal Reserve staff members are beginning a review of the major banks' internal credit risk-capital allocation models in order to understand better the strengths and weaknesses of these models We already know, however, that there has been an irreversible application of risk measurement technology without which banks would not be able to design, price, and manage many of the newer financial products, like credit derivatives These same or similar technologies can and are beginning to be used to price and manage traditional banking products Some of these developments are at an early stage, and all are evolving rapidly Today's technology allows us to measure risk in ways that were unthinkable a decade ago The next decade will likely produce further dramatic change But already today, the markets â€” including credit rating agencies â€” are using these quantitative tools Indeed, for the first time, we can seriously begin to contemplate a regulatory quantification of what we mean by "soundness " Recall that while the objective of bank regulation and supervision is to assure a minimum level of prudential soundness, the precise meaning of soundness has always been tenuous and illâ€”defined This is why judgment has been, and will continue to be, a critical component of prudential supervision However, the technology and techniques banks have developed, and are developing, allow us greatly to improve that judgment by constructing measures of soundness in probability terms If we can obtain reasonable estimates of portfolio loss distributions, soundness can be defined, for example, as the probability of losses exceeding capital In other words, soundness can be defined in terms of a quantifiable insolvency probability Moreover, one can conceive of definitions of soundness that go beyond simply the probability of insolvency to encompass also the level and variability of losses to the FDIC in the event of insolvency Going still further, regulatory targets for quantifiable soundness could be made to reflect market-based goals For example, soundness could be defined in terms of some implied, minimum credit rating for the bank's deposits, as if they were uninsured All of these approaches, however, require the regulators to establish targets regarding acceptable failure rates or the FDIC's exposure to potential losses Note that a bank could meet any particular quantitative soundness standard by increasing its capital or by reducing the risk of its portfolio I do not mean to suggest that we have reached the point at which we can now establish quantitatively precise soundness standards We have not These procedures are in their infancy and are hampered by the lack of historical micro data bases which have to be laboriously constructed at, or by, individual banks Moreover, ascertaining relevant probabilities, the basis of an evaluation of soundness, presupposes an estimation of the shape of these distributions, arguably the most difficult aspect of this process The technical methodology is also changing with experience and with conceptual progress in the academic and professional communities As I noted, we have already decided to use internal bank model approaches for measuring market risks at banks and allocating regulatory capital to those risks In addition, the Federal Reserve Board has been studying an alternative capital allocation process for market risk, the so-called "pre-commitment" approach This methodology would provide market and other financial incentives for banks to choose capital allocations for trading risk that are consistent with their own risk management capabilities, as well as with regulatory objectives With the Board's encouragement, the New York Clearing House Association is organizing a pilot study of the pre-commitment approach The next natural step is to begin to review ways to harness, for supervisory purposes, the banks' own models for the measurement of credit risk The private sector, for a considerable time, has been accustomed to product planning cycles â€” created by rapid technological change â€” in which the planning of the replacement product is begun, if not well along, by the time a new product is being introduced The United States banking system is not only the largest in the world, but it is also the most complex and the most innovative We cannot escape the reality that the banking supervisors and regulators will have to innovate to continue to carry out their responsibilities Bank, and more generally financial institution supervision, is, of necessity, a continually evolving process reflecting the continually changing structure and policies of the supervised institutions We will eventually correct, for example, all, or most, of the anomalies which we perceive in risk-based capital, only in a few years to be required to "correct" those corrections This is not a fault, but a description of an appropriate regulatory process Indeed, given our own long lead times, we, like banks and nonfinancial firms for their products, must begin designing the next generation of supervisory procedures even while introducing the latest modification What about principles that can be developed to address the original question of this conference What should regulators do? In light of my remarks this morning, let me suggest a basic principle Whenever possible, regulators should use approaches to regulation and supervision that include or simulate market techniques and signals Importantly, our soundness standards should be no more or no less stringent than those the market place would impose In the unregulated market, of course, a financial firm can take on any amount of insolvency risk it wishes, and the market will rate its liabilities, and price them, accordingly Unfortunately, we do not have a system in which deposit insurance premiums are permitted to vary as widely as simulating that response would require But, at least theoretically, we can adjust the individual bank's regulatory capital requirement to offset the reduction in market discipline attributed to the safety net Perfection would occur if bankers had a genuinely difficult choice deciding if they really wanted to remain an insured bank or become an unregulated financial institution In the final analysis, such an approach is the only way to control the moral hazard of the safety net, to square the circle in balancing stability requirements with risk-taking An important â€” and increasingly feasible â€” prerequisite in achieving that balance is for the regulators to quantify what their goals are, especially what is meant by "soundness " Measuring actual risks relative to these goals would be facilitated if regulators harness for supervisory purposes the market-oriented tools already used internally by banks for management purposes When seeking to implement this principle and utilize new technologies, we must take care to remember that we are unlikely ever to be able to measure risk in absolutely precise ways Quantification procedures are still extrapolations of the past, and behavior is always changing Models wil still doubtless be haunted by specification and estimation errors The world will still remain a highly complex place, and I have no doubt that financial participants and markets will continue to invent instruments and procedures that models will not be able to capture until sufficient experience is gained Thus, neither am I proposing nor do I anticipate that bank supervisors will be relying on a black box based on statistical and econometric rules I am suggesting, however, that new paradigms are in the process of evolving which will provide us with tools that will permit greater quantification of both risk standards and risk management Such quantification will not solve all of our problems, nor will it ever substitute for human judgment, which is the only technology we have available to parse the most difficult regulatory problems Nonetheless, quantification will facilitate great improvements in both risk management and what regulators will be able to do The financial world is dynamic and I have little doubt that there will be a continuous need to modify what we develop In the end, judgment must be augmented with technology, and technology must be tempered with judgment</t>
-  </si>
-  <si>
-    <t>Lord Mayor, ladies, and gentlemen, it is an honor to be in this city to talk about the evolution of global finance To be sure, participants in Frankfurt's financial markets have not been coronated as were some of the Holy Roman Emperors depicted in this magnificent room But the impact of the Bundesbank, of the private institutions active here, and of the prospective European Central Bank has been, and no doubt will be, profound This evening, I will not talk specifically about Frankfurt or the implications of EMU, and certainly not about the Holy Roman Empire, but rather about the evolution of global financial markets in general. World financial markets are far more efficient today than ever before Changes in communications and information technology, and the new instruments and nsk-management techniques they have made possible, enable an ever wider range of financial and nonfinancial firms to manage their financial risks more effectively They can now concentrate on managing the economic risks associated with their primary businesses Still, for central bankers with responsibilities for financial market stability, the new technologies and new instruments have presented new challenges Some argue that market dynamics have been altered in ways that increase the likelihood of significant market disruptions Whatever the merits of this argument, there is a clear sense that the new technologies, and the financial instruments and techniques they have made possible, have strengthened interdependencies between markets and market participants, both within and across national boundaries As a result, a disturbance in one market segment or one country is likely to be transmitted far more rapidly throughout the world economy than was evident in earlier eras A global financial system, of course, is not an end in itself It is the institutional structure that has developed over the centuries to facilitate the world-wide production of goods and services Accordingly, we can better understand the evolution of today's burgeoning financial markets by parsing the extraordinary changes that have emerged, in the past century or more, in what we conventionally call the real side of economies the production of goods and services The same technological forces currently driving finance were first evident in the production process and have had a profound effect on what we produce, how we produce it, and how it is financed Technological change or, more generally, ideas have increasingly altered the nature of output so that it has become progressively more conceptual and less physical In the United States, for example, the weight of our gross domestic product today measured in tons is only modestly higher than several decades ago The huge rise in the real, or price-adjusted, value of output since then is the result much more of the generation and development of ideas than of the exploitation and transformation of physical resources As a consequence, a much smaller proportion of the measured real gross domestic product constitutes physical bulk currently than in past generations Because the accretion of knowledge is, with rare exceptions, irreversible, this trend almost surely will continue into the 21st century and beyond The changes in what we usually view as physical product have been dramatic The purpose of production, of course, has remained the same to serve human needs and values But output of comparable utility now generally is smaller and lighter Our radios used to be activated by large vacuum tubes, today we have pocket-sized transistors to perform the same function Thin fiber optics have replaced huge tonnages of copper wire Advances in architecture and engineering, as well as the development of lighter but stronger materials, now give us the same working space in buildings but with significantly less concrete, glass, and steel tonnage than was required in an earlier era The process is interactive The development of the insights that brought us central heating enabled lighter-weight apparel fabrics to displace the heavier cloths of the past The breakthroughs in medical research that have revolutionized health care are only the beginning of a growing list of almost wholly conceptual elements in our economic output As the relative cost of transporting goods falls dramatically as a consequence of such physical downsizing, the rising conceptual content of output becomes a major factor in the increasingly rapid globalization of merchandise trade International trade in, say, construction gravel or scrap metal is limited by weight or bulk High-value computer products, in contrast, make up an expanding share of world trade Obviously, the less the bulk and the lower the weight, the easier goods are to move, especially over long distances and across national boundaries Thus, for the United States, after we adjust for average price changes, tons shipped per real dollar of both U S exports and imports are now less than half of what they were in 1970 The downsizing of American trade is patently a reflection of the extent to which conceptualization is also dominating the economies of our trading partners throughout the world Of course, a significant part of the pronounced expansion in international trade has resulted from the breaking down of trade barriers over the years However, the political processes that have led in that direction to an important extent have been themselves pushed by the technological changes in the composition of goods and services Not unexpectedly, as goods and services have moved across borders, the necessity to finance them has increased dramatically But what is particularly startling is how large the expansion in cross-border finance has become, relative to the trade it finances To be sure, much cross-border finance supports investment portfolios, doubtless some largely speculative But in the end, even they are part of the support systems for the efficient international movement of goods and services The relative expansion of cross-border financial transactions is, in itself, another manifestation of conceptual trade, as a single financial product is broken into many pieces that, in turn, are traded Specifically, world trade measured in nominal dollars was 2 1/3 times as large in 1994 as it was a decade earlier The stock of cross-border assets held on balance sheets by banks at the end of 1994, also in dollars, was more than 3 times as large as at the end of 1984 Off-balance-sheet growth has been, of course, much larger Nonbank cross-border transactions have also grown enormously Such rapid expansion in cross-border banking and finance should not be surprising given the extent to which low-cost information processing and communications technology have improved the ability of customers in one part of the world to avail themselves of opportunities offered anywhere in the world on a real-time basis These developments enhance the process whereby an excess of saving over investment in one country finds an appropriate outlet in another In short, they facilitate the drive to equate risk-adjusted rates of return on investments worldwide They thereby improve the worldwide allocation of scarce capital and, in the process, engender a huge increase in risk dispersion and hedging opportunities If we can resist protectionist pressures in our societies in the financial arena as well as in the interchange of goods and services, we can look forward to the benefits of the international division of labor on a much larger scale in the 21 st century What we don't know for sure, but strongly suspect, is that the accelerating expansion of global finance may be indispensable to the continued rapid growth in world trade in goods and services It is becoming increasingly evident that many layers of financial intermediation will be required if we are to capture the full benefits of our advances in finance Certainly, the emergence of a highly liquid foreign exchange market has facilitated basic forex transactions, and the availability of more complex hedging strategies enables producers and investors to achieve their desired risk positions This owes largely to the ability of modem financial products to unbundle complex risks in ways that enable each counterparty to choose the combination of risks necessary to advance its business strategy, and to eschew those that do not This process enhances cross-border trade in goods and services, facilitates portfolio investment strategies, enhances the lower-cost financing of real capital formation on a worldwide basis and, hence, leads to an expansion of international trade and rising standards of living Achieving those benefits surely will require the maintenance of a stable macroeconomic environment An environment conducive to stable product pnces and to maintaining sustainable economic growth is a prime responsibility of governments and, of course, central banks How well we central bankers do our job has implications for participants in financial markets We provide the backdrop against which individual market participants make their decisions In the context of rapid financial market changes, disruptions are inevitable The turmoil in the European Exchange Rate mechanism in 1992 and the plunge in the exchange value of the Mexican peso at the end of 1994 and early in 1995 have shown, for example, how the new world of financial trading can punish policy misalignments with amazing alacrity Notwithstanding, the economic consequences of such disruptions will be minimized if they are not further compounded by financial instability associated with fluctuations in underlying inflation trends Reserve currency countries, like the United States, have a special responsibility to provide an anchor of stability for themselves and the world at large Such countries face a high demand for their financial instruments, a substantial share of which is related to volatile portfolio motives As international financial markets continue to expand, central banks thus have twin objectives fostering macroeconomic stability and maintaining safe and sound financial institutions that can take advantage of stability while exploiting the advantages of new technological advances The changing dynamics of modern global financial systems require that central banks address the inevitable increase of potential systemic risk It is probably fair to say that the very efficiency of global financial markets, engendered by the rapid proliferation of financial products, also has the capability of transmitting mistakes at a far faster pace throughout the financial system in ways that were unknown a generation ago, and not even remotely imagined in the 19th century Certainly, last year's Barings Brothers collapse shows how much more rapidly losses can be generated in the current environment relative to a century earlier when Barings Brothers confronted a similar episode Current technology enables single individuals to initiate massive transactions with very rapid execution Clearly, not only has the productivity of global finance increased markedly, but so, obviously, has the ability to generate losses at a previously inconceivable rate Moreover, increasing global financial efficiency, by creating the mechanisms for mistakes to ricochet throughout the global financial system, has patently increased the potential for systemic risk Why not then, one might ask, bar or contain the expansion of global finance by capital controls, transaction taxes, or other market inhibiting initiatives Why not return to the less hectic and seemingly less threatening markets of earlier years' Endeavoring to thwart technological advance and new knowledge and innovation through the erection of barriers to the spread of knowledge would, as history amply demonstrates, have large, doubtless adverse, unintended consequences Suppressed markets in one location would be rapidly displaced by others outside the reach of government controls and taxes Of greater importance, risk-taking, so indispensable to the creation of wealth, would surely be curbed, to the detriment of rising living standards We cannot turn back the clock, and we should not try to do so Rather, we should recognize that, if it is technology that has imparted the current stress to markets, technology can be employed to contain it Enhancements to financial institutions' internal nsk-management systems arguably constitute one of the most effective countermeasures to the increased potential instability of the global financial system Improving the efficiency of the world's payment systems is clearly another The availability of new technology and new derivative financial instruments has facilitated new, more rigorous approaches to the conceptualization, measurement, and management of risk There are, however, limitations to the statistical models used in such systems owing to the necessity of overly simplifying assumptions Hence, human judgments, based on analytically looser but far more realistic evaluations of what the future may hold, are of critical importance in nsk management Although a sophisticated understanding of statistical modeling techniques is important to risk management, an intimate knowledge of the markets in which an institution trades, and of the customers it serves, is turning out to be far more important In one sense, risk-management systems were exposed to a very severe real-life stress test in 1994, when sharp increases in interest rates created large losses in fixed income markets I assume that as a consequence, firms' models and judgments are sounder today than those that prevailed in early 1994 But the Barings episode suggests that further improvements to internal risk-management systems as well as internal controls are needed, in some instances very significant improvements To be sure, we should recognize also that if we choose to have the advantages of a leveraged system of financial intermedianes the burden of managing risk in the financial system will not lie with the pnvate sector alone With leveraging there will always exist a remote possibility of a chain reaction, a cascading sequence of defaults that will culminate in financial implosion if it proceeds unchecked Only a central bank, with unlimited power to create money, can with a high probability thwart such a process before it becomes destructive Hence, central banks will of necessity be drawn into becoming lenders of last resort But implicit in the existence of such a role is that there will be some sort of allocation between the public and private sectors of the burden of risk of extreme outcomes Thus, central banks are led to provide what essentially amounts to catastrophic financial insurance coverage Such a public subsidy should be reserved for only the rarest of disasters, triggered, at most, a handful of times per century If the owners or managers of private financial institutions were to anticipate being propped up frequently by government support, it would only encourage reckless and irresponsible management practices In theory, the allocation of responsibility for risk-bearing between the private sector and the central bank depends upon an evaluation of the private cost of capital In order to attract, or at least retain, capital, a private financial institution must earn at minimum the overall economy's rate of return, adjusted for risk In competitive financial markets, the greater the leverage, the higher the rate of return, before adjustment for risk If private financial institutions have to absorb all financial risk, then the degree to which they can leverage will be limited, the financial sector small, and its contribution to economic growth, minimal On the other hand, if central banks effectively insulate private institutions from the largest potential losses, however incurred, increased laxity could threaten a major drain on taxpayers or produce inflationary instability as a consequence of excess money creation In practice, the policy choice of how much, if any, of the extreme market risk that central banks should absorb is fraught with many complexities Yet we central bankers make this decision every day, either explicitly or by default It does seem clear, however, that under the currently structured international financial system, if central banks do not choose to absorb the most extreme risks, private financial institutions will surely be daunted by the specter of unlikely, but enormous and unhedgable losses Private institutions would naturally adopt an attitude of caution that would render them far less effective in the financing of wealth creation Nonetheless, as experience amply demonstrates, all risk with limited and extreme exceptions must remain within the private financial system The probability that central banks can thwart the kind of chain reaction to which I just referred will be immeasurably enhanced if world payment systems can achieve something closer to real time settlement Herstatt and other time dependent risks are deceptively large, as the report issued in March by the BIS Committee on Payment and Settlement Systems has now made clear Technology has already markedly contained this nsk by shortening the payment and settlement cycle of a broad segment of financial transactions Reducing float, of course, requires costly investments in computer and telecommunications technology, as well as the opportunity costs associated with holding large cash and securities balances to effect settlements In that sense reducing float implies a significant tradeoff between risk reduction and cost But while technological advances and lower costs have increased the risk of systemic breakdown, so has the same technology enabled the financial community, both pnvate and public, to contain such nsks In conclusion, we must assure that our rapidly changing global financial system retains the capacity to contain market shocks This is a never-ending process Mutual self interest in an expanding global financial system is fostering broadening cooperation among the monetary authorities of the larger trading nations The markets are beginning to dictate a merging of interests not only on the monetary front, but in fiscal affairs, as well As last year's G-10 study on Saving, Investment and Real Interest Rates pointed out, "the effects on real interest rates of changes in fiscal deficits in one country are now spread across all countries integrated into the global financial system " Clearly, the challenges of the changing international environment in which we all operate dictate that public officials and pnvate market participants maintain and strengthen the sound working relationships that we have built up in recent years These relationships epitomize the kinds of contacts that will be essential in meeting the common challenges of the rest of this decade and into the 21st century</t>
-  </si>
-  <si>
-    <t>I regret that I was unable to join you for the earlier portions of this conference I know that you've had some important explorations of the process through which technology contributes to economic growth What I'd like to do in this session is perhaps augment these discussions by shifting gears a bit I would like to focus on the question of how people perceive the benefits of recent technological change Today a truly puzzling phenomenon confronts the American economy I refer to the pervasiveness of job insecurity in the context of an economic recovery that has been running for more than five years, inflation that has been contained, and a layoff rate that is historically quite low Yet, in the face of all this seemingly good news, a sense persists that something is fundamentally wrong This afternoon I want to try to explain where I believe the insecurity is coming from and, I hope, raise some suggestions as to how it might be assuaged The issue, as best I can judge, appears to be rooted in one of those rare, perhaps once-in-a-century events--a structural technological advance The advent of the transistor and the integrated circuit and, as a consequence, the emergence of modern computer, telecommunication, and satellite technologies have fundamentally changed the structure of the American economy Since the beginning of the industrial revolution, our economy and, to only a slightly lesser degree, the economies of our industrial trading partners have been progressing toward a regime in which abstract ideas and concepts are the dominant element in the creation of economic value A hundred years ago, physical brawn was critical to value-added determination People who personally could lift rolled sheet steel and help haul it from one part of the plant to another performed an activity that was valuable in the marketplace Today, several generations later, the structure of production has become, to a remarkable degree, idea-determined On the output side, at the turn of the twentieth century, we produced steel, industrial chemicals, and heavy fabrics in abundance, what impressed was the very size and bulk of the productive facilities and the output itself Today, the products that we find remarkable are those that are lighter, smaller, and in some cases, almost invisible Our radios used to be activated by large vacuum tubes, today we have pocket-sized transistors to perform the same function Thin fiber optic cables have replaced huge tonnages of copper wire In the past, buildings were so over-structured and sturdy that, when their time for replacement arrived, demolition was a Herculean task Owing to conceptual advances in metallurgy, engineering, and architectural design, we now can create as much or more space with fewer materials Indeed, such advances have created an overall national output whose physical weight probably is only modestly greater than that of whatever we produced a hundred years ago Real GDP, that is price-adjusted value-added, of course, is much higher today, and by far, ideas account for the difference That trend will doubtless continue because idea creation is irreversible Knowledge, once acquired, does not disappear If anything, this process has accelerated in recent years, and that acceleration seems to have had two important side effects First, it has had a major influence on the distribution of income in this country, and second, a related but different concept, it has imparted a degree of insecurity, uncertainty, and even fear to a vast segment of job holders The consequence of both effects, as I will explain shortly, has been to create a sense that something in the economy is awry, which is wholly at odds with what the macroeconomic data seemingly imply--economic success, tranquility, and progress The roots of this puzzling situation go back a few decades As ideas became especially valuable relative to physical activity in the creation of value-added, education and intellectual skill became increasingly major determinants of income Throughout the 1960s and 1970s, the rapid rise in the number of college graduates apparently kept the supply of educated workers moving up with the demand However, by the latter 1970s and into the 1980s, demand seemed to have outstripped supply, the apparent consequence was a fairly pronounced rise in compensation going to college graduates relative to the compensation going to those who had only high school diplomas A similar disparity of earnings developed between those who had graduated from high school and those who had dropped out After the mid -1970s, productivity slowed quite markedly, for reasons that are not wholly apparent, and so did average real incomes As a consequence, the widening disparity also means that a not insignificant portion of our work force--primarily those whose work involves less conceptual activities--has been experiencing either stagnant or falling real incomes in the past ten or fifteen years A substantial number of these people understandably feel that they have been on a treadmill and are barely able to make ends meet from their incomes That feeling has engendered significant concerns about economic and financial well-being among this part of our work force I suspect that other concerns affect an even larger group--composed of those who have average or above incomes and have been employed in their current jobs for a number of years These are the people with higher skills, who interact closely day by day with the high-tech part of our capital stock Because that stock, reflecting computer and telecommunications-based technologies, is turning over very rapidly, the involved workers have a high degree of uncertainty and insecurity about their jobs As one affected employee commented to a Wall Street Journal reporter a couple of weeks ago, "Is somebody getting ready to change my whole life for me?" These workers perceive the job skills that they have acquired through high school or college to be increasingly open to competitive challenge One must wonder how highly skilled, turn-of-the-century telegraphers felt with the onset of the telephone or the skilled buggy-whip craftsman with the advent of the automobile Today, large numbers of people have become so demonstrably insecure about whether their skills will still be relevant in, say, five years that they fear for their jobs This insecurity is evidenced by the fact that they have increasingly forgone wage hikes for job security As a consequence, the past few years have been a period of extraordinary labor peace In fact, 1995 had the lowest strike record for a half-century Moreover, labor contracts, which historically almost never extended beyond thirty-six months, are now sometimes going out five and six years, as people try to lock in job security, often willing to forgo significant wage increases in the process This sense of job insecurity is so deep that many workers are truly scared Some fear that their skills will no longer be appropriate for the future Some fear their ability to make ends meet in the future Many appear truly concerned about a prospective decline in their standard of living Journal, May 16, 1996, page A 16 This development is startling considering the overall state of the economy suggested by the macroeconomic data It is certainly the case that average real income has slowed and that the disparity in real incomes has widened After reaching a postwar low in the late 1960s, income disparities, as measured by Gini coefficients, climbed steadily through 1994--the most recent year for which data are available Moreover, disparities in the distribution of wealth (net worth) as measured by the Federal Reserve's Survey of Consumer Finances also widened significantly between the surveys taken in 1963 and 1992, with much of that increase in Gini coefficients occurring during the 1980s Doubtless, that disparity has widened further in recent years in the wake of major increases in stock and bond prices But the notion that the economic well-being of the lower-income segments of our workforce has deteriorated as much as might be suggested by the widening disparities in the income and wealth statistics is open to question I say this because there is a surprising difference between trends in the dispersion of holdings of claims to goods and services (that is, income and wealth) and trends in the dispersion of actual consumption, which is, of course, the ultimate determinant of material or economic well-being Put another way, well-being is determined by things people consume, either directly from their incomes and accumulated savings or indirectly from the stock of household goods they already own--automobiles, telephones, TVs, VCRs, and so forth, not to mention the homes themselves And disparities in consumption and ownership of hard goods don't appear to have widened nearly as much as income disparities I do not wish to disparage income as a partial antidote to insecurity Nevertheless, some aspects of economic well-being may be more accurately discerned by examining consumption A number of researchers have compared trends in the distribution of consumption with the distribution of income Many of these studies rely on data from the Consumer Expenditure Survey that the Bureau of Labor Statistics conducts, and much of the analytical research on distributional issues has been carried out by BLS economists A recent study by David Johnson and Stephanie Shipp of the BLS finds that "income inequality is more volatile than consumption and the level is about 3 0 percent more than that of consumption inequality " These findings are not surprising As is well known, consumers tend to maintain their levels of consumption in the face of temporary changes in income Variations in asset holdings and debt buffer changes in income In short, consumption patterns tend to look more like patterns in income that has been averaged over several years, rather than the one- year convention of our statistics But, besides finding differences in the levels of consumption and income inequality, Johnson and Shipp find differences in the inequality trends In particular, although consumption inequality has increased, on average, since 1981, the rise has been only three-fourths as large as that of income inequality (see table 1) An evaluation that views consumption not in terms of outlays but, rather, in terms of the flow of services that come from purchases indicates an additional qualification The reason, of course, for examining the flow of services from spending, and not just current-period spending alone, is that while outlays for food and haircuts, for example, are consumed immediately, a television set that is purchased today provides entertainment over its entire service life Thus, unless ownership of household appliances and other consumer durables is brought into the evaluation, the story of the dispersion of material well- being is incomplete What do the numbers show? During the 1960s and 1970s, the real net stock of consumer durables per household increased an average of 3 1 percent per year The average growth rate has slowed slightly since then--to a pace of 2-1/2 percent--but all of that slowing occurred during the recessions of 1980 and 1981-82 Indeed, since 1982 households have been adding to their stock of durables at an annual rate per household of 3 3 percent--slightly faster than in the 'sixties and 'seventies Moreover, we have apparently not had a widening disparity in holdings of hard assets like the one that appears in the income and wealth data Stephanie Shipp and her colleagues in the Division of Consumer Expenditure Surveys at the BLS generously provided the Board's staff with detailed tabulations of the ownership of consumer goods and vehicles by income decile To be sure, these data show that ownership rates for consumer durables clearly rise with income But the data also show that for motor vehicles and a number of appliances--for example, dishwashers, clothes dryers, microwave ovens, and even garbage disposals--the distribution of ownership rates by income decile moved toward greater equality between 1980 and 1994 For some consumer goods we are moving toward greater equality because the proportion of households with access to these items is moving close to saturation For example, nearly all poor families have access to a refrigerator, stove, and color TV In addition, three-fourths of poor households have telephones, and nearly two-thirds have microwave ovens and VCRs These encouraging findings are not without qualification, however As an example, for personal computers, which nowadays are critical for economic success, the disparity in ownership rates is quite large--around 10 percent for lower-income households in 1994 compared with more than 50 percent for the highest-income decile And, even when most families own a durable good or vehicle, the number owned by the low-income group typically is less than that owned by the upper-income groups For example, in 1994 lower-income families owned slightly more than one color television set, on average, whereas high-income families tended to own more than two The figures for motor vehicles are similar--slightly under one per household at the lower end of the income distribution and slightly more than two at the upper end Nonetheless, even though the inequality in the number of units owned per household is often greater than that in the ownership rate, the degree of inequality measured on this basis narrowed between 1984 and 1994 in a manner similar to the shifts for ownership rates (compare tables 2 and 3 ) But, even if the number of hard assets per family were the same for rich and poor, it is not evident how much this would assuage the current deep-seated sense of insecurity that pervades such a large segment of our workforce Clearly, there is more to economic security than owning consumer durables In fact, the very forces that load our households with every sort of gadget come from an economy that apparently is changing too quickly for many Americans to absorb readily Accelerated change fosters fear in all walks of life It is a rational human response to such an imperative Finding a solution to such insecurity is not simple If 30b insecurity is largely a fear of skill obsolescence, real or imagined, some way must be found to enhance skills People who believe that their skills are up to date and readily marketable do not inordinately fear job layoffs Bolstered by signals from the marketplace, education is clearly increasingly becoming a lifetime activity Resting on one's skills as the world rapidly goes by will only intensify a sense of job insecurity Ongoing schooling and training are becoming ever more relevant for the average worker Fortunately, developing human capital is rapidly being perceived by many corporations as adding to shareholder value If ideas are increasingly the factor that engenders value-added, then training and education are crucial to the expansion of company value-added and profitability As a consequence, corporate universities are emerging as a growth industry in this country A significant and expanding number of companies require that employees attend class, say, twice a week, at company expense, to augment their on-the-job techniques Moreover, there is a growing peripheral industry whose basic product is to train company employees in the latest technologies Such trends should decidedly be encouraged Hopefully, in that environment efforts to increase the competitive skills of workers in the lower half of the income distribution will succeed in narrowing income disparities At this point it is unclear whether the particular current surge of technology is peaking and will eventually slow down or whether we are in its early stages Much of this surge may well represent more wheel-spinning than real increases in production, as our subdued national productivity data suggest Nathan Rosenberg in his paper for this conference points out that organizational changes and further development of complementary technologies likely will be required before we see the productivity payoff to computer technology If so, as the infrastructure of the economy finally adjusts itself to the new semiconductor-based revolution, the rapid changes are likely to finally become more evident in increased measured productivity and growth In any event, a new world is emerging The twenty-first century will be different--much more rapidly paced and changing than any of us who have been around for a while have experienced in our lifetimes There will be a different America out there Fortunately, job insecurity does not appear to be a problem for a 21-year-old who has experienced nothing else, and even less for a 6-year-old who seems to be far more computer literate than grandfather As a consequence, with the inexorable turnover of the population, people will adjust When we go through a period of transition, inevitable symptoms of friction, uncertainty, and fear arise They will pass Technical Note The raw data on the ownership rates of consumer durables by income decile are not in a form that can be used directly to calculate standard measures of inequality ( e g , Gini coefficients or mean log deviations) However, William Cleveland of the Board's staff suggested a transformation of the raw data that allows one to calculate a measure of inequality that looks like a Gini coefficient This note describes the procedure The first step is to transform the raw data into a discrete probability distribution In the case of ownership rates for consumer durables, the calculation for a given consumer good is where p is the fraction of all households that own the consumer good who are in income decile 1, and r is the actual ownership rate for the 1 decile By construction, the sum of the p ' s is equal to one For goods that have ownership rates that are relatively equal across deciles (regardless of the level of the ownership rate), these probability distributions are fairly flat, with values of p close to 0 1 For goods that are more concentrated among the affluent households, the probability distributions tend to rise across income deciles The next step is to take the probability distributions and create cumulative probability distributions (CPD) (e g , the value of the CPD for the second decile equals p + p ) The CPDs look like Lorenz curves The standard formula for the Gini coefficient is then used to construct a measure of the degree of inequality implied by the CPDs These are shown in table 2 The calculation of "Gini coefficients" for the average number of units owned per household in each income decile (u ) is the same, except u is substitued for r in equation 1 These "Gini coefficients" are shown in table 3</t>
-  </si>
-  <si>
-    <t>I am honored to present the William Taylor Memorial Lecture to such a distinguished group of senior bank supervisors from around the world I am especially delighted to have with us Bill's wife, Sharon, and daughter, Claire This visit gives them the opportunity to meet more of Bill's colleagues and to appreciate, once again, the great importance of the work he did Those of you who had the opportunity to know Bill can recall him as a dedicated bank supervisor and an outstanding public servant We in the United States were certainly fortunate to have had him lead our bank supervisory functions at the Federal Reserve and the FDIC while the U S banking system was experiencing quite difficult times To me, no individual displayed the characteristics necessary for a successful senior bank supervisor better than Bill Taylor Well known for this integrity, tenacity, and professional dedication, Bill demanded the best from himself and from those around him He understood that a safe and sound banking system was essential to a healthy market system, and he was committed to maintaining such a system His contributions extended outside the United States and into the efforts of the Basle Committee on Banking Supervision and beyond Indeed, heâ€”as much as anyoneâ€”recognized that the changes occurring in our international banking system increased the importance of supervisors from around the world communicating and working together It is most fitting, therefore, that we remember him at this conference The dual themes of this year's conference of cross-border banking and qualitative supervision are highly relevant to our responsibilities as bank supervisors in a world economy that is becommg increasingly integrated and complex Banking has become more sophisticated, the volume of transactions has multiplied, and competitive pressures have grown These developments reflect the increased efficiency of financial markets worldwide, which have helped to bring about expanded international trade and economic growth However, by strengthening the interdependences among markets and market participants, they may also have increased the potential for significant, adverse events to spread quickly to other markets As bank supervisors, we must deal with both the positive and the potentially negative effects of rapid innovation and change We should also take the opportunity that change provides to promote sound risk management practices within our banking systems Meetmg these challenges will be a daunting task 3 During my comments this evening I will suggest ways supervisors can address these challenges and prepare for undoubtedly greater changes in the years to come First, though, I would like to discuss the interaction of governments and central banks with private commercial banks in free economies in terms of risk sharing By articulating and understanding that relationship, we may have a better framework for considering how to supervise and regulate our financial institutions In addressing these issues it is important to remember that many of the benefits banks provide modern societies derive from their willingness to take risks and from their use of a relatively high degree of financial leverage Through leverage, in the form principally of taking deposits, banks perform a critical role in the financial intermediation process, providing savers with additional investment choices and borrowers with a greater range of sources of credit, thereby facilitating a more efficient allocation of resources and contri- buting importantly to greater economic growth Indeed, it was the evident value of intermediation and leverage that has shaped the development of our financial systems from the earliest timesâ€”certainly since Renaissance goldsmiths discovered that lending out deposited gold was feasible and profitable Stockholm, itself, recognized the value of intermediation with the founding of the Riksbank more than 300 years ago as a private institution Of course, this same leverage and risk-taking also greatly increases the possibility of bank failure Indeed, without leverage, losses from risk-taking would be absorbed by the bank's owners, virtually eliminating the chance that the bank would be unable to meet its obligations in a "failure" Some failures can be of a bank's own making, resulting, for example, from poor credit judg- ments For the most part, these failures are a normal and important part of the market process and provide discipline and information to other participants regarding the level of business risks Other failures, can result from, and contribute to, the rare episodes of severe economic or market turmoil that affects broad segments of an economy and is not the consequence of the imprudence of individual banks Because of important roles banks and other financial inter- mediaries play in our financial systems, such failures could have large ripple effects that spread throughout business and financial markets at great costs Over time, societies concluded that leverage and intermediation were essential to economic performance, but also that some bank failures could have unacceptable economic costs In response, central banks were created and were accorded new responsibilities, and what we now call prudential regulation evolved In the United States, these initiatives took the shape of the creation of the Federal Reserve in 1913 after several financial panics in the late 19th and early 20th centuries, and of federal deposit insurance and a broadened role for bank supervisors in the 1930's While the responses in other countries were often less overt, they were generally still significant in their effects This expanded role of governments, central banks, and bank supervisors implies a complex approach to managmg and even sharing the risks of failure between governments and privately owned banks Some of what central banks do might be termed "shaping" or reducing some kinds of risks, primarily by providing liquidity in certain situations to reduce the odds of extreme market outcomes, in which uncertainty feeds market panics Traditionally this was accomplished by making discount or Lombard facilities available, so that depositories could turn illiquid assets into liquid resources and not exacerbate unsettled market conditions by selling such assets or calling loans Similarly, open market operations, in situations like that which followed the 1987 stock market crash, satisfy increased needs for liquidity that otherwise could feed cumulative, self-remforcing, contractions across many fmancial markets But guarding against systemic problems also has involved, on very rare occasions, an element of more overt risk-sharing, in which the governmentâ€”or more accurately the taxpayerâ€”is potentially asked to bear some of the cost of failure Activatmg such risk sharing quite appropriately occurs at most maybe two or three times a century The willingness to do so arises from society's judgment that some bank failures may have serious adverse effects on the entire economy and that requiring banks to carry enough capital to avoid any risk of failure under any circumstances itself would have unacceptable costs in terms of reduced intermediation If banks had to absorb all financial risk, then the degree to which they could leverage, of necessity, would be limited, and their contribution to economic growth, modest Risk-sharing encourages leverage and intermediation Eliminating nsk-sharing and asking banks to remove the possibility of failure would lead to a much smaller banking system To attract, or at least retain equity capital, a private financial institution must earn at a minimum the overall economy's rate of return, adjusted for risk The rate of return banks would need in order to compete for a large amount of extra equity capital would seriously constrain the assets they could hold In their management of market or credit risk, well-run banks carefully consider potential losses from most possible market outcomes, and they hold sufficient capital to protect themselves from all but the most extreme situations But banks and other private businesses recognize that to be safe against all possible risks implies a level of capital on which it would be difficult, if not impossible, to earn a competitive rate of return On the other hand, if central banks or governments effectively insulate private institutions from the largest potential losses, however incurred, increased laxity could be costly to society as well Leverage would escalate to the outer edge of prudence, if not beyond. Lenders to banks (as well as their owners or managers) would learn to anticipate central bank or government intervention and would become less responsible, perhaps reckless, in their practices Such laxity would hold the potential of a major call on taxpayers And central banks would risk inflationary instabilities from excess money creation if they acted too readily and too often to head off possible market turmoil In practice, the policy choice of how much, if any, of the extreme market risk that government authorities should absorb is fraught with many complexi- ties Yet we central bankers make this decision every day, either explicitly or by default Moreover, we can never know for sure whether the decisions we made were appropriate The question, though, is not whether our actions to support entire financial systems or to require major changes at specific insti- tutions are seen to have been necessary in retrospect The absence of a fire does not mean that we should not have paid for fire insurance Rather, the question is whether, ex ante, the probability of a systemic collapse was sufficient to warrant intervention Often, we cannot wait to see whether, in hindsight, the problem will be judged to have been an isolated event and largely benign Thus, governments have been given certain responsibilities related to their banking and financial systems that must be balanced We have the responsi- bility to prevent major financial market disruptions through development and enforcement of prudent regulatory standards and, if necessary in rare circum- stances, through direct intervention m market events But we also have the responsibility to assure that private sector institutions have the capacity to take prudent and appropriate risks, even though such risks will sometimes result in bank losses or even bank failures Providing institutions with the flexibility that may lead to failure is as important as permitting them the opportunity to succeed By its nature, all business investment is risky The role of banks to assist in the financmg of such risk thus implies the taking of risk by the bank itself Indeed, this is the economic role of banking in a market economy The purpose of risk manage- ment is not to eliminate risk, but to manage it m a prudent manner Our goal as supervisors, therefore, should not be to prevent all bank failures, but to maintain sufficient prudential standards so that banking problems do not become widespread We try to achieve the proper balance through official regulations, formal and informal supervisory policies and procedures To some extent, we do this over time by signalling to the market, through our actions, the kinds of circumstances in which we might be willing to inter- vene to quell financial turmoil, and conversely, what levels of difficulties we expect private institutions to resolve by themselves The market, then, responds by adjusting the cost of capital to banks Throughout most of this century, we have made our decisions largely in a domestic context However, in recent decades that situation has changed markedly for many countries and is rapidly changing for all With financial instruments and markets becoming more complex and closely linked, it is essential that bank supervisors around the globe get to know and trust one another and communicate openly, as necessary, when bankmg problems and potential crises emerge In recognition of such common interests, major industrial countries have worked together for years through the Basle Committee on Bankmg Supervision Conferences like this one also clearly help advance the goal of interaction International coordinating and educational efforts doubtless also help supervisors cope with the growing complexity of supervisory matters by providing them with a forum for dealing with issues of mutual interest and concern The Caribbean Banking Supervisors Group, the SEANZA Forum of Banking Supervisors, and other regional associations of bank supervisors in the Middle East, Africa, and elsewhere help to move us in the right direction We have also madeâ€”and continue to makeâ€”significant progress in developmg prudent mtemational supervisory standards that are both quantitative and qualitative in nature Bill Taylor played a critical role in crafting and negotiating the Basle Accord of 1988 for credit risk that helped greatly to strengthen capital standards worldwide and to provide a more equitable basis for international competition More recently, the internal models approach for measuring market risks in trading activities, adopted by the Basle Committee late last year, builds upon that framework and may illustrate how supervisory rules and practices can evolve As financial markets change, supervision must be prepared to adjust We have to adapt continuously to changmg technologies, changing bank practices and changmg market forces Supervision is an ever evolving process We must be careful, however, not to alter our modalities too often for fear of creating supervisory uncertainty To maintain a proper balance in the years ahead will be one of our greatest challenges The decision to craft a bank's capital requirements for trading activities around accepted and verifiable internal risk measures was an important step in the supervision and regulation of large, internationally active banks It is all the more noteworthy because it recognizes the importance of both quantitative and qualitative criteria in the measurement and management of trading risks As risk management techniques evolve for other bank activities, supervisors will need to understand the new procedures and how they affect overall banking risks Time and again, though, events are demonstrating that despite the com- plexity of transactions and the alleged sophistication of management systems, it is poor qualitative factorsâ€”that is, the lack of basic policies and controlsâ€”that so often undermine banks Fortunately, in many cases, the technology that has enabled institutions to design complex new products also provides the techniques with which the resulting risks can be identified, measured, and controlled Management also must have the knowledge and motivation to employ these techniques to ensure that the risks are adequately contained We must never forget that no matter how technologically complex our supervisory systems become, the basic unit of supervision on which all else rests remains the human judgment of the degree of risk on a specific loan, based on the creditworthiness and character of a borrower If those credit judgments are persistently flawed, no degree of complexity of supposed risk dispersion or elegance of credit models will help As the Barings and other episodes illustrate, proper controls include such basic elements as adequate management oversight and separation of duties Those of us who supervise banks with worldwide operations must recognize that, with today's telecommunications, management must extend its policies, procedures, and controls to all offices that have the ability to take risks In this respect, coordination and cooperation between home and host countries become not only important, but essential in mamtainmg financially sound institutions and financial markets Within the United States, the Federal Reserve and other bank supervisors are placing growing importance on a bank's risk management process and are strengthening our supervisory procedures, where necessary, to assist exammers in identifying management weaknesses and strengths We are also working to develop supervisory tools and techniques that utilize available technology and that help supervisors perform their duties with less disruption to banks These improvements range from software designed to download data about a bank's loan portfolio to an exammer's personal computer, to simply more thoughtful reviews of internal management reports Such automation enhancements will permit exammers, themselves, to analyze more efficiently the various concen- trations within loan or mvestment portfolios and, therefore, help them to identify the underlymg risks and discuss those risks with bank management Countries in which supervisors conduct on-site examinations or otherwise review specific loans or loan portfolios may find such technology particularly useful Within the United States, the growing volume and complexity of transactions, particularly at the largest institutions, is requiring such productivity enhancements and other modifications to our supervisory procedures For ex- ample, rather than evaluate a high percentage of a bank's loans and investment products by reviewing individual transactions, we will increasingly seek to ensure that the management process itself is sound, and that adequate policies and controls exist While still important, the amount of transaction testing, especially at large banks, will decline. However, supervisors everywhere should expect bank boards of directors and senior managements to perform their leadership and oversight roles By themselves supervisors cannot expect to detect or prevent every unsound practice, nor to ensure that all weak management processes are improved We can expect our banking systems to be sound only by ensurmg that directors and managers provide guidance regarding their appetite for risk, that they bring to the bank, personnel with the integrity and skills to do the job, and that they monitor compliance with their own directives Encouraging and promoting sound qualitative risk management and internal controls has been and should remain a high priority of bank supervisors Indeed, it is as important, in my view, as the development of quantitative prudential standards Thus, despite all the changes and innovations, commercial banking remains a business largely of extending credit and managing the related risks To prosper, bankers must be risk-takers, but risk-takers to an appropriate degree Banking is special in all of our countries because of its role in financial intermediation Accordingly, the industry has been given important privileges, including the direct or implicit support of a national safety net in most countries that effectively protects it from the most severe economic events If relied on too heavily, however, that safety net can be abused by banks, which then be- come undercapitalized and too willing to take on inappropriate risk In the decades ahead, supervisors will have to adjust to growing technol- ogies and increasingly sophisticated markets A generation ago a month-old bank balance sheet was a reasonable approximation of the current state of an institution Today, for some banks, day-old balance sheets are on the edge of obsolescence In the 21st century that will be true of most banks Future supervision will of necessity have to rely far more on a bank's risk management information system to protect against loss We supervisors will be appreciably more involved in evaluating individual bank risk management pro- cesses, than after-the-fact results In doing so, however, we must be assured that with rare and circumscribed exceptions we do not substitute supervisory judg- ments for management decisions That is the road to moral hazard and ineffi- cient bank management Fortunately, the same technology and innovation that is drivmg supervisors to focus on management processes will, through the development of sophisticated market structures and responses, do much of our job of ensuring safety and soundness We should be careful not to impede the process Bank supervisors play an important role in encouraging the proper balance of risk-taking by developing prudent standards and enforcing sound practices at banks Bill Taylor understood that role and worked vigorously to address the weaknesses he saw. The approach we take will convey our views regarding to what extent governments will share banking risks and how much responsibility rests with banks In a global financial system, the choices we make will clearly have widespread effects</t>
-  </si>
-  <si>
-    <t>Before I take this opportunity to discuss the performance of the U S economy and the conduct of monetary policy, I would first like to thank the Chairman and the other members of this Committee for their support during my confirmation process I am grateful for the opportunity to serve the nation in this capacity for another term Nineteen-ninety-six has been a good year for the American economy By all indications, spending and production were robust in the first half of this year GDP increased at a 2-1/4 percent annual rate in the first quarter Partial data suggest a significantly stronger increase in the second quarter as the economy, as expected, accelerated out of its soft patch around the turn of the year During the second quarter, industrial production rose at an annual rate of 5-1/2 percent, and manufacturers are currently running their plant and equipment at utilization rates that are a touch above their postwar averages About 1 4 million workers have been added to nonfarm payrolls in the first six months of the year, and the unemployment rate fell to 5 3 percent in June Even though the U S economy is using its productive resources intensively, inflation has remained quiescent The core inflation rate, measured by the consumer price index less food and energy prices, at a 2 8 percent annual rate over the first six months of the year, is about 1/2 percentage point slower than the same period one year ago While increases in energy prices have boosted the overall CPI inflation rate to 3 5 percent thus far in 1996, a partial reversal of the jump in petroleum product prices observed in the first half appears to be in train I shall be discussing in greater detail later some possible reasons for this favorable inflation experience and offering some thoughts about how long it might last Economic activity thus far this year has turned out to be better than many analysts expected An important supporting factor, as I pointed out in February, was favorable conditions in financial markets in the latter part of 1995 and early 1996 Intermediate- and longer-term interest rates were low Among the influences accounting for this were optimism about prospective budget-deficit reduction, small easings of the stance of monetary policy in the second half of 1995 and early 1996, and the possibility of a further moderation in credit demands owing to a potentially soft economy Credit remained readily available, with banks and other lenders in financial markets generally pursuing credit opportunities aggressively And a rising stock market reduced the cost of capital to businesses and bolstered household balance sheets Looking forward, there are a number of reasons to expect demands to moderate and economic activity to settle back toward a more sustainable pace in the months ahead First, the bond markets have taken a turn toward restraint this year as they have responded to incoming data depicting an economy that was stronger than had been anticipated Intermediate- and longer-term interest rates have risen from 1 to 1-1/4 percentage points since January Second, the value of the dollar on foreign exchange markets has appreciated significantly on a trade-weighted basis against the currencies of other industrial countries over the past year or so This appreciation importantly reflects the market perception that the U S economy has been performing better than those of many of our major trading partners The rise in the dollar helps to keep down price pressures, but it also tends to divert domestic demand toward imported goods and damp exports some Third, the support to economic growth provided by expenditures on durable goods, both for household consumption and business fixed investment, is likely to wane in coming quarters Consumer spending in the past few years has been boosted as households have made up for the purchases of big-ticket items that they had deferred during the recession and the early, weaker phase of the recovery Five years after the business-cycle trough, however, we should expect that this pent-up demand has been largely exhausted Moreover, many households have built up sizable debt burdens in recent years, and coping with debt repayments could hold down their spending The business sector has been adding considerably to capacity, opportunities to invest profitably in new capital should be increasing less rapidly as final demand slows some While these are all good reasons to anticipate that economic growth will moderate some, the timing and extent of that downshift are uncertain We have not, as yet, seen much effect of the rise in interest rates on, for example, the housing market In many other aspects, financial market conditions remain quite supportive to domestic spending, and the economies of many foreign countries are showing signs of achieving more solid growth, which should help support our export sales Moreover, and perhaps of most relevance, a desire to build inventories could add significantly to production in the near term Data available for 1996 through May show that inventories were reduced relative to sales and are now fairly lean in many important industries Although the use of just-in-time inventory and production systems encourages purchasing managers to keep stocks lean, any evidence that deliveries of previously ordered goods are being delayed for extended periods would quickly alert companies to the need for higher safety stocks Indeed, indications of some mounting delivery delays in June do raise warning flags in this regard The reversal of earlier draw-downs in inventories, of course, could potentially impart an important boost to incomes and production as we enter the second half of the year The economy is already producing at a high level-and some early signs of pressures on resources are emerging, especially in the labor market There are, to be sure, legitimate questions about how much margin in resource utilization currently exists Historically, current levels of slack, measured in terms of either the unemployment rate or capacity utilization, have often been associated with a gradual strengthening of price and wage pressures Yet, the recent evidence of such pressures is scant I have already noted the lack of a distinct trend in the growth rate of the so-called core CPI Increases in more comprehensive, and perhaps more representative, chain-weighted measures of consumer prices, based on the national income and product accounts, actually have continued to edge lower The same is true of a still broader measure of price change, the chain-weighted price index for gross domestic purchases, which covers both consumers and businesses Although nominal wage rates have accelerated recently, the rate of increase has been lagging significantly behind that predicted on the basis of historical relationships with unemployment and past inflation And domestic profit margins have held up far later into this economic expansion than is the norm Have we moved into a new environment where inflation imbalances no longer threaten the stability and growth of our economy in ways they once did? The simple answer, in our judgment, is no But the issue is not a simple one As we have discussed before, powerful forces have evolved in the past few years to help contain inflationary tendencies An ever-increasing share of our nation's workforce uses the tools of new technologies Microchips embodied in physical capital make it work more efficiently, and sophisticated software adds to intellectual capital The consequent waves of improvements in production techniques have quickly altered the economic viability of individual firms and sometimes even entire industries, as well as the market value of workers' skills With such fast and changeable currents, it is not surprising that workers may be less willing to test the waters of job change Indeed, voluntary job leaving to seek other employment appears to be quite subdued despite evidence of a tight labor market Because workers are more worried about their own job security and their marketability if forced to change jobs, they are apparently accepting smaller increases in their compensation at any given level of labor market tightness Moreover, a growing share of all output competes in an increasingly global marketplace, allowing fixed costs to be spread over ever broader markets, promoting greater specialization and efficiency, and enhancing price competition As I indicated in February, these forces, to the extent that they are operative, exert a transitory, not permanent, effect in reducing wage and price inflation These trends leave the level of both wages and prices lower than historical relationships would predict But, at some point, greater job security will no longer be worth the further sacrifice of gains in real wages The growth of wages will then again be more responsive to tightness of labor markets, potentially putting pressure on profit margins and ultimately prices Moreover, the reductions in unit costs that are a consequence of the ever expanding global reach of many companies must ultimately be bound by the limits of geography To be sure, production and sales will continue to be diversified across geographic areas, but the world can only figuratively shrink so far At some point, possibly well into the future, increasing returns from ever- greater globalization must also ebb Perhaps reflecting these unusual influences, we have yet to see early signs in prices themselves of intensifying pressures, despite anecdotal and statistical evidence that the amount of operating slack in our economy has been at low levels by historic standards for some time Among the encouraging indicators, industrial commodity prices have remained roughly flat and the list of reported shortages of materials has been exceptionally small This pattern is consistent with the view that American businesses, by and large, have felt comfortable that inflation has been subdued and offers little evidence of the advance buying and expanded commitments that would come if businesses were expecting significant price pressures in the reasonably near future Nonetheless, there are early indications that this episode of favorable inflation developments, especially with regard to labor markets, may be drawing to a close The surprising strength in the employment cost index for wages and salaries in the first quarter raises the possibility that workers' willingness to surrender wage gains for job security may be lessening Wage data since March have been somewhat difficult to read Average hourly earnings clearly accelerated in the second quarter However, in looking at those figures, one must be mindful that they can reflect not only changes in wage rates but also shifts in the composition of employment And in recent months, a significant part, although not all of the pickup, has been accounted for by a tendency for employment to shift to relatively high-pay industries, such as durable goods manufacturing Whether such shifts also imply a correspondingly higher level of output per worker will determine whether unit labor costs also accelerated to impart upward pressures to price inflation Increases in pay, of course, are not inflationary so long as they are matched by gains in productivity Without question, we would applaud such trends, which increase standards of living However, wage gains that increase unit costs and are eaten up by inflation help no one, and ultimately place economic growth in jeopardy Clearly, in this environment, the Federal Reserve has had to become especially vigilant to incipient inflation pressures that could ultimately threaten the health of the expansion The relatively good inflation performance of the past few years, as best we can judge, owes in part to transitional forces that are only temporarily damping the wage-price inflation process We cannot be confident that we can ascertain when that process will come to an end This makes policy responses more difficult than usual, because, as always, the impact of pohcy will be felt with a significant lag Of course, if the economy grows so strongly as to strain available resources, transitional forces notwithstanding, history persuasively indicates that imbalances will develop that will bring the expansion to a halt The forecasts of the governors of the Federal Reserve Board and presidents of the Federal Reserve Banks for economic performance over the remainder of this year and the next reflect the view that sustainable economic growth is likely in store The growth rate of real GDP is most commonly seen as between 2-1/2 and 2-3/4 percent over the four quarters of 1996 and 1-3/4 to 2-1/4 percent in 1997 Given the strong performance of real GDP in the last two quarters, this outcome implies slower growth in the second half of this year Nonetheless, for the remainder of this year and the next in these projections, the unemployment rate remains in the range of the past 1-1/2 years Inflation, as measured by the four-quarter percent change in the consumer price index, is expected to be 3 to 3-1/4 percent in 1996 The governors and bank presidents, however, view the prospects for inflation to be more favorable going forward The expected reversal of some of the recent run-up in energy prices would contribute to that result, but policy makers' forecasts also reflect their determination to hold the line on inflation The central tendency of their inflation forecasts for 1997 is 2-3/4 to 3 percent, returning to the range from 1991 to 1995 We at the Federal Reserve would welcome faster economic growth, provided that it were sustainable As I emphasized last February, we do not have firm judgments on the specific level or growth rate of output that would engender economic strains Instead, we respond to evidence that those strains themselves are developing Whatever the long-run potential for sustainable growth, we believe that a necessary condition for achieving it is low inflation As a consequence, the Federal Reserve remains committed to preventing a sustained pickup in inflation and ultimately achieving and preserving price stability Price stability is an appropriate and desirable goal for policy, not only because it allows financial markets and the economy to work most efficiently, but also because it most likely raises productivity and living standards in the long run Specifically, in an inflationary environment, business managers are distracted from their basic function of building profits through prudent investment and cost control My own observation of business practices over the years suggests that the inability to pass cost increases through to higher prices provides a powerful incentive to hrms to increase profit margins through innovation and greater efficiency, which boosts productivity and ultimately standards of living over time Holding the line on inflation, thus, does not impose a speed limit on economic growth On the contrary, it induces the private sector to focus more on efforts that yield faster long-term economic growth In this context, we can readily understand why financial markets welcome sustained low inflation Uncertainty about future inflation raises the risks associated with investing for that future Lowering that uncertainty by keeping inflation down diminishes those risks, so that all commitments concerning future income become more valuable During periods of low inflation, stock and bond prices tend to reflect the higher valuation that comes from harnessing our physical plant more efficiently to provide improved opportunities in the future, including higher wages and profits What investors fear, what all Americans should fear, are inflationary instabilities They diminish our ability to provide the wherewithal for the standards of living of the next generation and the retirement incomes of our current work force The interests of investors as expressed in bond and stock markets do not conflict with those of average Americans--they coincide In order to realize the benefits of low and declining inflation, Federal Reserve policy has, for some time now, been designed to act preemptively--as I indicated earlier-to look beyond current data readings and base action on its assessment of where the economy is headed Policy restraint initiated in February 1994 followed from the judgment that unchanged policy would encourage subsequent inflationary imbalances that would ultimately cut short the economic expansion The three easing steps in the past year were instituted when we anticipated that inflationary imbalances would be less threatening and that lower rates would be compatible with promoting sustainable economic expansion Similarly, I am confident that the Federal Open Market Committee would move to tighten reserve market conditions should the weight of incoming evidence persuasively suggest an oncoming intensification of inflation pressures that would jeopardize the durability of the economic expansion The Committee selected provisional ranges for the monetary aggregates in 1997 that once again encompass the growth rates associated with conditions of approximate price stability, provided that these aggregates act in accord with their historical relationships with nominal income and interest rates These ranges are identical to those endorsed for 1996--1 to 5 percent for M2 and 2 to 6 percent for M3 The Committee reaffirmed its range of 3 to 7 percent for the debt of the domestic nonfinancial sectors for this year and chose the same range provisionally for next year The Committee's expectations for inflation and nominal GDP expansion in 1996 and 1997 suggest growth of the monetary aggregates at the upper ends of their benchmark ranges as a distinct possibility this year and next, though debt should be in the middle portion of its range The experience of the first part of the 1990s--when money growth diverged from historical relationships with income and interest rates-severely set back most analysts' confidence in the usefulness of M2 Recently, there have been tentative signs that the historical relationship linking the velocity of M2--or the ratio of nominal GDP to the money stock-to the cost of holding M2 assets has reasserted itself For now, though, the Committee is satisfied with watching these developments carefully, waiting for more compelling evidence that M2 has some predictive content in forecasting current and prospective spending Such evidence, however, at best will only accumulate gradually over time Monetary policy is, of course, only one factor shaping the macroeconomic environment I thus would be remiss if I did not again emphasize the critical importance to our nation's economic welfare of continuing to reduce our federal budget deficit We have made significant and welcome progress on this score in recent years But unless further legislative steps are taken, that progress will be reversed Inevitably, such changes will require addressing the consequences for entitlement spending of the anticipated shift in the nation's demographics in the first few decades of the next century Lower budget deficits are the surest and most direct way to increase national saving Higher national saving would help to lower real interest rates, spurring spending on capital goods so as to put cutting-edge technology in the hands of more American workers With a greater volume of modern equipment at their disposal, American workers will be able to produce goods that compete even more effectively on world markets The rally in capital markets last year that trimmed as much as two percentage points from longer-term Treasury yields was almost surely, in part, a response to the developing positive dialogue on deficit reduction While the backup in intermediate- and longer-term market interest rates this year has mostly reflected the unexpected vigor of economic activity, market participants must also have been struck by the dying out of serious discussions that might lead to a bipartisan agreement to eliminate the budget deficit over time Conclusion Mr Chairman, our economy is now in its sixth year of economic expansion The staying power of the expansion has owed importantly to the initial small size and rapid correction of emerging imbalances, reflected in part in the persistence of low inflation To be sure, the economy is not free of problems But as we address those problems, policy makers also need to recognize the limitations of our influence and the wellspring of our success The good performance of the American economy in the most fundamental sense rests on the actions of millions of people, who have been given the scope to express themselves in free and open markets In this, we are a model for the rest of the world, which has come to appreciate the power of market economies to provide for the public's long-term welfare</t>
-  </si>
-  <si>
-    <t>I appreciate this opportunity to appear before the Banking Committee today to address certain recent reports on the Federal Reserve's operations Of most relevance, the GAO has raised some significant issues with respect to the management of the Federal Reserve System Both the GAO and the Congress deserve our full response We are strongly committed to ensuring that the Federal Reserve System is managed efficiently and effectively It is most important to us at the Federal Reserve Board and the Reserve Banks, not only to run a "tight ship," but to foster the attitudes and processes that will ensure continuous improvement in the effectiveness of the Federal Reserve's operations We recognize that spending non-appropriated funds places a special obligation on us to be particularly diligent in the use and application of those funds Accordingly, even though we may ultimately disagree with some of the specific suggestions of the GAO, we welcome all of them and their insights because they require us to rethink our positions and change them, if appropriate Certain GAO recommendations for review of specific aspects of our management clearly have merit and reviews of a number of issues highlighted in the GAO's report are currently underway. These reviews may lead to changes in the Federal Reserve's administration that will further enhance our effectiveness It is most important for any organization, including the Federal Reserve, periodically to reassess its businesses and how they are carried out. Strategic planning is particularly critical given our rapidly changing environment, in which technology is advancing at an extraordinary pace and the financial services industry is becoming ever more complex It is essential that the Federal Reserve adapt to this changing environment with some foresight and as effectively as possible To that end, in 1995 we formalized our strategic focus by establishing a System Strategic Planning Coordinating Group to assess how the Federal Reserve can most effectively meet its public policy objectives into the next century Our strategic focus is also reflected in recent significant changes that the Federal Reserve has made in the way it carries out its major responsibilities For example, we have undertaken a major redesign and upgrade of our computer systems, communications networks, and critical software applications to improve reliability, respond more quickly to changing business requirements, and improve our disaster recovery capabilities. We have placed an increasing reliance on automation to provide a more flexible approach to bank examinations -- an approach that is risk-oriented, cost-effective, and sensitive to the burden placed on banks. We have also consolidated certain fiscal agency functions that we provide for the government in order to improve cost effectiveness and quality, and a Reserve Bank policy committee has been established to coordinate the provision of Federal Reserve financial services. In addition, the Federal Reserve already had underway several specific initiatives related to recommendations made by the GAO For example, we recently engaged an independent accounting firm to audit and certify the combined financial statements of the Reserve Banks The firm issued an unqualified opinion on the 1995 financial statements, as prepared in accordance with the financial accounting manual for the Reserve Banks In addition, we are actively reviewing the appropriate infrastructure for providing certain financial services, taking into consideration both cost efficiency and service quality. One difficult issue that has and will confront the Federal Reserve Board in our oversight of the System is the appropriate degree of consolidation of various activities Certain Systemwide activities do appear to be more cost effective if consolidated For example, we anticipate that the consolidation of our critical electronic payment applications will reduce our costs of providing these services But it is also evident that the element of autonomy that is accorded to the Reserve Banks has created an environment within the Federal Reserve that attracts highly qualified staff who contribute importantly to the effectiveness and efficiency of the Federal Reserve System over the long run The advantages of this environment must be balanced against the possible savings from consolidation. Federal Reserve's Role as Service Provider Many of our resources are devoted to providing priced payment services The Federal Reserve has played an integral role in the nation's payments system since the System's inception Indeed, one of Congress' original goals in establishing the Federal Reserve System was to improve the efficiency of check clearmg Prior to the passage of the Monetary Control Act in 1980, the Federal Reserve provided payment services to its member banks, the banks paid for these services implicitly with non-interest bearing reserves rather than through explicit fees The MCA fundamentally changed the manner in which the Federal Reserve provided and received payment for these services. Because the Act expanded reserve requirements to all depository institutions, it also required that the Federal Reserve offer its payment services to all depository institutions To offset the Act's reduction in the level of required reserves, as well as to broaden and level the competitive market for interbank payment services, Congress required us to price our services at full cost with a rate of return comparable to that of private firms I believe that the increased competition resulting from the MCA requirements has benefited the payments system The GAO has recommended that we review our future role in providing payment services We are in the process of conducting such a review in the context of our overall strategic plan In general, we view our role as a payments service provider as crucial in carrying out our overall central bank mission We believe it is important for the Federal Reserve to foster the integrity, efficiency, and accessibility of the U S dollar payments system, which in turn is important to maintain financial stability and maximize sustainable economic growth The provision of services by the Federal Reserve has contributed directly to these goals In addition, the knowledge and operational expertise we have gained as a service provider strengthens our efforts in containing systemic risks and is crucial in managing potential financial crises. We regard the wholesale payments services we provide, such as Fedwire and net settlement, as essential central bank services and important in limiting payments system risk Our role in providing these services probably will not change significantly as the marketplace evolves, although the nature of the services themselves might It is quite possible, if not likely, that as changes occur in the financial services marketplace over time, or owing to other considerations, our role in providing other services, such as check collection, may change as well In this regard, we must be sensitive to the fact that, as the nation's central bank, we have an unsurpassable credit rating that must not be used to unfairly compete with private-sector providers We are continually assessing our available means of achieving our payments system goals, including our regulatory authority and our role as a direct participant in the payments system, with our public service role always kept paramount For example, the Federal Reserve has adopted regulations that have fostered competition and efficiency in the provision of check collection services, even though they resulted in a reduction in the Federal Reserve's direct participation in the check system At the same time, the Federal Reserve has encouraged other efficiencies in the payments system through innovations in its service offerings. To the extent that we can achieve our payments system goals most effectively through our direct participation, our continued provision of these services will remain appropriate Federal Reserve Cost Effectiveness In considering the cost structure of the Federal Reserve, it is necessary to keep in mind the unique combination of responsibilities that have been assigned to this institution. The Federal Reserve is responsible for conducting monetary policy; supervising and regulating certain financial institutions, promoting the efficiency and integrity of the payments system, and providing fiscal agency services to the Treasury and other government agencies at their direction Different factors affect the cost structure of each of these functions For example, priced services are subject to the inherent discipline of the marketplace as the Federal Reserve must control costs in order to meet the statutory directives for cost recovery in the Monetary Control Act. On the other hand, in providing depository and fiscal services to the Treasury, the Federal Reserve must respond to the instructions of the Treasury We endeavor to carry out Treasury's directives in a cost effective manner, but cannot refuse legitimate requests because of their effect on our costs or because they are inconsistent with other Federal Reserve plans In the areas of monetary policy and financial institution supervision, there are fewer external constraints on our expenses Here we must be particularly vigilant Given the critical nature of the Federal Reserve's responsibilities, particularly in the areas of monetary policy, financial stability, and financial institution supervision, our major initiatives must be judged not only in terms of cost but also in the context of risk management and the appropriate level of resources to be devoted to each function For example, Congress, in enacting the Foreign Bank Supervision Enhancement Act in 1991, clearly concluded that the additional costs of expanding the Federal Reserve's supervisory responsibilities for U S operations of foreign banks were justified by the greater financial stability and protection that the enhanced supervision would bring We focus our banking examination resources based on risk assessments, with the expectation that areas not covered extensively in the examinations will not become serious problems Had we devoted more resources to Daiwa, and perhaps less elsewhere, would we have uncovered its wrongdoing at an early stage? We can't know for sure, but the odds would have been higher But, if we had the foresight to divert these resources from other activities, would we have increased our risk exposure elsewhere? As another example, the Federal Reserve's recent investment in a major upgrade of our computer systems and personnel to adapt our surveillance and payments technologies to the major changes that have occurred in private financial markets was also driven in large part to improve risk management While the costs of these improvements were not trivial, they have enhanced our ability to ensure the smooth functioning of the financial markets, even during periods of financial or operational disruptions To hold the risk of systemic crises to acceptably low levels in both U.S markets and U S dollar markets abroad requires some redundancy of resources Given the vast scale of the value of payment transactions that flow through our systems--our Fedwire volume alone averages almost $1 5 trillion a day~we believe that the benefits of this redundancy far exceed the associated incremental costs. The risk-management decisions that we make concerning the way we provide payment services to depository institutions are tested directly in the marketplace These services comprise more than one-third of the Federal Reserve Banks' total budget and the Monetary Control Act requires that, over the long run, we price these services to recover their costs, as well as costs that would be borne by private businesses, such as taxes and a return on equity If we provide these services inefficiently, we price ourselves out of the market Over the past decade, our track record has been good The Reserve Banks have recovered 101 percent of their total cost of providing priced services, including the targeted return on equity I should also note that, by recovering not only our actual costs but also the imputed costs that a private firm would incur, the Federal Reserve's priced services have consistently contributed to the amount we have transferred to the Treasury. During the past decade, priced services revenue has exceed operating costs by almost $1 billion Our fiscal agency services, which comprise another one-sixth of the Reserve Banks' total budget, are provided at the direction of the Treasury and other federal government agencies for whom we provide these services and whose reimbursements to us are made primarily with appropriated funds Here our difficulty has been in obtaining full reimbursement over the years We understand that, as part of its FY97 funding request, the Treasury sought a permanent indefinite appropriation, similar to that in place for the Bureau of the Public Debt, for services provided to its Financial Management Service The Federal Reserve and our fiscal principals continue to work closely to identify and implement initiatives that improve further the efficiency of these operations With respect to staff compensation and some other aspects of our infrastructure that are necessary to support our varied responsibilities, only indirect market criteria are available to judge the Federal Reserve's costs For example, we try to set salary structures that can attract and retain the personnel with skills necessary to run the Federal Reserve System in a highly effective manner. In order to acquire and hold such personnel, we strive to provide salaries and benefits competitive with local private and public sector markets, tempered by the willingness of many professionals to accord a nonmonetary premium to Federal Reserve employment Although the GAO report suggests that the Federal Reserve does not adequately review Federal Reserve employee salary and benefit levels to determine whether they continue to be justified, I can assure the Committee that these costs are scrutinized regularly to ensure that they are appropriate We believe that the GAO's comparison of growth in Federal Reserve employee benefits with those of the federal government is incorrect The problem is that while we accrue such benefits according to generally accepted accounting principles (GAAP), the federal government does not. Were the federal government to use accrual accounting, presumably the comparisons would be straightforward The federal government, however, employs an outmoded cash accounting system, which makes it difficult for us to reverse our accruals in a manner consistent with it As best we can judge, when calculated on a comparable basis using federal government accounting principles, the cost of benefits per employee for the Federal Reserve and the federal government increased by approximately the same percentage during the 1988 to 1994 period -- 64 percent and 62 percent, respectively We believe the GAO significantly overstated the increase in Federal Reserve benefit costs by including the cost of future pension benefits related to Federal Reserve early retirement plans on an accrual basis without considering the associated future savings attributable to those programs. Each of the early retirement programs has a positive net present value, indicating a net cost savings from such plans Including the present value cost of early retirement plans without considering the present value of cost savings skews any comparison of the increase in total benefits costs for the Federal Reserve and federal government Applying peer analysis more broadly, during the 1988 to 1994 period reviewed by the GAO, the increase in Federal Reserve operating costs was slightly less than the 51 percent increase in federal discretionary non-defense spending, which has been subject to increasing Congressional restraint in recent years The GAO makes this as one of its comparisons The Federal Reserve effectively contained its costs despite a significant expansion in its mandated responsibilities and expanded resources required to monitor and contain the financial market turmoil of that period To also compare, however, as the GAO did in its report, the rate of our expense increases with that of total federal discretionary outlays, which are dominated by the major post-cold war retrenchment in defense, is clearly inappropriate. Moreover, with the significant expansion of our computer systems now close to completion and our adjustment to our expanded supervisory mandates reaching fruition, our costs during the past two years and those projected for the immediate future are definitely on a flattening trajectory More generally, we believe that the GAO is mistaken in its notion that the Federal Reserve does not regularly assess certain ongoing programs to determine whether they are reasonable and justified In particular, we do not use a "current services" approach to develop the Board and Reserve Bank budgets The significant reallocation of System resources among the various responsibility areas during recent years clearly demonstrates that this is not the case In summary, although the Board believes that much of the GAO's analysis and recommendations have merit, we take exception to the broad implication of the GAO report that the Federal Reserve has not exercised appropriate budget constraint and that it has not adequately addressed the changing technological and financial environment in which it operates In my experience, the Federal Reserve is as well run an organization as any with which I have been associated, private or public, over the decades Is there nonetheless room for improvement Certainly I am not aware of any complex organization for which this is not the case In particular, the Board plans to review several specific areas highlighted by the GAO related to management of health care benefits. Reserve Bank procurement and contracting procedures, and Reserve Bank travel reimbursement policies The Federal Reserve Surplus One area discussed in the GAO report-the elimination or reduction of the Federal Reserve's surplus-has received substantial, and often misleading, media coverage I agree with the assessment of the Conference Report on the FY97 budget resolution on this matter The Report concluded that a transfer of the Federal Reserve's surplus to the Treasury would be a "gimmick" that "has no real economic impact on the deficit " While a transfer of Federal Reserve surplus would increase "unified receipts" (because the Federal Reserve, for technical reasons, is not included in the unified budget), it would nonetheless be an intra-governmental transfer that would not change the government's true economic and financial position with respect to the private sector. The Federal Reserve holds government securities as the asset counterpart to its surplus, interest on which it returns to the Treasury If the Federal Reserve decreased its surplus, it would do so by selling government securities and transferring the proceeds to the Treasury Consequently, the Federal Reserve's future payments to the Treasury would decline permanently by the foregone amount of interest on the surplus funds transferred, exactly offsetting the Treasury's savings on gross interest payments The surplus is part of our capital account In that context, I believe retention by the Federal Reserve of some level of surplus is desirable, but I acknowledge that the appropriate level of the Federal Reserve's surplus is debatable We would welcome the opportunity to work with Congress to review this issue Other Recent Inquiries I would like to conclude my testimony by commenting on several recent inquiries into certain aspects of the Reserve Banks' operations -- specifically, the management of our Interdistrict Transportation System (ITS) and cash statistical reporting problems experienced by the Los Angeles Branch of the Federal Reserve Bank of San Francisco Earlier this year, Representative Henry Gonzalez issued a report on the administration of the Federal Reserve's ITS network The report asserts that the Federal Reserve may have violated the Monetary Control Act to the extent that it does not fully recover the costs of ITS through revenue attributable to its use The GAO and the courts reviewed this issue in the mid-1980s and concluded that such cost recovery was not required by the Act No integrated company in the private sector (such as one that provides check collection services) prices individual segments of its operation to achieve a uniform rate of return Optimum profitability, i e , minimum consolidated costs, is enhanced through transfer pricing flexibility Even aside from the imprecisions associated with allocating fixed costs, it would not make sense for us to separately recover the costs of each input to a service, such as transportation, data processing, or labor, as implied by Representative Gonzalez Rather, all of the costs the Reserve Banks incur in providing check services to depository institutions, including ITS costs (which represent less than 5 percent of the costs of our check service), are recovered through fees for their various check products. Representative Gonzalez's report also alleges that certain contracting practices used by the Boston Reserve Bank in managing ITS were improper and wasteful Administration of ITS requires Federal Reserve management to make numerous, rapid, and complex business decisions every day, constantly balancing efforts to improve service, reduce float, and control operating costs In hindsight, are there some decisions that should have been made differently Almost surely But from a broad perspective, ITS has been managed effectively in our judgment Finally, I would like to put in context the errors made by the Los Angeles Branch of the Federal Reserve Bank of San Francisco in reporting certain statistical cash information to the Federal Reserve Board Unfortunately, the press coverage of this matter, in our judgment, has significantly overstated the problem First, these reports are used for informational purposes only No taxpayer money has been lost No key decision-making has been compromised The errors have not affected the usefulness of the information derived from the Federal Reserve's financial statements, nor have they affected the Federal Reserve's calculation of the money supply, its conduct of monetary policy, or the amount of shipments of currency and coin to or from the Branch. Second, although there were reports of mistakes amounting to $178 million, the errors changed the Branch's reported production volume by less than one-half of one percent If the mistakes had not been discovered, at worst there would have been slight errors in forecasting future currency demand, which could have caused a slight increase to the Federal Reserve's order to the Treasury to print new currency The cost of this higher currency print order would have been offset, however, by a lower print order in the following year Third, the Los Angeles Branch had identified the problems internally and was in the process of resolving them before Representative Gonzalez began his inquiry The Los Angeles Branch is working diligently to ensure that all of the data used to prepare the cash statistical reports transmitted to the Board are accurate In closing, let me state that we appreciate the GAO's review in that it assists us in our ongoing evaluation of the Federal Reserve's structure and functions and our efforts to continually improve operations. As I noted, many recommendations are useful and we are pursuing them In my opinion, however, the general tenor of the report does not reflect the high level of effectiveness with which the Federal Reserve has fulfilled its mission While, as is likely the case with any organization, the Federal Reserve has opportunities for further improvement, I believe these opportunities should be put in the context of our significant accomplishments</t>
-  </si>
-  <si>
-    <t>I thank the members of the Public Securities .Association for bestowing upon me this award for distinguished public service I am particularly honored by the company that I keep as a winner of this award, as previous recipients have included Senators Daniel Patrick Moynihan, Christopher Dodd, and Kay Bailey Hutchison and my predecessor as Chairman of the Federal Reserve, Paul Volcker I trust that everyone in this audience would agree that the U S government securities market works as well as any on earth and generates widespread macroeconomic benefits In one sense, that is regrettable The market has become so efficient in part because of the economies of scale associated with the large volume of Treasury debt issued over the years While the massive federal debt has allowed traders to refine their skills, it has also implied that much of the small pool of national saving has gone toward funding the government Moreover, the interest burden of this debt has kept tax rates higher than we might have wanted In another sense, though, the efficiency of the government securities market stands as testimony to decisions by policy makers in the formative days of our nation that convinced the world that the United States honored its commitments and valued the rule of law Every time I visit Secretary Robert Rubin, I am reminded of the power of the first Secretary of the Treasury's decisions that laid the foundations for this nation's financial credibility Engraved at the base of the statue of Alexander Hamilton outside the Treasury building are the words of Daniel Webster "He touched the dead corpse of the public credit, and it sprung upon its feet" Everyone knows the short version of the events that prompted that praise 2 Hamilton convinced the new Congress to honor the debts of the Continental Congress Under his prodding, the federal government also assumed responsibility for the debts of the individual states incurred in fighting the War of Independence But there are five details of the debate at that time that we all would be well served to remember First, Hamilton insisted on full payment of the debt Many at that time counseled discrimination among those obligations-perhaps by favoring vendors and veterans over bond holders or perhaps by paying original holders of debt more than those who purchased securities in the secondary market Hamilton recognized that an obligation was an obligation, no matter how it was incurred or who held it Repayment had both a moral and practical dimension The debt, in Hamilton's words, was the "price of liberty" because it financed the successful completion of the War of Independence Those who extended aid at a time of peril, or supported the debt subsequently, deserved to be repaid But repayment would also send an important message to investors, particularly those abroad, that the United States could be trusted in the future Hamilton recognized, and we should never forget, that investors have many choices on world markets Even the whiff of the possibility that the United States would not honor its debt would push up the cost of borrowing for years to come Following Hamilton's lead, the Treasury has never defaulted on any debt security, notwithstanding the abrogation of the gold clauses in 1933 Second, Hamilton was practical in his understanding that economic policy 3 making cannot be divorced from the broader discourse on public priorities The debate on the assumption of state debts generated arguments so heated as to make our weekend television talk shows appear as civil as tea parties Reflecting on those days in his later years, Thomas Jefferson--by no means an admirer of the first Secretary of the Treasury-was led to write that "this measure produced the most bitter and angry contest ever known in Congress, before or since the Union of the States " But those bitter enemies, Hamilton and Jefferson, compromised with an old-fashioned horse trade Jefferson threw his support for the assumption of the state debts in return for Hamilton's advocacy of placing the nation's capital on the banks of the Potomac Political realities have not changed in that regard in the succeeding two centuries It is inevitable that consideration of the budget be included as part of a wider debate on public policies However, Alexander Hamilton drew a line that no one should cross The government of the United States must never default on its debt Third, Hamilton's plan to honor the old debt provided a sinking fund to help repay new debt as it came due The first Secretary saw that Treasury debt was a burden to future generations And it was his responsibility to provide the means to lighten that load In those simpler times, before we became too sophisticated for our own good, deficit financing was a necessity prompted solely by peril, not as a tool of active demand management or as an excuse to put off hard decisions In one sense, though, Hamilton's job of planning for the retirement of the debt he was issuing was 4 easier than the problems confronting today's policy makers In 1789, government obligations could be measured by the amount of debt outstanding Today, debt comes in many forms, including promises to pay that have become embodied in unfunded entitlement programs Fourth, Hamilton's refunding scheme provided for the issuance of securities of long maturity that would be repaid in specie Thus, his Treasury locked in longer- term funding and did not have to test continually the market's willingness to finance the new government At the same time, investors were given some assurance that holding government securities would preserve their purchasing power Those same incentives have led our present-day Treasury to issue securities across a wide range of maturities and, I am pleased to note, to begin soon to offer debt indexed to consumer prices Fifth, and this should come as no surprise from one of the authors of the Federalist Papers, Hamilton explained his policies in well written, logically constructed arguments that remain pleasures to read, even two hundred years later Hamilton's lessons speak across the generations, both to policy makers in mature democracies and those coping, as he did, with financing newly independent states If we are to protect his creation, the U S Treasury market, we must remember two facts he could not afford to forget For one, buyers of Treasury securities do so through their own volition Investors have alternatives, and more so now than ever before For another, the issuer of those securities, the U S Treasury, must finance an amount, on net, that is determined by the political judgments of 5 the congressional and executive branches of government If the government makes purchasing its debt harder--by imposing onerous reporting or bookkeeping requirements--or riskier-by following capricious macroeconomic policies-buyers will pull back and the cost of servicing the debt will rise We at the Federal Reserve will do our part to contribute to financial stability, which is to preserve the purchasing power of money over time To be sure, the dollar sums that preoccupied Alexander Hamilton were small The national debt totaled $75 million, or $18 per capita But the issues at stake were large I can only hope that, by following his precedent, today's policy makers show some of the same wisdom in dealing with the public debt the congressional and executive branches of government If the government makes purchasing its debt harder--by imposing onerous reporting or bookkeeping requirements--or riskier--by following capricious macroeconomic policies-buyers will pull back and the cost of servicing the debt will rise We at the Federal Reserve will do our part to contribute to financial stability, which is to preserve the purchasing power of money over time To be sure, the dollar sums that preoccupied Alexander Hamilton were small The national debt totaled $75 million, or $18 per capita But the issues at stake were large I can only hope that, by following his precedent, today's policy makers show some of the same wisdom in dealing with the public debt</t>
-  </si>
-  <si>
-    <t>I am privileged to accept the Union League of Philadelphia's Abraham Lincoln award This is the first time I have been at the Union League in nearly four decades, but I am gratified to learn that your organization remains as vital and active as it was in the 1950s when I visited friends here with some frequency Today I would like to address an issue that almost certainly will be at the forefront of American concerns over the next decade our largest federal entitlement program, social security It is becoming conventional wisdom that the social security system, as currently constructed, will not be fully viable after the so-called baby boom generation starts to retire in about fifteen years The most recent report by the social security trustees projected that the trust funds of the system will grow over approximately the next fifteen years However, beginning in the year 2012, the annual expected costs of social security are projected to exceed annual earmarked tax receipts, and the consequent deficits are projected to deplete the trust funds by the year 2029 While such evaluations are based on an uncertain future, the benefit per current retiree under existing law, adjusted for inflation, can be forecast with some precision over the next thirty years Somewhat less precision is possible for future retirees The price escalation of benefits, of course, is even more difficult to pin down But since price inflation has an equal effect on wages subject to social security taxation, for all practical purposes, the degree of inflation does not have a large direct effect on the net funding of the system over the long run However, the rate of inflation, because it affects the overall economy, presumably does affect the real wage base from which social security taxes and future benefits are derived The projection of inflation-adjusted taxes, which are subject to a wider degree of uncertainty than total benefits, is largely driven by real wage growth-that is, wage growth adjusted for inflation-which, in turn, is primarily determined by the growth of productivity Projecting productivity in line with the pattern of the last quarter century suggests a trend of revenue falling far short of the levels required to finance the benefits of the large baby-boomer bulge in retirees anticipated to start at about 2010 I should state, parenthetically, that if recent productivity trends are underestimated, as I suspect they are, for much the same reasons are the projected trends of both real benefits and payroll taxes The real future funding shortfall, therefore, would not be materially effected Our social security problem is, thus, not merely statistical, it is the consequence of a projected shortfall in real resources dedicated to social security In money terms, the current social security trust fund of a half trillion dollars falls far short of the levels required to fund the current obligations to pay promised benefits to those already retired and those who will retire in the years ahead Social security, unlike fully funded private retirement programs, is largely an intergenerational transfer Today's workers are essentially paying for today's retirees Under the current system, the social security benefits paid to today's workers when they retire in the future will be primarily dependent upon the payroll taxes acquired from future workers Accordingly, if the social security system is to survive in its current form, either real benefits must be curtailed, or real taxes increased The latter can come from either higher tax rates or higher real wage growth--in effect, higher productivity growth However, as I will be explaining shortly, higher productivity is unlikely alone to do the trick Moreover, increased social secunty tax rates, of course, are controversial in that many perceive them, myself included, to adversely affect employment A primary cause of social security's funding imbalance stems from the fact that, until very recently, the payments into the social security trust accounts by the average employee, plus employer contributions and interest earned, were inadequate, at retirement, to fund the total of retirement benefits This has started to change Under the most recent revisions to the law, and presumably conservative economic and demographic assumptions, today's younger workers will be paying social security taxes over their working years that appear sufficient to fund their benefits during retirement However, the huge unfunded liability for current retirees, as well as for much of the work force closer to retirement, leaves the system, as a whole, badly underfunded As longevity improved far beyond that contemplated by the creators of the system, and productivity growth slowed after 1973, the original premise of the system of intergenerational balance began to fail Today the official unfunded liability for the Old Age, Survivors and Disability funds, which takes into account expected future tax payments and benefits out to the year 2070, has reached a staggering $3 trillion The social security trustees currently project taxes and benefits, under existing, and of necessity, quite tentative economic assumptions, that imply that fully funding social security for the next 75 years would require an immediate and permanent increase in social security taxes of about 2 2 percentage points of taxable payrolls on top of the current 12 4 percent tax rate, assuming that such an increase would not impede economic growth Of course, benefit reductions of a similar magnitude, or a mix of tax hikes and benefit cuts, could also bring the system back into long-term actuarial balance, at least statistically. These types of program adjustments, which on the surface seem quite modest, might nonetheless be perceived as transforming what has until recently been a largely popular, subsidized, intergenerational transfer system into something quite contentious Moreover, the longer action is deferred, the greater will be the necessary tax increases or, more likely, benefit adjustments required to achieve the goal of long-term actuarial balance Clearly, something has to give The question is what? We cannot hope to grow our way out of the problem An immediate and sustained increase in annual productivity growth of about two percentage points apparently would be needed to close the long-run funding gap without an increase in taxes or a cut in benefits The improvement in productivity growth must be this large because higher productivity raises future benefits as well as current and future tax receipts However, given that we struggle to devise economic policies that might raise productivity growth by a few tenths of a percentage point per annum, a gain of two full points seems beyond the reach of credibility Nonetheless, this issue does underscore the critical elements in the forthcoming debate, since it focusses on the core of any retirement system, private or public Simply put, unless social security taxes increase, or as I just indicated, more likely, benefits are adjusted, domestic savings must increase. Potential beneficiaries must further abstain from consuming all of their incomes Enough must be set aside over a lifetime of work to fund the excess of consumption over any non-social security income a retiree may still enjoy. At the simplest level, one could envision households saving by actually storing goods purchased during their working years for consumption during retirement Even better, the resources that would have otherwise gone into the stored goods could be diverted to the production of new capital assets, which would, cumulatively, over a working lifetime, produce an even greater quantity of retirement goods and services In short, we would be getting more output per worker, our traditional measure of productivity, and a factor that is central in all calculations of long-term social security trust fund financing Hence, the bottom line in all retirement programs is physical resource availability The finance of any system is merely to facilitate the underlying system of allocating real resources that fund retirement consumption of goods and services The basic premise of our current largely pay-as-you-go social security system is that future productivity growth will be adequate to supply promised retirement benefits for current workers At existing rates of saving and investment this is becoming increasingly dubious Accordingly, there are a number of initiatives, at a minimum, that will surely have to be addressed As I argued at length in the Social Security Commission deliberations of 1983, with only marginal effect, some delaying of the age of eligibility for retirement benefits will become increasingly pressing For example, adjusting the full-benefits retirement age to keep pace with increases in life expectancy would keep the ratio of retirement years to expected lifespan approximately constant and would help to significantly narrow the funding gap Hopefully, other modifications to social security benefits also will be judged as necessary Moreover, it is becoming increasingly recognized that the Consumer Price Index overstates increases in the cost of living, and thus indexing social security benefits to the CPI goes far beyond the intent of the Congress to insulate retirees from inflation In that regard, the recently released report from the Boskin commission makes a valuable contribution to the emerging consensus on this issue But, unless future taxes and/or benefits are sufficiently adjusted, there is no substitute for increased domestic savings and investment currently. To be sure, for relatively short periods of time we can finance part of domestic investment in plant and equipment with foreign savings as we are doing today History, however, tells us that there is a limit to how far that can go We are also apparently increasing the productivity of our capital It is possible that the maturing of emerging technologies, and further substantial deregulation of industry and finance, will, in themselves, improve the growth rate of productivity without large capital investment and savings But, it would take implausible improvements in capital productivity from current rates to close very much of the social security funding gap from this source The necessary boost in domestic savings need not be derived from an improved social security system, but certainly a reduction in the social security funding gap would itself move in that direction In a sense, it could create a virtuous cycle with higher savings engendering higher productivity growth which, in turn, would narrow the funding gap still further. Of course, additional saving can be achieved through a reduction in the overall federal government budget deficit, and intensified efforts to encourage private household and business savings Some have argued for a provision in law to require the social security trust funds to invest in higher yielding, private securities, especially equities, rather than in U.S Treasuries only A higher rate of return, it is alleged, would help solve the social security funding problem That may in fact be the case, but if so, what would happen to private retirement programs? If social security trust funds are shifted in part, or in whole, from U S Treasury securities to private debt and equity instruments, holders of those securities in the private sector must be induced to exchange them, net, for U S Treasuries If, for example, social security funds were invested wholly in equities, presumably they would have to be purchased from the major holders of such equities Private pension and insurance funds, among other holders of equities, presumably would have to swap equities for Treasuries But, if the social security trust funds achieved a higher rate of return investing in equities than in lower yielding U S Treasuries, private sector incomes generated by their asset portfolios, including retirement funds, would fall by the same amount, potentially jeopardizing their financial condition This zero-sum result occurs because of the assumption that no new productive saving and investment has been induced by this portfolio reallocation process Proceeding further, one must presume that in such a circumstance, in order to induce the private sector to exchange their equities for Treasuries, equity prices must rise, and bond prices fall But, this would create great market tension. Bonds and equities are merely the paper claims to income earning assets, and the value of the income stream is not determined by short-run changes in the supply and demand for securities Rather, equity prices must, in the long run, reflect the underlying earnings of the corporations on which the equities are a claim, as well as society's need to be compensated for postponing consumption into the future and its perception and attitudes toward risk as a consequence of uncertainty about the future. Indeed, the total market value of debt plus equities, is, to a first approximation, likely to be unaffected by a shift in the balance of paper claims One might expect that this tension between the altered relative supply of equity and debt claims, on the one hand, and unaltered overall economic value of the nation's companies, on the other hand, would be resolved by an increase in the issuance of equity securities, relative to bonds This could reverse much, if not all, of the price shift in favor of equities However, to complicate the issue still further, it is not clear as to whether, and to what extent, bond prices would rise as corporations cut back on debt issuance Certainly with the social security trust funds no longer investing all of their surplus in U.S. Treasuries, the federal debt held by the public would rise, presumably placing downward pressure on bond prices. At best, the results of this restricted form of privatization are ambiguous Thus, the dilemma for the social security trust funds is that a shift to equity investments without an increase in domestic savings may not appreciably increase the rate of return of social security trust fund assets, and to whatever extent that it does, would likely be mirrored by a comparable decline in the incomes of private pension and retirement funds I should stress that this does not mean that at least a partial privatization of our social security system does not provide a potentially viable solution to current funding problems There are a number of thoughtful initiatives that, through the process of privatization, could increase domestic saving rates These are clearly worthy of intensive evaluation Perhaps the strongest argument for privatization is that replacing the current unfunded system, which apparently discourages saving, with a fully funded system, is that such a change could boost domestic saving But, in any event, we must remember it is because privatization plans might increase savings that makes them potentially viable, not their particular form of financing The types of changes that will be required to restore fiscal balance to our social secunty accounts, in the broader scheme of things, are significant but manageable More important, most entail changes that are less unsettling if they are put into effect in the near term rather than waiting five or ten years or longer Minimizing the potential disruptions associated with the inevitable changes to social security is made all the more essential because of the pressing financial problems in the Medicare system, social security's companion program for retirees Medicare currently is in an even more precarious position than social security The fmancing of Medicare faces some of the same problems associated with demographics and productivity as social security but faces different, and currently greater, pressures owing to the behavior of medical costs and utilization rates Reform of the Medicare system will require more immediate and potentially more dramatic changes than those necessary to reform social security. We owe it to those who will retire after the turn of the century to be given sufficient advance notice to make what alterations in retirement planning may be required The longer we wait to make what are surely inevitable adjustments, the more difficult they will become If we procrastinate too long, the adjustments could be truly wrenching. Our citizens deserve better.</t>
-  </si>
-  <si>
-    <t>Mr Chairman and members of the Committee, I am pleased to appear here today In just a few weeks the Federal Reserve Board will submit its semiannual report on monetary policy to the Congress That report and my accompanying testimony will cover in detail our assessment of the outlook for the U S economy and the challenges facing monetary policy This morning, I would like to offer some personal perspectives on the current economic situation I think it is fair to say that the overall performance of the U S economy has continued to surpass most forecasters' expectations The current cyclical upswing is now approaching six years in duration, and the economy has retained considerable vigor, with few signs of the imbalances and inflationary tensions that have disrupted past expansions Although the data for the fourth quarter are still incomplete, it is apparent that real gross domestic product posted an increase in the neighborhood of 3 percent over the four quarters of 1996 This increase may seem quite moderate compared with the gains registered in some earlier years of the postwar period, however, at a time when the working-age population is expanding relatively slowly and unemployment is already low, this economic growth is appreciable indeed It was enough to generate more than 2-1/2 million new payroll jobs last year and to cause the unemployment rate to edge down to 5- 1/4 percent--a figure roughly matching the low of the last cyclical upswing, in the late 1980s But, in contrast to that earlier period, we have not experienced a broad increase in inflation, in fact, by some important measures of price trends, inflation actually slowed a bit in 1996 The balance and solidity of the expansion last year can be seen in the composition of the growth Notably, consumers appear to have been rather conservative in their spending In some instances, they may have been constrained by the debt-service burdens accumulated over the previous few years, but in the aggregate, households experienced an enormous further accretion of net worth as the stock market continued to climb at a breathtaking rate Judging from historical patterns, such an increase in wealth might have inspired households to spend an enlarged share of their current income, but, if we take the available data at face value, households appear instead to have set aside a greater share of their income for financial investment Perhaps Americans are finally becoming conscious of the need to accumulate additional assets to ensure not only that they can handle temporary interruptions in employment but also that they will have the wherewithal to enjoy a lengthy retirement down the road Be that as it may, the increased flow of private savings--and a reduced call upon those savings by the Treasury--helped to fund substantial increases in fixed investment last year Homebuilding activity was up considerably, notably, single-family housing starts were robust once again and helped to push the nation's homeownership rate to a fifteen-year high In addition, business fixed investment posted another strong advance Firms acquired large amounts of computing and telecommunications equipment in particular, seeking to enhance the efficiency of their operations as well as their overall productive capacity At the same time, they accumulated inventories rather cautiously Stock-to-sales ratios, which had risen in 1995, were in many cases near historic lows as of November 1996, the most recent month for which statistical information is available The growing economy had beneficial effects on the finances of many states and localities, which consequently could spend more on needed infrastructure and vital services and, in some instances, trim taxes Of course, overall government sector purchases were held down by the ongoing efforts to reduce the federal deficit It clearly was private demand that drove economic growth last year To be more specific, it was domestic private demand that did so, for net exports fell, on balance, in 1996 The volume of goods and services we sold abroad grew appreciably, despite moderate economic expansion by our major trading partners, but our imports continued to grow at a rapid clip In fact, imports provided a safety valve in a U S economy marked by a high degree of resource utilization I've already noted that our unemployment rate reached the lowest level in some time Moreover, throughout the year, we heard reports from around the country that qualified workers were in tight supply Although increases in hourly compensation remained relatively subdued--an important fact to which I shall return in a few moments-- they did become more sizable, and they raised unit costs when employers were unable to enhance productivity commensurately Thanks to the very substantial additions to facilities in the past few years, physical capacity in the manufacturing sector was not greatly strained The question is, of course, where do we go from here? Can we continue to achieve significant gains in real activity while avoiding inflationary excesses? Because monetary policy works with a lag, it is not the conditions prevailing today that are critical but rather those likely to prevail six to twelve months, or even longer, from now Hence, as difficult as it is, we must arrive at some judgment about the most probable direction of the economy and the distribution of risks around that expectation Fortunately, economic events are not wholly random and unforecastable There are certain principles, and certain empirical regularities in behavioral relations, that we can follow with some degree of confidence For example, capital investment responds in a predictable way to the rate of growth of the economy, expected profitability, and the cost of capital Similarly, housing activity, with some qualifications, moves inversely with mortgage rates And the largest component of final demand, personal consumption expenditures, generally follows income over time Many of these relationships are embedded in the traditional notion of the business cycle developed by Wesley Clair Mitchell three-quarters of a century ago and worked out with Arthur F Burns, one of my predecessors, in the definitive tome, Measuring Business Cycles Their insights remain relevant today Even so, each cycle tends to have its own identifying characteristic For example, in the late 1980s and the recessionary period of the early 1990s, the economy was dominated by the sharp fall in the market value of commercial real estate, because such real estate served as a major source of loan collateral, the drop in its value had a profoundly restrictive influence on the willingness and ability of commercial banks to lend As you may recall, at that time, I characterized the economy as trying to advance in the face of fifty- mile-an-hour headwinds The severe credit restraint was only grudgingly responsive to the extended efforts of the Federal Reserve to ease monetary conditions Similarly, the dramatic rise of inflation and of inflation expectations in the 1970s was key in shaping the cyclical patterns of that period One manifestation was the impetus to spending on houses, cars, and other consumer durables from buyers' efforts to beat future price increases Countering this inflation required a major monetary tightening, which moved both nominal and real interest rates up sharply and led to substantial contractions in housing and other interest-sensitive sectors in the early 1980s In contrast, as I've mentioned several times to the Congress over the past few years, perhaps the dominant characteristic of the current expansion is low inflation and quiescent inflation expectations, which have helped create a financial environment conducive to strong capital spending and longer-range planning generally I emphasized this point in our Humphrey-Hawkins testimony of a year ago Since then, increases in hourly compensation as measured by the employment cost index have continued to fall far short of what they would have been had historical relationships between compensation gains and the degree of labor market tightness held Reaching some judgment about the reasons for this departure from past patterns is important As I see it, heightened job insecurity explains a significant part of the restraint on compensation and the consequent muted price inflation Surveys of workers have highlighted this extraordinary state of affairs In 1991, at the bottom of the recession, a survey of workers at large firms indicated that 25 percent feared being laid off In 1996, despite the sharply lower unemployment rate and the demonstrably tighter labor market, the same survey organization found that 46 percent were fearful of a job layoff The continued reluctance of workers to leave their jobs to seek other employment as the labor market has tightened provides further evidence of such concern, as does the tendency toward longer labor union contracts For many decades, contracts rarely exceeded three years Today, one can point to five- and six-year contracts-- contracts that are commonly characterized by an emphasis on job security and that involve only modest wage increases The low level of work stoppages of recent years also attests to concern about job security Thus, the willingness of workers to trade off smaller increases in wages for greater job security seems to be reasonably well-documented for this particular business-cycle expansion The unanswered question is why this insecurity has persisted even as the labor market has, by all objective measures, tightened considerably One possibility is the ongoing concern of workers about job skill obsolescence The reality of this obsolescence is evidenced by the marked expansion of on-the-job training programs, especially in technical areas, in many of the nation's corporations No longer can one expect to obtain all of one's lifetime job skills with a high- school or college diploma Indeed, continuing adult education is perceived to be increasingly necessary to retain a job Certainly, there are other possible explanations of the softness in compensation growth in the past few years The sharp deceleration in health care costs, of course, is cited frequently Another possibility is the heightened pressure on firms and their workers in industries that compete internationally Domestic deregulation has had similar effects on the intensity of competitive forces in some industries In addition, the continued decline in the share of the private workforce in labor unions has likely made wages more responsive to market forces --indeed, the converse is also true in that the new competitive realities have in many instances undermined union strength In any event, although I do not doubt that all these explanations are relevant, I would be surprised if any were dominant Another potential explanation is that persistently low price inflation is constraining wage increases Historical evidence clearly indicates that price inflation is a factor in wage change But, if the causation is running mainly from product markets, where prices are set, "to labor markets, where wages are set, then we would expect to see some squeeze on profit margins Clearly, this is not the case at present Rather, owing in part to the subdued behavior of wages, profits and rates of return on capital have risen to high levels The high rates of return, in turn, seem to be inducing competitive pressures that limit the ability of firms to raise prices relative to their underlying cost structures because they fear that competitors anxious to capture a greater share of the market will not follow suit Thus, the evidence seems more consistent with the view that wage restraint is damping price increases than the other way around If the job insecurity paradigm that I have outlined is the key, then we must recognize that, as I indicated in last February's Humphrey-Hawkins testimony, "suppressed wage cost growth as a consequence of job insecurity can be carried only so far At some point in the future, the trade-off of subdued wage growth for job security has to come to an end " In short, this implies that even if the level of real wages remains permanently lower as a result of the experience of the past few years, the relatively modest wage gains we've seen are a transitional rather than a lasting phenomenon The unknown is how long the transition will last Indeed, the recent pickup in some measures of wages suggests that the transition may already be running its course If so, the important question from a monetary policy point of view is whether prospective labor market conditions will be consistent with the maintenance of satisfactory price performance I would like to conclude with a brief discussion of some issues of measurement and economic data that may be useful as you begin your deliberations on the 1998 budget One issue you will have to grapple with is the growing consensus that the consumer price index--and other broad price measures that rely heavily on CPI data in their construction--are substantially overstating changes in the true cost of living From your perspective, one important implication of the CPI bias is that it creates an automatic and presumably unintended real increase in social security and other indexed federal benefits and a real cut in indexed individual income taxes each year Less widely recognized is the fact that, for a given level of nominal spending, the upward bias in the CPI in many cases is mirrored in a downward bias in estimates of real spending, this muddies the interpretation of both recent economic developments and longer-run trends in our economic performance Several researchers have attempted to quantify the bias In the CPI and other broad measures of prices One set of studies has examined the detailed microstatistical evidence on price measurement The Boskin Commission drew heavily on these studies and concluded that the CPI is currently overstating changes In the true cost of living by approximately 1 percentage point per year In addition to some technical factors associated with its construction, the CPI overstates inflation because of the slow introduction of new products and inadequate adjustment for quality improvements Recently, researchers at the Federal Reserve Board have looked at the measurement Issue from a macroeconomic perspective This analysis, which questions whether the pattern implied by the published price, output, and productivity statistics makes sense, also suggests that the inflation rate is overstated In particular, the research finds that measured real output and productivity in the service sector of the economy are implausibly weak, given that the return to the owners of these businesses that is implicit in our aggregate statistics on GDP apparently has been well-maintained The published data indicate that the level of output per hour in several service-producing industries has been falling for more than two decades --that is, that firms in these industries have been getting less and less efficient for more than twenty years This pattern is highly unlikely Price mismeasurement seems to be the most probable explanation of the data anomalies, and the order of magnitude appears consistent with the microstatistical results The evidence that inflation has been slower and that real growth has been faster than the official measures indicate is welcome, in part because it suggests that the nation's current level of economic well-being is higher than we had thought But I want to make clear that revising our historical estimates of real growth to incorporate better price data would have no material effect on measures of the degree of resource utilization, because such a revision implies faster growth in potential output, as well as actual output, accordingly, it does not alter the relationship between resource utilization and inflation Nor does it change the outlook for the federal budget deficit, apart from any modifications to the indexing formulas for entitlements and income taxes Certainly, the judgment that aggregate productivity has been growing faster than indicated by the official statistics seems reasonable in light of the significant business restructurings and extraordinary improvements in technology in recent years I do not mean to imply, however, that we should assume that the full productivity gain from information technology has already been reaped Clearly, it takes some time for firms to adopt production techniques that translate a major new technology into increased output In an intriguing parallel, electric motors in the late nineteenth century were well-known as a technology but were initially integrated into production systems that were designed for steam-driven power plants Not until the gradual conversion of previously vertical factories into horizontal facilities, mainly in the 1920s, were firms able to take full advantage of the synergies implicit in the electric dynamo and thus achieve dramatic increases in productivity Analogously, not all of today's production systems can be easily integrated with new information and communication technologies Some existing equipment cannot be controlled by computer, for example Thus, the full exploitation of even the current generation of information and communication equipment may occur over quite a few years and only after a considerably updated stock of physical capital has been put in place While such a scenario is quite plausible, we cannot be certain when, or if, it will occur Thus, we must be vigilant to ensure that our economy remains sufficiently flexible for entrepreneurial initiatives And we must continue our efforts to further enhance productivity growth by raising national saving and spurring capital formation Attaining a higher national saving rate quite soon is crucial, particularly in view of the anticipated shift in the nation's demographics and associated pressures on federal retirement and health programs in the first few decades of the next century Reducing the size of the federal budget deficit, and over time moving the unified budget into surplus, would go a substantial way in that direction</t>
-  </si>
-  <si>
-    <t>Mr. Chairman and members of the Committee, I appreciate the opportunity to appear before you today. The Committee is faced with a number of complex policy issues that will have an important bearing on the fiscal health of the nation and the welfare of our people well into the next century. I will be happy to respond to questions relating to any of those issues, but in my formal comments this morning I intend to focus on the accuracy of the consumer price index. I would like to begin by commending this Committee for having done so much to bring the issue of possible bias in the CPI to the attention of the Congress and of the nation in general. The hearings conducted by this Committee in 1995, as well as the report produced by the advisory commission that was sponsored by this Committee, have advanced the discussion considerably. These efforts, along with the continuing contributions of the Bureau of Labor Statistics research staff, have added importantly to our understanding of the sources of measurement error in the CPI. Any index that endeavors to measure the cost of living should aim to be unbiased. That is, a serious examination of all available evidence should yield the conclusion that there is just as great a chance that the index understates the rate of growth of the target concept as there is that it overstates the truth. The present-day consumer price index does not meet this standard. In fact, the best available evidence suggests that there is virtually no chance that the CPI as currently published understates the rate of growth of the appropriate concept. In other words, there is almost a 100 percent probability that we are overcompensating the average social security recipient for increases in the cost of living, and almost a 100 percent probability that we are causing the inflation-adjusted burden of the income tax system to decline more rapidly than I presume the Congress intends. A major reason for this is that consumers respond to changes in relative prices by changing the composition of their actual marketbasket. At present, however, the marketbasket used in constructing the CPI changes only once every decade or so. Moreover, new goods and services deliver value to consumers even at the relatively elevated prices that often prevail early in their life cycles; currently, that value is not reflected in the CPI. For that and other reasons outlined in the Boskin Commission report and other studies, we know with near certainty that the current CPI is off. We do not know precisely by how much, however. There is, nonetheless, a very high probability that the upward bias ranges between 1/2 percentage point per year and 1-1/2 percentage points per year. Although this range happens to coincide with the one I gave two years ago, it does reflect both the improvements in the index that the BLS has implemented since then and the emergence of evidence suggesting that the initial problem was of a slightly greater dimension than had previously been estimated. This estimate is consistent with a number of microstatistical studies as well as an independently derived macroevaluation by staff at the Federal Reserve Board, which I will discuss shortly. In judging these evaluations, it is incumbent upon us to resist the evident strong inclination to believe that precision is the equivalent of accuracy in price bias estimation. If we cannot find a precise estimate for a certain bias, we should not implicitly choose zero as though that was a more scientifically supportable estimate. There is no sharp dividing line between a pristine estimate of a price and one that is not. All of the estimates in the CPI are approximations, in some cases very rough approximations. Further, even very rough approximations can give us a far better judgment of the cost of living, than holding to a false precision of accuracy. We would be far better served following the wise admonition of John Maynard Keynes that "it is better to be roughly right than precisely wrong." Estimates of the magnitude of the bias in our price measures are available from a number of sources. Most have been developed from detailed examinations of the microstatistical evidence. However, recent work by staff economists at the Federal Reserve Board has added strong corroborating evidence of price mismeasurement using a macroeconomic approach that is essentially independent of the exercises performed by other researchers, including those on the Boskin Commission. In particular, employing the statistical system from which the Commerce Department estimates the national income and product accounts, the research finds that measured real output and productivity in the service sector are implausibly weak, given that the return to owners of businesses in that sector apparently has been well- maintained. Taken at face value, the published data indicate that the level of output per hour in a number of service- producing industries has been falling for more than two decades. In other words, the data imply that firms in these industries have been becoming less and less efficient for more than twenty years. These circumstances simply are not credible. On the reasonable assumption that nominal output and hours worked and paid of the various industries are accurately measured, faulty price statistics are almost surely the likely cause of the implausible productivity trends. The source of a very large segment of these prices is the CPI. For this exercise, the study used the GDP chain-weight price measures. Although these price measures are based on many of the same individual price indexes included in the CPI, they do not suffer from upper-level substitution bias. Hence, the price mismeasurement revealed by this data system largely reflects shortcomings in quality adjustment and in the treatment of new goods and services. If, instead of declining, productivity in these selected service industries was flat, to up a modest one percentage point per year, the implicit aggregate price bias associated with these service industries alone would be on the order of 1/2 percentage point or so per annum in recent yearsâ€”very similar in magnitude to the Boskin Commission estimate of total quality adjustment and new products bias. To be sure, it is theoretically possible that some of the measured productivity declines in these service industries merely reflect mispricing of intermediate transfers among various industries. Such an occurrence would cause an understatement of productivity in some sectors, but a corresponding overstatement in others. But the available evidence suggests that for these particular service industries this theoretical possibility is not of a sufficiently large empirical magnitude to overturn the basic conclusion that there are serious measurement problems in our price statistics. Moreover, the study did not attempt to evaluate possible quality and new products bias in other industries. Some observers who are skeptical that the bias in the CPI could be very large have noted that the evidence on the magnitude of unmeasured quality change and the importance of new items bias is incomplete and inconclusive. Without a doubt, quality change and new items are among the most difficult of the problems currently confronting the BLS. But since I raised this issue two years ago in my testimony before this committee, a number of studies have documented significant new examples of cases in which the current treatment in the CPI results in an overstatement of the rate of growth of the cost of living. There doubtless are certain components of the CPI that are biased downward because quality change is handled inappropriately. One instance in which there may well be a problem in this regard pertains to new vehicles, where it may be more appropriate to treat pollution control and mandatory safety equipment, at least in part, as raising price to a consumer rather than improving quality, as is the present practice. But the potential downward bias introduced by current methodology for such equipment can only be slight. We should be prepared to embrace credible new research on quality adjustment, regardless of whether that research points to additional sources of upward bias or previously undetected instances of downward bias. Nonetheless, currently available evidence very strongly supports the view that, on balance, the bias is decidedly toward failing to appropriately capture quality improvements in our price indexes. There is little reason to believe that this conclusion will change unless we alter our procedures. A more difficult quality related issue is whether to reflect changes in broad environmental and social conditions in price measures that are used for indexing various components of federal outlays and receipts. That is, should the CPI reflect the influence of factors such as the level of crime, air and water quality, and the emergence of new diseases, which are not specifically related to products that consumers purchase? There is little in the record to suggest that, when it enacted the indexation of social security benefits in 1972, the Congress intended for the beneficiaries of that program to be compensated for changes in such environmental and social factors. Nor do these issues appear to have been raised when Congress debated the indexation of various tax parameters during the 1980s. Taking account of such conditions, particularly those that lie outside of the markets for goods and services, would be an interesting exercise in its own right, but would appear to extend well beyond the original intent of the Congress. A considerable professional consensus already exists for at least two actions that would almost surely bring the CPI into closer alignment with a true cost-of-living index. First, we should move away from the concept of a fixed marketbasket at the upper level of aggregation, and move toward an aggregation formula that takes into account the tendency of consumers to alter the composition of their purchases in response to changes in relative prices. The BLS already calculates such an index on an experimental basis with a lag of about a year. If the Bureau adopts the Boskin Commission's recommendation that it publish a "best practice" version of the CPI with a lag of a year, it should, without question, build that index on the foundation of a variable marketbasket. There is a somewhat more difficult issue as to whether the concept of a variable marketbasket can be applied in "real time," that is, with the same degree of timeliness that characterizes the current CPI. It is not possible to implement the textbook versions of any of the so-called "superlative" index formulas in real time, because those formulas require contemporaneous data on expenditures, and those data are not presently available until about a year after the fact. However, this hardly forecloses the possibility of implementing an approximation to a superlative formula, and work should continue on the development of such an approximation. A second area that will require attention is the aggregation of prices at the most detailed level of the index. This is a highly technical area, and an important example of how research by the staff at the BLS has advanced our knowledge. Without going into the details of the matter, it is sufficient to say that a selective move away from the current aggregation formula is warranted, and would probably make a modest further contribution to bringing the index more in line with the concept of a cost-of-living index. Beyond these rather limited steps, most of the needed developments will require time, effort, and quite possibly additional resources. It is important that the Congress provide the Bureau with sufficient resources to pursue the agenda vigorously. These are difficult problems, and cannot be solved tomorrow or next week. But with adequate support and diligent effort, the pace of improvement should quicken. Moreover, an accelerated pace of BLS activity, and heightened congressional interest should galvanize analysts outside the government to contribute to the research effort. Where will this longer-term effort be required? One of the key areas, by all accounts, is quality adjustment. As the Bureau has rightly noted, they do indeed already employ a variety of methods to control for quality change, but available evidence suggests that these are not sufficient to the task. Unfortunately, making improvements on this front will be difficult: Each item will have to be considered on its own, and there may well be limited transfer of knowledge from one item to the next. Another key area on the longer-term agenda will be the estimation of the value of new products to consumers. Significant innovations, such as the personal computer, the cellular telephone, and the heart bypass operation create value for consumers, even at their typically high initial prices; moreover, this value is even greater at the much lower prices that often prevail when new products are, in fact, introduced into the CPI. A true cost-of-living index would reflect this value and its implication for the true rate of growth of the cost of living. The CPI does not reflect it, and accordingly fails to capture a significant offset to price rises in other products. Deriving an estimate of this value and building it into the CPI will not be an easy undertaking. But conceptually, it is unquestionably the right direction to be heading, and some recent research suggests that it could measurably affect the index. Over time, we will need to investigate alternative sources of data. Already, there is interesting work being done to develop techniques for processing data collected from bar-code scanners at the check-out counter. Scanner data will allow the BLS to track not just a small sample of products, but virtually the entire universe of products in selected lines of business and, perhaps most importantly, virtually the universe of transactions, regardless of whether those transactions happen on a weekday, at night, or on a holiday. We should also move to improve our understanding of the value that consumers place on their own time. Absent such knowledge, it will be impossible for the BLS to estimate the value of many goods and services that mainly serve to enhance convenience and save time. Finally, we will have to attempt to build an understanding of why consumers shop at the places they do: What characteristics of an outlet are important, and how much so? Location, hours of operation, inventory, and quality of service all are likely influences on the value that consumers place on their shopping experience, and all will be important in helping the BLS to develop a more sophisticated statistical method for dealing with the appearance of new consumer outlets, including those that operate over the Internet. Even if the BLS moves aggressively, some upward bias will almost surely remain in the CPI, at least for the next several years. Two years ago, in testimony before this committee, I suggested that a workable structure for dealing with this situation might involve a two-track approach. That suggestion still seems to me to make sense. The first track would involve action by the BLS to address those aspects of the bias that can be dealt with in relatively short order, say within the next year. The second track would involve the establishment of an independent national commission to set annual cost-of-living adjustment factors for federal receipt and outlay programs. The Commission would examine available evidence on a periodic basis, and estimate the bias in the CPI taking into account both the latest research on the sources and magnitudes of the bias, and any corrective actions that had been taken by the BLS. This type of approach would have the benefit of being objective, nonpartisan, and sufficiently flexible to take full account of the latest information. Moreover, there is no reason why the two tracks could not proceed in parallel. Without the second track, we are implicitly assuming, contrary to overwhelming evidence, that the most accurate estimate of the bias is zero. There has been considerable objection that such a second track procedure would be a political fix. To the contrary, assuming zero for the remaining bias is the political fix. On this issue, we should let evidence, not politics, drive policy. We have an overarching national interest in building a better measure of consumer prices and in implementing more rational indexation procedures. Through these efforts, we are most likely to ensure that the original intent of the relevant pieces of legislation will be fulfilled in insulating taxpayers and benefit recipients from the effects of ongoing changes in the cost of living. At present this objective is not being met.</t>
-  </si>
-  <si>
-    <t>Madam Chairwoman, members of the Subcommittee on Financial Institutions and Consumer Credit, it is a pleasure to appear here today to present the views of the Federal Reserve Board on some broad issues associated with financial modernization The unremitting pressures of technology and the market are drastically changing the financial landscape and eroding traditional positions of competitors, inducing new competitive strategies and participants, forcing new regulatory responses, and building pressures on the Congress to shape developments in the public interest Madam Chairwoman, I know that you have been an active sponsor and supporter of legislation to modernize the financial system The Board also has been a strong proponent both of expanded financial activities for banking organizations and enhanced opportunities for nonbank financial institutions to enter banking We continue to support financial modernization because we believe it would provide improved financial services for our citizens Moreover, both our expenence and analysis suggest that the additional risks of new financial products are modest and manageable Indeed, technology already has resulted in a blurring of product and service-defining lines so dramatic as to make many financial products virtually indistinguishable from each other and the old rules inapplicable In the process, we have already seen the public benefits, benefits that removal of old barriers could only enhance But, as we proceed down the path of reform, reforms both desired for their benefits to the public and required by global markets and new technologies, the Board urges that any modifications be tested against certain standards In particular, the Board believes that the changes we adopt should be consistent with (1) continuing the safety and soundness of the banking system, (2) limiting systemic risks, (3) contributing to macroeconomic stability, and (4) limiting the spread of both the moral hazard and the subsidy implicit in the safety net Thus, if my comments today sound cautious, I want the subcommittee to understand that my observations do not reflect opposition to further freeing of constraints on financial competition To the contrary We strongly urge an extensive increase in the activities permitted to banking organizations and other financial institutions, provided these activities are financed at nonsubsidized market rates and do not pose unacceptable risks to our financial system. While a level playing field requires broader powers, it does not require subsidized ones. Safety Net Implications In this century the Congress has delegated the use of the sovereign credit-the power to create money and borrow unlimited funds at the lowest possible rate-to support the banking system It has done so indirectly as a consequence of deposit insurance, Federal Reserve discount window access, and final riskless settlement of payment system transactions The public policy purpose was to protect depositors, stem bank runs, and lower the level of risk to the financial system from the insolvency of individual institutions In insuring depositors, the government, through the FDIC, substituted its unsurpassable credit rating for those of banks Similarly, provisions of the Federal Reserve Act enabled banks to convert illiquid assets, such as loans, into riskless assets (deposits at the central bank) through the discount window, and to complete payments using Federal Reserve credits All these uses of the sovereign credit have dramatically improved the soundness of our banking system and the public's confidence in it In the process, it has profoundly altered the risks and returns in banking Sovereign credit guarantees have significantly reduced the amount of capital banks and other depositones need to hold, since creditors demand less of a buffer to protect themselves from the failure of institutions that are the beneficiaries of such guarantees In different language, these entities have been able to operate with a much higher degree of leverage-that is, to obtain more of their funds from other than the owners of the organizationâ€”than virtually all other financial institutions At the same time, depositories have been able to take greater risk in their portfolios than would otherwise be the case, because private creditors-depositors and others-are less affected by the illiquidity of, or losses on, the banks' portfolios The end result has been a higher risk-adjusted rate of return on depository institution equity Moreover, the enhanced ability to take risk has contnbuted to economic growth, while the discount window and deposit insurance have contributed to our macroeconomic stability But all good things have their pnce The use of the sovereign credit in bankingâ€”even its potential use-creates a moral hazard that distorts the incentives for banks the banks determine the level of risk-taking and receive the gains therefrom, but do not bear the full costs of that risk The remainder of the risk is transferred to the government. This then creates the necessity for the government to limit the degree of risk it absorbs by writing rules under which banks operate, and imposing on these entities supervision by its agentsâ€”the banking regulatorsâ€”to assure adherence to these rules The expenence in the 1980s with many insured thrift institutions showed just how dangerous lax enforcement of supervisory rules can be In the end, some hard lessons were learned, many of which were legislated into the FDIC Improvement Act of 1991 The subsidy to the banking and other depositories created by the use of the unsurpassable sovereign credit rating of the United States government is an undesirable but unavoidable consequence of creating a safety net Indeed, one measure of the effectiveness of a safety net is our ability to minimize the subsidy and limit its incidence outside of the area to which it was directed Some of the value of the subsidy has been passed to depositors of, and borrowers from, banks, for example, as well as to the original bank shareholders But, the United States government has been remarkably successful in containing the value of most of the subsidy within depository institutions The bank holding company organizational structure has, on balance, provided an effective means of limiting the use of the sovereign credit subsidy by other parts of the banking organization To be sure, bank holding companies have indirectly benefitted from the subsidy because their major assets are subsidiary banks The value of the subsidy given to the subsidiary banks has no doubt been capitalized in part into the share prices of holding companies and has improved their debt ratings, lowering their cost of capital But, holding companies also own nonsubsidized entities that have no direct access to the safety net Accordingly, both bank holding companies and their nonbank subsidiaries have a higher cost of capital than banks This is clear in the debt ratings of bank subsidiaries of bank holding companies, which are virtually always higher than those of their parent holding companies Moreover, existing law and regulation under Sections 23A and 23B of the Federal Reserve Act require that any credit extended by a bank to its parent or affiliate not only be totally collateralized and subject to quantitative limits, but also be extended at arms-length and at market rates, making a direct transfer of the safety net subsidy difficult It is true that a bank could pay dividends from its earnings, earnings which have been enhanced by the safety net subsidy, to fund its parent's nonbank affiliates However, the evidence appears to be that such transfers generally do not occur Existing holding company powers are limited and do not offer a broad spectrum of profitable opportunities Accordingly, it is not surprising that data for the top 50 bank holding companies indicate that transfers from bank subsidiaries to their parents which, like dividends, embody the subsidy, appear to have approximately equaled holding company net transfers to their own shareholders and long-term creditors This indicates that few subsidized dollars in the aggregate found their way into the equity accounts of holding company nonbank affiliates from the upstreaming of bank funds We must, I think, be continually on guard that the subsidy provided by the safety net does not leak outside the institutions for which it was intended and provide a broad subsidy to other kinds of activities Put another way, we must remain especially vigilant in maintaining a proper balance between a safety net that fosters economic and financial stabilization and one that benefits the competitive position of private businesses for no particular public purpose As I noted, safety net subsidies have costs in terms of distorted incentives and misallocated resources That is why the Congress must be cautious in how the sovereign credit is used It has been suggested that the bank holding company structure imposes inefficiencies on banking organizations, and that these organizations should thus be given the option of conducting expanded financial activities in a direct subsidiary of the bank The bank subsidiary may be a marginally more efficient way of delivering such services, but we believe it cannot avoid being a funnel for transferring the sovereign credit subsidy directly from the bank to finance the new powers, thereby imparting a subsidized competitive advantage to the subsidiary of the bank One can devise rulesâ€”such as 23A and 23B-to assure that loans from the bank to its own subsidiaries are limited and at market rates One can even devise rules to limit the aggregate equity investment made by banks in their subsidiaries But one cannot eliminate the fact that the equity invested in subsidiaries is funded by the sum of insured deposits and other bank borrowings that directly benefit from the subsidy of the safety net Thus, inevitably, a bank subsidiary must have lower costs of capital than an independent entity and even a subsidiary of the bank's parent Indeed, one would expect that a rational banking organization would, as much as possible, shift its nonbank activity from the bank holding company structure to the bank subsidiary structure Such a shift from affiliates to bank subsidiaries would increase the subsidy and the competitive advantage of the entire banking organization relative to its nonbank competitors I am aware that these are often viewed as only highly technical issues, and hence ones that are in the end, of little significance I do not think so The issue of the use of the sovereign credit is central to how our financial system will allocate credit, and hence real resources, the kinds of risk it takes, and the degree of supervision it requires If the Congress wants to extend the use of the sovereign credit further, to achieve a wider range over which the benefits of doing so can accrue, it ought to make that decision explicitly, and accept the consequences of the subsidy on the financial system that come with it But, it should not, in the name of some technical change, or in search of some minor efficiency, inadvertently expand the use of the sovereign credit This issue would not be so important were we not in the process of addressing what must surely be a watershed in the revamping of our regulatory structure We must avoid inadvertently extending the safety net and its associated subsidy without a thorough understanding of the implications of such an extension to the competitive balance and systemic risks of our financial system Central to the Board's choice of a financial structure is its desire for one that will be most effective in fostering both a viable financial system and a vibrant economy These objectives, in our view, would be thwarted if the safety net subsidy directly benefitted new activities With the safety net comes the moral hazard of which I spoke earlier, and its attendant misallocation of resources, and uneven competitive playing field If the government subsidies directed to banks were channeled to bank subsidiaries, in my judgement, both the benefits and enumerated costs to the financial system and the public would occur If banks were permitted to engage in new activities in their own subsidiaries, inevitably virtually all holding companies would shift those activities now conducted in holding company affiliates to bank subsidiaries, eviscerating the holding company structure Were such shifts to happen solely as the result of operational efficiencies, no one, including the Board, should mourn the demise of the holding company But if, as I suspect, such shifts occurred because of the attraction of a government subsidy, we should be concerned because the insidious effects of such subsidies would have spread The evidence from flows between banks and their parents, relative bond ratings, and the administration of Sections 23A and B of the Federal Reserve Act, all strongly suggest that the holding company structure is far more capable of containing the sovereign credit subsidy whose purpose is support of the safety net, not providing expanded competitive advantage As new activities hopefully expand for banking organizations, we believe that it is essential that we assure they are financed at market rates, not subsidized ones This will not always be easy Containment of subsidies is often implemented through firewalls and other devices which could also inhibit the very synergies which the expansion of activities is meant to achieve But we have dealt with these trade-offs before and should be able to in the future as well Umbrella Supervision Whether new activities are authorized in bank subsidiaries, bank holding companies, or both, Congress, in its review of financial modernization, must consider legal entity supervision versus umbrella supervision The Board believes that umbrella supervision is a realistic necessity for the protection of our financial system and to limit any misuse of the sovereign credit The bank holding company organization is increasingly being managed so as to take advantage of the synergies between its component parts in order to deliver better products to the market and higher returns to stockholders Such synergies cannot occur if the model of the holding company is one in which the parent is just, in effect, a portfolio investor in its subsidiary Indeed, virtually all of the large holding companies now operate as integrated units and are managed as such As bank holding companies began to widen their activities, and as new technologies permitted not only the development of new products but also the systems for controlling them, the banking organization was impelled to develop centralized risk control techniques that crossed legal entities Today, risk management for the entire company is increasingly centralized not only at the larger and more sophisticated banking organizations, but at other large financial services providers as well This development reflects the demands of the marketplace, which views banks and their affiliates and other financial businesses and their affiliates as integrated organizations in terms of financial condition, management and reputation To understand the risk controls of the bank, we have first to come to grips with the fact that the organization is interested in risk and its control, not by instrument or legal entity, but for the entire business This type of control is being adopted by more and more organizations each year, and can only increase as more activities are authorized by the regulators and the Congress Regulatory policies and operating procedures have had to respond to these realities, to focus on the process of decisionmaking for the total organization Thus, the Federal Reserve-the historical umbrella supervisorâ€”also has found it necessary to concentrate more on the process that banking organizations use to manage market, credit, operating and exchange rate risk, and less on the traditional after- the-fact evaluation of balance sheets that can and often do change dramatically the day after they have been reviewed by the supervisors In such a world, process, if not everything, is critical, and that process is determined increasingly at the parent holding company for all of the units of the organization on a consolidated basis One could argueâ€”as several witnesses appearing before this subcommittee did on Tuesdayâ€”that regulators should only be interested in the entities they regulate and, hence, review the risk evaluation process only as it relates to their regulated entity Presumably each regulator of each entityâ€”the bank regulators, the SEC, the state insurance and finance company authonties-would look only at how the risk management process affected their units It is our belief that this simply will not be adequate Risks managed on a consolidated basis cannot be reviewed on an individual legal entity basis by different supervisors Indeed, our expenence has been that a problem in one legal entity can have a contagion effect in other entities If a bank affiliate begins to have difficulty, the market evaluates the problem as the consolidated entity's problem and can bring pressure on all the units These pressures usually take the form of funding or liquidity difficulties, as creditors seek to reduce their exposure to all units of an organization that seems to be having trouble Better safe than sorry Indeed, it is in the cauldron of the payments and settlement system, where decisions involving large sums must be made in short periods, that this contagion effect might be first seen as participants understandably seek to protect themselves from the uncertainty that accompanies this contagion effect And that is how crises often begin These concerns were part of the motivation for the congressional decision just five years ago to require that foreign banks could enter the United States if, and only if, they were subject to consolidated supervision, This decision, which is consistent with the international standards for consolidated supervision of banking organizations, was a good decision then It is a good decision today, especially for those banking organizations whose disruption could cause major financial disturbances in United States and foreign markets For foreign and for U S banking organizations, retreat from consolidated supervision would, the Board believes, be a significant step backward We have to be careful, however, that consolidated umbrella supervision does not inadvertently so hamper the decisionmaking process of banking organizations as to render them ineffectual The Federal Reserve Board is accordingly in the process of reviewing its supervisory structure and other procedures in order to reflect the aforementioned market-directed shift from conventional balance sheet auditing to evaluation of the internal risk management process Although focussed on the key risk management processes, it would sharply reduce routine supervisory umbrella presence in holding companies As the Committee knows, the Board has recently published for comment proposals to expedite the applications process, and the legislation Congress enacted last year eased such procedures as well Nonetheless, the Board requests even greater modification to its existing statutory mandate so that the required applications process could be sharply cut back, particularly in the area of nonbank financial services. We would hope that should the Congress authorize wider activities for financial services holding companies that it recognize that a bank which is a minor part of such an organization (and its associated safety net) can be protected through adequate bank capital requirements and the application of Sections 23A and 23B of the Federal Reserve Act The case is weak, in our judgment, for umbrella supervision of a holding company which, because it owns only a small bank, does not have material access to the safety net As I noted when discussing the safety net and bank subsidiaries, attached to all uses of the sovereign credit come efforts by the government to protect the taxpayer Those entities interested in banks are really interested in access to the safety net, since it is far easier to engage in the nonsafety net activities of banks without acquiring a bank If an organization chooses to deliver some of its services with the aid of the sovereign credit by acquiring a bank, it should not be excused from efforts of the government to look out for the stability of the overall financial system For bank holding companies that own more than a small bank, this implies umbrella supervision Although that process will increasingly be designed to reduce supervisory presence and be as nonintrusive as possible, umbrella supervision should not be eliminated, but recognized for what it is: the cost of obtaining a subsidy Banking and Commerce Finally, let me turn to an issue that has bedeviled supervisory and regulatory discussions for years the potential separation of commerce and banking As I indicated earlier, it is clear that rapidly changing technologies are altering the nature of what constitutes finance Indeed, just as the lines between banking and other financial institutions are often already difficult to discern, the boundaries between finance and nonfinance are likely to become increasingly indistinct as we move into the 21st century For example, computer and software firms will certainly be offenng ever more sophisticated financial products And doubtless financial firms will be offenng an increasingly sophisticated array of nonfinancial services In addition, some of the financial firms who mainly produce products and services that many observers believe should be permissible to banks are also engaged in, or affiliated with, nonfinancial businesses Newer technologies will make it highly unlikely that the walling off of any ownership of financial institutions by nonfinancial businesses and vice-versa can be continued very far into the 21st century Nonetheless, the Board has concluded that it would be wise to move with caution in addressing the removal of the current legal barriers between commerce and banking The free and open legal association of banking and commerce would be a profound and surely irreversible structural change in the American economy Hence, we must be careful to assure ourselves that whatever changes are made in our supervisory structure, that it not distort our evolution to the most efficient financial structure as we move into the next century Were we fully confident of how the structure would evolve, we could presumably construct today the regulations which would foster that evolution But we cannot be certain We thus run the risk of locking in a set of inappropriate regulations that could adversely alter the development of market structures We cannot be confident we know what the true synergies between finance and nonfinance will be in ten or even five years Our ability to foresee accurately the future implications of technologies and market developments in banking, as in other industries, has not been particularly impressive As Professor Rosenberg of Stanford University has pointed out, " mistaken forecasts of future structure litter our financial landscape " Consider the view of the 1960s that the "cashless society" was imminent Nonetheless, the public preference for paper has declined only gradually Similarly, just a few years ago conventional wisdom argued that banks were dinosaurs that were becoming extinct The reality today is far from it Even more recently, it was argued that banks and nonfinancial firms had to merge in order to save the capital-starved banking system Today, as you know, virtually all of our banks are very well capitalized. All these examples suggest that if we change the rules now about banking and commerce under circumstances of uncertainty about future synergies between finance and nonfinance we might end up doing more harm than good And, as with all rule changes by government, we are likely to find it impossible to correct our errors promptly Modifications of such a fundamental structural rule as the separation of banking and commerce should accordingly proceed at a deliberate pace, testing the response of markets and technological innovation to the altered rules in the years ahead The public needs to have confidence in the regulatory structure, implying that we proceed slowly and cautiously Excessive delay, however, would doubtless produce some inequities Expanded financial activities for banking organizations requires, the Board believes, that those firms operating in markets that banks can enter should, in turn, be authorized to engage in banking However, some of these nonbanking financial firms already own-or are owned byâ€”nonfinancial entities A complete commerce and banking prohibition would thus require the divestiture of all nonfinancial activities by those organizations that wanted to acquire or establish banks The principle of caution suggests an approach which may prove useful Perhaps those organizations that either have or establish well-capitalized and well-managed bank subsidiaries should be permitted a small basket of nonfinancial assetsâ€”a certain percentage of either consolidated assets or capital A small permissible basket would establish, in effect, a pilot program to evaluate the efficacy of further breaching of the banking and commerce wall We found that such a slow and deliberate policy worked well with Section 20 affiliates Of course, some nonbanking firms would find that their nonfinancial activities would exceed a small basket exemption Such excess nonconforming assets might be addressed on a case-by-case basis with a scheduled longer-term divestiture to avoid the worst short-term inequities A basket clause plus case-by-case review of individual situations might also provide a way to make available a common bank and thrift charter to those unitary thrifts that are affiliated with nonfinancial businesses The Board has no firm opinion on just exactly how such trade-offs might be made, constrained only by the general concerns I summanzed earlier</t>
-  </si>
-  <si>
-    <t>I am pleased to participate once again in the Federal Reserve Bank of Atlanta's annual Financial Markets Conference As in previous years, the Reserve Bank has developed a conference program that is quite timely Changes in technology have permitted the development in recent years of increasingly diverse financial instruments and intensely competitive market structures The rapid evolution of products and markets has led many to conclude that market regulatory structures, many of which were established in the 1920s and 1930s, have become increasingly outdated Some see new products and markets not covered by government regulation and fear the consequences of so-called "regulatory gaps" Others see old government regulations applied to new instruments and markets and fear the unintended consequences of what seems unnecessary and burdensome regulation Nowhere have these tensions been more evident than in the ongoing debate over the appropriate government regulation of derivative contracts, a debate which has varied in intensity but has never fully subsided for at least ten years Recent efforts by members of the Senate Agriculture Committee to clarify and rationalize the regulation of derivative contracts under the Commodity Exchange Act have once again placed these contentious issues on the front burner In my remarks today I shall proffer a set of considerations that I find quite valuable as a guide to decisions about the need for government regulation of financial markets I shall then review the history of government regulation of derivative contracts and markets in the United States and consider the current regulatory structure for those products and markets in light of these considerations I would argue that the first imperative when evaluating market regulation is to enunciate clearly the public policy objectives that government regulation would be intended to promote What market characteristics do policymakers seek to encourage? Efficiency? Fair and open access? What phenomena do we wish to discourage or eliminate? Fraud, manipulation, or other unfair practices? Systemic instability? Without explicit answers to these questions, government regulation is unlikely to be effective More likely, it will prove unnecessary, burdensome, and perhaps even contrary to what more careful consideration would reveal to be the underlying objectives A second imperative, once public policy objectives are clearly specified, is to evaluate whether government regulation is necessary for those purposes In making such evaluations, it is critically important to recognize that no market is ever truly unregulated The self- interest of market participants generates private market regulation Thus, the real question is not whether a market should be regulated Rather, the real question is whether government intervention strengthens or weakens private regulation If incentives for private market regulation are weak or if market participants lack the capabilities to pursue their interests effectively, then the introduction of government regulation may improve regulation But if private market regulation is effective, then government regulation is at best unnecessary At worst, the introduction of government regulation may actually weaken the effectiveness of regulation if government regulation is itself ineffective or undermines incentives for private market regulation We must be aware that government regulation unavoidably involves some element of moral hazard--if private market participants believe that government is protecting their interests, their own efforts to protect their interests will diminish to some degree Whether government regulation is needed, and if so, what form of government regulation is optimal, depends critically on a market's characteristics A "one-size-fits-all" approach to financial market regulation is almost never appropriate The degree and type of government regulation needed, if any, depends on the types of instruments traded, the types of market participants, and the nature of the relationships among market participants To cite just one example, a government regulatory framework designed to protect retail investors from fraud or insolvency of brokers is unlikely to be necessaryâ€”and is almost sure to be suboptimalâ€”if applied to a market in which large institutions transact on a principal-to- principal basis Recognizing that a one-size-fits-all approach is seldom appropriate, it may be useful to offer transactors a choice between seeking the benefits and accepting the burdens of government regulation, or forgoing those benefits and avoiding those burdens by transacting in financial markets that are only privately regulated In such circumstances, the privately regulated markets in effect provide a market test of the net benefits of government regulation Migration of activity from government-regulated to privately regulated markets sends a signal to government regulators that many transactors believe the costs of regulation exceed the benefits When such migration occurs, government regulators should consider carefully whether less regulation or different regulation would provide a better cost-benefit tradeoff without compromising public policy objectives Before evaluating the current regulation of derivatives in light of these considerations, it is quite useful to know something of the history of these instruments and their regulation Derivative contracts (forward contracts and options) appear to have been utilized throughout American history Indeed, it will probably come as a surprise even to this audience that 15 to 25 percent of trades on the New York Stock Exchange in its early years were time bargains, that is, forward contracts, rather than transactions for cash settlement (in those days, same-day settlement) or regular-way settlement (next-day settlement) In the case of commodities, forward contracts for corn, wheat, and other grains came into common use by 1850 in Chicago, where they were known as "to arrive" contracts The first organized futures exchange in the United States, the Chicago Board of Trade, evolved through the progressive standardization of the terms of to arrive contracts, including lot sizes, grades of grain, and delivery periods Trading apparently was centralized on the Board of Trade by 1859, and in 1865 it set out detailed rules for the trading of highly standardized contracts quite similar to the grain futures contracts traded today The first recorded instance of federal government regulation of derivatives was the Anti-Gold Futures Act of 1864, which prohibited the trading of gold futures The government had been unhappy that its fiat currency issues, the infamous greenbacks, were at that time trading at a substantial discount to gold Unwilling to accept this result as evidence of failure of the government's monetary policies, Congress concluded that it was evidence of a serious failure of private market regulation In the event, Congress's action was followed by a further sharp drop in the value of the greenbacks Although it took the government many years to restore monetary policy to a sound footing, it took Congress only two weeks to conclude that its prohibition of gold futures was having unintended consequences and to repeal the act It has been the trading of agricultural futures, however, that from its inception has produced calls for government intervention Throughout the late nineteenth and early twentieth centuries, farmers were often opposed to futures trading, particularly during periods when prices of their products were low or declining They presumed that dreaded speculators were depressing their prices The states were the first to respond to calls for government regulation of futures For the most part, state legislation on futures was limited to prohibitions on bucket shops, that is, operations that purport to act as brokers of exchange- traded futures but "bucket" rather than execute their clients' trades An Illinois statute of 1874 signaled early concerns about market integrity The statute criminalized the spreading of false rumors to influence commodity prices and attempts to corner commodity markets After its misadventure with futures regulation during the Civil War, the federal government appears not to have given further consideration to regulating futures trading until 1883, when a bill was introduced in Congress to prohibit use of the mails to market futures Thereafter, repeated efforts were made to regulate or prohibit trading of futures and options on agricultural products When the Agriculture Department reviewed the Congressional Record in 1920, it found that 164 measures of this sort had previously been introduced These efforts culminated in passage of the Futures Trading Act of 1921 That act was promptly declared unconstitutional by the Supreme Court, on the grounds that it was a regulatory measure masquerading as a tax measure But in 1922 Congress restated the purpose of the 1921 act as "an act for the prevention and removal of obstructions and burdens upon interstate commerce in grain, by regulating transactions on grain futures exchanges," and renamed it the Grain Futures Act of 1922 As an explicitly regulatory measure, it was later upheld by the Court The objective of the Grain Futures Act was to reduce or eliminate "sudden or unreasonable fluctuations" in the prices of grain on futures exchanges The framers of the act believed that such sudden or unreasonable fluctuations of grain futures prices reflected their susceptibility to "speculation, manipulation, or control" Moreover, such fluctuations in price were seen to have broad ramifications that affected the national public interest Grain futures contracts were widely used by producers and distributors of grain to hedge the risks of price fluctuations Futures prices also were widely disseminated and widely used as the basis for pricing grain transactions off the futures exchanges Indeed, given the relative size of the agricultural sector of the time, fluctuations in futures prices no doubt had the potential to affect the economy as a whole It is not entirely clear that the view that futures trading was exacerbating volatility in agricultural prices was well-founded To be sure, evidence abounds that market participants talked incessantly about corners and bear raids Moreover, the design of the contracts may, indeed, have made such contracts susceptible to manipulation However, empirical studies of more recent experience cast doubt on whether the use of derivatives adds to price volatility And, while charges of market manipulation are heard to this day, they typically are difficult, if not impossible, to prove Professional speculators were easy to blame for fluctuations in market prices that actually reflected fundamental shifts in supply or demand, as they are today The market clearing process is a very abstract concept It is sometimes far easier to envisage price changes as the consequence of individual manipulators Indeed, for a lot of 19th century ring traders, it was some measure of manhood (women were few) that they could squeeze or corner a market The evidence suggests that this was largely Walter Middy- type fantasy In any event, the Grain Futures Act of 1922 established many of the key elements of our current regulatory framework for derivatives In general, the act was designed to confine futures trading to regulated futures exchanges The act made it unlawful to trade futures on exchanges other than those designated as contract markets by the Secretary of Agriculture The Secretary was permitted to so designate an exchange only if certain conditions were met These included the establishment of procedures for recordkeeping and reporting of futures transactions, for prevention of dissemination of false or misleading crop or market information, and for prevention of price manipulation or cornering of markets Finally, the act recognized the need to permit bona fide derivatives transactions to be executed off of the regulated exchanges, it explicitly excluded forward contracts for the delivery of grain from the exchange-trading requirement Forward contracts were essentially defined as contracts for future delivery to which farmers or farm interests were counterparties or in which the seller, if not a farmer, owned the grain at the time of making the contract The next major piece of federal legislation affecting futures regulation was the Commodity Exchange Act (CEA) of 1936 As in the case of the Grain Futures Act, an important objective of the CEA was to discourage forms of speculation that were seen as exacerbating price volatility In addition, the CEA introduced provisions designed primarily to protect small investors in commodity futures, whose participation had been increasing and was viewed as beneficial These provisions included requirements for the registration of futures commission merchants (FCMs), that is, futures brokers, and for the segregation of customer funds from FCM funds The CEA also expanded the coverage of futures regulation to cover contracts for cotton, rice, and certain other specifically enumerated commodities traded on futures exchanges, and prohibited the trading of options on commodities traded on futures exchanges The federal regulatory framework for derivatives market regulation then remained substantially unchanged until 1974, when Congress enacted the Commodity Futures Trading Commission Act The act did not make any fundamental changes in the objectives of derivatives regulation However, it expanded the scope of the CEA quite significantly In addition to creating the Commodity Futures Trading Commission (CFTC) as an independent agency and giving the CFTC exclusive jurisdiction over commodity futures and options, the 1974 amendments expanded the CEA's definition of "commodity" beyond a specific list of agricultural commodities to include "all other goods and articles, except onions, and all services, rights, and interests in which contracts for future delivery are presently or in the future dealt in " In one respect, this was sweeping deregulation, in that it explicitly allowed the trading on futures exchanges of contracts on virtually any underlying assets, including financial instruments Only onion futures, banned in 1958 as the presumed favorite plaything of manipulators, remained beyond the pale In another respect, however, this was a sweeping extension of regulation Given this broad definition of a commodity and an equally broad interpretation of what constitutes a futures contract, this change brought a tremendous range of off-exchange transactions potentially within the scope of the CEA In particular, it could 8 be interpreted to extend the broad prohibition on off-exchange trading of futures to an immense volume of diverse transactions that never had been traded on exchanges The potential for the legality of a wider range of transactions to be called into question did not go unnoticed during debate on the 1974 act In particular, the Treasury Department proposed language excluding off-exchange derivative transactions in foreign currency, government securities, and certain other financial instruments from the newly expanded CEA This proposal was adopted by Congress and is known as the Treasury Amendment In proposing the amendment, Treasury was primarily concerned with protecting foreign exchange markets from what it considered unnecessary and potentially harmful regulation The foreign exchange markets clearly have quite different characteristics from markets for agricultural futures-the markets for the major currencies are deep and, as some central banks have learned the hard way, they are extremely difficult to manipulate Furthermore, participants in those markets, primarily banks and other financial institutions, and large corporations, would not seem to need, and certainly are not seeking, the protection of the CEA Thus, there was, and is, no reason to presume that the regulatory framework of the CEA needs to be applied to the foreign exchange markets to achieve the public policy objectives that motivated the CEA Indeed, the wholesale foreign exchange markets provide a clear and compelling example of how private parties can regulate markets quite effectively without government assistance What the Treasury did not envision and the Treasury Amendment did not protect was the subsequent development and spectacular growth of privately negotiated derivative contractsâ€”swaps, forwards, and options on interest rates, exchange rates, and prices of commodities and securities The rapid growth of these instruments primarily reflected the value-added in specially crafted, individualized contracts that the standardized, one-size-fits-all contracts traded on exchanges did not provide By the mid-1980s, concerns already had surfaced that such contracts could prove unenforceable if they were found to be illegal off- exchange futures The CFTC recognized that the development of swaps and similar contracts provided important public benefits and eventually issued various rules and interpretations intended to allay concerns about their enforceability Nonetheless, substantial legal uncertainty about the reach of the CEA persisted Moreover, some were questioning the CFTC's interpretations of the CEA and its authority to exempt transactions that were futures from the exchange-trading requirement Congress sought to provide legal certainty for interest rate swaps and many of the other questioned transactions through a provision in the Futures Trading Practices Act of 1992 That provision granted the CFTC explicit authority to exempt off-exchange transactions between "appropriate persons" from most provisions of the CEA, including the exchange-trading requirement, "appropriate persons" are regulated financial intermediaries, other larger businesses, and others deemed appropriate by the CFTC The CFTC promptly utilized this authority to exempt interest rate swaps and most other OTC derivative contracts from the exchange-trading requirement and most other provisions of the CEA However, the CFTC reserved its anti-fraud and anti-manipulation authority with respect to any swaps that might be regarded as futures and also included provisions that would deny legal certainty to swaps that were executed through an exchange or cleared through a clearing house Later, the CFTC, which had been directed by Congress to promote fair competition between futures exchanges and the off-exchange markets, initiated a pilot program under which the futures 10 exchanges would be permitted to develop a new class of exchange-traded markets that would be exempt from some provisions of the CEA However, no exchange has taken advantage of this opportunity Despite the CFTC's efforts, uncertainty about the scope of the CEA and debate about the appropriateness of the CEA regulatory framework have continued Litigation has called into question the types of contracts and counterparties that are covered by the Treasury Amendment Because Congress prohibited the CFTC from exempting equity derivatives from the CEA, the enforceability of some OTC equity swaps has remained uncertain And the futures exchanges continue to argue that unnecessary and burdensome regulation is making it impossible for them to compete with off-exchange markets in the United States and with foreign futures exchanges Solutions to these problems can be identified by applying the key considerations relating to market regulation that I set out earlier There appears to be a fair degree of consensus on the objectives of public policy Most would agree that the objectives of derivatives regulation are endeavoring to ensure the integrity of markets, especially deterring manipulation, and to protect market participants from losses resulting from fraud or the insolvency of counterparties Where there is disagreement is on the need for government regulation to achieve these objectives, and where government regulation is agreed to be appropriate, on whether the CEA provides the optimal regulatory framework In the case of the institutional off-exchange derivatives markets, it seems abundantly clear that private market regulation is quite effectively and efficiently achieving what have been identified as the public policy objectives of government regulation I am aware of no evidence that the prices of OTC contracts have been manipulated Participants in these markets have been savvy enough to limit their activity to contracts that are very difficult to manipulate The vast majority of OTC contracts are settled in cash rather than through delivery The cash settlement typically is based on a rate or price in a highly liquid market with a very large or even unlimited deliverable supply, for example, LIBOR or the spot dollar-yen exchange rate Those OTC contracts that require delivery typically limit the costs of failing to deliver to actual damages Thus, attempts to corner an OTC market, even if successful, could not induce sellers to pay significantly higher prices to offset their contracts or to purchase the underlying assets In any event, prices of off-exchange contracts are not used directly or indiscriminately as the basis for pricing other transactions, so any price distortions would not affect other buyers or sellers of the underlying asset and certainly would not affect the economy as a whole Institutional participants in the off-exchange derivative markets also have demonstrated their ability to protect themselves from losses from fraud and counterparty insolvencies Participants in those markets have insisted that dealers have financial strength sufficient to warrant a credit rating of A or higher When such dealers have engaged in deceptive practices, their victims have been able to obtain restitution by going to court or simply threatening to do so The threat of legal damages provides dealers with incentives to avoid misconduct A far more powerful incentive, however, is the fear of loss of the dealer's good reputation, without which it cannot compete effectively, regardless of its financial strength or financial engineering capabilities Institutional participants in the off-exchange markets also 12 have demonstrated their ability to manage credit risks quite effectively through careful evaluation of counterparties, the setting of internal credit limits, and the judicious use of netting agreements and collateral Actual losses to institutional counterparties in the United States from dealer defaults have been negligible Thus, there appears to be no need for government regulation of off-exchange derivative transactions between institutional counterparties In particular, the CEA, which was designed for markets with completely different characteristics, seems an inappropriate framework for regulating such transactions Because many retail investors may lack the ability to evaluate their counterparties effectively, some government regulation of off- exchange transactions with such counterparties may be appropriate to protect them against unrecoverable losses from fraud or dealer insolvencies But, even for those transactions, it is not obvious that the CEA provides the best regulatory framework In particular, it seems to me that the marketing of off-exchange derivatives to retail customers by banks and broker- dealers is more appropriately regulated by the banking regulatory agencies and the Securities and Exchange Commission, respectively There is no evidence that the existing regulatory frameworks applicable to these institutions are not adequate to protect retail counterparties to off-exchange derivative contracts Some may argue that CEA-style regulation of all entities marketing derivatives to retail counterparties is necessary to achieve a level playing field for competitors However, a level playing field does not require identical regulation of all competitors Nor would identical regulation of one product line of multi-product firms by itself achieve a truly level playing field The government regulatory framework for exchange-trading may also need to be re- examined As we have seen, the key provisions of the CEA were put in place in the 1920s and 1930s to regulate the trading of grain futures by the general public, including retail investors Since then, U S futures exchanges have undergone profound changes Financial futures, not agricultural futures, now account for the great bulk of activity on the exchanges For many of the actively traded financial contracts, participation by retail investors is negligible Finally, in recent years trading volumes for most financial futures have been declining or growing very slowly, while the volume of off-exchange financial derivatives transactions has continued to grow very rapidly As I noted earlier, such migration of activity from regulated to unregulated markets presumably reflects in part the value-added of specially crafted, risk-unbundling contracts But almost surely as well many market participants perceive the costs of government regulation of exchanges to exceed the benefits Specifically, we need to think carefully about the characteristics of exchange trading per se that differentiate such markets from the off-exchange markets One argument is that the exchange markets perform a price-basing or price-discovery function that off-exchange markets do not This argument probably is valid for certain exchange-traded agricultural contracts However, I am not aware that any significant volume of off-exchange transactions is being priced solely on the basis of prices of exchange-traded financial contracts In the case of interest rate and exchange rate contracts, deep and liquid cash markets provide an alternative source of information that market participants find is quite adequate for price- discovery purposes 14 Another argument points to the existence of clearing houses for exchange-traded contracts, which act as counterparties to all trades on their affiliated exchanges and provide centralized management of counterparty risks To be sure, clearing houses concentrate and mutualize risks in ways that make regulation of clearing houses desirable from a systemic stability perspective But here again, we need to recognize the potential effectiveness of private market regulation Any government regulation of clearing houses must be carefully designed to avoid impairing private regulation This may not be possible if a one-size-fits-all regulatory approach is adopted Clearing houses that recently have been established for foreign exchange contracts have involved innovative approaches to risk management that differ from the approaches of futures exchanges in ways that are intended to preserve the private market discipline that has proven so effective One way of ensuring the necessary regulatory flexibility would be to allow such clearing houses a choice of federal regulatory regimes In addition to the CFTC, federal banking regulators or the Securities and Exchange Commission would seem quite capable of providing oversight to clearing houses for exchange-traded or OTC instruments It would also seem unwise to unnecessarily impede competition in the provision of centralized trading or clearing facilities to derivatives transactions that are currently negotiated and cleared bilaterally In particular, if institutional counterparties desire such services, futures exchanges should be allowed to compete as providers The trading and clearing systems for institutional markets undoubtedly should be kept separate from the existing futures trading and clearing systems But no further restrictions on their ability to compete would seem necessary In particular, it is not obvious why otherwise identical contracts could 15 not be traded on regulated exchanges open to the general public and on affiliated unregulated exchanges open only to institutions Institutional counterparties then would be free to choose whether to seek the benefits and accept the burdens of regulation under the CEA To sum up, the need for U S government regulation of derivatives instruments and markets should be carefully re-examined The application of the Commodity Exchange Act to off-exchange transactions between institutions seems wholly unnecessaryâ€”private market regulation appears to be achieving public policy objectives quite effectively and efficiently There also appears to be a strong case for allowing the centralized trading or clearing of financial derivatives that currently are bilaterally negotiated and cleared, and such evolution should not be obstructed by the threat of application of the CEA Although a case can be made for regulating clearing systems for such markets, alternatives to regulation under the CEA should be offered to avoid the potential dangers of a one-size-fits-all regulatory approach Furthermore, subject to a few restrictions, futures exchanges should be allowed to create affiliates to compete as providers of such services I would note in conclusion that the bipartisan legislation recently introduced in the Senate manifests a willingness to contemplate such fundamental changes in government regulation 16</t>
-  </si>
-  <si>
-    <t>I appreciate the opportunity to appear before this Committee to present the Federal Reserve's semiannual report on monetary policy. The performance of the U.S. economy over the past year has been quite favorable. Real GDP growth picked up to more than three percent over the four quarters of 1996, as the economy progressed through its sixth year of expansion Employers added more than two-and-a-half million workers to their payrolls in 1996, and the unemployment rate fell further Nominal wages and salaries have increased faster than prices, meaning workers have gained ground in real terms, reflecting the benefits of rising productivity. Outside the food and energy sectors, increases in consumer prices actually have continued to edge lower, with core CPI inflation only 2-1/2 percent over the past twelve months Low inflation last year was both a symptom and a cause of the good economy. It was symptomatic of the balance and solidity of the expansion and the evident absence of major strains on resources. At the same time, continued low levels of inflation and inflation expectations have been a key support for healthy economic performance. They have helped to create a financial and economic environment conducive to strong capital spending and longer-range planning generally, and so to sustained economic expansion. Consequently, the Federal Open Market Committee (FOMC) believes it is crucial to keep inflation contained in the near term and ultimately to move toward price stability. Looking ahead, the members of the FOMC expect inflation to remain low and the economy to grow appreciably further However, 2 as I shall be discussing, the unusually good inflation performance of recent years seems to owe in large part to some temporary factors, of uncertain longevity. Thus, the FOMC continues to see the distribution of inflation risks skewed to the upside and must remain especially alert to the possible emergence of imbalances in financial and product markets that ultimately could endanger the maintenance of the low-inflation environment. Sustainable economic expansion for 1997 and beyond depends on it. For some, the benign inflation outcome of 1996 might be considered surprising, as resource utilization rates-- particularly of labor--were in the neighborhood of those that historically have been associated with building inflation pressures. To be sure, an acceleration in nominal labor compensation, especially its wage component, became evident over the past year. But the rate of pay increase still was markedly less than historical relationships with labor market conditions would have predicted. Atypical restraint on compensation increases has been evident for a few years now and appears to be mainly the consequence of greater worker insecurity. In 1991, at the bottom of the recession, a survey of workers at large firms by International Survey Research Corporation indicated that 25 percent feared being laid off. In 1996, despite the sharply lower unemployment rate and the tighter labor market, the same survey organization found that 46 percent were fearful of a job layoff. 3 The reluctance of workers to leave their jobs to seek other employment as the labor market tightened has provided further evidence of such concern, as has the tendency toward longer labor union contracts. For many decades, contracts rarely exceeded three years Today, one can point to five- and six-year contractsâ€”contracts that are commonly characterized by an emphasis on job security and that involve only modest wage increases. The low level of work stoppages of recent years also attests to concern about job security. Thus, the willingness of workers in recent years to trade off smaller increases in wages for greater job security seems to be reasonably well documented. The unanswered question is why this insecurity persisted even as the labor market, by all objective measures, tightened considerably One possibility may lie in the rapid evolution of technologies in use in the work place. Technological change almost surely has been an important impetus behind corporate restructuring and downsizing. Also, it contributes to the concern of workers that their job skills may become inadequate No longer can one expect to obtain all of one's lifetime job skills with a high-school or college diploma. Indeed, continuing education is perceived to be increasingly necessary to retain a job. The more pressing need to update job skills is doubtless also a factor in the marked expansion of on- the-job training programs, especially in technical areas, in many of the nation's corporations 4 Certainly, other factors have contributed to the softness in compensation growth in the past few years. The sharp deceleration in health care costs, of course, is cited frequently. Another is the heightened pressure on firms and their workers in industries that compete internationally. Domestic deregulation has had similar effects on the intensity of competitive forces in some industries. In any event, although I do not doubt that all these factors are relevant, I would be surprised if they were nearly as important as job insecurity. If heightened job insecurity is the most significant explanation of the break with the past in recent years, then it is important to recognize that, as I indicated in last February's Humphrey-Hawkins testimony, suppressed wage cost growth as a consequence of job insecurity can be carried only so far. At some point, the tradeoff of subdued wage growth for job security has to come to an end. In other words, the relatively modest wage gains we have experienced are a temporary rather than a lasting phenomenon because there is a limit to the value of additional job security people are willing to acquire in exchange for lesser increases in living standards. Even if real wages were to remain permanently on a lower upward track than otherwise as a result of the greater sense of insecurity, the rate of change of wages would revert at some point to a normal relationship with inflation. The unknown is when this transition period will end. 5 Indeed, some recent evidence suggests that the labor markets bear especially careful watching for signs that the return to more normal patterns may be in process. The Bureau of Labor Statistics reports that people were somewhat more willing to quit their jobs to seek other employment in January than previously The possibility that this reflects greater confidence by workers accords with a recent further rise in the percent of households responding to a Conference Board survey who perceive that job availability is plentiful. Of course, the job market has continued to be quite good recently; employment in January registered robust growth and initial claims for unemployment insurance have been at a relatively low level of late. Wages rose faster in 1996 than in 1995 by most measures, perhaps also raising questions about whether the transitional period of unusually slow wage gains may be drawing to a close. To be sure, the pickup in wage gains has not shown through to underlying price inflation. Increases in the core CPI, as well as in several broader measures of prices, have stayed subdued or even edged off further in recent months. As best we can judge, faster productivity growth last year meant that rising compensation gains did not cause labor costs per unit of output to increase any more rapidly. Non-labor costs, which are roughly a quarter of total consolidated costs of the nonfinancial corporate sector, were little changed in 1996. Owing in part to this subdued behavior of unit costs, profits and rates of return on capital have risen to high levels 6 As a consequence, businesses believe that, were they to raise prices to boost profits further, competitors with already ample profit margins would not follow suit; instead, they would use the occasion to capture a greater market share. This interplay is doubtless a significant factor in the evident loss of pricing power in American business. Intensifying global competition also may be further restraining domestic firms' ability to hike prices as well as wages. Clearly, the appreciation of the dollar on balance over the past eighteen months or so, together with low inflation in many of our trading partners, has resulted in a marked decline in non-oil import prices that has helped to damp domestic inflation pressures. Yet it is important to emphasize that these influences, too, would be holding down inflation only temporarily; they represent a transition to a lower price level than would otherwise prevail, not to a permanently lower rate of inflation. Against the background of all these considerations, the FOMC has recognized the need to remain vigilant for signs of poten- tially inflationary imbalances that might, if not corrected promptly, undermine our economic expansion. The FOMC in fact has signaled a state of heightened alert for possible policy tightening since last July in its policy directives. But, we have also taken care not to act prematurely. The FOMC refrained from changing policy last summer, despite expectations of a near-term policy firming by many financial market participants. 7 In light of the developments I've just discussed affecting wages and prices, we thought inflation might well remain damped, and in any case was unlikely to pick up very rapidly, in part because the economic expansion appeared likely to slow to a more sustainable pace In the event, inflation has remained quiescent since then. Given the lags with which monetary policy affects the economy, however, we cannot rule out a situation in which a preemptive policy tightening may become appropriate before any sign of actual higher inflation becomes evident. If the FOMC were to implement such an action, it would be judging that the risks to the economic expansion of waiting longer had increased unduly and had begun to outweigh the advantages of waiting for uncertainties to be reduced by the accumulation of more information about economic trends Indeed, the hallmark of a successful policy to foster sustainable economic growth is that inflation does not rise. I find it ironic that our actions in 1994-95 were criticized by some because inflation did not turn upward. That outcome, of course, was the intent of the tightening, and I am satisfied that our actions then were both necessary and effective, and helped to foster the continued economic expansion. To be sure, 1997 is not 1994. The real federal funds rate today is significantly higher than it was three years ago Then we had just completed an extended period of monetary ease which addressed the credit stringencies of the early 1990s, and with 8 the abatement of the credit crunch, the low real funds rate of early 1994 was clearly incompatible with containing inflation and sustaining growth going forward. In February 1997, in contrast, our concern is a matter of relative risks rather than of expected outcomes. The real funds rate, judging by core inflation, is only slightly below its early 1995 peak for this cycle and might be at a level that will promote continued non-inflationary growth, especially considering the recent rise in the exchange value of the dollar. Nonetheless, we cannot be sure. And the risks of being wrong are clearly tilted to the upside. I wish it were possible to lay out in advance exactly what conditions have to prevail to portend a buildup of inflation pressures or inflationary psychology. However, the circumstances that have been associated with increasing inflation in the past have not followed a single pattern. The processes have differed from cycle to cycle, and what may have been a useful leading indicator in one instance has given off misleading signals in another. I have already discussed the key role of labor market developments in restraining inflation in the current cycle and our careful monitoring of signs that the transition phase of trading off lower real wages for greater job security might be coming to a close. As always, with resource utilization rates high, we would need to watch closely a situation in which demand was clearly unsustainable because it was producing escalating pressures on resources, which could destabilize the economy. And 9 we would need to be watchful that the progress we have made in keeping inflation expectations damped was not eroding. In general, though, our analysis will need to encompass all potentially relevant information, from financial markets as well as the economy, especially when some signals, like those in the labor market, have not been following their established patterns The ongoing economic expansion to date has reinforced our conviction about the importance of low inflation--and the public's confidence in continued low inflation. The economic expansion almost surely would not have lasted nearly so long had monetary policy supported an unsustainable acceleration of spending that induced a buildup of inflationary imbalances. The Federal Reserve must not acquiesce in an upcreep in inflation, for acceding to higher inflation would countenance an insidious weakening of our chances for sustaining long-run economic growth. Inflation interferes with the efficient allocation of resources by confusing price signals, undercutting a focus on the longer run, and distorting incentives This year overall inflation is anticipated to stay restrained. The central tendency of the forecasts made by the Board members and Reserve Bank presidents has the increase in the total CPI slipping back into a range of 2-3/4 to 3 percent over the four quarters of the year. This slight falloff from last year's pace is expected to owe in part to a slower rise in food prices as some of last year's supply limitations ease. More importantly, world oil supplies are projected by most analysts to 10 increase relative to world oil demand, and futures markets project a further decline in prices, at least in the near term. The recent and prospective declines in crude oil prices not only should affect retail gasoline and home heating oil prices but also should relieve inflation pressures through lower prices for other petroleum products, which are imbedded in the economy's underlying cost structure. Nonetheless, the trend in inflation rates in the core CPI and in broader price measures may be somewhat less favorable than in recent years. A continued tight labor market, whose influence on costs would be augmented by the scheduled increase in the minimum wage later in the year and perhaps by higher growth of benefits now that considerable health-care savings already have been realized, could put upward pressure on core inflation. Moreover, the effects of the sharp rise in the dollar over the last eighteen months in pushing down import prices are likely to ebb over coming quarters. The unemployment rate, according to Board members and Bank presidents, should stay around 5-1/4 to 5-1/2 percent through the fourth quarter, consistent with their projections of measured real GDP growth of 2 to 2-1/4 percent over the four quarters of the year. Such a growth rate would represent some downshifting in output expansion from that of last year. The projected moderation of growth likely would reflect several influences: (1) declines in real federal government purchases should be exerting a modest degree of restraint on overall demand; (2) the lagged effects of the increase in the exchange value of the dollar in 11 recent months likely will damp U.S net exports somewhat this year; and (3) residential construction is unlikely to repeat the gains of 1996. On the other hand, we do not see evidence of widespread imbalances either in business inventories or in stocks of equipment and consumer durables that would lead to a substan- tial cutback in spending. And financial conditions overall remain supportive; real interest rates are not high by historical standards and credit is readily available from intermediaries and in the market. The usual uncertainties in the overall outlook are especially focused on the behavior of consumers. Consumption should rise roughly in line with the projected moderate expansion of disposable income, but both upside and downside risks are present. According to various surveys, sentiment is decidedly upbeat. Consumers have enjoyed healthy gains in their real incomes along with the extraordinary stock-market driven rise in their financial wealth over the last couple of years. Indeed, econometric models suggest that the more than $4 trillion rise in equity values since late 1994 should have had a larger positive influence on consumer spending than seems to have actually occurred. It is possible, however, that households have been reluctant to spend much of their added wealth because they see a greater need to keep it to support spending in retirement. Many households have expressed heightened concern about their financial security in old age, which reportedly has led to 12 increased provision for retirement. The results of a survey conducted annually by the Roper Organization, which asks individuals about their confidence in the Social Security system, shows that between 1992 and 1996 the percent of respondents expressing little or no confidence in the system jumped from about 45 percent to more than 60 percent. Moreover, consumer debt burdens are near historical highs, while credit card delinquencies and personal bankruptcies have risen sharply over the past year. These circumstances may make both borrowers and lenders a bit more cautious, damping spending. In fact, we may be seeing both wealth and debt effects already at work for different segments of the population, to an approximately offsetting extent. Saving out of current income by households in the upper income quintile, who own nearly three- fourths of all non-pension equities held by households, evidently has declined in recent years. At the same time, the use of credit for purchases appears to have leveled off after a sharp runup from 1993 to 1996, perhaps because some households are becoming debt constrained and, as a result, are curtailing their spending. The Federal Reserve will be weighing these influences as it endeavors to help extend the current period of sustained growth. Participants in financial markets seem to believe that in the current benign environment the FOMC will succeed indefinitely. There is no evidence, however, that the business cycle has been repealed. Another recession will doubtless occur some day owing 13 to circumstances that could not be, or at least were not, perceived by policymakers and financial market participants alike. History demonstrates that participants in financial markets are susceptible to waves of optimism, which can in turn foster a general process of asset-price inflation that can feed through into markets for goods and services. Excessive optimism sows the seeds of its own reversal in the form of imbalances that tend to grow over time When unwarranted expectations ultimately are not realized, the unwinding of these financial excesses can act to amplify a downturn in economic activity, much as they can amplify the upswing. As you know, last December I put the question this way. "...how do we know when irrational exuberance has unduly escalated asset values, which then become subject to unexpected and prolonged contractions . ..? We have not been able, as yet, to provide a satisfying answer to this question, but there are reasons in the current environment to keep this question on the table. Clearly, when people are exposed to long periods of relative economic tranquility, they seem inevitably prone to complacency about the future. This is understandable. We have had fifteen years of economic expansion interrupted by only one recession--and that was six years ago. As the memory of such past events fades, it naturally seems ever less sensible to keep up one's guard against an adverse event in the future. Thus, it should come as no surprise that, after such a long period of balanced expansion. 14 risk premiums for advancing funds to businesses in virtually all financial markets have declined to near-record lows. Is it possible that there is something fundamentally new about this current period that would warrant such complacency? Yes, it is possible. Markets may have become more efficient, competition is more global, and information technology has doubtless enhanced the stability of business operations. But, regrettably, history is strewn with visions of such "new eras" that, in the end, have proven to be a mirage. In short, history counsels caution. Such caution seems especially warranted with regard to the sharp rise in equity prices during the past two years. These gains have obviously raised questions of sustainability. Analytically, current stock-price valuations at prevailing long- term interest rates could be justified by very strong earnings growth expectations. In fact, the long-term earnings projections of financial analysts have been marked up noticeably over the last year and seem to imply very high earnings growth and continued rising profit margins, at a time when such margins are already up appreciably from their depressed levels of five years ago. It could be argued that, although margins are the highest in a generation, they are still below those that prevailed in the 1960s. Nonetheless, further increases in these margins would evidently require continued restraint on costs: labor compensa- tion continuing to grow at its current pace and productivity growth picking up. Neither, of course, can be ruled out. But we 15 should keep in mind that, at these relatively low long-term interest rates, small changes in long-term earnings expectations could have outsized impacts on equity prices. Caution also seems warranted by the narrow yield spreads that suggest perceptions of low risk, possibly unrealistically low risk. Considerable optimism about the ability of businesses to sustain this current healthy financial condition seems, as I indicated earlier, to be influencing the setting of risk premiums, not just in the stock market but throughout the financial system This optimistic attitude has become especially evident in quality spreads on high-yield corporate bonds--what we used to call "junk bonds." In addition, banks have continued to ease terms and standards on business loans, and margins on many of these loans are now quite thin Many banks are pulling back a little from consumer credit card lending as losses exceed expectations. Nonetheless, some bank and nonbank lenders have been expanding aggressively into the home equity loan market and so-called "subprime" auto lending, although recent problems in the latter may already be introducing a sense of caution. Why should the central bank be concerned about the possibil- ity that financial markets may be overestimating returns or mispricing risk? It is not that we have a firm view that equity prices are necessarily excessive right now or risk spreads patently too low Our goal is to contribute as best we can to the highest possible growth of income and wealth over time, and we would be pleased if the favorable economic environment 16 projected in markets actually comes to pass. Rather, the FOMC has to be sensitive to indications of even slowly building imbalances, whatever their source, that, by fostering the emergence of inflation pressures, would ultimately threaten healthy economic expansion. Unfortunately, because the monetary aggregates were subject to an episode of aberrant behavioral patterns in the early 1990s, they are likely to be of only limited help in making this judgment. For three decades starting in the early 1960s, the public's demand for the broader monetary aggregates, especially M2, was reasonably predictable. In the intermediate term, M2 velocity--nominal income divided by the stock of M2--tended to vary directly with the difference between money market yields and the return on M2 assets--that is, with its short-term opportunity cost. In the long run, as adjustments in deposit rates caused the opportunity cost to revert to an equilibrium, M2 velocity also tended to return to an associated stable equilibrium level. For several years in the early 1990s, however, the velocities of M2 and M3 exhibited persisting upward shifts that departed markedly from these historical patterns. In the last two to three years, velocity patterns seem to have returned to those historical relationships, after allowing for a presumed permanent upward shift in the levels of velocity. Even so, given the abnormal velocity behavior during the early 1990s, FOMC members continue to see considerable uncertainty in the relationship of broad money to opportunity costs and nominal 17 income. Concern about the possibility of aberrant behavior has made the FOMC hesitant to upgrade the role of these measures in monetary policy. Against this background, at its February meeting, the FOMC reaffirmed the provisional ranges set last July for money and debt growth this year- 1 to 5 percent for M2, 2 to 6 percent for M3, and 3 to 7 percent for the debt of domestic nonfinancial sectors. The M2 and M3 ranges again are designed to be consis- tent with the FOMC's long-run goal of price stability: For, if the velocities of the broader monetary aggregates were to continue behaving as they did before 1990, then money growth around the middle portions of the ranges would be consistent with noninflationary, sustainable economic expansion. But, even with such velocity behavior this year, when inflation is expected to still be higher than is consistent with our long-run objective of reasonable price stability, the broader aggregates could well grow around the upper bounds of these ranges The debt aggregate probably will expand around the middle of its range this year. I will conclude on the same upbeat note about the U.S. economy with which I began Although a central banker's occupational responsibility is to stay on the lookout for trouble, even I must admit that our economic prospects in general are quite favorable The flexibility of our market system and the vibrancy of our private sector remain examples for the whole world to emulate. The Federal Reserve will endeavor to do its part by continuing to foster a monetary framework under which our citizens can prosper to the fullest possible extent</t>
-  </si>
-  <si>
-    <t>Mr Chairman and members of the Committee, I appreciate the opportunity to appear before you today As you know, my colleagues and I who serve on the Federal Reserve Board just recently submitted to Congress our semiannual report on monetary policy and the economy In brief, the performance of the U S economy over the past year has been quite favorable, with few signs of the imbalances that might typically have been expected by the sixth year of a cyclical expansion Indeed, we believe that the most likely prospect is for continued sustainable economic growth accompanied by low and stable inflation, and our objective will be to foster the conditions most likely to produce that outcome In that regard, continued low levels of inflation and inflation expectations have been a key support for the healthy economic performance of the past year They have helped to create a financial and economic environment conducive to strong capital spending and longer-range planning generally, and so to sustained economic expansion Consequently, it is crucial to keep inflation contained in the near term and ultimately to move toward price stability If we are successful, a stable macroeconomic environment will contribute to your efforts to place the fiscal health of the nation on a firmer footing But achieving your fiscal objectives will require this Committee to confront additional issues of extraordinary complexity and importance I would like to devote the remainder of my prepared remarks to one of these issues, namely the bias in the consumer price index I want to begin by commending this Committee for your continuing interest in this subject Indeed, our conversation about potential bias in the CPI goes back some two years, when I testified before a joint meeting of this Committee and your counterparts from the Senate The topic remains just as important now as it was then A useful starting point for discussion of this issue is to be clear that any index that endeavors to measure the cost of living should aim to be unbiased That is, a serious examination of all available evidence should yield the conclusion that there is just as great a chance that the index understates the rate of growth of the true cost of living as there is that it overstates it The present-day consumer price index does not meet this standard In fact, the best available evidence suggests that there is almost a 100 percent probability that we are overcompensating the average social security recipient for increases in the cost of living, and almost a 100 percent probability that we are causing the inflation-adjusted burden of the income tax system to decline more rapidly than I presume the Congress intends A major reason for this is that consumers respond to changes in relative prices by changing the composition of their actual marketbasket At present, however, the marketbasket used in constructing the CPI changes only once every decade or so Moreover, new goods and services deliver value to consumers even at the relatively elevated prices that often prevail early in their life cycles, currently, that value is not reflected in the CPI For these and other reasons outlined in the Boskin Commission report and other studies, we know with near certainty that the current CPI is off Although we do not know precisely by how much, there is a very high probability that the upward bias ranges between 1/2 percentage point per year and 1-1/2 percentage points per year In thinking about how to remedy this situation, we must recognize that there is no sharp dividing line between a pristine estimate of a price and one that is not Although the concept of price is clear enough in theory, it is often extremely difficult to implement in practice In order to construct a fully satisfactory measure of the price of a given item, one would first have to specify all the characteristics of that item that deliver value to consumers Then one would have to reprice the identical bundle of characteristics month in and month out In practice, both of these steps are difficult because we are often not precisely certain about what consumers value, and because the items that are available to consumers are constantly changing, often in subtle ways As a result, virtually all of the components that make up the CPI are approximations, in some cases very rough approximations But the essential fact remains that even combinations of very rough approximations can give us a far better judgment of the overall cost of living than would holding to a false precision of accuracy and thereby delimiting the range of goods and services evaluated We would be far better served following the wise admonition of John Maynard Keynes that "it is better to be roughly right than precisely wrong " Estimates of the magnitude of the bias in our price measures are available from a number of sources Most have been developed from detailed examinations of the microstatistical evidence However, recent work by staff economists at the Federal Reserve Board has added strong corroborating evidence of price mismeasurement using a macroeconomic approach that is essentially independent of the exercises performed by other researchers, including those on the Boskin Commission In particular, employing the statistical system from which the Commerce Department estimates the national income and product accounts, this research finds that the measured growth of real output and productivity in the service sector are implausibly weak, given that the return to owners of businesses in that sector apparently has been well-maintained Taken at face value, the published data indicate that the level of output per hour in a number of service-producing industries has been falling for more than two decades In other words, the data imply that firms in these industries have been becoming less and less efficient for more than twenty years These circumstances simply are not credible On the reasonable assumption that nominal output and hours worked and paid of the various industries are accurately measured, faulty price statistics are by far the most likely cause of the implausible productivity trends The source of a very large segment of these prices is the CPI Some observers who are skeptical that the bias in the CPI could be very large have noted that the evidence on the magnitude of unmeasured quality change and the importance of new items bias is incomplete and inconclusive Without a doubt, quality change and new items are among the most difficult of the problems currently confronting the BLS But since I raised this issue two years ago, the accumulating evidence continues to support the view that the current treatment of quality change and new items in the CPI results in an overstatement of the rate of growth of the cost of living An even more difficult quality-related issue is whether changes in broad environmental and social conditions should be reflected in price measures that are used for indexing various components of federal outlays and receipts That is, should the CPI reflect the influence of factors such as the level of crime, air and water quality, and the emergence of new diseases, which are not specifically related to products that consumers purchase There is little in the record to suggest that, when it enacted the indexation of social security benefits in 1972, the Congress meant to insure the beneficiaries of that program against changes in such environmental and social factors Nor do these issues appear to have been raised when Congress debated the indexation of various tax parameters during the 1980s Taking account of such conditions, particularly those that lie outside of the markets for goods and services, would be an interesting exercise in its own right, but would appear to extend well beyond the original intent of the Congress A considerable professional consensus already exists for at least two actions that would almost surely bring the CPI into closer alignment with a true cost-of-living index First, we should move away from the concept of a fixed marketbasket at the upper level of aggregation, and move toward an aggregation formula that takes into account the tendency of consumers to alter the composition of their purchases in response to changes in relative prices Second, we should selectively move away from the current aggregation formula at the lower level of aggregation Beyond these rather limited steps, most of the needed developments will require time, effort, and quite possibly additional resources It is important that the Congress provide the Bureau with sufficient resources to pursue the agenda vigorously Where will this longer-term effort be required One of the key areas, by all accounts, is quality adjustment As the Bureau has rightly noted, they do indeed already employ a variety of methods to control for quality change, but available evidence suggests that these are not sufficient to the task Unfortunately, making improvements on this front will be difficult Each item will have to be considered on its own, and there may well be limited transfer of knowledge from one item to the next The longer-term agenda should also include concentrated attention to the methods for introducing new items into the index, the development of new sources of data such as the information collected by bar-code scanners, and the analysis of time use, the latter being important in understanding the value of time-saving and convenience-enhancing innovations Even if the BLS moves aggressively, some upward bias will almost surely remain in the CPI, at least for the next several years Two years ago, I suggested that a workable structure for dealing with this situation might involve a two-track approach That suggestion still seems to me to make sense The first track would involve action by the BLS to address those aspects of the bias that can be dealt with in relatively short order, say within the next year The second track would involve the establishment of an independent national commission to set annual cost-of-living adjustment factors for federal receipt and outlay programs The Commission would examine available evidence on a periodic basis, and estimate the bias in the CPI taking into account both the latest research on the sources and magnitudes of the bias, and any corrective actions that had been taken by the BLS This type of approach would have the benefit of being objective, nonpartisan, and sufficiently flexible to take full account of the latest information Moreover, there is no reason why the two tracks could not proceed in parallel Without the second track, we are implicitly assuming, contrary to overwhelming evidence, that the most accurate estimate of the bias due to quality adjustment problems and introduction of new items is zero There has been considerable objection that such a second track procedure would be a political fix To the contrary, assuming zero for the remaining bias is the political fix On this issue, we should let evidence, not politics, drive policy We have an overarching national interest in building a better measure of consumer prices and in implementing more rational indexation procedures These efforts are essential if we are to ensure that the original intent of the relevant pieces of legislation will be fulfilled in insulating taxpayers and benefit recipients from the effects of ongoing changes in the cost of living At present this objective is not being met</t>
-  </si>
-  <si>
-    <t>Mr Chairman, members of the Subcommittee, thank you for inviting me to present the views of the Federal Reserve Board on the supervision of our nation's banking organizations should they be authorized by the Congress to engage in a wider range of activities As you know, the Board has supported financial modernization for many years and hopes that the Congress will act to facilitate reforms that, by enhancing competition within the financial services industry, would benefit the consumers of financial products in the United States Financial modernization may well mean that future banking organizations will be sufficiently different from today as to require perhaps substantial changes in the supervisory process for the entire organization Just how much modification may be needed will depend on the kinds of reforms the Congress adopts In evaluating those modifications, I would like to underline the significant supervisory role required by the Federal Reserve to carry out its central bank responsibilities I also would like briefly to discuss the continued importance of umbrella supervision and the implications of a wider role for bank subsidiaries in the modernization process Supervision and Central Banking There are compelling reasons why the central bank of the United States- the Federal Reserveâ€”should continue to be involved in the supervision of banks The supervisory activities of the Federal Reserve, for example, have benefited from its economic stabilization responsibilities and its recognition that safety and soundness goals for banks must be evaluated jointly with its responsibilities for the stability and growth of the economy The Board believes that these joint responsibilities make for better supervisory and monetary policies than would result from either a supervisor divorced from economic responsibilities or a macroeconomic policymaker with no practical experience in the review of individual bank operations To carry out its responsibilities, the Federal Reserve has been required to develop extensive, detailed knowledge of the intricacies of the U S, and indeed the world, financial system That expertise is the result of dealing constantly over many decades with changing financial markets and institutions and their relationships with each other and with the economy, and from exercising supervisory responsibilities It comes as well from ongoing interactions with central banks and financial institutions abroad These international contacts are critical because today crises can spread more rapidly than in earlier timesâ€” in large part reflecting new technologiesâ€”and require a coordinated international response Crisis Management and Systemic Risk Second only to its macrostability responsibilities is the central bank's responsibility to use its authority and expertise to forestall financial crises (including systemic disturbances in the banking system) and to manage such crises once they occur In a crisis, the Federal Reserve, to be sure, could always flood the market with liquidity through open market operations and discount window loans, at times it has stood ready to do so, and it does not need supervisory and regulatory responsibilities to exercise that power But while sometimes necessary in times of crises, such an approach may be costly and distortive to economic incentives and long-term growth, as well as an insufficient remedy Supervisory and regulatory responsibilities give the Federal Reserve both the insight and the authority to use techniques that are less blunt and more precisely calibrated to the problem at hand Such tools improve our ability to manage crises and, more importantly, to avoid them The use of such techniques requires both the authority that comes with supervision and regulation and the understanding of the linkages among supervision and regulation, prudential standards, risk taking, relationships among banks and other financial market participants, and macroeconomic stability Our financial systemâ€”market oriented and characterized by innovation and rapid changeâ€”imparts significant benefits to our economy But one of the consequences of such a dynamic system is that it is subject to episodes of stress In the 1980s and early 1990s we faced a series of international debt crises, a major stock market crash, the collapse of the most important player in the junk bond market, the virtual failure of the S&amp;L industry, and extensive losses at many banking institutions More recently, we faced another Mexican crisis and, while in the event less disruptive, the failure of a large British merchant bank In such situations the Federal Reserve stands ready to provide liquidity, if necessary, and monitors continuously the condition of depository institutions to contain the secondary consequences of any problem The objectives of the central bank in crisis management are to contain financial losses and prevent a contagious loss of confidence so that difficulties at one institution do not spread more widely to others The focus of its concern is not to avoid the failure of entities that have made poor decisions or have had bad luck, but rather to see that such failures-or threats of failuresâ€”do not have broad and serious impacts on financial markets and the national, and indeed the global, economy The Federal Reserve's ability to respond expeditiously to any particular incident does not necessitate comprehensive information on each banking institution But it does require that the Federal Reserve have in-depth knowledge of how institutions of various sizes and other characteristics are likely to behave, and what resources are available to them in the event of severe financial stress Even for those events that might, but do not, precipitate financial crises, the authorities turn first to the Federal Reserve, not only because, as former Chairman Volcker noted last month, we have the money, but also because we have the expertise and the experience We currently gain the necessary insight by having a broad sample of banks subject to our supervision and through our authority over bank holding companies Payment and Settlement Systems Virtually all of the U S dollar transactions made worldwideâ€”for securities transfers, foreign exchange and other international capital flows, and for payment for goods and services-are settled in the United States banking system A small number of transactions that comprise the vast proportion of the total value of transactions are transferred over large-dollar payment systems Banks use two of these systemsâ€”Fed wire, operated by the Federal Reserve, and CHIPS, operated by the New York Clearing Houseâ€”currently to transfer $1 6 trillion and $1 3 trillion a day, respectively CHIPS settles its members' net positions on Fedwire These interbank transfers, for banks' own accounts and for those of their customers, occur and are settled over a network and structure that is the backbone of the U S financial system Indeed, it is arguably the linchpin of the international system of payments that relies on the dollar as the major international currency for trade and finance Disruptions and disturbances in the U S payment system thus can easily have global implications Fedwire, CHIPS, and the specialized depositories and clearinghouses for securities and other financial instruments, are crucial to the integrity and stability not only of our financial markets and economy, but those of the world Similarly, adverse developments in transfers in London, Tokyo, Singapore, and a host of other centers could rapidly be transferred here, given the financial interrelationships among the individual trading nations In all these payment and settlement systems, commercial banks play a central role, both as participants and providers of credit to nonbank participants Day-in and day-out, the settlement of payment obligations and securities trades requires significant amounts of bank credit In periods of stress, such credit demands surge just at the time when some banks are least willing or able to meet them These demands, if unmet, could produce gridlock in payment and settlement systems, halting activity in financial markets Indeed, it is in the cauldron of the payments and settlement systems, where decisions involving large sums must be made quickly, that all of the risks and uncertainties associated with problems at a single participant become focussed as participants seek to protect themselves from uncertainty Better solvent than sorry, they might well decide, and refuse to honor a payment request Observing that, others might follow suit And that is how crises often begin Limiting, if not avoiding, such disruptions and ensuring the continued operation of the payment system requires broad and indepth knowledge of banking and markets, as well as detailed knowledge and authority with respect to the payment and settlement arrangements and their linkages to banking operations This type of understanding and authorityâ€”as well as knowledge about the behavior of key participants-cannot be created on an ad hoc basis It requires broad and sustained involvement in both the payment infrastructure and the operation of the banking system Supervisory authority over the major bank participants is a necessary element Monetary Policy While financial crises and payment systems disruptions arise only sporadically, the Federal Reserve conducts monetary policy on an ongoing basis In this area, too, the Federal Reserve's role in supervision and regulation provides an important perspective to the policy process Monetary policy works through financial institutions and markets to affect the economy, and depository institutions are a key element in those markets Indeed, banks and thrifts are more important in this regard than might be suggested by a simple arithmetic calculation of their share of total credit flows While diverse securities markets handle the lion's share of credit flows these days, banks are the backup source of liquidity to many of the securities firms and large borrowers participating in these markets Moreover, banks at all times are the most important source of credit to most small- and intermediate-sized firms that do not have ready access to securities markets These firms are the catalyst for U S economic growth and the prime source of new employment opportunities for our citizens The Federal Reserve must make its monetary policy with a view to how banks are responding to the economic environment This was especially important during the "credit crunch" of 1990 Our supervisory responsibilities give us important qualitative and quantitative information that not only helps us in the design of monetary policy, but provides important feedback on how our policy stance is affecting bank actions The macroeconomic stabilization responsibilities of the Federal Reserve make us particularly sensitive to how regulatory and supervisory postures can influence bank behavior and hence how banks respond to monetary policy actions For example, capital, liquidity, loan loss reserve, and asset quality evaluation policies of supervisors will directly influence the manner and speed with which monetary policy actions work In the development of interagency rules and policies, the Federal Reserve brings to the table its unique concerns about the impact of these rules on credit availability, potential responses to changes in interest rates, and the consequences for the economy We believe that, as a result, supervisory policy is improved Federal Reserve's Supervisory Role For all of these reasons, the Board believes the Federal Reserve needs to retain a significant supervisory role in the banking system Just exactly how that is achieved depends critically on the types of reforms the Congress enacts and the direction the banking industry takes in structuring and conducting its activities In the Board's view, its current authority is adequate for the current structure For today's financial system, we are able to meet our obligations by the intelligence we gain from, and the authorities we have over the modest number of large banks we directly supervise and the holding companies of these and other large banks over which we have a direct umbrella supervisory role Our information is importantly supplemented by our supervision of a number of other banks of all sizes, namely state member banks Currently, the latter group gives us a good representative sample of organizations of all sizes outside the largest entities The large entities are essential if we are to address the Federal Reserve's crisis management and systemic risk responsibilities, deal with international financial issues involving foreign central banks, manage risk exposures in payment systems, and retain our practical knowledge and skill base in rapidly changing financial markets Large bank holding companies are typically at the forefront in financial innovation and in developing sophisticated techniques for managing risks It is crucial that the Federal Reserve stay informed of these events and understand directly how they work in practice Directly supervising both these large organizations and a sample of others is also critical to our ability to conduct monetary policy by permitting us to gain first- hand on-the-spot intelligence on how changes in financial marketsâ€”including those induced by monetary policyâ€”are affecting money and credit flows If in the future the holding company becomes a less clear window into the banking system, the Board believes that the Congress would need to change the supervisory structure if the central bank is to carry out the responsibilities I have discussed today Umbrella Supervision The Congress, in its review of financial modernization, must consider legal entity supervision alone versus legal entity supervision supplemented by umbrella supervision The Board believes that umbrella supervision is a realistic necessity for the protection of our financial system and to limit any misuse of the sovereign credit, that is, the government's guarantees that support the banking system through the safety net The bank holding company organization increasingly is being managed so as to take advantage of the synergies between its component parts in order to deliver better products to the market and higher returns to stockholders Such synergies cannot occur if the model of the holding company is one in which the parent is just, in effect, a portfolio investor in its subsidiary Indeed, virtually all of the large holding companies now operate as integrated units and are managed as such, especially in their management of risk One could argue that regulators should be interested only in the entities they regulate and, hence, review the risk evaluation process only as it relates to their regulated entity Presumably each regulator of each entityâ€”the bank regulators, the SEC, the state insurance and any state finance company authoritiesâ€”would look only at how the risk management process affected their units It is our belief that this simply will not be adequate Risks managed on a consolidated basis cannot be reviewed on an individual legal entity basis by different supervisors The latter logic motivated the congressional decision just five years ago to require that foreign banks could enter the United States if, and only if, they were subject to consolidated supervision This decision, which is consistent with the international standards for consolidated supervision of banking organizations, was a good decision then It is a good decision today, especially for those banking organizations whose disruption could cause major financial disturbances in United States and foreign markets For foreign and for U S banking organizations, retreat from consolidated supervision would, the Board believes, be a significant step backward We have to be careful, however, that consolidated umbrella supervision does not inadvertently so hamper the decisionmaking process of banking organizations as to render them ineffectual The Federal Reserve Board is accordingly in the process of reviewing its supervisory structure and other procedures in order to reflect a market-directed shift from conventional balance sheet auditing to evaluation of the internal risk management process Although focussed on the key risk management processes, it would sharply reduce routine supervisory umbrella presence in holding companies As the Committee knows, the Board has recently published for comment proposals to expedite the applications process, and the legislation Congress enacted last year eased such procedures as well Nonetheless, the Board requests even greater modification to its existing statutory mandate so that the required applications process could be sharply cut back, particularly in the area of nonbank financial services In the Board's view, those entities interested in banks are really interested in access to the safety net, since it is far easier to engage in the nonsafety net activities of banks without acquiring a bank If an organization chooses to deliver some of its services with the aid of the sovereign credit by acquiring a bank, it should not be excused from efforts of the government to look out for the stability of the overall financial system For bank holding companies, this implies umbrella supervision Although that process will increasingly be designed to reduce supervisory presence and be as nonmtrusive as possible, umbrella supervision should not be eliminated, but recognized for what it is the cost of obtaining a subsidy Nonetheless, we would hope that should the Congress authorize wider activities for financial services holding companies that it recognize that a bank which is a minor part of such an organization (and its associated safety net) can be protected through adequate bank capital requirements and the application of Sections 23A and 23B of the Federal Reserve Act The case is weak, in our judgment, for umbrella supervision of a holding company in which the bank is not the dominant unit and is not large enough to induce systemic problems should it fail Subsidiaries, Subsidies, and Safety Nets The members of this Subcommittee are, I think, aware of the Board's concerns that the safety net constructed for banks inherently contains a subsidy, that conducting new activities in subsidiaries of banks will inadvertently extend that subsidy, and that extension of any subsidy is undesriable The Subcommittee recently heard testimony that there is no net subsidy and, therefore, the authorization of nonbank activities in bank subsidiaries would neither inadvertently extend this undesirable side effect of the safety net nor reduce the importance of the holding company as a consequence of the increased incentives to shift activities from the holding company to the bank Mr Chairman, I would like briefly to comment on these latter views Subsidy valuesâ€”net or grossâ€”vary from bank to bank, riskier banks clearly get a larger subsidy from the safety net than safer banks In addition, the value of the subsidy varies over time, in good times, markets incorporate a low risk premium and when markets turn weak, financial asset holders demand to be compensated by higher yields for holding claims on riskier entities It is at this time that subsidy values are the most noticeable What was it worth in the late 1980s and early 1990s for a bank with a troubled loan portfolio to have deposit liabilities guaranteed by the FDIC, to be assured that it could turn illiquid to liquid assets at once through the Federal Reserve discount window, and to tell its customers that payment transfers would be settled on a riskless Federal Reserve Bank For many, it was worth not basis points but percentage points For some, it meant the difference between survival and failure It is argued by some that the cost of regulation exceeds the subsidy I have no doubt that the costs of regulation are large, too large in my judgment But no bank has turned in its charter in order to operate without the cost of banking regulation, which would require that it operate also without deposit insurance or access to the discount window or payments system To do so would require both higher deposit costs and higher capital Indeed, it is a measure of the size of banks' net subsidy that most nonbank financial institutions are required by the market to operate with significantly higher capital-to-asset ratios than banks Most finance companies, for example, with credit ratings and debenture interest costs equal to banks are forced by today's market to hold six or seven percentage points higher capital-to-asset ratios than those of banks It is instructive that there are no private deposit insurers competing with the FDIC For the same product offered by the FDIC, private insurers would have to charge premiums far higher than those of government insurance, and still not be able to match the certainty of payments in the event of default, the hallmark of a government insurer backed by the sovereign credit of the United States The Federal Reserve has a similar status with respect to the availability of the discount window and riskless final settlement during a period of national economic stress Providing such services is out of the reach of all private institutions The markets place substantial values on these safety net subsidies, clearly in excess of the cost of regulation To repeat, were it otherwise, some banks would be dropping their charters if there were not a net subsidy In fact it is apparently the lower funding costs at banks, that benefit directly from the subsidy of the safety net, that has created the tendency for banking organizations to return to the bank and its subsidiaries many activities that are authorized to banks These activities previously had been conducted in nonbank affiliates for reasons such as geographic and other inflexibilities, which have gradually eased Indeed, over the last decade the share of consolidated assets of bank holding companies associated with nonbank affiliatesâ€”other than Section 20 securities affiliatesâ€”has declined almost half to just 5 2 percent This tendency reflects the fact that asset growth that earlier had been associated with nonbank affiliates of bank holding companies- consumer and commercial finance, leasing, and mortgage bankingâ€”has most recently occurred largely in the bank or in a subsidiary of the bank To be sure, as Chairman Heifer indicated to the Subcommittee earlier this month, many banking organizations still retain nonbank subsidiaries Our discussions with bank holding companies, however, suggest that in some cases, these affiliates were acquired in the past and have established names and an interstate network whose value would be reduced if subsumed within a bank There are also often adverse tax implications for the shift And, finally, some of these activities may not be asset intensive and hence may not benefit significantly from bank funding Clearly, the authorization of new activities in bank subsidiaries that are not now permitted either to banks or their affiliates would tend to accelerate the trend to reduce holding company activity, even if these activities were also permitted to holding company subsidiaries The subsidy inherent in the safety net would assure that result, extending the spread of the safety net and requiring that the Federal Reserve's authority and ability to meet its responsibilities be shifted to a different paradigm Such a result is reason enough for our concern about the spreading of the safety net subsidy But we should also be concerned because of the distortions subsidies bring to the financial system more generally After all, the broad premise underlying financial modernizationâ€”with its removal of legislative and regulatory restrictionsâ€”is that free and often intense competition will create the most efficient and customer-oriented business system This principle has proved itself, generation by generation, with ever higher standards of living In financial, as well as most other, markets the principle is rooted in another premiseâ€”that the interaction of private competitive forces will, with rare exceptions, create a stable error self-correcting system This premise is very seriously called into question if government subsidies are supplied at key balancing points By their nature, subsidies distort the establishment of competitive market prices, and create incentives that misalign private risks with private gains Such distortions undermine the error self-correcting mechanisms that support strong financial markets We must be very careful that in the name of free market efficiency we do not countenance greater powers and profits subsidized directly or indirectly by government Conclusion Mr Chairman, in conclusion, the Board believes that as the Congress moves toward financial modernization the newly created structure of financial organizations should limit, in so far as possible, the real and perceived transfer of the subsidy inherent in the safety net to nonbank activities To maintain a level playing field for all competitors, nonbank activities must be financed at market, not subsidized, rates The Board also believes that financial modernization should not undermine the ability and authority of the central bank of the United States to manage crises, assure an efficient and safe payment system, and conduct monetary policy We believe all of these require that the Federal Reserve retain a significant and important role as a bank supervisor In today's structure, we have adequate authority and coverage to meet our responsibilities But should erosion occur, as would likely be the case if new activities are authorized in bank subsidiaries, the Congress would have to consider what changes would be required in the Board's supervisory authority to assure that it continues to be able to meet its central bank responsibilities</t>
-  </si>
-  <si>
-    <t>Mr Chairman and members of the Committee, I am pleased to appear here today Last month, the Federal Reserve Board submitted its semiannual report on monetary policy to the Congress That report and my accompanying testimony covered in detail our assessment of the outlook for the U S economy This morning, I would like to highlight some of the key aspects of the current economic situation As I told the Congress last month, the performance of the U S economy remains quite favorable Real GDP growth picked up to more than 3 percent over the four quarters of 1996 Moreover, recently released data suggest that activity has retained a great deal of vigor in early 1997 In addition, nominal hourly wages and salaries have risen faster than prices over the past several quarters, meaning that workers have reaped some of the benefits of rising productivity and thus gained ground in real terms Outside the food and energy sectors, increases in consumer prices have actually continued to edge lower, with core CPI inflation of only 2-1/2 percent over the past twelve months The low inflation of the past year is both a symptom and a cause of the good economy It is symptomatic of the balance and solidity of the expansion and the evident absence of major strains on resources At the same time, continued low levels of inflation and inflation expectations have been a key support for healthy economic performance They have helped to create a financial and economic environment conducive to strong capital spending and longer-range planning generally, and so to sustained economic expansion These types of results are why we stressed in our monetary policy testimony the importance of acting promptly--ideally pre-emptively--to keep inflation low over the intermediate term and to promote price stability over time For some, the benign inflation outcome of the past year might be considered surprising, as resource utilization rates--particularly of labor--have been in the neighborhood of those that historically have been associated with building inflation pressures To be sure, nominal hourly labor compensation, especially its wage component, accelerated in 1996 But the rate of pay increase still was markedly less than historical relationships with labor market conditions would have predicted Atypical restraint on compensation increases has been evident for a few years now Almost certainly, it reflects a number of factors, including the sharp deceleration in health care costs and the heightened pressure on firms and workers in industries that compete internationally Domestic deregulation has also intensified the competitive forces in some industries But, as I outlined in some detail in testimony last month, I believe that job insecurity has played the dominant role For example, in 1991, at the bottom of the recession, a survey of workers at large firms by International Survey Research Corporation indicated that 25 percent feared being laid off In 1996, despite the sharply lower unemployment rate and the tighter labor market, the same survey organization found that 46 percent were fearful of a job layoff Whatever the reasons for its persistence, job insecurity cannot suppress wage growth indefinitely Clearly, there is a limit to how long workers will remain willing to accept smaller increases in living standards in exchange for additional job security Even if real wages were to remain permanently on a lower upward track than otherwise as a result of the greater sense of insecurity, the rate of change of wages would revert at some point to a normal relationship with price Inflation The unknown Is when a more normal pattern will resume Indeed, the labor markets bear especially careful watching for signs that such a process is under way So far this year, the demand for labor has stayed strong Payroll employment grew briskly in January and February, and the unemployment rate remained around 5-1/4 percent-- roughly matching the low of the last cyclical upswing, in the late 1980s. Also, initial claims for unemployment insurance remained low into March In addition, the percentage of households telling the Conference Board that jobs are plentiful has risen sharply of late, which suggests that workers may be growing more confident about the job situation Finally, wages rose faster in 1996 than in 1995 by most measures--in fact, the acceleration was quite sizable by some measures. This, too, raises questions about whether the transitional period of unusually slow wage gains may be drawing to a close In any event, further increases in labor utilization rates would heighten the risk of additional upward pressure on wage costs, and ultimately prices To be sure, the pickup in wage gains to date has not shown through to underlying price inflation Increases in the core CPI, as well as in several other broad measures of prices, have stayed subdued or even edged off further of late As best I can judge, faster productivity growth last year offset the pressure from rising compensation gains on labor costs per unit of output And non-labor costs, which are roughly a quarter of total consolidated costs of the nonfinancial corporate sector, were little changed in 1996 Owing in part to this subdued behavior of unit costs, profits and rates of return on capital have risen to high levels As a consequence, a substantial number of businesses apparently believe that, were they to raise prices to boost profits further, competitors with already ample profit margins would not follow suit, instead, they would use the occasion to capture a greater market share This interplay is doubtless a significant factor in the evident loss of pricing power in American business Intensifying global competition may also be limiting the ability of domestic firms to hike prices as well as wages Competitive pressures here and abroad should continue to act as a restraint on inflation in the months ahead In addition, crude oil prices have largely retraced last year's run-up, and, with the worldwide supply of oil having moved up relative to demand, futures markets project stable prices over the near term Food prices should also rise less rapidly than they did in 1996 as some of last year's supply limitations ease Nonetheless, the trends in the core CPI and in broader price measures are likely to come under pressure from a continued tight labor market, whose influence on costs will be augmented by the scheduled increase in the minimum wage later in the year And, with considerable health-care savings already having been realized, larger increases in fringe benefits could put upward pressure on overall compensation Moreover, although non-oil import prices should remain subdued in 1997 as the sharp rise in the dollar over the past year-and-a-half continues to feed through to domestic prices, their damping effects on U S inflation probably will not be as great as in 1996 The lagged effects of the increase in the exchange value of the dollar will also likely restrain real U S net exports this year In addition, declines in real federal government purchases should exert a modest degree of restraint on overall demand, and residential construction will probably not repeat the gains of 1996 On the other hand, financial conditions overall remain supportive to the real economy, and creditworthy borrowers are finding funding to be readily available from intermediaries and in the securities markets Moreover, we do not see evidence of widespread imbalances either in business inventories or in stocks of capital equipment and consumer durables that would lead to a substantial cutback in spending The trends in consumer spending on items other than durables also look solid Retail sales posted robust gains in January and February, and, according to various surveys, sentiment is decidedly upbeat Moreover, consumers have enjoyed healthy increases in their real incomes over the past couple of years, along with the extraordinary stock-market driven rise in their financial wealth Should the higher wealth be sustained, it could provide important support to consumption in 1997 But, looking at the data through 1996, the surging stock market does not seem to have imparted as big a boost to spending as past relationships would have predicted The lack of a more substantial wealth effect is especially surprising because we have also seen a noticeable widening in the ownership of stocks over the past several years Indeed, the Federal Reserve's recently released Survey of Consumer Finances suggests that of the total value of all families' holdings of publicly traded stocks and mutual funds, the share held by those with incomes below $100,000 (in 1995 dollars) rose from 32 percent in 1989 to 46 percent in 1995 It is possible, however, that the wealth effect is being offset by other factors In particular, families may be reluctant to spend their added wealth because they see a greater need to keep it to support spending in retirement. Many have expressed heightened concern about their financial security in old age, in part because of growing skepticism about the viability of the Social Security system This concern has reportedly led to stepped-up saving for retirement The sharp increase in debt burdens in recent years may also be constraining spending by some families, Indeed, although our consumer survey showed that debt usage rose between 1992 and 1995 for almost all income groups, changes in financial conditions were not uniform across families Notably, the median ratio of debt payments to income for families with debt--a useful measure of the typical debt burden--held steady or declined for families with incomes of at least $50,000, but it rose for those with incomes below $50,000 We don't know whether these latter families took on the additional debt because they perceived brighter future income prospects, or simply to accelerate purchases they would have made later Nonetheless, these families are probably the most vulnerable to disruptions in income, and the rise in their debt burdens is likely to make both borrowers and lenders a bit more cautious as we move forward Both household and business balance sheets have expanded at a pace considerably faster than income and product flows over the past decade Accordingly, any percentage change in assets or liabilities has a greater effect on economic growth than it used to However, identifying such influences in the aggregate data is not always easy At present, the difficulty is compounded by concern that the currently published national statistics may not provide an accurate reading of the trends in recent years, especially for productivity In any event, other data suggest that wealth and debt effects may be exerting a measurable influence on the consumption and saving decisions of different segments of the population According to the Consumer Expenditure Survey conducted by the Bureau of Labor Statistics, saving out of current income by families in the upper- income quintile evidently has declined in recent years At the same time. Federal Reserve estimates suggest that the use of credit for purchases has leveled off after a sharp run-up from 1993 to 1996, perhaps because some families are becoming debt constrained and, as a result, are curtailing their spending The Federal Reserve, of course, will be weighing these and other influences as it makes future policy decisions Demand has been growing quite strongly in recent months, and the FOMC, at its meeting next week, will have to judge whether that pace of expansion will be maintained, and, if so, whether it will continue to be met by solid productivity growth, as it apparently has been--official figures to the contrary notwithstanding Alternatively, if strong demand is expected to persist, and does not seem likely to be matched by productivity improvement, the FOMC will have to decide whether increased pressures on supply will eventually produce the types of inflationary imbalances that, if not addressed early, will undermine the long expansion Should we choose to alter monetary policy, we know from past experience that, although the financial markets may respond immediately, the main effects on inflationary pressures may not be felt until late this year and in 1998 Because forecasts that far out are highly uncertain, we rarely think in terms of a single outlook Rather, we endeavor to assess the likely consequences of our decisions in terms of a reasonable range of possible outcomes Part of our evaluation is to judge not only the benefits that are likely to result from appropriate policy, but also the costs should we be wrong In any action--including leaving policy unchanged--we seek to assure ourselves that the expected benefits are large enough to risk the cost of a mistake In closing, I would like to note that the current economic expansion is now entering its seventh year That makes it already a long upswing by historical standards And yet, looking ahead, the prospects for sustaining the expansion are quite favorable The flexibility of our market system and the vibrancy of our private sector remain examples for the whole world to emulate We will endeavor to do our part by continuing to foster a monetary framework under which our citizens can prosper to the fullest possible extent</t>
-  </si>
-  <si>
-    <t>It is a pleasure to be here today I will take this occasion to offer some thoughts related to the upcoming G-7 economic summit meeting, which will be held in Denver in less than two months One theme in recent summit meetings -- starting in Halifax in 1995 and continuing in Lyon last year â€” has been the promotion of stability in international financial markets My purpose today is not to describe all the efforts that have been made in that regard, which relate primarily to supervision and regulation Rather, I would like to step back a bit and offer a framework for thinking about those efforts To begin with, we should not lose sight of the fact that government regulation, if not carefully designed, can undermine the effectiveness of private market regulation and can itself be ineffective in protecting the public interest No market is ever truly unregulated in that the self-interest of participants generates private market regulation Counterparties thoroughly scrutinize each other, often requiring collateral and special legal protections, self-regulated clearing houses and exchanges set margins and capital requirements to protect the interests of the members Thus, the real question is not whether a market should be regulated Rather, it is whether government intervention strengthens or weakens private regulation, and at what cost At worst, the introduction of government rules may actually weaken the effectiveness of regulation if government regulation is itself ineffective or, more importantly, undermines incentives for private market regulation Regulation by government unavoidably involves some element of perverse incentives, that is, moral hazard If private market participants believe that government is protecting their interests, their own efforts to do so will diminish 2 At the same time, societies have judged that it is not sufficient to rely exclusively on the private sector to ensure the adequacy of the management of risk in our financial systems There is a perceived need for supervision and regulation by the public sector, as well As I will point out shortly, this need arises largely to counter the potential moral hazard that arises as a consequence of the development of large safety nets for our financial systems Many of the benefits banks provide modern societies derive from their willingness to take risks and from their use of a relatively high degree of financial leverage Through leverage, in the form principally of taking deposits, banks perform a critical role in the financial intermediation process, they provide savers with additional investment choices and borrowers with a greater range of sources of credit, thereby facilitating a more efficient allocation of resources and contributing importantly to greater economic growth Indeed, it has been the evident value of intermediation and leverage that has shaped the development of our financial systems from the earliest times -- certainly since Renaissance goldsmiths discovered that lending out deposited gold was feasible and profitable Central bank provision of mechanisms for converting highly illiquid portfolios into liquid ones in extraordinary circumstances â€” a key element of our safety nets -- has led to a greater degree of leverage in banking than market forces alone would support Traditionally these mechanisms involve making discount or Lombard facilities available, so that individual depositories could turn illiquid assets into liquid resources and not exacerbate unsettled market conditions by the forced selling of such assets or the calling of loans More broadly, open market operations, in situations like that which followed the crash of stock markets 3 around the world in 1987, satisfy increased needs for liquidity for the system as a whole that otherwise could feed cumulative, self-reinforcing contractions across many financial markets Of course, this same leverage and risk-taking also greatly increase the possibility of bank failures Without leverage, losses from risk-taking would be absorbed by a bank's owners, virtually eliminating the chance that the bank would be unable to meet its obligations in the case of a "failure " Some failures can be of a bank's own making, resulting, for example, from poor credit judgments For the most part, these failures are a normal and important part of the market process and provide discipline and information to other participants regarding the level of business risks However, because of the important roles that banks and other financial intermediaries play in our financial systems, such failures could have large ripple effects that spread throughout business and financial markets at great cost The presence of the safety net, which inevitably imparts a subsidy to banks, has created a disconnect between risk-taking by banks and banks' cost of capital It is this disconnect that has made necessary a degree, of supervision and regulation that would not be necessary without the existence of the safety net That is, regulators are compelled to act as a surrogate for market discipline since the market signals that usually accompany excessive risk-taking are substantially muted, and because the prices to banks of government deposit guarantees, or of access to the safety net more generally, do not, and probably cannot, vary sufficiently with risk to mimic market prices The problems that arise from the retarding of the pressures of market discipline have led us increasingly to accept supervision and regulation that endeavors to simulate the market responses that would occur if there were no safety net, but without giving up its protections To be sure, we should recognize that if we choose to have the advantages of a safety net and a leveraged system of financial intermediaries, the burden of managing risk in the financial system will not lie with the private sector alone With leveraging there will always exist a remote possibility of a chain reaction, a cascading sequence of defaults that will culminate in financial implosion if it proceeds unchecked Only a modern central bank, with its unlimited power to create money, can with a high probability thwart such a process before it becomes destructive Hence, central banks will of necessity be drawn into becoming lenders of last resort But implicit in the existence of such a role is that there will be some form of allocation between the public and private sectors of the burden of risk of extreme outcomes Thus, central banks are led to provide what essentially amounts to catastrophic financial insurance coverage Such a public subsidy should be reserved for only the rarest of disasters If the owners or managers of private financial institutions were to anticipate being propped up frequently by government support, it would only encourage reckless and irresponsible practices In theory, the allocation of responsibility for risk-bearing between the private sector and the central bank depends upon an evaluation of the private cost of capital In order to attract, or at least retain, capital, a private financial institution must earn at minimum the overall economy's rate of return, adjusted for risk In competitive financial markets, the greater the leverage, the higher the rate of return, before adjustment for risk If private financial institutions have to absorb all financial risk, then the degree to which they can leverage will be limited, the financial sector smaller, and its contribution to the economy more limited On the other hand, if central banks effectively insulate private institutions from 5 the largest potential losses, however incurred, increased laxity could threaten a major drain on taxpayers or produce inflationary instability as a consequence of excess money creation Thus, governments, including central banks, have been given certain responsibilities related to their banking and financial systems that must be balanced We have the responsibility to prevent major financial market disruptions through development and enforcement of prudent regulatory standards and, if necessary in rare circumstances, through direct intervention in market events But we also have the responsibility to ensure that private sector institutions have the capacity to take prudent and appropriate risks Our goal as supervisors should not be to prevent all bank failures, but to maintain sufficient prudential standards so that banking problems that do occur do not become widespread We try to achieve the proper balance through official regulations, as well as through formal and informal supervisory policies and procedures The revolution in information and data processing technology has transformed our financial markets and the way our financial institutions conduct their operations In most respects, these technological advances have enhanced the potential for reducing transactions costs, to the benefit of consumers of financial services, and for managing risks But in some respects they have increased the potential for more rapid and widespread disruption The efficiency of global financial markets, engendered by the rapid proliferation of financial products, has the capability of transmitting mistakes at a far faster pace throughout the financial system in ways that were unknown a generation ago, and not even remotely imagined in the 19th century Financial crises in the early 19th century, for example, particularly those associated with the Napoleonic Wars, were often related to military and 6 other events in faraway places Communication was still comparatively primitive An investor's speculative position could be wiped out by a military setback, and he might not even know about it for days or even weeks, which, from the perspective of central banking today, might be considered bliss Similarly, the collapse of Barings Brothers in 1995 showed how much more rapidly losses can be generated in the current environment relative to a century earlier when Barings Brothers confronted a similar episode Current technology enables single individuals to initiate massive transactions with very rapid execution Clearly, not only has the productivity of global finance increased markedly, but so, obviously, has the ability to generate losses at a previously inconceivable rate These technological forces also have been central to the process of globalization, that is, the growing integration of national economies â€” including national financial markets They are, of course, not the only forces The gradual removal of barriers to trade, deregulation and reform of financial systems, and simply the enormous creation of wealth have all generated the demand and opportunities for the expansion of investment and business horizons beyond national boundaries Technological changes have facilitated such an expansion The growing importance of emerging market economies in international financial markets is one manifestation not just of the impressive growth of those economies but also of increasing global integration Thus, it is not surprising that the need to promote financial stability, and in particular to enhance prudential supervision, in emerging market economies was identified at the Lyon summit as an important objective It is important for those economies individually and for all of us collectively One element of the follow-up to the Lyon summit that is especially fitting in the context of my earlier remarks has been efforts to enhance market transparency, including more -- and more meaningful -- public disclosure Meaningful public disclosures by firms about the nature of their risk exposures and their procedures for managing those risks contribute significantly to the constructive role of market discipline Not surprisingly, the market itself is probably the most powerful source of pressure for improved disclosures I might mention one specific accomplishment related to market transparency Central banks have agreed to establish a system of regular reporting of derivatives activities by the world's major dealers, beginning as of June 1998 The system has been designed to yield aggregate data on global trading activities in a manner that avoids double counting and is sensitive to reporting burden The aggregate data will be publicly released to enable firms to assess their own activities in relation to the market as a whole The globalization of international financial markets and of the operations of individual firms clearly calls for international cooperation among supervisors Correspondingly, supervisory cooperation is an important element of the G-7 summit agenda on financial stability Much of the recent work has related to the desirability of a more systematic exchange of information among national supervisors, including consideration of what kinds of information need to be exchanged and under what circumstances The possible need for and 8 possible roles of an "information coordinator" have been central issues in the Joint Forum discussions The objective of a more systematic exchange of information is easy to support in principle However, when it comes to implementation, there are questions that need to be addressed Even more questions arise when one thinks of going beyond the exchange of information to other forms of supervisory coordination, involving a "lead regulator" of some kind that is intended to fill so-called supervisory gaps What are the supervisory gaps that need to be filled? Each of us could probably point to episodes where problems could have been avoided, or the degree of disruption could have been reduced, if better information had been available sooner to supervisory authorities Perhaps Barings is one example It is more difficult to point to episodes when the absence of formal arrangements for coordination of supervisory actions inhibited a response to a problem Conversely, might arrangements that are too formal, too rigid, or too cumbersome themselves inhibit appropnate responses in emergency situations, each of which is likely-to be unique"? Another question is whether supervisory authorities have the expertise and resources to provide meaningful oversight and develop accurate assessments of the risk-taking activities of large, diversified, globally active financial institutions If the answer is no, as might well be the case, should we nevertheless convey to market participants the sense that we are in fact adequately supervising such activities? Wouldn't that reduce the incentives for market participants themselves to provide discipline? 9 Would a statement that all major financial firms, even the most diversified ones, are subject to coordinated supervision suggest a degree of support that effectively extends, to an unwarranted extent, the subsidy associated with national safety nets? Would it generate a degree of moral hazard that could itself be the source of systemic risk? The answers to these questions are not straightforward However, while many firms should reassess and upgrade their risk management procedures, and supervisors should improve their procedures as well, I do not believe that the need for a radical change in our framework for the supervision of internationally active financial firms has been demonstrated The paradigm of supervision itself is, of necessity, continuously adjusted to the rapidly changing, technologically driven, financial system In recent years, firms and supervisors alike have sought to harness technological advances to enhance risk management procedures Much thought has been given to how to make public disclosure more meaningful and to reinforce market discipline Supervisors around the world, not just in the major industrial countries, have gotten to know each, other better and to understand better each others' problems and policies The legal and institutional infrastructure of financial markets has been significantly improved Along with good macroeconomic policy -- a topic for another day -- a continuation of this ongoing process of careful and measured progress represents the most constructive strategy for ensuring financial stability</t>
-  </si>
-  <si>
-    <t>For more than three decades, this conference has focused our attention on key issues facing banks, their customers, and regulators Its proceedings have chronicled a remarkable and ongoing transformation of the U S financial services industry At the time of the first gathering in 1963, our financial system was highly segmented, with commercial banks, savings and loans, investment banks, insurance companies, and finance companies providing distinctly separate products Statutes and regulations greatly restricted competition between banks and nonbanks, and among banks themselves Today, the marketplace for financial services is intensely competitive, innovative, and global Banks and nonbanks, domestic and foreign, now compete aggressively across a broad range of on- and off-balance sheet financial activities It is noteworthy that, for the most part, this transformation has not been propelled by sweeping legislative reforms Rather, the primary driving forces have been advances in computing, telecommunications, and theoretical finance that, taken together, have eroded economic and regulatory barriers to competition, de facto Technology has fundamentally reshaped how financial products are created, and how these products are delivered, received, and employed by end-users In my remarks this morning, I plan to discuss two aspects of this process of technological change First is the recurring theme of financial products being unbundled into their component parts, including the unbundling of credit, market, and other risks These developments have worked to enhance the competitiveness and efficiency of the financial system, and at the same time to provide financial institutions and then customers with better tools for managing risks A by-product is that our largest and most complex financial organizations increasingly are measuring and managing risk on a centralized basis This trend seems irreversible, and in my view provides a compelling reason for maintaining some type of umbrella supervision over banking organizations, especially as we contemplate repeal of Glass-Steagall and other restrictions on the activities of banking organizations The second theme I want to explore is the large element of uncertainty underlying technological progress Reflecting this uncertainty, it is inherently very difficult to predict the extent to which government policies may distort the private sector's incentives to innovate This argues for supervisory and regulatory policies that are more "incentive-compatible," in the sense that they are reinforced by market discipline and the profit-maximizing incentives of bank owners and managers To the extent this can be achieved, and I believe we have taken some innovative steps in this direction, supervisory and regulatory policies will be both less burdensome and more effective Unbundling of Financial Services The unbundling of financial products is now extensive throughout our financial system Perhaps the most obvious example is the ever expanding array of financial derivatives available to help firms manage interest rate risk, other market risks, and, increasingly, credit risks Derivatives are now used routinely to separate the total risk of more generic products into component parts associated with various risk factois These components frequently are repackaged into synthetic products having risk profiles that mimic financial instruments in other markets The synthetic products can then be lesold to those investors most willing and able to bear the associated risks Another far-reaching innovation is the technology of securitization -- a form of derivative ~ which has encouraged unbundling of the production processes for many credit services Securitization permits separate financial institutions to originate, service, fund, and assume the credit or market risks of a portfolio of loans or other assets Thus, a financial institution may specialize in those activities where it has parucular expertise or other comparative advantages For example, to reduce the costs of originating and securitizing certain types of household loans, the underwriting processes used by some financial institutions rely on highly automated credit-scoring models developed by third-party vendors These models, in turn, typically are linked to huge databases on borrower characteristics maintained independently by national credit bureaus Numerous types of assets are now routinely securitized, including residential mortgages, commercial mortgages, auto loans, and credit card loans In addition, medium- and large-size businesses, including some that are below investment-grade, legulaily access the commeicial paper market by securitizing their trade accounts or other assets Recently, securitization and credit-scoring are beginning to be applied to small business lending These and other developments facilitating the unbundling of financial products have surely improved the efficiency of our financial markets One benefit is greater economic specialization, as banks and other financial institutions are able to create market niches, for example, in cash management, investment management, or the origination or servicing of certain loans Moreover, by lowering the costs of hedging and financial arbitrage, derivatives and securitization work to enhance market liquidity and reduce both absolute risk premiums and disparities in risk premiums across financial instruments and geographic regions Unbundling also has lowered economic barriers to competition, affording households and businesses a greater choice of potential providers for financial products The ability to unbundle permits potential competitors to target highly specific product- or market-attributes, for which existing providers are earning excessive "rents " Through credit-scoring and direct-mail marketing, for instance, a financial institution can identify and recruit potentially profitable credit card customers over a wide geographic area, without incurring the costs associated with a large branch network According to our Survey of Consumer Finances, for example, 84 percent of general purpose credit cards held by U S households in 1995 were issued by financial institutions from which the card holder received no other financial service In addition, unbundling has helped erode legal barriers to competition, by enabling one or more attributes of a product to be modified in order to exploit statutory or regulatory "loopholes " A classic example, of course, is the introduction of money market mutual funds, which ultimately forced the removal of Regulation Q interest rate ceilings on deposit accounts It is important to recognize that these developments would not have been possible without complementary advances in technology across several disciplines First, innovations in finance theory, such as the principle of financial arbitrage and models for pricing contingent claims, provided a conceptual framework for understanding and modeling financial risks Second, advances in computer and communications technologies have made these conceptual innovations economically feasible, by lowering the costs associated with information processing and with the transmission of large volumes of data over long distances 5 Besides promoting competition and improved products and production efficiencies, these same technological advances have spawned a sea-change in the risk management practices of financial institutions The largest and most sophisticated banking organizations increasingly have centralized their risk management at the parent level -- cutting across legal entities and financial instruments This new management paradigm is grounded in the same conceptual techniques employed by financial engineers to unbundle the total risk of an individual asset Such techniques rely on the financial engineer's ability to model the relationship between an individual asset's economic value and a number of separate risk factors Carrying this process further, the relationship between these risk factors and the value of an overall portfolio can be obtained by summing the relationships foi the individual underlying assets With the processing power of modern computers, it is now possible to estimate the joint probability distribution of many risk factors and, given this distribution, to simulate the probability distributions of losses for large, complex portfolios Over the past decade or so, the largest banking organizations have invested substantial sums to hire the staff and to create the software, databases, and related management information systems to carry out such computations Most of you are aware of the application of this technology in VaR, or "value-at-risk," models, which are used to estimate loss distributions for trading portfolios More recently, many large banking organizations have begun using similar technologies to measure the credit risk in their loan portfolios In both applications, the measurements of overall portfolio risk are used to determine the prices for loans and other products needed to achieve hurdle rates-of-return on shareholder equity, to assess the adequacy of an organization's overall equity capital, as well as for other management purposes These efforts to develop more centralized risk management systems are being driven by normal competitive pressures to maximize synergies within financial organizations, such as joint-production and cross-selling opportunities involving multiple subsidiaries This, in turn, is the logical outcome of the organization's desire to produce and market its products most efficiently, and to achieve the highest risk-adjusted returns for shareholders Such synergies cannot occur if the parent is merely a passive portfolio investor in its subsidiaries Reflecting this economic reality, vntually all large bank holding companies are now operated and managed as integrated units The trend toward centralized risk management raises some fundamental policy issues for how we should regulate and supervise large, complex banking organizations Chief among these, this trend raises serious doubts regarding suggestions that we rely solely on decentralized "functional regulation" as we move to expand further the permissible activities of banking organizations The traditional view of the functional approach to regulating a banking organization would involve a bank regulator supervising the insured bank, the SEC supervising any broker/dealer subsidiary, a state insurance department supervising any insurance subsidiary, and so on Each functional regulator would look only at the risk management practices of the regulated entity under its supervision, unregulated subsidiaries, including the parent, would be unsupervised Before technology advanced to a point where substantial oversight and control of large banking organizations could be consolidated at the parent level, functional regulation conformed with practical limitations on the abilities of managers to coordinate resources, and evaluate risks, for the organizations as a whole In essence, a decentralized approach to regulation followed from the decentralized financial decision-making process of its day To borrow a concept from architecture form followed function In today's world, however, the "form," decentralized regulation, no longer follows the "function," centralized risk management Almost by definition, the synergies upon which centralized management is predicated imply that neither a subsidiary's economic condition on a going-concern basis, nor its exposure to potential risks, can be evaluated independently of the condition and management policies of the consolidated organization Regulation must fit the architecture of what is being regulated To give one example, it is common for complex banking organizations to manage the relationships with large customers centrally, even though the underlying cash management, credit, 01 capital maikets services piovided to the customer may transcend several subsidiaries Under this framework, the way the organization's internal transfer pricing system allocates costs, revenues, and risks to a specific regulated entity may be somewhat arbitrary, or even misleading Yet, a functional regulator -- looking only at the entity under its supervision -- generally would have insufficient information to validate the reasonableness of these allocations A purely decentralized regulatory approach would also greatly diminish our ability to evaluate and contain potential systemic disruptions in the financial system, since no legulator would be responsible for monitoring the consolidated banking organization We should lemember that one of the primary motivations of a society having a central bank and a safety net is precisely to limit systemic risk Partly in recognition of the fact that financial organizations are managed on a consolidated basis, financial markets generally view them as single economic entities Thus, troubles in the non-government-regulated portion of a bank holding company cannot be expected to leave the government-regulated subsidiaries unscathed In a worst case scenario, problems in one part of an organization could precipitate a run at a healthy affiliate bank, and could even generate spillover effects onto nonaffiliated banks It is worth noting that recent deposit insurance and depositor preference legislation may increase these concerns, by exposing uninsured creditors of banks to a greater risk of loss than in the past While these new initiatives have the significant benefit of strengthening market discipline, they may also induce some additional systemic risks, even for healthy banks, in periods characterized by heightened levels of economic uncertainty We don't have much experience, yet, in operating under these new ground rules For all of these leasons, I believe we must continue to have some type of umbrella supervision for banking organizations, especially for the largest and most complex organizations that pose the greatest systemic risk concerns In my judgment, therefore, the critical challenge is to develop approaches to implementing umbrella supervision that are effective in limiting systemic risk without distorting economic incentives or being unduly burdensome to banking organizations If history is our guide, market innovations - with or without supporting legislation -- will continue to stimulate financial modernization As this process unfolds, we can expect banking organizations to undertake an increasing number of financial activities Under these cricumstances, policymakers face a very difficult 9 tradeoff namely, balancing the need for financial stability and umbrella supervision, on the one hand, against our desire to avoid extending bank-like regulation and the safety net over these new activities In addressing this tradeoff, policymakers also have an obligation to consider the potential effects of their policies, unintended as well as intended, on the process of financial innovation Technological progress has been a critical element in rising living standards This is not surprising, because the creation and diffusion of innovations have represented voluntary decisions by individuals and firms acting in then own self-interests Government policies always pose some risk of misdirecting or distorting this process by interfering with normal competitive market mechanisms This concern is particularly relevant to the financial sector, whose innovations seem to be especially attuned to the risk-return incentives created by the safety net and regulatory policies Designing government policies that minimize the potentially disruptive effects on private incentives to innovate is complicated by how little we really understand the process of innovation and technological change Forecasting the direction or pace of technological change has proven to be especially precarious over the generations, even for relatively mature industries While uncertainty is inherent in any creative process, Nathan Rosenberg of Stanford suggests that even after an innovation's technical feasibility has been clearly established, its ultimate effect on society is often highly unpredictable He notes at least two sources of this uncertainty First, the range of applications for a new technology may not be immediately apparent For instance, Alexander Graham Bell initially viewed the telephone as solely a business instrument - merely an enhancement of the telegraph â€” for use in transmitting very specific messages, such as the terms of a contract Indeed, he offered to sell his telephone patent to Western Union for only $100,000, but was turned down Similarly, Guglielmo Marconi initially overlooked the radio's value as a public broadcast medium, instead believing its principal application would be in the transmission of point-to-point messages, such as ship-to-ship, where communication by wire was infeasible A second source of technological uncertainty reflects the possibility that an innovation's full potential may be realizable only after extensive improvements, or after complementary innovations in other fields of science According to Charles Townes, a Nobel Prize winner for his work on the laser, the attorneys for Bell Labs initially refused, in the 1960s, to patent the laser because they believed it had no applications in the field of telecommunications Only in the 1980s, after extensive improvements in fiber optics technology, did the laser's importance for telecommunications become apparent It's not hard to find examples of such uncertainties within the financial services mdustry The evolution of the OTC derivatives market over the past decade has been nothing less than spectacular But as the theoretical underpinnings of financial arbitrage were being pubbshed by Modigliani and Miller in the late 1950s, few observers could have predicted how their insights would eventually revolutionize global financial markets This is because, in addition to their insights, at least two complementary innovations had to fall into place The first was further conceptual advances in contingent claims theory, such as the Black-Scholes option pricing model The second was several generations of advances in computer and communications technologies that were necessary to make these concepts computationally practicable Given the high degree of uncertainty inherent in the development of new products and processes, policymakers should be cautious when attempting to anticipate the future path of innovation, or the effects new regulations may have on innovation There are several aspects to this interaction between government policies and market innovation First, banking organizations may develop new products or innovations to exploit regulatory "loopholes," or they may decline to develop new products whose bkely regulatory treatments are viewed as burdensome or unclear Another unintended consequence is that a policy action may establish an inappropriate unofficial government standard for how certain activities should be conducted In contrast to government standards, which can be extremely difficult to change, when the private sector adopts a standard that subsequently becomes outmoded, market forces generally can be expected to remedy the situation The history of retail electronic payments provides a useful illustration In the 1970s, when many were heralding the advent of a "cashless society," the Federal Reserve and the Treasury played an important role in developing and promoting what was seen as a key component of this vision - the automated clearinghouse system Now, twenty yeais later, we know that while the ACH has been successful in some areas, it has failed to replace a substantial portion of the daily flow of paper checks in the economy This experience leads me to conclude that the experimentation with innovative electronic payment methods that we are seeing today in the private sector is likely to have a much better chance of meeting the needs of consumers and businesses than did the government-led initiatives two decades ago Within the context of banking regulation, concerns about setting a potentially inappropriate regulatory standard were an important factor in the decision by the banking agencies several years ago not to incorporate interest rate risk and asset concentration risk into the formal risk-based capital standards In the end, we became convinced that the technologies for measuring and managing interest rate risk and concentration risk were evolving so rapidly that any regulatory standard would quickly become outmoded or, worse, inhibit private market innovations Largely for these reasons, ultimately we chose to address the relationship between these risks and capital adequacy through the supervisory process I believe that in many cases, policymakers can reduce potential distortions by structuring policies to be more "incentive-compatible" -- that is, by working with, rather than around, the profit-maximizing goals of investors and firm managers In light of the underlying uncertainties illustrated in my earlier examples, I readily acknowledge this is often easier said than done Nevertheless, I believe some useful guiding principles can be formulated The first guiding principle is that, where possible, we should attempt to strengthen market discipline, without compromising financial stability As financial transactions become increasingly rapid and complex, I believe we have no choice but to harness market forces, as best we can, to reinforce our supervisory objectives The appeal of market-led discipline lies not only in its cost-effectiveness and flexibility, but also in its limited intrusiveness and its greater adaptability to changing financial environments Measures to enhance market discipline involve providing private investors the incentives and the means to reward good bank performance and penalize poor performance Expanded risk management disclosures by financial institutions is a significant step in this direction In addition, Congress has undertaken important initiatives, including a national depositor preference statute and the least-cost resolution and prompt corrective action provisions of the FDIC Improvement Act Of course, the value of these initiatives will depend on the credibility of regulators in implementing the legislative mandates consistently over time A second guiding principle is that, to the extent possible, our regulatory policies should attempt to simulate what would be the private market's response in the absence of the safety net Such a principle suggests that supervisory and regulatory policies, like market responses, should be capable of evolving over time, along with changes in institutional practices and financial technologies Almost certainly, such a principle impbes that we avoid locking ourselves into formulaic, one-size-fits-all approaches to measunng and affecting bank safety and soundness Foi example, as a bank's internal systems for measuring and managing market, credit, and operating risks improve with advances in technology and finance, our supervisory policies should become more tailored to that bank's specific needs and internal management processes Recently, we have taken several steps that attempt to operationalize this concept, including the introduction of an internal models approach to assessing capital for market risks in large banks' trading accounts Also, as I am sure most of you are aware, the Board is currently pilot-testing with the New York Clearing House Association an alternative capital allocation procedure for market risk, called the "pre-commitment" approach The pre-commitment approach would permit capital lequnements for market risk to reflect not only the estimates of risk derived from a bank's internal market-risk model, but also other features of the bank's trading risk management system that help limit its overall risk exposure - such as 14 the effectiveness of its internal controls and other risk-management tools Over the last three decades, the folly of attempting to legislate or regulate against the primal forces of the market is one of the most fundamental lessons learned by banking regulators If those market forces are driving financial firms toward centralized decision-making regarding risk, pricing, and other operational issues, it will be difficult, at best, to implement a decentralized approach to prudential regulation, however attractive its apparent simplicity Similarly, in the face of continual market-driven innovations in banks' risk measmement and management systems, regulatory approaches based on rigid, one-size-fits-all rules are likely to become quickly outdated, ineffectual, and, worse, potentially counterproductive Incentive-compatible regulation, flexibly constructed and applied, is the logical alternative to an increasingly complex system of rigid rules and regulations that inevitably have unintended consequences, including possible deleterious effects on the innovation process While I have discussed some examples of incentive- compatible regulation that appear to be working, we have a very long way to go For example, banking regulators have yet to reach a consensus on some of the most basic questions associated with prudential supervision ~ questions such as what is an appropnate conceptual basis for assessing a financial institution's overall risk exposure, how should such risk exposures be measured, and if we use internal management models for such measurements, how can these models be validated? The revolution in risk measurement techniques makes the answers to these questions approachable, but not without significant effort on the part of the regulators and the 15 financial industry itself I am confident that all parties are both willing and able to solve the challenges that confront us It is clearly in our mutual self-interest to do so Our success will pieserve not only the benefits of the most competitive and innovative financial markets in the world, but also the benefits of financial stability that are cntical to our economy</t>
-  </si>
-  <si>
-    <t>I am pleased to be here today to present the views of the Board of Governors of the Federal Reserve System on the financial modernization legislation introduced by Chairman Leach, H R 10, the Financial Services Competitiveness Act of 1997 This bill would reform the Glass-Steagall prohibitions to permit the affiliation of banks and securities firms It would also permit bank and insurance company affiliations and provide the flexibility for banking organizations to engage in other "financial" or "incidental" activities The Competitiveness Act would facilitate the ownership of banks by other financial firms by creating a category of uninsured wholesale banks that may have some commercial affiliations H R. 10 would produce identical rules for banks and federally chartered thrifts and rationalize their regulation and supervision The Board strongly supports the approach to financial modernization embodied in H R 10. We believe it would improve the efficiency and competitiveness of the financial services industry and result in more choices and better service for consumers However, as the Committee knows, the Board opposes one aspect of the bill, the authorization for so- called operating subsidiaries of banks to engage in some financial activities not permitted to their parent bank Our concern is the transference of the safety net subsidy directly to those activities that the bill would authorize for subsidiaries of banks. The Board believes that the Congress should widen the permissible range of affiliations for banking organizations in order to expand the choices for consumers and increase the efficiency of financial markets Financial modernization should remove outdated restrictions that serve no useful purpose, that decrease economic efficiency, and that, as a result, limit choices and options for the consumer of financial services Such statutory prohibitions result in higher costs and lower quality services for the public Their removal would permit banking organizations to compete more effectively in their natural markets The result would be a more efficient financial system providing better services to the public Indeed, the Board urges that, as you consider the reforms before you, the focus not be on which set of financial institutions should be permitted to take on a new activity, or which would, as a result, get a new competitor All are doing similar things now and are currently in competition with each other, offering similar products Securities firms have for some time offered checking-like accounts linked to mutual funds, their affiliates routinely extend significant credit directly to businesses , and they are becoming increasingly important in the syndicated loan market Banking organizations are already conducting a securities business While indicative of the need for reform, which institution has hurdled some earlier restraint is not the issue The Board believes that the focus should be do H R 10 and the other proposed bills promote a financial system that makes the maximum contribution to the growth and stability of the U S economy? Is the removal of existing restraints in these bills consistent with a safe and sound banking system and containment of the federal safety net? Do the proposals increase the compatibility of our laws and regulations with the changing technological and global market realities in order to ensure that these goals are achieved? Are they consistent with increased alternatives and convenience for the public at a manageable risk to both the bank insurance fund and financial market stability? With the previously noted caveat, Mr. Chairman, the Board believes that these questions can be answered in the affirmative for your bill Banking organizations are in a particularly good position to provide securities underwriting, insurance, and other financial services to investors They are knowledgeable about the institutional structure of the market, skilled at evaluating risk, knowledgeable about the financial needs of their customers, and operate from locations that are convenient for the public Moreover, for centuries, the special expertise of banking organizations has been to accumulate borrower-specific information that they can use to make credit and related judgments that less well-informed savers and depositors cannot make Using such information asymmetries has been the value added of banking on the credit side It would appear that many companies and individuals want to deal with a full-service provider that can handle then- entire range of financing needs This preference for "one-stop shopping" is easy to understand Starting a new financial relationship is costly for companies and individuals and, by extension, for the economy as a whole It takes considerable time and effort for a customer to convey to an outsider a deep understanding of its financial situation This process, however, can be short-circuited by allowing the customer to rely on a single organization for deposit services, loans, strategic advice, the underwriting of debt and equity securities, and other financial services As evidence that there are economies from this sharing of information, most of the Section 20 underwriting has been for companies that had a prior relationship with the banking organization The economic benefits of "one-stop shopping" can readily be seen for small and medium-sized firms These firms, as a rule, do not attract the interest of major investment banks, and regional brokerage houses do not provide the full range of financial services these companies require Rather, their primary financial relationship is with the commercial banking organizations where they borrow and obtain their services From the borrower's perspective, it makes sense to leverage this relationship when the time comes to access the capital markets for financing It is thus reasonable to anticipate that if secunties activities are authorized for bank affiliates, banking organizations, especially regional and smaller banking organizations, would use their information base to facilitate securities offerings for smaller, regional firms The same efficiencies are likely to benefit local municipal revenue bond issues The Board's recent action to raise the Section 20 limits on ineligible revenues to 25 percent of the total will increase the number of banking organizations that can engage in secunties underwriting However, there are still a large number of banks that do not have the necessary volume of government, agency, and municipal bonds transactions to meet the other 75 percent of the total that would permit them to engage in an economically viable volume of corporate and/or municipal revenue bond underwriting, and hence to service their smaller customers Investment banking services are now available for some of these smaller issuers, but at a relatively high cost Moreover, the Board's recent decision does not address other important aspects of secunties activities that are dealt with by H R 10, such as authorizing merchant banking and mutual fund sponsorship The convenience and cost savings for companies issuing securities will also accrue to individuals seeking other financial services There are real potential benefits to consumers of "one-stop shopping" for loans, deposits, money market accounts, securities, and insurance It is only artificial and outdated restrictions that stand in the way of lower cost and convenient delivery systems for our citizens The Need for Congress to Shape Developments Three major forces are rapidly changing our financial system and rendering old structures obsolete These forces offer Congress the opportunity to restructure the financial services industry in a way that will serve the public interest by assuring minimum cost, maximum service, and prudent risk management The most profound force is, of course, technology the rapid growth of computers and telecommunications Their spread has lowered the cost and broadened the scope of financial services, making possible new product development that would have been inconceivable a short time ago, and, in the process, challenging the institutional and market boundaries that in an earlier day seemed so well defined Technological innovation has accelerated the second major trend, financial globalization, that has been in process for at least three decades Both developments have expanded cross-border asset holdings, trading, and credit flows and, in response, both securities firms and U S and foreign banks have increased their cross-border locations Under a congressional mandate, foreign offices of U S banking organizations have for some time been permitted, within limits, to meet the competitive pressures of the local markets in which they operate by conducting activities not permitted to them in the United States In the evolving international environment, these off-shore activities have included global secunties underwriting and dealing, through subsidiaries, an activity in which U S banking organizations have been among the world leaders, despite limitations on their authority to distribute securities in the United States Such a response to competition abroad is an example of the third major trend reshaping financial marketsâ€”market innovationâ€”which has been as much a reaction to technological change and globalization as an independent factor These developments make it virtually impossible to maintain some of the rules and regulations established for a different economic environment As a result, the kinds of activities our banking organizations are conducting no longer fit the traditional paradigms of deposit taking and loan making Technological change, globalization, and regulatory erosion will eventually make it impossible to sustain outdated restrictions That is what we are here today to discussâ€”the need to remove outdated restrictions and to rationalize our system for delivering financial services To be sure, with the benefits of financial modernization come some risks, but the Board believes the evidence indicates that the risks in securities underwriting and dealing are manageable Underwriting primarily is a deals oriented, purchase and rapid resale, mark-to- market business in which losses, if any, are quickly cut as the firm moves to the next deal Since the enactment of the Securities Actsâ€”with their focus on investor protectionâ€”the broker/dealer regulator, the SEC, is quick to liquidate a firm with insufficient capital relative to the market value of its assets, constraining the size of any disturbance to the market or affiliates The SEC now applies such supervision to Section 20 affiliates, and it would do so to securities affiliates under H R 10 and similar bills introduced in this Congress Section 20 affiliates have operated during a period in which sharp swings have occurred in world financial markets, but they still were able to manage their risk exposures well with no measurable risks to their parent or affiliated banks Indeed, in order to limit the exposure of the safety net, the supervisors have insisted that securities affiliates have risk management and control systems that assure that risk can be managed and contained As would be the case for securities affiliates with the Competitiveness Act, the Federal Reserve has required that such an infrastructure exist before individual Section 20 affiliates are authorized and that organizations engaging in these activities through nonbank affiliates have bank subsidiaries with strong capital positions The bill proposed by Chairman Leach attempts to accommodate the merchant banking business currently conducted by independent securities firms Both bank holding companies with Section 20 subsidiaries and independent securities firms engage in securities underwriting and dealing activities However, independent securities firms also directly provide equity capital to a wide variety of companies without any intention to manage or operate them The Leach bill would permit securities firms that acquire commercial banks, as well as securities firms acquired or established by bank holding companies, to engage in all of these activitiesâ€”underwriting and dealing in securities, as well as merchant and investment banking through equity investment in any business without becoming involved in the day-to- day operations of that business These powers are crucial to permit securities firms to remain competitive domestically and internationally Under the bill, the Board could establish rules to ensure that these activities do not pose significant risks to banks affiliated with securities firms, serve as a "back door" to the commingling of banking and commerce, or unduly spread the subsidy impact in the safety net As for insurance, the evidence is clear that, where risk is diversifiable and, hence, predictable, such as life and certain property insurance lines, the resultant business risks are manageable The evidence is less clear for catastrophe-related property insurance Other risks come from the same sorts of credit and interest rate risks about which banks are already knowledgeable Life, automobile, and other insurance sales are virtually riskless and authorizing insurance brokerage sales by banks is likely to add additional convenience and service, as well as lower prices, for the public. H R 10 would continue the holding company framework for nonbank activities, which the Board believes is important in order to limit the direct risk of new financial activities to banks and the safety net The Board is of the view that the risks from securities and insurance underwriting are manageable using the holding company framework proposed in the Competitiveness Act But there is another risk the risk of transference to nonbank affiliates of the subsidy implicit in the federal safety netâ€”deposit insurance, the discount window, and access to the payments systemâ€”with the attendant moral hazard As the Committee knows, the Board believes that the subsidy is more readily transferred to a subsidiary of an insured depository institution than to its affiliates, and that the holding company structure creates the best framework for limiting this leakage We have concluded accordingly that the further the separation from the bank, the better the insulation We are concerned that conducting securities and similar activities as principal in subsidiaries of U S banks does not create sufficient distance from the bank Let me be clear that bank holding companies and their subsidiaries also benefit from the subsidy implicit in the safety net Their capital costs are lower since a portionâ€”currently a large part ofâ€”the consolidated assets of the organization are in subsidiary depository institutions that have direct access to the safety net This transfer, of course, is significantly smaller than the direct transfer to a bank subsidiary But it is large enough to suggest that we should be cautious about extending permissible activities of bank or financial services holding companies to include nonfinancial commercial enterprises Generally, public policy should give wide range to free market competition, including business decisions on affiliations However, when such affiliations may imply subsidy transfers at bestâ€”and taxpayer support at worstâ€”we should be very careful The world is changing rapidly and it may well become increasingly difficult to distinguish between banking and aspects of commerce However, the free and open legal association of banking and commerce would be a profound and surely irreversible structural change in the American economy We should, as a result, be careful to assure ourselves that whatever changes are made in our financial system do not distort our continued evolution to the most efficient financial system In earlier testimony, I suggested that we would have to review carefully the kinds of combinations that could occur with a permissible basket for nonfinancial firms As we have done so, the problems exposed have led us to a more cautious position More generally, the subsidy transfer concerns and our uncertainty about the ultimate impact of free affiliation between banking and commerce on our financial system suggest to the Board that at least any wider authonzation of banking and commerce should be postponed while we focus on financial modernization Concerns about ensuring a two-way street should be addressed without attempting to make final decisions now about any future wider combinations of banking and commerce The legislation proposed by Chairman Leach also provides for oversight of the consolidated activities of a financial services holding company The Board believes such oversight is essential to a sound financial system in which the public can have confidence Some, however, have expressed concerns that such oversight is incompatible with an institution that owns a number of otherwise unregulated subsidiaries That view is presumably directed at an expected level of significant supervisory intrusion and possibly from fear of new regulatory constraints by those acquiring a bank for the first time The Board also has concerns about excessive oversight, although for somewhat different reasons In an environment of greater deregulation and financial reform, market discipline becomes ever more critical Such discipline requires that market participants correctly perceive that nonbanking entities are not covered by the federal safety net Providing bank-like supervision to nonbank affiliates of banks in the context of financial reform would send the wrong signal, creating difficult moral hazard issues For these reasons, the agency charged with consolidated oversight should have a clearly defined roleâ€”one that permits it to protect affiliated banks and the safety net from abuse and excessive risk, while permitting operational synergies and imposing minimal interference with the growth or activities of the bank's affiliates The Board believes that combination of the holding company vehicle and Federal Reserve supervision and regulation under the Bank Holding Company Act has limited the transfer of the safety net from the banks to the holding company parent and its nonbank subsidiaries The historical experience in supervising bank holding companies also has shown that knowledge of the financial strength and risks inherent in a consolidated holding company can be critical to protecting an insured subsidiary bank and resolving problems once they arise Examples are easy to recall BCCI, Continental Illinois, Barings PLC, thrifts, and Texas banks all exhibited problems that spread quickly among their affiliates, or required a consolidated approach to resolve the problems at least cost and disruption to the financial system By approaching matters from the perspective of a consolidated organization, the Federal Reserve, the agency historically charged with conducting consolidated oversight, has also helped to prevent banking problems by addressing operational or capital deficiencies within a subsidiary bank, or elsewhere in the organization. Moreover, continued gains in technology and in innovative risk management techniques permit organizations of all kinds to manage and control their activities on an increasingly centralized basis, with less attention paid to the individual legal entities that make up the organization In that environment, it seems to the Board that oversight on a consolidated basis of an organization's broad-based activities becomes more crucial, not less Bank supervisors throughout the world recognize this point, and have adopted consolidated oversight as a fundamental principle The Congress also recognized the necessity of consolidated oversight for the U S banking system, by requiring, as a condition for a foreign bank's entry into this country, that the bank be subject to consolidated home country supervision What is necessary for foreign banks entering the United States is surely just as necessary for U S banks and the U S banking system While important, consolidated oversight need not become unduly intrusive to financial services holding companies The necessity to understand and review centralized risk management and control mechanisms, and similarly to review intra-organizational fund transfers involving the insured depositories, does not require bank-like supervision of nonbank affiliates H R 10 recognizes this It would require the banking agencies to rely to the fullest extend possible on examination reports and other information collected by supervisors of other regulated entities It would also provide for quite limited consolidated oversight for those organizations in which the bank subsidiaries represent a modest part of the overall organization and do not exceed a maximum size In addition, the bill would require the banking agencies to defer to the SEC in interpretations and enforcement of the federal securities laws It further eliminates the current legal requirements for applications for nonbanking activities by holding companies that own relatively small banks, an approach we believe could also be extended quite usefully to bank acquisition proposals These are extremely important provisions both for existing bank holding companies and for securities firms and insurance companies that wish to affiliate with banks. Such provisions would greatly enhance the "two-way street" by eliminating unnecessary burden and red tape The Board not only supports these changes, but also recognizes that its own traditional approach to supervising and regulating bank holding companies must change as technology changes Indeed, such changes are already well underway They include a much streamlined application process, a more risk-focused/less transaction-testing approach to inspections, fewer firewalls between banking and securities affiliates of bank holding companies to accommodate operating synergies, and greater reliance on internal and external auditors In anticipation of financial modernization legislation, the Board is considering alternative approaches to evaluating the capital adequacy of heterogeneous financial conglomerates, when banking is not the dominant activity Such flexibility would be required to ensure that bank-like standards are not indirectly imposed on insurance or securities firms and that the standards of their primary regulator prevail and allow them to compete effectively As the affiliates of banks increasingly conduct a nonbanking business, the desirability of avoiding the extension of bank-like regulation will require that the agency with oversight responsibility rely heavily on published financial reports, agency reviews of existing management information, examinations by other supervisors, and evaluations by market analysts when assessing the overall strength and potential riskiness of a bank's parent and affiliates Such information can alert the oversight agency to look more closely at the organization and, if necessary, take steps to protect an affiliated bank Indeed, that agency should be empowered and expected to prevent or curtail abusive practices and undue risks in an organization when they threaten affiliated banks and the safety net Similarly, it should be just as responsible to assure that the transfer of the subsidy of the safety net from the bank to its affiliate, through intra-organizational funds transfers and othe means, is kept to a minimum I believe the United States currently has a strong and effective supervisory process, and one that has also permitted its banking and financial system to fuel economic growth to a degree unmatched in the world today While we have had our problems, most notably with thrifts, we must not forget our experience as we work toward a still-better approach Our domestic banking system is also widely recognized as the most innovative and best capitalized system in the world, and its profits have reached new record levels in recent years As I have pointed out previously, advancing technology will inevitably require increasing reliance on pnvate counterparty surveillance to contain credit and market risks Nonetheless, we should recall that just six or seven years ago, events created pressures to expand and increase government banking supervision at all levels In the present environment of prosperity and financial stability, it is easy to forget that experience and to believe that little or no oversight is now needed for consolidated entities We must move forward, but with proper balance, Mr Chairmanâ€”with a balance that I believe your bill maintains, with the exception noted The agency conducting consolidated oversight must be permitted to monitor both the financial condition of the organization and the potential transfer of risks to its insured depository affiliates Moreover, we reiterate our concern that, regardless of how restructuring is addressed, the Congress not impair the ability of the Federal Reserve to monitor large banking organizations and respond effectively to systemic crises "Mr Chairman, members of the Committee, the question is not whether we will have changes in financial markets Technology, globalization, and market innovations are bringing rapid changes that cannot be reversed The open questions are how banking organizations will participate, and will they do so in ways that appropriately balance the tradeoffs among risk, minimal use of the sovereign credit, and maximum competition, public benefit and convenience If Congress does not act, the balancing will be done by market forces and, where possible, regulators forced to take positions by events The Board believes that the Congress needs to act and that the Leach proposalâ€”excluding authorization for new activities in bank subsidiariesâ€”accomplishes a balancing of the risks and benefits of banks' participation in financial modernization The Board also urges that the Congress resist efforts to so limit consolidated oversight of banking organizations as to raise questions about our ability to limit risk exposures of insured depositones, to limit the transference of the safety net subsidy, or to prevent and manage financial market crises</t>
-  </si>
-  <si>
-    <t>Mr Chairman, I appreciate the opportunity to present the views of the Board of Governors on the Financial Services Competition Act of 1997 The Banking Committee is to be commended for addressing the complex issues associated with financial modernization The Committee has taken a major step forward in permitting affiliations of banking, securities, and insurance organizations within an appropriate framework for consolidated oversight We believe such affiliations would improve the efficiency and competitiveness of the financial services industry, and result in more choices and better services for consumers However, in addressing financial modernization the bill encompasses a large number of far ranging provisions The Board has difficulty with the way some of the issues are resolved in the bill before you, Thus, while reemphasizing our support for much of the general thrust of the bill, I would like today to highlight our major concerns The need to respond to the effects of technology is one of the major reasons we are here today Technology has already eroded many of the previous distinctions between banking and nonbank finance, thereby supporting the desirability, if not the necessity, of permitting the merging of all financial activities It seems clear that the same forces are in the process of blurring the boundaries between financial and nonfinancial businesses Most of us are aware of software companies interested in the financial services business, but some financial firms, leveraging off their own internal skills, are also seeking to produce software for third parties Shipping companies' tracking software lends itself to payment services Manufacturers have financed their customers' purchases for a long time, but now increasingly are using the resultant financial skills to finance noncustomers Moreover, many nonbank financial institutions are now profitably engaged in nonfinancial activities Current facts and future trends, in short, are creating market pressures to permit the common ownership of financial and nonfinancial firms The Board, in fact, has concluded that it is quite likely that in future years it will be close to impossible to distinguish where one type of activity ends and another begins Nonetheless, the Federal Reserve Board also has concluded that it would be wise to move with caution in addressing the removal of the current legal barriers between commerce and banking, since the unrestricted association of banking and commerce would be a profound and surely irreversible structural change in the American economy Were we fully confident of how emerging technologies would affect the evolution of our economic and financial structure, we could presumably develop today the regulations which would foster that evolution But we are not, and history suggests we cannot We thus run the risk of locking in a set of inappropriate rules that could adversely alter the development of market structures Our ability to foresee accurately the future implications of technologies and market developments in banking, as in other industries, has not been particularly impressive As Professor Rosenberg of Stanford University has pointed out, mistaken forecasts of future structure litter our financial landscape " Consider the view of the 1960s that the "cashless society" was imminent Nonetheless, the public preference for paper has declined only gradually Similarly, just a few years ago conventional wisdom argued that banks were dinosaurs that were becoming extinct The reality today is far from it Even more recently, it was argued that banks and nonfinancial firms had to merge in order to save the capital-starved banking system Today, as you know, virtually all of our banks are very well capitalized. All these examples, and more, suggest that if we dramatically change the rules now about banking and commerce under circumstances of great uncertainty about future synergies between finance and nonfinance we may well end up doing more harm than good And, as with all rule changes by government, we are likely to find it impossible to correct our errors promptly, if at all Modifications of such a fundamental structural rule as the separation of banking and commerce accordingly should proceed at a deliberate pace in order to test the response of markets and technological innovations to the altered rules in the years ahead Excessive delay would doubtless produce inequities Expanded financial activities for banking organizations require, and the Banking Committee's Financial Services Competition Act provides, that those firms operating in markets that banks can enter, in turn, be authorized to engage in banking However, some securities and insurance firms, as well as some thrifts, already own-or are owned by-nonfinancial entities Continuing the commerce and banking prohibitions would thus require the divestiture or grandfathenng of all nonfinancial activities by those organizations that wanted to acquire or establish banks But, the fact is that we do not-and the Board's view is that we need notâ€”have to make today as sweeping a banking and commerce decision as the Competition Act proposes That bill would permit both banks and nonfinancial corporations each to originate up to 15 percent of their revenue from the other's activities While there is some limit on the original size of each nonfinancial firm acquired by a bank holding company and on the original size of the one bank that a nonfinancial company could purchase, the subsequent growth is only constrained by the 15 percent revenue limit This constraint may be more apparent than real, given the ongoing growth and consolidation of the financial services industry In our judgment, these baskets are far larger than what is needed either as a controlled experiment or to permit unfettered consolidation with banks of those financial firms that have commercial affiliates Moreover, the Banking Committee bill would permit additional bank and commercial affiliations beyond these holding company affiliate baskets and permit some affiliation within the bank or a bank subsidiary Any commercial (or financial) activity that had been authorized by the Office of Thrift Supervision for thrifts or by the Federal Reserve Board's regulation for overseas operations of U S banks would be permitted to banks in the United States by the Banking Committee bill Thus, over and above the basket, U S banks could create subsidiaries that invest up to 3 percent of the bank's assets in the equity of OTS- approved commercial enterprises. In addition, applying the Board's foreign market rule to domestic operations would mean that banks themselves could invest in the equity of individual nonfinancial firms The Board's foreign market rule, authorized by statute, was promulgated to assist American banks to achieve a level playing field with their foreign competitors in foreign markets We see no compelling need to apply that rule to American banks' domestic operations We are also concerned that the grandfather date for savings and loan holding companies continues to shift with the date of enactment of the bill, thereby encouraging an increase in the number of commercial firms that seek to affiliate with insured savings associations before new rules come into effect The Competition Act, in the Board's view, goes well beyond what both commercial banks and nonfinancial firms need to meet the requirements of today, as well as in the foreseeable future The Board believes it would be virtually impossible to reverse such a change in the legal framework without major damage to established business relationships Thus, any errors from larger-than-needed initial authorizations could result in significant problems Moreover, the authorization of commercial activities through banks and their subsidiaries directly extends the subsidy of the safety net over a much wider range of activities, not to mention potentially undermining the safety and soundness of insured banks Mr Chairman, a number of observers have argued that there is no subsidy associated with the federal safely net for depository institutions-deposit insurance, and direct access to the Federal Reserve's discount window and payment system guarantees The Board strongly rejects this view In saying this, the Board fully agrees that mandated government supervision and regulation impose significant costs on banks, costs which, in many cases, can and should be reduced But given that these costs cannot be avoided by a bank, no rational bank manager would ignore the opportunity to take advantage of the lower cost of funds, or equivalently, the lower capital ratio, that access to the safety net demonstrably provides While it is true that the safety net does increase the possibility of loss to taxpayers, a far larger public policy concern is that it provides banks with a government-sanctioned competitive advantage over nonbank firms In the Board's view, unless Congress explicitly desires to expand access to the safety net and tilt the competitive playing field further, a core component of any prudent financial modernization strategy should be to minimize the chances that safety net subsidies will be expanded into new activities and beyond the confines of insured depository institutions Because the subsidy created by the federal safety net grants access to the "sovereign credit" of the United States, bank creditors are willing to accept a lower risk premium on bank liabilities and capital than otherwise would be the case For fully insured deposits this risk premium is reduced essentially to zero But other debt instruments also benefit, and the capital ratio demanded by the market is lower The end result is that banks enjoy a lower total and marginal cost of funding, including lower capital ratios, than would otherwise be required by the market While some benefits of the safety net are always available to banks, it is critical to understand that the value of the subsidy is smallest for very healthy banks during good economic times, and greatest at weak banks during a financial crisis What was it worth in the late 1980s and early 1990s for a bank with a troubled loan portfolio to have deposit liabilities guaranteed by the FDIC, to be assured that it could turn illiquid assets to liquid assets at once through the Federal Reserve discount window, and to tell its customers that payment transfers would be settled on a nskless Federal Reserve Bank? For many, it was worth not basis points but percentage points For some, it meant the difference between survival and failure In contrast today, when the economy is performing well and the banking industry has just experienced its fifth straight year of record profits, it is perhaps too easy to ignore the value of the safety net and see only its costs The Board believes that prudent public policy should take a longer view In the Board's judgment, the bank holding company organizational form has, by the record, proved to be an effective means for limiting the safety net subsidy primarily to banks There is clear evidence that market participants understand that regulatory policy is focused on the bank, and thus markets distinguish between the bank and its holding company parent and affiliates Given this success, the holding company structure should, in the Board's view, not be abandoned Indeed, our strong preference is for the holding company format to be retained for new activities that will under expanded authonties benefit from direct access to the federal safety net Thus, we would recommend that the Financial Services Competition Act's provisions that allow expanded activities to be conducted either in a holding company subsidiary or in a direct operating subsidiary of a bank be amended to require that new activities be conducted only in a holding company subsidiary The Board supports the provisions of the Banking Committee's Competition Act that continue consolidated oversight of the bank holding company In our judgment, it is essential that these provisions be retained and not weakened The historical experience in supervising bank holding companies has shown that knowledge of the financial strength and risks inherent in a consolidated holding company can be critical to protecting an insured subsidiary bank and resolving problems once they arise Examples are easy to recall BCCI, Continental Illinois, Barings PLC, thrifts, and Texas banks all exhibited problems that spread quickly among their affiliates, or required a consolidated approach to resolve the problems at least cost and disruption to the overall financial system Moreover, continued gains in technology and in innovative risk management techniques permit organizations of all kinds to manage and control their activities on an increasingly centralized basis, with less attention paid to the individual legal entities that make up the organization In that environment, it seems to the Board that oversight on a consolidated basis of an organization's broad-based activities has become more crucial in recent years, not less Bank supervisors throughout the world recognize this point, and have adopted consolidated oversight as a fundamental principle The Congress also recognized the necessity of consolidated oversight for the U S banking system, by requiring, as a condition for a foreign bank's entry into this country, that the bank be subject to consolidated home country supervision What is necessary for foreign banks entering the United States is surely just as necessary for U S banks and the U S banking system Crisis Management and Systemic Risk Mr Chairman, we believe that the Federal Reserve needs to continue to have consolidated oversight authority, especially for organizations in which the bank is large enough that its failure could cause disruptions in financial markets sufficient to affect economic activity Critically, the central bank has the responsibility to forestall financial crises (including systemic disturbances in the banking system) and to manage such crises once they occur Supervisory and regulatory responsibilities afford the Federal Reserve both the insight and the authority to use crisis management techniques that are less blunt than open market operations, and more precisely calibrated to the problem at hand Such tools not only improve our ability to manage crises but, more importantly, help us to avoid them Indeed, we measure our degree of success in this area not by the number of crises we assist in containing, but rather in the number of crises which could have erupted but did not The use of cnses management techniques requires both the authority that comes with supervision and regulation and the understanding of the linkages among supervision and regulation, prudential standards, risk-taking, relationships among banks and other financial market participants, and macroeconomic stability The objectives of the central bank in crisis management are to contain financial losses and prevent a contagious loss of confidence so that difficulties at one institution do not spread more widely to others The focus of its concern is not to avoid the failure of entities that have made poor decisions or have had bad luck, but rather to see that such failuresâ€”or threats of failures-do not have broad and serious impacts on financial markets and the national, and indeed the global, economy The Federal Reserve's ability to respond expeditiously to any particular incident does not necessitate comprehensive information on each banking institution But it does require that the Federal Reserve have in-depth knowledge of how institutions of vanous sizes and other characteristics are likely to behave, and what resources are available to them in the event of severe financial stress We currently gain the necessary insight by having a broad sample of banks subject to our supervision and through our authority over bank holding companies Payment and Settlement Systems A key element of avoiding systemic concerns is management of the payment system Virtually all of the U S dollar transactions made worldwideâ€”for securities transfers, foreign exchange and other international capital flows, and for payment for goods and servicesâ€”are settled in the United States banking system A small number of transactions that comprise the vast proportion of the total value of transactions are transferred over large-dollar payment systems A critical component of these systems is the Federal Reserve's wire transfer network, Fedwire Fedwrre and a very small number of private clearinghouses are arguably the linchpin of the international system of payments that relies on the dollar as the major international currency for trade and finance Disruptions and disturbances in the U S payment system thus can easily have global implications In all of these payment and settlement systems, commercial banks play a central role, both as participants and as providers of credit to nonbank participants Day-in and day-out, the settlement of payment obligations and securities trades requires significant amounts of bank credit In periods of stress, such credit demands surge just at the time when some banks are least willing or able to meet them These demands, if unmet, could produce gridlock in payment and settlement systems, exposing financial markets to dangerous stress Indeed, it is in the cauldron of the payment and settlement systems, where decisions involving large sums must be made quickly, that all of the risks and uncertainties associated with problems at a single participant become focussed as participants seek to protect themselves from uncertainty Better solvent than sorry, they might well decide, and refuse to honor a payment request Observing that, others might follow suit And that is how crises often begin Limiting, if not avoiding, such disruptions and ensuring the continued operation of the payment system requires broad and indepth knowledge of banking and markets, as well as detailed knowledge and authority with respect to the payment and settlement arrangements and their linkages to banking operations This type of insight and authonty-as well as knowledge about the behavior of key participants-cannot be created on an ad hoc basis It requires broad and sustained involvement in both the payment infrastructure and the operation of the banking system Supervisory authority over the major bank participants is a necessary element Changing Role of Consolidated Oversight The modernizing of our financial systemâ€” especially the combining of banks, securities firms, and insurance companies, as well as possibly banking and commerce-requires that the role of consolidated oversight also be reviewed The necessity to understand and review centralized risk management and control mechanisms, and similarly to review intra-organizational fund transfers involving the insured depositories, does not require bank-like supervision of nonbank affiliates The Competition Act appropriately recognizes this It would require that the banking agencies rely to the fullest extent possible on examination reports and other information collected by supervisors of other regulated entities In addition, the bill would require the banking agencies to defer to the Securities and Exchange Commission in interpretations and enforcement of the federal securities laws and to the state insurance commissioners and to state insurance laws The bill continues to allow the Federal Reserve Board to establish capital adequacy guidelines at the holding company level However, the bill sets important limits on these holding company guidelines For example, the consolidated supervisor may not impose capital requirements on any nonbank subsidiary that is in compliance with applicable capital requirements of another federal or state agency In addition, holding company capital guidelines must take full account of the capital position of these regulated nonbank subsidiaries when establishing consolidated capital guidelines, and full account of capital levels in unregulated subsidiaries when those levels are consistent with industry norms The bill requires the Federal Reserve Board to address the use of double leverage (that is, the use of debt at the holding company to fund equity and subordinated debt at a regulated institution), but prohibits the establishment of a capital ratio that is not risk weighted In addition, the bill requires that the consolidated supervisor consult with other supervisors, including in particular, supervisors of nonbanking entities, prior to establishing capital guidelines for holding companies All of these--the capital and examination rules-are extremely important provisions both for existing bank holding companies and for secunties firms and insurance companies that wish to affiliate with banks Such provisions would greatly enhance the "two-way street" by eliminating unnecessary burden and red tape Mr Chairman, the Board believes that bank holding companies need to continue to have consolidated oversight in order both to protect the safety net and to limit the transference of the safety net subsidy We believe that the Federal Reserve must not have its ability impaired to monitor banking organizations in order to respond effectively to systemic crises, to manage the nsk in the payment system, and to ensure the safety and stability of our financial system Mr Chairman, to summarize The Board supports the overall thrust of the Banking Committee bill that is now being reviewed by this Committee We strongly support the bill's approach to affiliations of banking, secunties, and insurance organizations We are, nonetheless, concerned that the bill goes unnecessarily far at this time in mixing commerce and banking There is no reason not to proceed in incremental steps, first to integrate banking and finance with the minor and quite limited combinations of banking and commerce that this requires, and only later, as these developments mature, assess the desirability of fully dismantling the barriers between banking and commerce In addition, we think it unwise to permit banks to conduct new activities in their own subsidiaries because of the extension of the safety net subsidy directly to those subsidiaries We have concluded that the holding company framework provides the best insulation against the transference of that subsidy beyond the bank, and creates the most level playing field for affiliations of banks and other financial firms Consolidated oversight of bank holding companies is critical both to protect the safety net and to minimize its transference We believe that the central bank's role in the prevention and containment of financial cnses and as guarantor of the payment system requires that we continue to have consolidated oversight responsibility for most holding companies</t>
-  </si>
-  <si>
     <t>The Committee (FOMC) decided today to leave its target for the FFR unchanged. Strengthening productivity growth has been fostering favorable trends in unit costs and prices, and much recent information suggests that these trends have been sustained. Nonetheless, the growth of demand has continued to outpace that of supply, as evidenced by a decreasing pool of available workers willing to take jobs. In these circumstances, the Committee (FOMC) will need to be especially alert in the months ahead to the potential for costs to increase significantly in excess of productivity in a manner that could contribute to inflation pressures and undermine the impressive performance of the economy. Against this background, the Committee adopted a directive that was biased toward a possible firming of policy going forward. Committee members emphasized that such a directive did not signify a commitment to near-term action. The Committee will need to evaluate additional information on the balance of aggregate supply and demand and conditions in financial markets.</t>
   </si>
   <si>
@@ -951,16 +860,35 @@
   </si>
   <si>
     <t>Although overall economic activity edged down in the first quarter, household spending and business fixed investment remained strong. Job gains have been robust in recent months, and the unemployment rate has declined substantially. Inflation remains elevated, reflecting supply and demand imbalances related to the pandemic, higher energy prices, and broader price pressures. The invasion of Ukraine by Russia is causing tremendous human and economic hardship. The implications for the U.S. economy are highly uncertain. The invasion and related events are creating additional upward pressure on inflation and are likely to weigh on economic activity. In addition, COVID-related lockdowns in China are likely to exacerbate supply chain disruptions. The Committee is highly attentive to inflation risks. The Committee seeks to achieve maximum employment and inflation at the rate of 2 percent over the longer run. With appropriate firming in the stance of monetary policy, the Committee expects inflation to return to its 2 percent objective and the labor market to remain strong. In support of these goals, the Committee decided to raise the target range for the FFR to 0.75 to 1 percent and anticipates that ongoing increases in the target range will be appropriate. In addition, the Committee decided to begin reducing its holdings of Treasury securities and agency debt and agency mbs on June 1, as described in the Plans for Reducing the Size of the FR's Balance Sheet that were issued in conjunction with this statement. In assessing the appropriate stance of monetary policy, the Committee will continue to monitor the implications of incoming information for the economic outlook. The Committee would be prepared to adjust the stance of monetary policy as appropriate if risks emerge that could impede the attainment of the Committee's goals. The Committee's assessments will take into account a wide range of information, including readings on public health, labor market conditions, inflation pressures and inflation expectations, and financial and international developments. Voting for the monetary policy action were Jerome H. Powell, Chair; John C. Williams, Vice Chair; Michelle W. Bowman; Lael Brainard; James Bullard; Esther L. George; Patrick Harker; Loretta J. Mester; and Christopher J. Waller. Patrick Harker voted as an alternate member at this meeting.</t>
+  </si>
+  <si>
+    <t>FOMC Communication Text Cleaning Procedure:</t>
+  </si>
+  <si>
+    <t>Federal Open Market Committee = Committee (FOMC)
+federal funds rate = FFR
+Board of Governors = BOG
+Federal Reserve = FR
+basis points = bps
+basis point = bps
+-basis-point =  bps (extra space at the beginning)
+mortgage-backed securities = mbs
+Term Asset-Backed Securities = TABS
+Information received since the Committee (FOMC) met in [Month] = Information received</t>
+  </si>
+  <si>
+    <t>Repetitive and technical terms are replaced with corresponding single abbreviations that themselves have been used by the Federal Reserve System
+at least one time in their released statements. The last substitution is specific to FOMC statements and is to prevent look-ahead bias from neural
+networks for text analysis. The following terms and abbreviations are as follows:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
     <numFmt numFmtId="165" formatCode="hh:mm:ss;@"/>
-    <numFmt numFmtId="166" formatCode="yyyy;@"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -1016,7 +944,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1027,7 +955,6 @@
     <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1363,11 +1290,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="110" customWidth="1"/>
-    <col min="2" max="2" width="92" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="107.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="75.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="96" x14ac:dyDescent="0.2">
@@ -1393,10 +1320,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -1541,6 +1468,19 @@
       </c>
       <c r="B25" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="160" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -1591,7 +1531,7 @@
         <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -1608,7 +1548,7 @@
         <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>91</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -1625,7 +1565,7 @@
         <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>173</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -1642,7 +1582,7 @@
         <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -1659,7 +1599,7 @@
         <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>126</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -1676,7 +1616,7 @@
         <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -1693,7 +1633,7 @@
         <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>174</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -1710,7 +1650,7 @@
         <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>127</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -1727,7 +1667,7 @@
         <v>29</v>
       </c>
       <c r="E10" t="s">
-        <v>128</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -1744,7 +1684,7 @@
         <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>129</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -1761,7 +1701,7 @@
         <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>130</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -1778,7 +1718,7 @@
         <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>131</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -1795,7 +1735,7 @@
         <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>132</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
@@ -1812,7 +1752,7 @@
         <v>29</v>
       </c>
       <c r="E15" t="s">
-        <v>133</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -1829,7 +1769,7 @@
         <v>29</v>
       </c>
       <c r="E16" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -1846,7 +1786,7 @@
         <v>29</v>
       </c>
       <c r="E17" t="s">
-        <v>134</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -1863,7 +1803,7 @@
         <v>29</v>
       </c>
       <c r="E18" t="s">
-        <v>135</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -1880,7 +1820,7 @@
         <v>29</v>
       </c>
       <c r="E19" t="s">
-        <v>136</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -1897,7 +1837,7 @@
         <v>29</v>
       </c>
       <c r="E20" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -1914,7 +1854,7 @@
         <v>29</v>
       </c>
       <c r="E21" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -1931,7 +1871,7 @@
         <v>29</v>
       </c>
       <c r="E22" t="s">
-        <v>138</v>
+        <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -1948,7 +1888,7 @@
         <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -1965,7 +1905,7 @@
         <v>29</v>
       </c>
       <c r="E24" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -1982,7 +1922,7 @@
         <v>29</v>
       </c>
       <c r="E25" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -1999,7 +1939,7 @@
         <v>29</v>
       </c>
       <c r="E26" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -2016,7 +1956,7 @@
         <v>29</v>
       </c>
       <c r="E27" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -2033,7 +1973,7 @@
         <v>29</v>
       </c>
       <c r="E28" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -2050,7 +1990,7 @@
         <v>29</v>
       </c>
       <c r="E29" t="s">
-        <v>200</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -2067,7 +2007,7 @@
         <v>29</v>
       </c>
       <c r="E30" t="s">
-        <v>201</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -2084,7 +2024,7 @@
         <v>29</v>
       </c>
       <c r="E31" t="s">
-        <v>202</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -2101,7 +2041,7 @@
         <v>29</v>
       </c>
       <c r="E32" t="s">
-        <v>203</v>
+        <v>173</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -2118,7 +2058,7 @@
         <v>29</v>
       </c>
       <c r="E33" t="s">
-        <v>292</v>
+        <v>262</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -2135,7 +2075,7 @@
         <v>29</v>
       </c>
       <c r="E34" t="s">
-        <v>97</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -2152,7 +2092,7 @@
         <v>29</v>
       </c>
       <c r="E35" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -2169,7 +2109,7 @@
         <v>29</v>
       </c>
       <c r="E36" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -2186,7 +2126,7 @@
         <v>29</v>
       </c>
       <c r="E37" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -2203,7 +2143,7 @@
         <v>29</v>
       </c>
       <c r="E38" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -2220,7 +2160,7 @@
         <v>29</v>
       </c>
       <c r="E39" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -2237,7 +2177,7 @@
         <v>29</v>
       </c>
       <c r="E40" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -2254,7 +2194,7 @@
         <v>29</v>
       </c>
       <c r="E41" t="s">
-        <v>82</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -2271,7 +2211,7 @@
         <v>29</v>
       </c>
       <c r="E42" t="s">
-        <v>83</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -2288,7 +2228,7 @@
         <v>29</v>
       </c>
       <c r="E43" t="s">
-        <v>84</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -2305,7 +2245,7 @@
         <v>29</v>
       </c>
       <c r="E44" t="s">
-        <v>85</v>
+        <v>55</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -2322,7 +2262,7 @@
         <v>29</v>
       </c>
       <c r="E45" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -2339,7 +2279,7 @@
         <v>29</v>
       </c>
       <c r="E46" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -2356,7 +2296,7 @@
         <v>29</v>
       </c>
       <c r="E47" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -2373,7 +2313,7 @@
         <v>29</v>
       </c>
       <c r="E48" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -2390,7 +2330,7 @@
         <v>29</v>
       </c>
       <c r="E49" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -2407,7 +2347,7 @@
         <v>29</v>
       </c>
       <c r="E50" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -2424,7 +2364,7 @@
         <v>29</v>
       </c>
       <c r="E51" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -2441,7 +2381,7 @@
         <v>29</v>
       </c>
       <c r="E52" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -2458,7 +2398,7 @@
         <v>29</v>
       </c>
       <c r="E53" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -2475,7 +2415,7 @@
         <v>29</v>
       </c>
       <c r="E54" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -2492,7 +2432,7 @@
         <v>29</v>
       </c>
       <c r="E55" t="s">
-        <v>144</v>
+        <v>114</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
@@ -2509,7 +2449,7 @@
         <v>29</v>
       </c>
       <c r="E56" t="s">
-        <v>182</v>
+        <v>152</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -2526,7 +2466,7 @@
         <v>29</v>
       </c>
       <c r="E57" t="s">
-        <v>94</v>
+        <v>64</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -2543,7 +2483,7 @@
         <v>29</v>
       </c>
       <c r="E58" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -2560,7 +2500,7 @@
         <v>29</v>
       </c>
       <c r="E59" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
@@ -2577,7 +2517,7 @@
         <v>30</v>
       </c>
       <c r="E60" t="s">
-        <v>183</v>
+        <v>153</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
@@ -2594,7 +2534,7 @@
         <v>30</v>
       </c>
       <c r="E61" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
@@ -2611,7 +2551,7 @@
         <v>30</v>
       </c>
       <c r="E62" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
@@ -2628,7 +2568,7 @@
         <v>30</v>
       </c>
       <c r="E63" t="s">
-        <v>106</v>
+        <v>76</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
@@ -2645,7 +2585,7 @@
         <v>30</v>
       </c>
       <c r="E64" t="s">
-        <v>107</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
@@ -2662,7 +2602,7 @@
         <v>30</v>
       </c>
       <c r="E65" t="s">
-        <v>108</v>
+        <v>78</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
@@ -2679,7 +2619,7 @@
         <v>30</v>
       </c>
       <c r="E66" t="s">
-        <v>109</v>
+        <v>79</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
@@ -2696,7 +2636,7 @@
         <v>30</v>
       </c>
       <c r="E67" t="s">
-        <v>110</v>
+        <v>80</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -2713,7 +2653,7 @@
         <v>30</v>
       </c>
       <c r="E68" t="s">
-        <v>111</v>
+        <v>81</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -2730,7 +2670,7 @@
         <v>30</v>
       </c>
       <c r="E69" t="s">
-        <v>112</v>
+        <v>82</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
@@ -2747,7 +2687,7 @@
         <v>30</v>
       </c>
       <c r="E70" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
@@ -2764,7 +2704,7 @@
         <v>30</v>
       </c>
       <c r="E71" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
@@ -2781,7 +2721,7 @@
         <v>30</v>
       </c>
       <c r="E72" t="s">
-        <v>184</v>
+        <v>154</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.2">
@@ -2798,7 +2738,7 @@
         <v>30</v>
       </c>
       <c r="E73" t="s">
-        <v>146</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
@@ -2815,7 +2755,7 @@
         <v>30</v>
       </c>
       <c r="E74" t="s">
-        <v>185</v>
+        <v>155</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
@@ -2832,7 +2772,7 @@
         <v>30</v>
       </c>
       <c r="E75" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -2849,7 +2789,7 @@
         <v>30</v>
       </c>
       <c r="E76" t="s">
-        <v>148</v>
+        <v>118</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
@@ -2866,7 +2806,7 @@
         <v>30</v>
       </c>
       <c r="E77" t="s">
-        <v>149</v>
+        <v>119</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
@@ -2883,7 +2823,7 @@
         <v>30</v>
       </c>
       <c r="E78" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -2900,7 +2840,7 @@
         <v>30</v>
       </c>
       <c r="E79" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -2917,7 +2857,7 @@
         <v>30</v>
       </c>
       <c r="E80" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -2934,7 +2874,7 @@
         <v>30</v>
       </c>
       <c r="E81" t="s">
-        <v>89</v>
+        <v>59</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -2951,7 +2891,7 @@
         <v>30</v>
       </c>
       <c r="E82" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
@@ -2968,7 +2908,7 @@
         <v>30</v>
       </c>
       <c r="E83" t="s">
-        <v>116</v>
+        <v>86</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -2985,7 +2925,7 @@
         <v>30</v>
       </c>
       <c r="E84" t="s">
-        <v>283</v>
+        <v>253</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
@@ -3002,7 +2942,7 @@
         <v>30</v>
       </c>
       <c r="E85" t="s">
-        <v>204</v>
+        <v>174</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
@@ -3019,7 +2959,7 @@
         <v>30</v>
       </c>
       <c r="E86" t="s">
-        <v>205</v>
+        <v>175</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -3036,7 +2976,7 @@
         <v>30</v>
       </c>
       <c r="E87" t="s">
-        <v>206</v>
+        <v>176</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
@@ -3053,7 +2993,7 @@
         <v>30</v>
       </c>
       <c r="E88" t="s">
-        <v>207</v>
+        <v>177</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
@@ -3070,7 +3010,7 @@
         <v>30</v>
       </c>
       <c r="E89" t="s">
-        <v>208</v>
+        <v>178</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
@@ -3087,7 +3027,7 @@
         <v>30</v>
       </c>
       <c r="E90" t="s">
-        <v>209</v>
+        <v>179</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
@@ -3104,7 +3044,7 @@
         <v>30</v>
       </c>
       <c r="E91" t="s">
-        <v>210</v>
+        <v>180</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
@@ -3121,7 +3061,7 @@
         <v>30</v>
       </c>
       <c r="E92" t="s">
-        <v>211</v>
+        <v>181</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
@@ -3138,7 +3078,7 @@
         <v>30</v>
       </c>
       <c r="E93" t="s">
-        <v>212</v>
+        <v>182</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
@@ -3155,7 +3095,7 @@
         <v>30</v>
       </c>
       <c r="E94" t="s">
-        <v>213</v>
+        <v>183</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -3172,7 +3112,7 @@
         <v>30</v>
       </c>
       <c r="E95" t="s">
-        <v>214</v>
+        <v>184</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -3189,7 +3129,7 @@
         <v>30</v>
       </c>
       <c r="E96" t="s">
-        <v>215</v>
+        <v>185</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
@@ -3206,7 +3146,7 @@
         <v>30</v>
       </c>
       <c r="E97" t="s">
-        <v>216</v>
+        <v>186</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
@@ -3223,7 +3163,7 @@
         <v>30</v>
       </c>
       <c r="E98" t="s">
-        <v>217</v>
+        <v>187</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
@@ -3240,7 +3180,7 @@
         <v>30</v>
       </c>
       <c r="E99" t="s">
-        <v>218</v>
+        <v>188</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -3257,7 +3197,7 @@
         <v>30</v>
       </c>
       <c r="E100" t="s">
-        <v>219</v>
+        <v>189</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.2">
@@ -3274,7 +3214,7 @@
         <v>30</v>
       </c>
       <c r="E101" t="s">
-        <v>220</v>
+        <v>190</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
@@ -3291,7 +3231,7 @@
         <v>30</v>
       </c>
       <c r="E102" t="s">
-        <v>221</v>
+        <v>191</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
@@ -3308,7 +3248,7 @@
         <v>30</v>
       </c>
       <c r="E103" t="s">
-        <v>222</v>
+        <v>192</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
@@ -3325,7 +3265,7 @@
         <v>30</v>
       </c>
       <c r="E104" t="s">
-        <v>223</v>
+        <v>193</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
@@ -3342,7 +3282,7 @@
         <v>30</v>
       </c>
       <c r="E105" t="s">
-        <v>224</v>
+        <v>194</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
@@ -3359,7 +3299,7 @@
         <v>30</v>
       </c>
       <c r="E106" t="s">
-        <v>225</v>
+        <v>195</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
@@ -3376,7 +3316,7 @@
         <v>30</v>
       </c>
       <c r="E107" t="s">
-        <v>226</v>
+        <v>196</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
@@ -3393,7 +3333,7 @@
         <v>30</v>
       </c>
       <c r="E108" t="s">
-        <v>227</v>
+        <v>197</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
@@ -3410,7 +3350,7 @@
         <v>30</v>
       </c>
       <c r="E109" t="s">
-        <v>228</v>
+        <v>198</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
@@ -3427,7 +3367,7 @@
         <v>30</v>
       </c>
       <c r="E110" t="s">
-        <v>229</v>
+        <v>199</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
@@ -3444,7 +3384,7 @@
         <v>30</v>
       </c>
       <c r="E111" t="s">
-        <v>230</v>
+        <v>200</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.2">
@@ -3461,7 +3401,7 @@
         <v>30</v>
       </c>
       <c r="E112" t="s">
-        <v>231</v>
+        <v>201</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.2">
@@ -3478,7 +3418,7 @@
         <v>30</v>
       </c>
       <c r="E113" t="s">
-        <v>232</v>
+        <v>202</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.2">
@@ -3495,7 +3435,7 @@
         <v>30</v>
       </c>
       <c r="E114" t="s">
-        <v>233</v>
+        <v>203</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.2">
@@ -3512,7 +3452,7 @@
         <v>30</v>
       </c>
       <c r="E115" t="s">
-        <v>234</v>
+        <v>204</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.2">
@@ -3529,7 +3469,7 @@
         <v>30</v>
       </c>
       <c r="E116" t="s">
-        <v>235</v>
+        <v>205</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
@@ -3546,7 +3486,7 @@
         <v>30</v>
       </c>
       <c r="E117" t="s">
-        <v>236</v>
+        <v>206</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
@@ -3563,7 +3503,7 @@
         <v>30</v>
       </c>
       <c r="E118" t="s">
-        <v>237</v>
+        <v>207</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
@@ -3580,7 +3520,7 @@
         <v>30</v>
       </c>
       <c r="E119" t="s">
-        <v>238</v>
+        <v>208</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
@@ -3597,7 +3537,7 @@
         <v>30</v>
       </c>
       <c r="E120" t="s">
-        <v>239</v>
+        <v>209</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.2">
@@ -3614,7 +3554,7 @@
         <v>30</v>
       </c>
       <c r="E121" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.2">
@@ -3631,7 +3571,7 @@
         <v>30</v>
       </c>
       <c r="E122" t="s">
-        <v>241</v>
+        <v>211</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
@@ -3648,7 +3588,7 @@
         <v>30</v>
       </c>
       <c r="E123" t="s">
-        <v>242</v>
+        <v>212</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
@@ -3665,7 +3605,7 @@
         <v>30</v>
       </c>
       <c r="E124" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.2">
@@ -3682,7 +3622,7 @@
         <v>30</v>
       </c>
       <c r="E125" t="s">
-        <v>244</v>
+        <v>214</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.2">
@@ -3699,7 +3639,7 @@
         <v>31</v>
       </c>
       <c r="E126" t="s">
-        <v>245</v>
+        <v>215</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.2">
@@ -3716,7 +3656,7 @@
         <v>31</v>
       </c>
       <c r="E127" t="s">
-        <v>246</v>
+        <v>216</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.2">
@@ -3733,7 +3673,7 @@
         <v>31</v>
       </c>
       <c r="E128" t="s">
-        <v>247</v>
+        <v>217</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.2">
@@ -3750,7 +3690,7 @@
         <v>31</v>
       </c>
       <c r="E129" t="s">
-        <v>248</v>
+        <v>218</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.2">
@@ -3767,7 +3707,7 @@
         <v>31</v>
       </c>
       <c r="E130" t="s">
-        <v>249</v>
+        <v>219</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
@@ -3784,7 +3724,7 @@
         <v>31</v>
       </c>
       <c r="E131" t="s">
-        <v>250</v>
+        <v>220</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
@@ -3801,7 +3741,7 @@
         <v>31</v>
       </c>
       <c r="E132" t="s">
-        <v>251</v>
+        <v>221</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.2">
@@ -3818,7 +3758,7 @@
         <v>31</v>
       </c>
       <c r="E133" t="s">
-        <v>252</v>
+        <v>222</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.2">
@@ -3835,7 +3775,7 @@
         <v>31</v>
       </c>
       <c r="E134" t="s">
-        <v>253</v>
+        <v>223</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.2">
@@ -3852,7 +3792,7 @@
         <v>31</v>
       </c>
       <c r="E135" t="s">
-        <v>254</v>
+        <v>224</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.2">
@@ -3869,7 +3809,7 @@
         <v>31</v>
       </c>
       <c r="E136" t="s">
-        <v>255</v>
+        <v>225</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.2">
@@ -3886,7 +3826,7 @@
         <v>31</v>
       </c>
       <c r="E137" t="s">
-        <v>256</v>
+        <v>226</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.2">
@@ -3903,7 +3843,7 @@
         <v>31</v>
       </c>
       <c r="E138" t="s">
-        <v>257</v>
+        <v>227</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.2">
@@ -3920,7 +3860,7 @@
         <v>31</v>
       </c>
       <c r="E139" t="s">
-        <v>258</v>
+        <v>228</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.2">
@@ -3937,7 +3877,7 @@
         <v>31</v>
       </c>
       <c r="E140" t="s">
-        <v>284</v>
+        <v>254</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.2">
@@ -3954,7 +3894,7 @@
         <v>31</v>
       </c>
       <c r="E141" t="s">
-        <v>285</v>
+        <v>255</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.2">
@@ -3971,7 +3911,7 @@
         <v>31</v>
       </c>
       <c r="E142" t="s">
-        <v>293</v>
+        <v>263</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.2">
@@ -3988,7 +3928,7 @@
         <v>31</v>
       </c>
       <c r="E143" t="s">
-        <v>294</v>
+        <v>264</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.2">
@@ -4005,7 +3945,7 @@
         <v>31</v>
       </c>
       <c r="E144" t="s">
-        <v>286</v>
+        <v>256</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.2">
@@ -4022,7 +3962,7 @@
         <v>31</v>
       </c>
       <c r="E145" t="s">
-        <v>295</v>
+        <v>265</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.2">
@@ -4039,7 +3979,7 @@
         <v>31</v>
       </c>
       <c r="E146" t="s">
-        <v>296</v>
+        <v>266</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.2">
@@ -4056,7 +3996,7 @@
         <v>31</v>
       </c>
       <c r="E147" t="s">
-        <v>297</v>
+        <v>267</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.2">
@@ -4073,7 +4013,7 @@
         <v>31</v>
       </c>
       <c r="E148" t="s">
-        <v>298</v>
+        <v>268</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.2">
@@ -4090,7 +4030,7 @@
         <v>31</v>
       </c>
       <c r="E149" t="s">
-        <v>299</v>
+        <v>269</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.2">
@@ -4107,7 +4047,7 @@
         <v>31</v>
       </c>
       <c r="E150" t="s">
-        <v>300</v>
+        <v>270</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.2">
@@ -4124,7 +4064,7 @@
         <v>31</v>
       </c>
       <c r="E151" t="s">
-        <v>301</v>
+        <v>271</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.2">
@@ -4141,7 +4081,7 @@
         <v>31</v>
       </c>
       <c r="E152" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
@@ -4158,7 +4098,7 @@
         <v>31</v>
       </c>
       <c r="E153" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.2">
@@ -4175,7 +4115,7 @@
         <v>31</v>
       </c>
       <c r="E154" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.2">
@@ -4192,7 +4132,7 @@
         <v>31</v>
       </c>
       <c r="E155" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.2">
@@ -4209,7 +4149,7 @@
         <v>31</v>
       </c>
       <c r="E156" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.2">
@@ -4226,7 +4166,7 @@
         <v>31</v>
       </c>
       <c r="E157" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.2">
@@ -4243,7 +4183,7 @@
         <v>32</v>
       </c>
       <c r="E158" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.2">
@@ -4260,7 +4200,7 @@
         <v>32</v>
       </c>
       <c r="E159" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.2">
@@ -4277,7 +4217,7 @@
         <v>32</v>
       </c>
       <c r="E160" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.2">
@@ -4294,7 +4234,7 @@
         <v>32</v>
       </c>
       <c r="E161" t="s">
-        <v>190</v>
+        <v>160</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.2">
@@ -4311,7 +4251,7 @@
         <v>32</v>
       </c>
       <c r="E162" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.2">
@@ -4328,7 +4268,7 @@
         <v>32</v>
       </c>
       <c r="E163" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.2">
@@ -4345,7 +4285,7 @@
         <v>32</v>
       </c>
       <c r="E164" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.2">
@@ -4362,7 +4302,7 @@
         <v>32</v>
       </c>
       <c r="E165" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.2">
@@ -4379,7 +4319,7 @@
         <v>32</v>
       </c>
       <c r="E166" t="s">
-        <v>154</v>
+        <v>124</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.2">
@@ -4396,7 +4336,7 @@
         <v>32</v>
       </c>
       <c r="E167" t="s">
-        <v>155</v>
+        <v>125</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.2">
@@ -4413,7 +4353,7 @@
         <v>32</v>
       </c>
       <c r="E168" t="s">
-        <v>156</v>
+        <v>126</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.2">
@@ -4430,7 +4370,7 @@
         <v>32</v>
       </c>
       <c r="E169" t="s">
-        <v>157</v>
+        <v>127</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.2">
@@ -4447,7 +4387,7 @@
         <v>32</v>
       </c>
       <c r="E170" t="s">
-        <v>191</v>
+        <v>161</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.2">
@@ -4464,7 +4404,7 @@
         <v>32</v>
       </c>
       <c r="E171" t="s">
-        <v>192</v>
+        <v>162</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.2">
@@ -4481,7 +4421,7 @@
         <v>32</v>
       </c>
       <c r="E172" t="s">
-        <v>193</v>
+        <v>163</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.2">
@@ -4498,7 +4438,7 @@
         <v>32</v>
       </c>
       <c r="E173" t="s">
-        <v>194</v>
+        <v>164</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.2">
@@ -4515,7 +4455,7 @@
         <v>32</v>
       </c>
       <c r="E174" t="s">
-        <v>287</v>
+        <v>257</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.2">
@@ -4532,7 +4472,7 @@
         <v>32</v>
       </c>
       <c r="E175" t="s">
-        <v>302</v>
+        <v>272</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.2">
@@ -4549,7 +4489,7 @@
         <v>32</v>
       </c>
       <c r="E176" t="s">
-        <v>259</v>
+        <v>229</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.2">
@@ -4566,7 +4506,7 @@
         <v>32</v>
       </c>
       <c r="E177" t="s">
-        <v>260</v>
+        <v>230</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.2">
@@ -4583,7 +4523,7 @@
         <v>32</v>
       </c>
       <c r="E178" t="s">
-        <v>261</v>
+        <v>231</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.2">
@@ -4600,7 +4540,7 @@
         <v>32</v>
       </c>
       <c r="E179" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.2">
@@ -4617,7 +4557,7 @@
         <v>32</v>
       </c>
       <c r="E180" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.2">
@@ -4634,7 +4574,7 @@
         <v>32</v>
       </c>
       <c r="E181" t="s">
-        <v>264</v>
+        <v>234</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.2">
@@ -4651,7 +4591,7 @@
         <v>32</v>
       </c>
       <c r="E182" t="s">
-        <v>265</v>
+        <v>235</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.2">
@@ -4668,7 +4608,7 @@
         <v>32</v>
       </c>
       <c r="E183" t="s">
-        <v>266</v>
+        <v>236</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.2">
@@ -4685,7 +4625,7 @@
         <v>32</v>
       </c>
       <c r="E184" t="s">
-        <v>267</v>
+        <v>237</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.2">
@@ -4702,7 +4642,7 @@
         <v>32</v>
       </c>
       <c r="E185" t="s">
-        <v>268</v>
+        <v>238</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.2">
@@ -4719,7 +4659,7 @@
         <v>32</v>
       </c>
       <c r="E186" t="s">
-        <v>269</v>
+        <v>239</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.2">
@@ -4736,7 +4676,7 @@
         <v>32</v>
       </c>
       <c r="E187" t="s">
-        <v>270</v>
+        <v>240</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.2">
@@ -4753,7 +4693,7 @@
         <v>32</v>
       </c>
       <c r="E188" t="s">
-        <v>271</v>
+        <v>241</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.2">
@@ -4770,7 +4710,7 @@
         <v>32</v>
       </c>
       <c r="E189" t="s">
-        <v>272</v>
+        <v>242</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.2">
@@ -4787,7 +4727,7 @@
         <v>32</v>
       </c>
       <c r="E190" t="s">
-        <v>273</v>
+        <v>243</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.2">
@@ -4804,7 +4744,7 @@
         <v>32</v>
       </c>
       <c r="E191" t="s">
-        <v>274</v>
+        <v>244</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.2">
@@ -4821,7 +4761,7 @@
         <v>32</v>
       </c>
       <c r="E192" t="s">
-        <v>303</v>
+        <v>273</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.2">
@@ -4838,7 +4778,7 @@
         <v>32</v>
       </c>
       <c r="E193" t="s">
-        <v>304</v>
+        <v>274</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.2">
@@ -4855,7 +4795,7 @@
         <v>32</v>
       </c>
       <c r="E194" t="s">
-        <v>195</v>
+        <v>165</v>
       </c>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.2">
@@ -4872,7 +4812,7 @@
         <v>32</v>
       </c>
       <c r="E195" t="s">
-        <v>158</v>
+        <v>128</v>
       </c>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.2">
@@ -4889,7 +4829,7 @@
         <v>32</v>
       </c>
       <c r="E196" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.2">
@@ -4906,7 +4846,7 @@
         <v>32</v>
       </c>
       <c r="E197" t="s">
-        <v>196</v>
+        <v>166</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.2">
@@ -4923,7 +4863,7 @@
         <v>32</v>
       </c>
       <c r="E198" t="s">
-        <v>159</v>
+        <v>129</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.2">
@@ -4940,7 +4880,7 @@
         <v>32</v>
       </c>
       <c r="E199" t="s">
-        <v>197</v>
+        <v>167</v>
       </c>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.2">
@@ -4957,7 +4897,7 @@
         <v>32</v>
       </c>
       <c r="E200" t="s">
-        <v>198</v>
+        <v>168</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.2">
@@ -4974,7 +4914,7 @@
         <v>32</v>
       </c>
       <c r="E201" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.2">
@@ -4991,7 +4931,7 @@
         <v>32</v>
       </c>
       <c r="E202" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.2">
@@ -5008,7 +4948,7 @@
         <v>32</v>
       </c>
       <c r="E203" t="s">
-        <v>160</v>
+        <v>130</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.2">
@@ -5025,7 +4965,7 @@
         <v>32</v>
       </c>
       <c r="E204" t="s">
-        <v>161</v>
+        <v>131</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.2">
@@ -5042,7 +4982,7 @@
         <v>32</v>
       </c>
       <c r="E205" t="s">
-        <v>162</v>
+        <v>132</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.2">
@@ -5059,7 +4999,7 @@
         <v>32</v>
       </c>
       <c r="E206" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.2">
@@ -5076,7 +5016,7 @@
         <v>32</v>
       </c>
       <c r="E207" t="s">
-        <v>164</v>
+        <v>134</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.2">
@@ -5093,7 +5033,7 @@
         <v>32</v>
       </c>
       <c r="E208" t="s">
-        <v>165</v>
+        <v>135</v>
       </c>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.2">
@@ -5110,7 +5050,7 @@
         <v>32</v>
       </c>
       <c r="E209" t="s">
-        <v>166</v>
+        <v>136</v>
       </c>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.2">
@@ -5127,7 +5067,7 @@
         <v>32</v>
       </c>
       <c r="E210" t="s">
-        <v>167</v>
+        <v>137</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.2">
@@ -5144,7 +5084,7 @@
         <v>32</v>
       </c>
       <c r="E211" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.2">
@@ -5161,7 +5101,7 @@
         <v>32</v>
       </c>
       <c r="E212" t="s">
-        <v>288</v>
+        <v>258</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.2">
@@ -5178,7 +5118,7 @@
         <v>32</v>
       </c>
       <c r="E213" t="s">
-        <v>275</v>
+        <v>245</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.2">
@@ -5195,7 +5135,7 @@
         <v>32</v>
       </c>
       <c r="E214" t="s">
-        <v>276</v>
+        <v>246</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.2">
@@ -5212,7 +5152,7 @@
         <v>32</v>
       </c>
       <c r="E215" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.2">
@@ -5229,7 +5169,7 @@
         <v>32</v>
       </c>
       <c r="E216" t="s">
-        <v>170</v>
+        <v>140</v>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.2">
@@ -5246,7 +5186,7 @@
         <v>32</v>
       </c>
       <c r="E217" t="s">
-        <v>171</v>
+        <v>141</v>
       </c>
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.2">
@@ -5263,7 +5203,7 @@
         <v>32</v>
       </c>
       <c r="E218" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.2">
@@ -5280,7 +5220,7 @@
         <v>32</v>
       </c>
       <c r="E219" t="s">
-        <v>277</v>
+        <v>247</v>
       </c>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.2">
@@ -5297,7 +5237,7 @@
         <v>32</v>
       </c>
       <c r="E220" t="s">
-        <v>289</v>
+        <v>259</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.2">
@@ -5314,7 +5254,7 @@
         <v>32</v>
       </c>
       <c r="E221" t="s">
-        <v>290</v>
+        <v>260</v>
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.2">
@@ -5331,7 +5271,7 @@
         <v>32</v>
       </c>
       <c r="E222" t="s">
-        <v>291</v>
+        <v>261</v>
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.2">
@@ -5348,7 +5288,7 @@
         <v>32</v>
       </c>
       <c r="E223" t="s">
-        <v>278</v>
+        <v>248</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.2">
@@ -5365,7 +5305,7 @@
         <v>32</v>
       </c>
       <c r="E224" t="s">
-        <v>279</v>
+        <v>249</v>
       </c>
     </row>
     <row r="225" spans="1:6" x14ac:dyDescent="0.2">
@@ -5382,7 +5322,7 @@
         <v>32</v>
       </c>
       <c r="E225" t="s">
-        <v>280</v>
+        <v>250</v>
       </c>
     </row>
     <row r="226" spans="1:6" x14ac:dyDescent="0.2">
@@ -5399,7 +5339,7 @@
         <v>33</v>
       </c>
       <c r="E226" t="s">
-        <v>199</v>
+        <v>169</v>
       </c>
       <c r="F226" s="1"/>
     </row>
@@ -5417,7 +5357,7 @@
         <v>33</v>
       </c>
       <c r="E227" t="s">
-        <v>281</v>
+        <v>251</v>
       </c>
       <c r="F227" s="1"/>
     </row>
@@ -5435,7 +5375,7 @@
         <v>33</v>
       </c>
       <c r="E228" t="s">
-        <v>282</v>
+        <v>252</v>
       </c>
     </row>
     <row r="229" spans="1:6" x14ac:dyDescent="0.2">
@@ -5672,7 +5612,7 @@
         <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.2">
@@ -5689,7 +5629,7 @@
         <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>91</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.2">
@@ -5706,7 +5646,7 @@
         <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>173</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.2">
@@ -5723,7 +5663,7 @@
         <v>29</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
@@ -5740,7 +5680,7 @@
         <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>126</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
@@ -5757,7 +5697,7 @@
         <v>29</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
@@ -5774,7 +5714,7 @@
         <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>174</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
@@ -5791,7 +5731,7 @@
         <v>29</v>
       </c>
       <c r="E9" t="s">
-        <v>127</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
@@ -5808,7 +5748,7 @@
         <v>29</v>
       </c>
       <c r="E10" t="s">
-        <v>128</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
@@ -5825,7 +5765,7 @@
         <v>29</v>
       </c>
       <c r="E11" t="s">
-        <v>129</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
@@ -5842,7 +5782,7 @@
         <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>130</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
@@ -5859,7 +5799,7 @@
         <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>131</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
@@ -5876,7 +5816,7 @@
         <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>132</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
@@ -5893,7 +5833,7 @@
         <v>29</v>
       </c>
       <c r="E15" t="s">
-        <v>133</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
@@ -5910,7 +5850,7 @@
         <v>29</v>
       </c>
       <c r="E16" t="s">
-        <v>175</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
@@ -5927,7 +5867,7 @@
         <v>29</v>
       </c>
       <c r="E17" t="s">
-        <v>134</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
@@ -5944,7 +5884,7 @@
         <v>29</v>
       </c>
       <c r="E18" t="s">
-        <v>135</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
@@ -5961,7 +5901,7 @@
         <v>29</v>
       </c>
       <c r="E19" t="s">
-        <v>136</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
@@ -5978,7 +5918,7 @@
         <v>29</v>
       </c>
       <c r="E20" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
@@ -5995,7 +5935,7 @@
         <v>29</v>
       </c>
       <c r="E21" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
@@ -6012,7 +5952,7 @@
         <v>29</v>
       </c>
       <c r="E22" t="s">
-        <v>138</v>
+        <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
@@ -6029,7 +5969,7 @@
         <v>29</v>
       </c>
       <c r="E23" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
@@ -6046,7 +5986,7 @@
         <v>29</v>
       </c>
       <c r="E24" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
@@ -6063,7 +6003,7 @@
         <v>29</v>
       </c>
       <c r="E25" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
@@ -6080,7 +6020,7 @@
         <v>29</v>
       </c>
       <c r="E26" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
@@ -6097,7 +6037,7 @@
         <v>29</v>
       </c>
       <c r="E27" t="s">
-        <v>178</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
@@ -6114,7 +6054,7 @@
         <v>29</v>
       </c>
       <c r="E28" t="s">
-        <v>179</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
@@ -6131,7 +6071,7 @@
         <v>29</v>
       </c>
       <c r="E29" t="s">
-        <v>200</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
@@ -6148,7 +6088,7 @@
         <v>29</v>
       </c>
       <c r="E30" t="s">
-        <v>201</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
@@ -6165,7 +6105,7 @@
         <v>29</v>
       </c>
       <c r="E31" t="s">
-        <v>202</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
@@ -6182,7 +6122,7 @@
         <v>29</v>
       </c>
       <c r="E32" t="s">
-        <v>203</v>
+        <v>173</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
@@ -6199,7 +6139,7 @@
         <v>29</v>
       </c>
       <c r="E33" t="s">
-        <v>292</v>
+        <v>262</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
@@ -6216,7 +6156,7 @@
         <v>29</v>
       </c>
       <c r="E34" t="s">
-        <v>97</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
@@ -6233,7 +6173,7 @@
         <v>29</v>
       </c>
       <c r="E35" t="s">
-        <v>98</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
@@ -6250,7 +6190,7 @@
         <v>29</v>
       </c>
       <c r="E36" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
@@ -6267,7 +6207,7 @@
         <v>29</v>
       </c>
       <c r="E37" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
@@ -6284,7 +6224,7 @@
         <v>29</v>
       </c>
       <c r="E38" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
@@ -6301,7 +6241,7 @@
         <v>29</v>
       </c>
       <c r="E39" t="s">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
@@ -6318,7 +6258,7 @@
         <v>29</v>
       </c>
       <c r="E40" t="s">
-        <v>81</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
@@ -6335,7 +6275,7 @@
         <v>29</v>
       </c>
       <c r="E41" t="s">
-        <v>82</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
@@ -6352,7 +6292,7 @@
         <v>29</v>
       </c>
       <c r="E42" t="s">
-        <v>83</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
@@ -6369,7 +6309,7 @@
         <v>29</v>
       </c>
       <c r="E43" t="s">
-        <v>84</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
@@ -6386,7 +6326,7 @@
         <v>29</v>
       </c>
       <c r="E44" t="s">
-        <v>85</v>
+        <v>55</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.2">
@@ -6403,7 +6343,7 @@
         <v>29</v>
       </c>
       <c r="E45" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
@@ -6420,7 +6360,7 @@
         <v>29</v>
       </c>
       <c r="E46" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.2">
@@ -6437,7 +6377,7 @@
         <v>29</v>
       </c>
       <c r="E47" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
@@ -6454,7 +6394,7 @@
         <v>29</v>
       </c>
       <c r="E48" t="s">
-        <v>180</v>
+        <v>150</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.2">
@@ -6471,7 +6411,7 @@
         <v>29</v>
       </c>
       <c r="E49" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.2">
@@ -6488,7 +6428,7 @@
         <v>29</v>
       </c>
       <c r="E50" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.2">
@@ -6505,7 +6445,7 @@
         <v>29</v>
       </c>
       <c r="E51" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.2">
@@ -6522,7 +6462,7 @@
         <v>29</v>
       </c>
       <c r="E52" t="s">
-        <v>181</v>
+        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.2">
@@ -6539,7 +6479,7 @@
         <v>29</v>
       </c>
       <c r="E53" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.2">
@@ -6556,7 +6496,7 @@
         <v>29</v>
       </c>
       <c r="E54" t="s">
-        <v>103</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.2">
@@ -6573,7 +6513,7 @@
         <v>29</v>
       </c>
       <c r="E55" t="s">
-        <v>144</v>
+        <v>114</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.2">
@@ -6590,7 +6530,7 @@
         <v>29</v>
       </c>
       <c r="E56" t="s">
-        <v>182</v>
+        <v>152</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.2">
@@ -6607,7 +6547,7 @@
         <v>29</v>
       </c>
       <c r="E57" t="s">
-        <v>94</v>
+        <v>64</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.2">
@@ -6624,7 +6564,7 @@
         <v>29</v>
       </c>
       <c r="E58" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
@@ -6641,7 +6581,7 @@
         <v>29</v>
       </c>
       <c r="E59" t="s">
-        <v>145</v>
+        <v>115</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.2">
@@ -6658,7 +6598,7 @@
         <v>30</v>
       </c>
       <c r="E60" t="s">
-        <v>183</v>
+        <v>153</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
@@ -6675,7 +6615,7 @@
         <v>30</v>
       </c>
       <c r="E61" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.2">
@@ -6692,7 +6632,7 @@
         <v>30</v>
       </c>
       <c r="E62" t="s">
-        <v>105</v>
+        <v>75</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.2">
@@ -6709,7 +6649,7 @@
         <v>30</v>
       </c>
       <c r="E63" t="s">
-        <v>106</v>
+        <v>76</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.2">
@@ -6726,7 +6666,7 @@
         <v>30</v>
       </c>
       <c r="E64" t="s">
-        <v>107</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.2">
@@ -6743,7 +6683,7 @@
         <v>30</v>
       </c>
       <c r="E65" t="s">
-        <v>108</v>
+        <v>78</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.2">
@@ -6760,7 +6700,7 @@
         <v>30</v>
       </c>
       <c r="E66" t="s">
-        <v>109</v>
+        <v>79</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.2">
@@ -6777,7 +6717,7 @@
         <v>30</v>
       </c>
       <c r="E67" t="s">
-        <v>110</v>
+        <v>80</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.2">
@@ -6794,7 +6734,7 @@
         <v>30</v>
       </c>
       <c r="E68" t="s">
-        <v>111</v>
+        <v>81</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.2">
@@ -6811,7 +6751,7 @@
         <v>30</v>
       </c>
       <c r="E69" t="s">
-        <v>112</v>
+        <v>82</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.2">
@@ -6828,7 +6768,7 @@
         <v>30</v>
       </c>
       <c r="E70" t="s">
-        <v>113</v>
+        <v>83</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.2">
@@ -6845,7 +6785,7 @@
         <v>30</v>
       </c>
       <c r="E71" t="s">
-        <v>114</v>
+        <v>84</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
@@ -6862,7 +6802,7 @@
         <v>30</v>
       </c>
       <c r="E72" t="s">
-        <v>184</v>
+        <v>154</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.2">
@@ -6879,7 +6819,7 @@
         <v>30</v>
       </c>
       <c r="E73" t="s">
-        <v>146</v>
+        <v>116</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
@@ -6896,7 +6836,7 @@
         <v>30</v>
       </c>
       <c r="E74" t="s">
-        <v>185</v>
+        <v>155</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.2">
@@ -6913,7 +6853,7 @@
         <v>30</v>
       </c>
       <c r="E75" t="s">
-        <v>147</v>
+        <v>117</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.2">
@@ -6930,7 +6870,7 @@
         <v>30</v>
       </c>
       <c r="E76" t="s">
-        <v>148</v>
+        <v>118</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.2">
@@ -6947,7 +6887,7 @@
         <v>30</v>
       </c>
       <c r="E77" t="s">
-        <v>149</v>
+        <v>119</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2">
@@ -6964,7 +6904,7 @@
         <v>30</v>
       </c>
       <c r="E78" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.2">
@@ -6981,7 +6921,7 @@
         <v>30</v>
       </c>
       <c r="E79" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.2">
@@ -6998,7 +6938,7 @@
         <v>30</v>
       </c>
       <c r="E80" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
@@ -7015,7 +6955,7 @@
         <v>30</v>
       </c>
       <c r="E81" t="s">
-        <v>89</v>
+        <v>59</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
@@ -7032,7 +6972,7 @@
         <v>30</v>
       </c>
       <c r="E82" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
@@ -7049,7 +6989,7 @@
         <v>30</v>
       </c>
       <c r="E83" t="s">
-        <v>116</v>
+        <v>86</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
@@ -7066,7 +7006,7 @@
         <v>30</v>
       </c>
       <c r="E84" t="s">
-        <v>283</v>
+        <v>253</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
@@ -7083,7 +7023,7 @@
         <v>30</v>
       </c>
       <c r="E85" t="s">
-        <v>204</v>
+        <v>174</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
@@ -7100,7 +7040,7 @@
         <v>30</v>
       </c>
       <c r="E86" t="s">
-        <v>205</v>
+        <v>175</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
@@ -7117,7 +7057,7 @@
         <v>30</v>
       </c>
       <c r="E87" t="s">
-        <v>206</v>
+        <v>176</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
@@ -7134,7 +7074,7 @@
         <v>30</v>
       </c>
       <c r="E88" t="s">
-        <v>207</v>
+        <v>177</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
@@ -7151,7 +7091,7 @@
         <v>30</v>
       </c>
       <c r="E89" t="s">
-        <v>208</v>
+        <v>178</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
@@ -7168,7 +7108,7 @@
         <v>30</v>
       </c>
       <c r="E90" t="s">
-        <v>209</v>
+        <v>179</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
@@ -7185,7 +7125,7 @@
         <v>30</v>
       </c>
       <c r="E91" t="s">
-        <v>210</v>
+        <v>180</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
@@ -7202,7 +7142,7 @@
         <v>30</v>
       </c>
       <c r="E92" t="s">
-        <v>211</v>
+        <v>181</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
@@ -7219,7 +7159,7 @@
         <v>30</v>
       </c>
       <c r="E93" t="s">
-        <v>212</v>
+        <v>182</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
@@ -7236,7 +7176,7 @@
         <v>30</v>
       </c>
       <c r="E94" t="s">
-        <v>213</v>
+        <v>183</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
@@ -7253,7 +7193,7 @@
         <v>30</v>
       </c>
       <c r="E95" t="s">
-        <v>214</v>
+        <v>184</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
@@ -7270,7 +7210,7 @@
         <v>30</v>
       </c>
       <c r="E96" t="s">
-        <v>215</v>
+        <v>185</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
@@ -7287,7 +7227,7 @@
         <v>30</v>
       </c>
       <c r="E97" t="s">
-        <v>216</v>
+        <v>186</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
@@ -7304,7 +7244,7 @@
         <v>30</v>
       </c>
       <c r="E98" t="s">
-        <v>217</v>
+        <v>187</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
@@ -7321,7 +7261,7 @@
         <v>30</v>
       </c>
       <c r="E99" t="s">
-        <v>218</v>
+        <v>188</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
@@ -7338,7 +7278,7 @@
         <v>30</v>
       </c>
       <c r="E100" t="s">
-        <v>219</v>
+        <v>189</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.2">
@@ -7355,7 +7295,7 @@
         <v>30</v>
       </c>
       <c r="E101" t="s">
-        <v>220</v>
+        <v>190</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
@@ -7372,7 +7312,7 @@
         <v>30</v>
       </c>
       <c r="E102" t="s">
-        <v>221</v>
+        <v>191</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
@@ -7389,7 +7329,7 @@
         <v>30</v>
       </c>
       <c r="E103" t="s">
-        <v>222</v>
+        <v>192</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
@@ -7406,7 +7346,7 @@
         <v>30</v>
       </c>
       <c r="E104" t="s">
-        <v>223</v>
+        <v>193</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
@@ -7423,7 +7363,7 @@
         <v>30</v>
       </c>
       <c r="E105" t="s">
-        <v>224</v>
+        <v>194</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
@@ -7440,7 +7380,7 @@
         <v>30</v>
       </c>
       <c r="E106" t="s">
-        <v>225</v>
+        <v>195</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
@@ -7457,7 +7397,7 @@
         <v>30</v>
       </c>
       <c r="E107" t="s">
-        <v>226</v>
+        <v>196</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
@@ -7474,7 +7414,7 @@
         <v>30</v>
       </c>
       <c r="E108" t="s">
-        <v>227</v>
+        <v>197</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
@@ -7491,7 +7431,7 @@
         <v>30</v>
       </c>
       <c r="E109" t="s">
-        <v>228</v>
+        <v>198</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
@@ -7508,7 +7448,7 @@
         <v>30</v>
       </c>
       <c r="E110" t="s">
-        <v>229</v>
+        <v>199</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
@@ -7525,7 +7465,7 @@
         <v>30</v>
       </c>
       <c r="E111" t="s">
-        <v>230</v>
+        <v>200</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.2">
@@ -7542,7 +7482,7 @@
         <v>30</v>
       </c>
       <c r="E112" t="s">
-        <v>231</v>
+        <v>201</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.2">
@@ -7559,7 +7499,7 @@
         <v>30</v>
       </c>
       <c r="E113" t="s">
-        <v>232</v>
+        <v>202</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.2">
@@ -7576,7 +7516,7 @@
         <v>30</v>
       </c>
       <c r="E114" t="s">
-        <v>233</v>
+        <v>203</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.2">
@@ -7593,7 +7533,7 @@
         <v>30</v>
       </c>
       <c r="E115" t="s">
-        <v>234</v>
+        <v>204</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.2">
@@ -7610,7 +7550,7 @@
         <v>30</v>
       </c>
       <c r="E116" t="s">
-        <v>235</v>
+        <v>205</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.2">
@@ -7627,7 +7567,7 @@
         <v>30</v>
       </c>
       <c r="E117" t="s">
-        <v>236</v>
+        <v>206</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.2">
@@ -7644,7 +7584,7 @@
         <v>30</v>
       </c>
       <c r="E118" t="s">
-        <v>237</v>
+        <v>207</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.2">
@@ -7661,7 +7601,7 @@
         <v>30</v>
       </c>
       <c r="E119" t="s">
-        <v>238</v>
+        <v>208</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
@@ -7678,7 +7618,7 @@
         <v>30</v>
       </c>
       <c r="E120" t="s">
-        <v>239</v>
+        <v>209</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.2">
@@ -7695,7 +7635,7 @@
         <v>30</v>
       </c>
       <c r="E121" t="s">
-        <v>240</v>
+        <v>210</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.2">
@@ -7712,7 +7652,7 @@
         <v>30</v>
       </c>
       <c r="E122" t="s">
-        <v>241</v>
+        <v>211</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.2">
@@ -7729,7 +7669,7 @@
         <v>30</v>
       </c>
       <c r="E123" t="s">
-        <v>242</v>
+        <v>212</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.2">
@@ -7746,7 +7686,7 @@
         <v>30</v>
       </c>
       <c r="E124" t="s">
-        <v>243</v>
+        <v>213</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.2">
@@ -7763,7 +7703,7 @@
         <v>30</v>
       </c>
       <c r="E125" t="s">
-        <v>244</v>
+        <v>214</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.2">
@@ -7780,7 +7720,7 @@
         <v>31</v>
       </c>
       <c r="E126" t="s">
-        <v>245</v>
+        <v>215</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.2">
@@ -7797,7 +7737,7 @@
         <v>31</v>
       </c>
       <c r="E127" t="s">
-        <v>246</v>
+        <v>216</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.2">
@@ -7814,7 +7754,7 @@
         <v>31</v>
       </c>
       <c r="E128" t="s">
-        <v>247</v>
+        <v>217</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.2">
@@ -7831,7 +7771,7 @@
         <v>31</v>
       </c>
       <c r="E129" t="s">
-        <v>248</v>
+        <v>218</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.2">
@@ -7848,7 +7788,7 @@
         <v>31</v>
       </c>
       <c r="E130" t="s">
-        <v>249</v>
+        <v>219</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
@@ -7865,7 +7805,7 @@
         <v>31</v>
       </c>
       <c r="E131" t="s">
-        <v>250</v>
+        <v>220</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
@@ -7882,7 +7822,7 @@
         <v>31</v>
       </c>
       <c r="E132" t="s">
-        <v>251</v>
+        <v>221</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.2">
@@ -7899,7 +7839,7 @@
         <v>31</v>
       </c>
       <c r="E133" t="s">
-        <v>252</v>
+        <v>222</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.2">
@@ -7916,7 +7856,7 @@
         <v>31</v>
       </c>
       <c r="E134" t="s">
-        <v>253</v>
+        <v>223</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.2">
@@ -7933,7 +7873,7 @@
         <v>31</v>
       </c>
       <c r="E135" t="s">
-        <v>254</v>
+        <v>224</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.2">
@@ -7950,7 +7890,7 @@
         <v>31</v>
       </c>
       <c r="E136" t="s">
-        <v>255</v>
+        <v>225</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.2">
@@ -7967,7 +7907,7 @@
         <v>31</v>
       </c>
       <c r="E137" t="s">
-        <v>256</v>
+        <v>226</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.2">
@@ -7984,7 +7924,7 @@
         <v>31</v>
       </c>
       <c r="E138" t="s">
-        <v>257</v>
+        <v>227</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.2">
@@ -8001,7 +7941,7 @@
         <v>31</v>
       </c>
       <c r="E139" t="s">
-        <v>258</v>
+        <v>228</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.2">
@@ -8018,7 +7958,7 @@
         <v>31</v>
       </c>
       <c r="E140" t="s">
-        <v>284</v>
+        <v>254</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.2">
@@ -8035,7 +7975,7 @@
         <v>31</v>
       </c>
       <c r="E141" t="s">
-        <v>285</v>
+        <v>255</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.2">
@@ -8052,7 +7992,7 @@
         <v>31</v>
       </c>
       <c r="E142" t="s">
-        <v>293</v>
+        <v>263</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.2">
@@ -8069,7 +8009,7 @@
         <v>31</v>
       </c>
       <c r="E143" t="s">
-        <v>294</v>
+        <v>264</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.2">
@@ -8086,7 +8026,7 @@
         <v>31</v>
       </c>
       <c r="E144" t="s">
-        <v>286</v>
+        <v>256</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.2">
@@ -8103,7 +8043,7 @@
         <v>31</v>
       </c>
       <c r="E145" t="s">
-        <v>295</v>
+        <v>265</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.2">
@@ -8120,7 +8060,7 @@
         <v>31</v>
       </c>
       <c r="E146" t="s">
-        <v>296</v>
+        <v>266</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.2">
@@ -8137,7 +8077,7 @@
         <v>31</v>
       </c>
       <c r="E147" t="s">
-        <v>297</v>
+        <v>267</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.2">
@@ -8154,7 +8094,7 @@
         <v>31</v>
       </c>
       <c r="E148" t="s">
-        <v>298</v>
+        <v>268</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.2">
@@ -8171,7 +8111,7 @@
         <v>31</v>
       </c>
       <c r="E149" t="s">
-        <v>299</v>
+        <v>269</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.2">
@@ -8188,7 +8128,7 @@
         <v>31</v>
       </c>
       <c r="E150" t="s">
-        <v>300</v>
+        <v>270</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.2">
@@ -8205,7 +8145,7 @@
         <v>31</v>
       </c>
       <c r="E151" t="s">
-        <v>301</v>
+        <v>271</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.2">
@@ -8222,7 +8162,7 @@
         <v>31</v>
       </c>
       <c r="E152" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
@@ -8239,7 +8179,7 @@
         <v>31</v>
       </c>
       <c r="E153" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.2">
@@ -8256,7 +8196,7 @@
         <v>31</v>
       </c>
       <c r="E154" t="s">
-        <v>119</v>
+        <v>89</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.2">
@@ -8273,7 +8213,7 @@
         <v>31</v>
       </c>
       <c r="E155" t="s">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.2">
@@ -8290,7 +8230,7 @@
         <v>31</v>
       </c>
       <c r="E156" t="s">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.2">
@@ -8307,7 +8247,7 @@
         <v>31</v>
       </c>
       <c r="E157" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.2">
@@ -8324,7 +8264,7 @@
         <v>32</v>
       </c>
       <c r="E158" t="s">
-        <v>187</v>
+        <v>157</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.2">
@@ -8341,7 +8281,7 @@
         <v>32</v>
       </c>
       <c r="E159" t="s">
-        <v>188</v>
+        <v>158</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.2">
@@ -8358,7 +8298,7 @@
         <v>32</v>
       </c>
       <c r="E160" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.2">
@@ -8375,7 +8315,7 @@
         <v>32</v>
       </c>
       <c r="E161" t="s">
-        <v>190</v>
+        <v>160</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.2">
@@ -8392,7 +8332,7 @@
         <v>32</v>
       </c>
       <c r="E162" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.2">
@@ -8409,7 +8349,7 @@
         <v>32</v>
       </c>
       <c r="E163" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.2">
@@ -8426,7 +8366,7 @@
         <v>32</v>
       </c>
       <c r="E164" t="s">
-        <v>152</v>
+        <v>122</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.2">
@@ -8443,7 +8383,7 @@
         <v>32</v>
       </c>
       <c r="E165" t="s">
-        <v>153</v>
+        <v>123</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.2">
@@ -8460,7 +8400,7 @@
         <v>32</v>
       </c>
       <c r="E166" t="s">
-        <v>154</v>
+        <v>124</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.2">
@@ -8477,7 +8417,7 @@
         <v>32</v>
       </c>
       <c r="E167" t="s">
-        <v>155</v>
+        <v>125</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.2">
@@ -8494,7 +8434,7 @@
         <v>32</v>
       </c>
       <c r="E168" t="s">
-        <v>156</v>
+        <v>126</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.2">
@@ -8511,7 +8451,7 @@
         <v>32</v>
       </c>
       <c r="E169" t="s">
-        <v>157</v>
+        <v>127</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.2">
@@ -8528,7 +8468,7 @@
         <v>32</v>
       </c>
       <c r="E170" t="s">
-        <v>191</v>
+        <v>161</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.2">
@@ -8545,7 +8485,7 @@
         <v>32</v>
       </c>
       <c r="E171" t="s">
-        <v>192</v>
+        <v>162</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.2">
@@ -8562,7 +8502,7 @@
         <v>32</v>
       </c>
       <c r="E172" t="s">
-        <v>193</v>
+        <v>163</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.2">
@@ -8579,7 +8519,7 @@
         <v>32</v>
       </c>
       <c r="E173" t="s">
-        <v>194</v>
+        <v>164</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.2">
@@ -8596,7 +8536,7 @@
         <v>32</v>
       </c>
       <c r="E174" t="s">
-        <v>287</v>
+        <v>257</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.2">
@@ -8613,7 +8553,7 @@
         <v>32</v>
       </c>
       <c r="E175" t="s">
-        <v>302</v>
+        <v>272</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.2">
@@ -8630,7 +8570,7 @@
         <v>32</v>
       </c>
       <c r="E176" t="s">
-        <v>259</v>
+        <v>229</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.2">
@@ -8647,7 +8587,7 @@
         <v>32</v>
       </c>
       <c r="E177" t="s">
-        <v>260</v>
+        <v>230</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.2">
@@ -8664,7 +8604,7 @@
         <v>32</v>
       </c>
       <c r="E178" t="s">
-        <v>261</v>
+        <v>231</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.2">
@@ -8681,7 +8621,7 @@
         <v>32</v>
       </c>
       <c r="E179" t="s">
-        <v>262</v>
+        <v>232</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.2">
@@ -8698,7 +8638,7 @@
         <v>32</v>
       </c>
       <c r="E180" t="s">
-        <v>263</v>
+        <v>233</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.2">
@@ -8715,7 +8655,7 @@
         <v>32</v>
       </c>
       <c r="E181" t="s">
-        <v>264</v>
+        <v>234</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.2">
@@ -8732,7 +8672,7 @@
         <v>32</v>
       </c>
       <c r="E182" t="s">
-        <v>265</v>
+        <v>235</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.2">
@@ -8749,7 +8689,7 @@
         <v>32</v>
       </c>
       <c r="E183" t="s">
-        <v>266</v>
+        <v>236</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.2">
@@ -8766,7 +8706,7 @@
         <v>32</v>
       </c>
       <c r="E184" t="s">
-        <v>267</v>
+        <v>237</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.2">
@@ -8783,7 +8723,7 @@
         <v>32</v>
       </c>
       <c r="E185" t="s">
-        <v>268</v>
+        <v>238</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.2">
@@ -8800,7 +8740,7 @@
         <v>32</v>
       </c>
       <c r="E186" t="s">
-        <v>269</v>
+        <v>239</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.2">
@@ -8817,7 +8757,7 @@
         <v>32</v>
       </c>
       <c r="E187" t="s">
-        <v>270</v>
+        <v>240</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.2">
@@ -8834,7 +8774,7 @@
         <v>32</v>
       </c>
       <c r="E188" t="s">
-        <v>271</v>
+        <v>241</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.2">
@@ -8851,7 +8791,7 @@
         <v>32</v>
       </c>
       <c r="E189" t="s">
-        <v>272</v>
+        <v>242</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.2">
@@ -8868,7 +8808,7 @@
         <v>32</v>
       </c>
       <c r="E190" t="s">
-        <v>273</v>
+        <v>243</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.2">
@@ -8885,7 +8825,7 @@
         <v>32</v>
       </c>
       <c r="E191" t="s">
-        <v>274</v>
+        <v>244</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.2">
@@ -8902,7 +8842,7 @@
         <v>32</v>
       </c>
       <c r="E192" t="s">
-        <v>303</v>
+        <v>273</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.2">
@@ -8919,7 +8859,7 @@
         <v>32</v>
       </c>
       <c r="E193" t="s">
-        <v>304</v>
+        <v>274</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.2">
@@ -8936,7 +8876,7 @@
         <v>32</v>
       </c>
       <c r="E194" t="s">
-        <v>195</v>
+        <v>165</v>
       </c>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.2">
@@ -8953,7 +8893,7 @@
         <v>32</v>
       </c>
       <c r="E195" t="s">
-        <v>158</v>
+        <v>128</v>
       </c>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.2">
@@ -8970,7 +8910,7 @@
         <v>32</v>
       </c>
       <c r="E196" t="s">
-        <v>123</v>
+        <v>93</v>
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.2">
@@ -8987,7 +8927,7 @@
         <v>32</v>
       </c>
       <c r="E197" t="s">
-        <v>196</v>
+        <v>166</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.2">
@@ -9004,7 +8944,7 @@
         <v>32</v>
       </c>
       <c r="E198" t="s">
-        <v>159</v>
+        <v>129</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.2">
@@ -9021,7 +8961,7 @@
         <v>32</v>
       </c>
       <c r="E199" t="s">
-        <v>197</v>
+        <v>167</v>
       </c>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.2">
@@ -9038,7 +8978,7 @@
         <v>32</v>
       </c>
       <c r="E200" t="s">
-        <v>198</v>
+        <v>168</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.2">
@@ -9055,7 +8995,7 @@
         <v>32</v>
       </c>
       <c r="E201" t="s">
-        <v>124</v>
+        <v>94</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.2">
@@ -9072,7 +9012,7 @@
         <v>32</v>
       </c>
       <c r="E202" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.2">
@@ -9089,7 +9029,7 @@
         <v>32</v>
       </c>
       <c r="E203" t="s">
-        <v>160</v>
+        <v>130</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.2">
@@ -9106,7 +9046,7 @@
         <v>32</v>
       </c>
       <c r="E204" t="s">
-        <v>161</v>
+        <v>131</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.2">
@@ -9123,7 +9063,7 @@
         <v>32</v>
       </c>
       <c r="E205" t="s">
-        <v>162</v>
+        <v>132</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.2">
@@ -9140,7 +9080,7 @@
         <v>32</v>
       </c>
       <c r="E206" t="s">
-        <v>163</v>
+        <v>133</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.2">
@@ -9157,7 +9097,7 @@
         <v>32</v>
       </c>
       <c r="E207" t="s">
-        <v>164</v>
+        <v>134</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.2">
@@ -9174,7 +9114,7 @@
         <v>32</v>
       </c>
       <c r="E208" t="s">
-        <v>165</v>
+        <v>135</v>
       </c>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.2">
@@ -9191,7 +9131,7 @@
         <v>32</v>
       </c>
       <c r="E209" t="s">
-        <v>166</v>
+        <v>136</v>
       </c>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.2">
@@ -9208,7 +9148,7 @@
         <v>32</v>
       </c>
       <c r="E210" t="s">
-        <v>167</v>
+        <v>137</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.2">
@@ -9225,7 +9165,7 @@
         <v>32</v>
       </c>
       <c r="E211" t="s">
-        <v>168</v>
+        <v>138</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.2">
@@ -9242,7 +9182,7 @@
         <v>32</v>
       </c>
       <c r="E212" t="s">
-        <v>288</v>
+        <v>258</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.2">
@@ -9259,7 +9199,7 @@
         <v>32</v>
       </c>
       <c r="E213" t="s">
-        <v>275</v>
+        <v>245</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.2">
@@ -9276,7 +9216,7 @@
         <v>32</v>
       </c>
       <c r="E214" t="s">
-        <v>276</v>
+        <v>246</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.2">
@@ -9293,7 +9233,7 @@
         <v>32</v>
       </c>
       <c r="E215" t="s">
-        <v>169</v>
+        <v>139</v>
       </c>
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.2">
@@ -9310,7 +9250,7 @@
         <v>32</v>
       </c>
       <c r="E216" t="s">
-        <v>170</v>
+        <v>140</v>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.2">
@@ -9327,7 +9267,7 @@
         <v>32</v>
       </c>
       <c r="E217" t="s">
-        <v>171</v>
+        <v>141</v>
       </c>
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.2">
@@ -9344,7 +9284,7 @@
         <v>32</v>
       </c>
       <c r="E218" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.2">
@@ -9361,7 +9301,7 @@
         <v>32</v>
       </c>
       <c r="E219" t="s">
-        <v>277</v>
+        <v>247</v>
       </c>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.2">
@@ -9378,7 +9318,7 @@
         <v>32</v>
       </c>
       <c r="E220" t="s">
-        <v>289</v>
+        <v>259</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.2">
@@ -9395,7 +9335,7 @@
         <v>32</v>
       </c>
       <c r="E221" t="s">
-        <v>290</v>
+        <v>260</v>
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.2">
@@ -9412,7 +9352,7 @@
         <v>32</v>
       </c>
       <c r="E222" t="s">
-        <v>291</v>
+        <v>261</v>
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.2">
@@ -9429,7 +9369,7 @@
         <v>32</v>
       </c>
       <c r="E223" t="s">
-        <v>278</v>
+        <v>248</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.2">
@@ -9446,7 +9386,7 @@
         <v>32</v>
       </c>
       <c r="E224" t="s">
-        <v>279</v>
+        <v>249</v>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.2">
@@ -9463,7 +9403,7 @@
         <v>32</v>
       </c>
       <c r="E225" t="s">
-        <v>280</v>
+        <v>250</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.2">
@@ -9480,7 +9420,7 @@
         <v>33</v>
       </c>
       <c r="E226" t="s">
-        <v>199</v>
+        <v>169</v>
       </c>
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.2">
@@ -9497,7 +9437,7 @@
         <v>33</v>
       </c>
       <c r="E227" t="s">
-        <v>281</v>
+        <v>251</v>
       </c>
     </row>
     <row r="228" spans="1:5" x14ac:dyDescent="0.2">
@@ -9514,7 +9454,7 @@
         <v>33</v>
       </c>
       <c r="E228" t="s">
-        <v>282</v>
+        <v>252</v>
       </c>
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.2">
@@ -9655,513 +9595,6 @@
       </c>
       <c r="D238" t="s">
         <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="4.83203125" style="8" customWidth="1"/>
-    <col min="2" max="2" width="12" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="8">
-        <v>35100.520833333336</v>
-      </c>
-      <c r="B2" s="6">
-        <v>35100.520833333336</v>
-      </c>
-      <c r="C2" s="3">
-        <v>35100.520833333336</v>
-      </c>
-      <c r="D2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="8">
-        <v>35103.375</v>
-      </c>
-      <c r="B3" s="6">
-        <v>35103.375</v>
-      </c>
-      <c r="C3" s="3">
-        <v>35103.375</v>
-      </c>
-      <c r="D3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="8">
-        <v>35115.541666666664</v>
-      </c>
-      <c r="B4" s="6">
-        <v>35115.541666666664</v>
-      </c>
-      <c r="C4" s="3">
-        <v>35115.541666666664</v>
-      </c>
-      <c r="D4" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="8">
-        <v>35118.319444444445</v>
-      </c>
-      <c r="B5" s="6">
-        <v>35118.319444444445</v>
-      </c>
-      <c r="C5" s="3">
-        <v>35118.319444444445</v>
-      </c>
-      <c r="D5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="8">
-        <v>35129.4375</v>
-      </c>
-      <c r="B6" s="6">
-        <v>35129.4375</v>
-      </c>
-      <c r="C6" s="3">
-        <v>35129.4375</v>
-      </c>
-      <c r="D6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="8">
-        <v>35143.375</v>
-      </c>
-      <c r="B7" s="6">
-        <v>35143.375</v>
-      </c>
-      <c r="C7" s="3">
-        <v>35143.375</v>
-      </c>
-      <c r="D7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="8">
-        <v>35151.375</v>
-      </c>
-      <c r="B8" s="6">
-        <v>35151.375</v>
-      </c>
-      <c r="C8" s="3">
-        <v>35151.375</v>
-      </c>
-      <c r="D8" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="8">
-        <v>35187.350694444445</v>
-      </c>
-      <c r="B9" s="6">
-        <v>35187.350694444445</v>
-      </c>
-      <c r="C9" s="3">
-        <v>35187.350694444445</v>
-      </c>
-      <c r="D9" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="8">
-        <v>35192.541666666664</v>
-      </c>
-      <c r="B10" s="6">
-        <v>35192.541666666664</v>
-      </c>
-      <c r="C10" s="3">
-        <v>35192.541666666664</v>
-      </c>
-      <c r="D10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="8">
-        <v>35222.479166666664</v>
-      </c>
-      <c r="B11" s="6">
-        <v>35222.479166666664</v>
-      </c>
-      <c r="C11" s="3">
-        <v>35222.479166666664</v>
-      </c>
-      <c r="D11" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="8">
-        <v>35229.479166666664</v>
-      </c>
-      <c r="B12" s="6">
-        <v>35229.479166666664</v>
-      </c>
-      <c r="C12" s="3">
-        <v>35229.479166666664</v>
-      </c>
-      <c r="D12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="8">
-        <v>35264.375</v>
-      </c>
-      <c r="B13" s="6">
-        <v>35264.375</v>
-      </c>
-      <c r="C13" s="3">
-        <v>35264.375</v>
-      </c>
-      <c r="D13" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="8">
-        <v>35272.34375</v>
-      </c>
-      <c r="B14" s="6">
-        <v>35272.34375</v>
-      </c>
-      <c r="C14" s="3">
-        <v>35272.34375</v>
-      </c>
-      <c r="D14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E14" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="8">
-        <v>35345.322916666664</v>
-      </c>
-      <c r="B15" s="6">
-        <v>35345.322916666664</v>
-      </c>
-      <c r="C15" s="3">
-        <v>35345.322916666664</v>
-      </c>
-      <c r="D15" t="s">
-        <v>29</v>
-      </c>
-      <c r="E15" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="8">
-        <v>35405.510416666664</v>
-      </c>
-      <c r="B16" s="6">
-        <v>35405.510416666664</v>
-      </c>
-      <c r="C16" s="3">
-        <v>35405.510416666664</v>
-      </c>
-      <c r="D16" t="s">
-        <v>29</v>
-      </c>
-      <c r="E16" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="8">
-        <v>35451.375</v>
-      </c>
-      <c r="B17" s="6">
-        <v>35451.375</v>
-      </c>
-      <c r="C17" s="3">
-        <v>35451.375</v>
-      </c>
-      <c r="D17" t="s">
-        <v>29</v>
-      </c>
-      <c r="E17" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="8">
-        <v>35460.385416666664</v>
-      </c>
-      <c r="B18" s="6">
-        <v>35460.385416666664</v>
-      </c>
-      <c r="C18" s="3">
-        <v>35460.385416666664</v>
-      </c>
-      <c r="D18" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="8">
-        <v>35474.375</v>
-      </c>
-      <c r="B19" s="6">
-        <v>35474.375</v>
-      </c>
-      <c r="C19" s="3">
-        <v>35474.375</v>
-      </c>
-      <c r="D19" t="s">
-        <v>29</v>
-      </c>
-      <c r="E19" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="8">
-        <v>35482.319444444445</v>
-      </c>
-      <c r="B20" s="6">
-        <v>35482.319444444445</v>
-      </c>
-      <c r="C20" s="3">
-        <v>35482.319444444445</v>
-      </c>
-      <c r="D20" t="s">
-        <v>29</v>
-      </c>
-      <c r="E20" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="8">
-        <v>35487.375</v>
-      </c>
-      <c r="B21" s="6">
-        <v>35487.375</v>
-      </c>
-      <c r="C21" s="3">
-        <v>35487.375</v>
-      </c>
-      <c r="D21" t="s">
-        <v>29</v>
-      </c>
-      <c r="E21" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="8">
-        <v>35493.375</v>
-      </c>
-      <c r="B22" s="6">
-        <v>35493.375</v>
-      </c>
-      <c r="C22" s="3">
-        <v>35493.375</v>
-      </c>
-      <c r="D22" t="s">
-        <v>29</v>
-      </c>
-      <c r="E22" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="8">
-        <v>35508.375</v>
-      </c>
-      <c r="B23" s="6">
-        <v>35508.375</v>
-      </c>
-      <c r="C23" s="3">
-        <v>35508.375</v>
-      </c>
-      <c r="D23" t="s">
-        <v>29</v>
-      </c>
-      <c r="E23" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="8">
-        <v>35509.375</v>
-      </c>
-      <c r="B24" s="6">
-        <v>35509.375</v>
-      </c>
-      <c r="C24" s="3">
-        <v>35509.375</v>
-      </c>
-      <c r="D24" t="s">
-        <v>29</v>
-      </c>
-      <c r="E24" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="8">
-        <v>35549.520833333336</v>
-      </c>
-      <c r="B25" s="6">
-        <v>35549.520833333336</v>
-      </c>
-      <c r="C25" s="3">
-        <v>35549.520833333336</v>
-      </c>
-      <c r="D25" t="s">
-        <v>29</v>
-      </c>
-      <c r="E25" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="8">
-        <v>35551.350694444445</v>
-      </c>
-      <c r="B26" s="6">
-        <v>35551.350694444445</v>
-      </c>
-      <c r="C26" s="3">
-        <v>35551.350694444445</v>
-      </c>
-      <c r="D26" t="s">
-        <v>29</v>
-      </c>
-      <c r="E26" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="8">
-        <v>35572.375</v>
-      </c>
-      <c r="B27" s="6">
-        <v>35572.375</v>
-      </c>
-      <c r="C27" s="3">
-        <v>35572.375</v>
-      </c>
-      <c r="D27" t="s">
-        <v>29</v>
-      </c>
-      <c r="E27" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="8">
-        <v>35628.375</v>
-      </c>
-      <c r="B28" s="6">
-        <v>35628.375</v>
-      </c>
-      <c r="C28" s="3">
-        <v>35628.375</v>
-      </c>
-      <c r="D28" t="s">
-        <v>29</v>
-      </c>
-      <c r="E28" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="8">
-        <v>35633.458333333336</v>
-      </c>
-      <c r="B29" s="6">
-        <v>35633.458333333336</v>
-      </c>
-      <c r="C29" s="3">
-        <v>35633.458333333336</v>
-      </c>
-      <c r="D29" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Folded in October 2026 FOMC statement
</commit_message>
<xml_diff>
--- a/fomcCommunication_master.xlsx
+++ b/fomcCommunication_master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11023"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranlephu/Documents/github/fomc-communication/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0BCF0BF-5CC4-A641-85C0-1CCE6608D5D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E96684F-2950-2F4B-ADA6-9FECF99D4573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="279">
   <si>
     <t>Explanation:</t>
   </si>
@@ -880,6 +880,9 @@
     <t>Repetitive and technical terms are replaced with corresponding single abbreviations that themselves have been used by the Federal Reserve System
 at least one time in their released statements. The last substitution is specific to FOMC statements and is to prevent look-ahead bias from neural
 networks for text analysis. The following terms and abbreviations are as follows:</t>
+  </si>
+  <si>
+    <t>The Committee (FOMC) approved the following statement for release by a 10 - 2 vote: The Committee decided to maintain the target range for the FFR at 3.75 to 4 percent, in support of the FR's dual mandate. The Committee is continuing its policy of maintaining ample reserves in the banking system. Economic activity is expanding at a strong pace. While uncertainty remains elevated owing, in part, to geopolitical developments, domestic spending has been resilient. Productivity growth is strong, and capital investment is robust. Job gains have kept pace with the workforce, and the unemployment rate has changed little. Inflation remains elevated. The accumulation of more information will help the Committee determine the policy stance appropriate to ensure a timely return of inflation to the Committee's 2 percent goal. The Committee will deliver price stability. Voting against the monetary policy action were Lisa D. Cook and Beth M. Hammack, who preferred to raise the target range for the FFR by 0.25 percentage point at this meeting.</t>
   </si>
 </sst>
 </file>
@@ -9470,6 +9473,9 @@
       <c r="D229" t="s">
         <v>33</v>
       </c>
+      <c r="E229" t="s">
+        <v>278</v>
+      </c>
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A230">

</xml_diff>

<commit_message>
Corrected 2027 meeting date
</commit_message>
<xml_diff>
--- a/fomcCommunication_master.xlsx
+++ b/fomcCommunication_master.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11027"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranlephu/Documents/github/fomc-communication/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E96684F-2950-2F4B-ADA6-9FECF99D4573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{842572AC-0255-8B45-B01E-FD693E6F893E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9538,7 +9538,7 @@
         <v>2027</v>
       </c>
       <c r="B234" s="6">
-        <v>46182</v>
+        <v>46547</v>
       </c>
       <c r="C234" s="3">
         <v>0.54166666666666663</v>

</xml_diff>